<commit_message>
update readme & ajustes dash
</commit_message>
<xml_diff>
--- a/SQL para análise de dados - Material de apoio/Exercícios/09-Projeto1-Dashboard de vendas/Projeto+1+-+Dashboard+de+vendas.xlsx
+++ b/SQL para análise de dados - Material de apoio/Exercícios/09-Projeto1-Dashboard de vendas/Projeto+1+-+Dashboard+de+vendas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Área de Trabalho\sql\SQL para análise de dados - Material de apoio\Exercícios\09-Projeto1-Dashboard de vendas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0670B2-D012-4F35-AD44-339AF5DC0461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0906A52E-A898-4946-8F8B-D8E26C01AD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,42 +17,13 @@
     <sheet name="Resultados" sheetId="3" r:id="rId2"/>
     <sheet name="Queries" sheetId="4" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$M$3:$N$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Resultados!$S$3:$U$10</definedName>
     <definedName name="_xlchart.v5.0" hidden="1">Resultados!$I$3:$J$3</definedName>
-    <definedName name="_xlchart.v5.1" hidden="1">Resultados!$I$3:$K$3</definedName>
-    <definedName name="_xlchart.v5.10" hidden="1">Resultados!$I$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.11" hidden="1">Resultados!$J$3</definedName>
-    <definedName name="_xlchart.v5.12" hidden="1">Resultados!$J$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.13" hidden="1">Resultados!$K$2</definedName>
-    <definedName name="_xlchart.v5.14" hidden="1">Resultados!$K$3</definedName>
-    <definedName name="_xlchart.v5.15" hidden="1">Resultados!$K$4:$K$8</definedName>
-    <definedName name="_xlchart.v5.16" hidden="1">[1]Resultados!$I$3:$J$3</definedName>
-    <definedName name="_xlchart.v5.17" hidden="1">[1]Resultados!$I$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.18" hidden="1">[1]Resultados!$K$3</definedName>
-    <definedName name="_xlchart.v5.19" hidden="1">[1]Resultados!$K$4:$K$8</definedName>
-    <definedName name="_xlchart.v5.2" hidden="1">Resultados!$I$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.20" hidden="1">Resultados!$I$3:$J$3</definedName>
-    <definedName name="_xlchart.v5.21" hidden="1">Resultados!$I$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.22" hidden="1">Resultados!$K$2</definedName>
-    <definedName name="_xlchart.v5.23" hidden="1">Resultados!$K$3</definedName>
-    <definedName name="_xlchart.v5.24" hidden="1">Resultados!$K$4:$K$8</definedName>
-    <definedName name="_xlchart.v5.25" hidden="1">Resultados!$I$3:$J$3</definedName>
-    <definedName name="_xlchart.v5.26" hidden="1">Resultados!$I$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.27" hidden="1">Resultados!$K$2</definedName>
-    <definedName name="_xlchart.v5.28" hidden="1">Resultados!$K$3</definedName>
-    <definedName name="_xlchart.v5.29" hidden="1">Resultados!$K$4:$K$8</definedName>
-    <definedName name="_xlchart.v5.3" hidden="1">Resultados!$J$3</definedName>
-    <definedName name="_xlchart.v5.4" hidden="1">Resultados!$J$4:$J$8</definedName>
-    <definedName name="_xlchart.v5.5" hidden="1">Resultados!$K$2</definedName>
-    <definedName name="_xlchart.v5.6" hidden="1">Resultados!$K$3</definedName>
-    <definedName name="_xlchart.v5.7" hidden="1">Resultados!$K$4:$K$8</definedName>
-    <definedName name="_xlchart.v5.8" hidden="1">Resultados!$I$3:$J$3</definedName>
-    <definedName name="_xlchart.v5.9" hidden="1">Resultados!$I$3:$K$3</definedName>
+    <definedName name="_xlchart.v5.1" hidden="1">Resultados!$I$4:$J$8</definedName>
+    <definedName name="_xlchart.v5.2" hidden="1">Resultados!$K$3</definedName>
+    <definedName name="_xlchart.v5.3" hidden="1">Resultados!$K$4:$K$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -131,9 +102,6 @@
     <t>5 - Dias da semana com maior número de visitas ao site</t>
   </si>
   <si>
-    <t>Brasil</t>
-  </si>
-  <si>
     <t>SP</t>
   </si>
   <si>
@@ -198,6 +166,9 @@
   </si>
   <si>
     <t>Domingo</t>
+  </si>
+  <si>
+    <t>Brazil</t>
   </si>
 </sst>
 </file>
@@ -2821,11 +2792,11 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v5.2</cx:f>
+        <cx:f>_xlchart.v5.1</cx:f>
         <cx:nf>_xlchart.v5.0</cx:nf>
       </cx:strDim>
       <cx:numDim type="colorVal">
-        <cx:f>_xlchart.v5.7</cx:f>
+        <cx:f>_xlchart.v5.3</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2871,7 +2842,7 @@
         <cx:series layoutId="regionMap" uniqueId="{00000001-8848-41A7-9E79-20C89709F016}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v5.6</cx:f>
+              <cx:f>_xlchart.v5.2</cx:f>
               <cx:v>vendas (#)</cx:v>
             </cx:txData>
           </cx:tx>
@@ -2882,2185 +2853,2221 @@
           <cx:layoutPr>
             <cx:geography cultureLanguage="pt-BR" cultureRegion="BR" attribution="Da plataforma Bing">
               <cx:geoCache provider="{E9337A44-BEBE-4D9F-B70C-5C5E7DAFC167}">
-                <cx:binary>3HxZc9zGsuZfUfh5INe+3LjnRkwB3c3mJoraLL8gaIlGFdYq7MCvn2x5OWSrzR7dh4m4owhbJtHo
-rNwzv8zyf36Z/+NL+fjQvpqrsu7+48v8r59s3/v/+Pnn7ot9rB6615X70jZd83v/+ktT/dz8/rv7
-8vjz1/ZhcnX2M0GY/fzFPrT94/zTf/0nfFv22Fw3Xx5619Rvh8d2uX/shrLvXnh28tGrL81Q94fX
-M/imf/1k2ofOlT+9evhauTpxXd+6Lz3+10/373569Vj3rl/eL/7xXz89e/7Tq5+Pv/y7g7wq4az9
-8BXejSh6jajmRKufXpVNnf31e45fEyw0hYfo2x/yF9HbhwpevHfNq137UH99fPW1efVugHP+85m+
-nejh69f2seuAnW9/n/yKZ6z8wek/CMV1TfyHuOLmwIi5/8b5z8/V8V//efQLkMXRb55o7Fhw5x79
-Xyvs8iXh/KDCCHmtkVIIYaL/+PNccYy+xlpIqskfekP0L+L/Vhwo7fKhfnRt89ezU5b0z1p7+v6x
-yoDX/4Eqe2q7z47/o/6E0Wv67Q8Ch3nmUPT1HxqR4qRD/eXt/3yS0/r4671np/538Pif5Cfv4pfM
-8eAn/+9992Z37kzPI86LwRbr1xorwSCD/GED+LmNgO9qygV8hv7x/Mh3b1z90L3aPbYPrnvpWKct
-5fnbR3574PP/BxO6e0ku50zon83rb7UmD/3D5lvyfZIdXn76V1o5evWFfPnno/3Xf/0kmH4Sgg5f
-8efDP6L5//7SPv7F8d8ff3zoekjtQrwWWGuGJcaMcKnA2qbHb48kGBrYGGFcSyykFkCkbtrewmvy
-NcYUccgtknPFNYXKoGuGb88wfo2ZpFAXKCYFF4T/XQHdNeWSNfXfovjz51f1UN01ru67f/0kJZzA
-//G5b4elXBEsuVYSDsg0UUDKf3m4hzILPo7/VzbLvtBThpIuH0P5gBZcJlMbap54QsfGFHxYRlMM
-Mk+8Zz5Oc+dudGeLy2bU/V2hi/BLGir5xq9qNr6i0TumS2eGppxKM+ssd8k6Dx2K12Kat5kv04vQ
-+tHUNOrfcj2LjWe6YDssxyR1476zfVubJorCJ78u/hfdyKxOShqQiHFZKSNLVn5Vi+CPs2X9bT9F
-WWumGdtLGfpit7I0vSvlsubx5Dtxw3AhjbdIyrjh62SEYMW2nFYVt6vON6Qclp3vV2+iRVSXDRvG
-/hoVI7me8qF9O7nFxnWZF5c9puJ3PtajiwNL9Zu84MWuK3FrDQmkvM6XiO3LKGR7jqcPhErUGUar
-9BPxKr1uB5Fdylzq6zpr37s+dxs0BnpZNIXBrOovonV1d+u8FJd+wfY+FOVdZrti42mb3frRkRvm
-xu5TGtb6YlZO7peooZmZEc0+drxOXbwoThMp+mjXzwV67/uCp6bQ6uOUjz5Zp8VvGGuKC0LKsJmb
-KKOmG3i6kfWYKcPnajH10GSdieaexG6wy40X9bqRqsnjsIzrfqgzval4ke+DxffjUl7yvP7Ua2wU
-ze9yNTiTySmNSeEHg+sexysTfeIWrmJGcL5bHEpjl0HSNtns5y2okpgV0fIy62t7tVYoxKp1tdHE
-hS0JK0pYIUKyBNFt+z5qE656uhVzNMetbMjeFq7+bVVk2Kxl4CimNl+NWOZ6NGymZSwCTd/Unt3j
-2lGjWGPmisdt1rF4zXy4X1qUbdcCzffRmsqLSfZLTGfgtxBlfiudGjeDpuItUGjuo4HMSdHhbEu1
-HTdV76uLfCyYCWpskhGMq39bzXxSW6J4MNx1hTC5tOXItxGtiuUyHXCf/1rxXndsM06Tdvw260gq
-VpO1Na8uqiBtt8TM6oKybREypyaTE2zHKGFrsA2+8TiKytnMpKat6I2ty2Lq7xc3Lqu7EsUwF/gu
-F67eTyJkCe2KJvFtaIz3y/ioOg1flBVs21adu8qWsfkq7Bo+pJWYE1Qsy77Vi/ulyrO8MhNH+m7k
-aRV3LQjLhjGrTLC22wxKNfdll/vtzApqzbCk9AK3k7geyrLIDcUh+rwqP1xlJeljMdPqrpxJeYs4
-Lj6XqdS7Ok39bzXxetf6VN6soVtRzEla7GxD7f06Z2E03BfWmRC67P04sepKrK0m29EqCFLTPAaj
-+kGQGKg3m4IN4lb51L6bpyFcdKLVwL5ftzYrcSJLXUdJWat6s+aMX+bjIi5IlPZ3UyppZTL9nqo2
-XBPry8rkVuncpO0QPnNUFvdK4z6WgRdmVj35yqVbPi5FqbCJbBeuGcVv15raTTWAwwiZk3cLH6p7
-2a3yWg6o2TiX0ztEB/pJNmvNTYkqejGRmk+XeG6HzBTUgxzrzrLfLcHkfetl9mYi5UrjLq/dpzmK
-ujs76WE2rMfyHWLOJmPlWghcmecfa9vsmjb4OZHEVjuSz3mCIzrVxka53nmpVrOsFW0M43wcTEZy
-EW0aFHW3VloLEbMs3s59NRq0NlabJltQZpYocnFWM1skaZGub8I4kCZhQS+xgy49M1ZO7tcsTcPl
-3NezMFnj0IXN5jXu6lLAz3nP3pO00w9V7cZ0Szjtb1C68Hf5MrsLvCJ0p8tQvlutppdudOxhajV+
-W0nFb+auJDG2i1zN3PU0mWUtfw8IjmOixo93y8DJRuSuuClwF/3iIsLDzs2RvJ0oX7aMzuMeYhEt
-IdAtw1Yuons74zAbpGZ+5cBWvjRBtLt50SgkcFRhaju4Kk9Y5+kejX5IWNl7IygdTUfkb0j0ahcy
-NHdmdraHj4xuSAZIlUmEvTZENDZhkvmLPOJT0o2i/yKmIbvGkC3NHKi6rdM6nwzONbrFlVovx5JP
-b6Uuyt7MUdptbZr3cZNSbFjWV/eRxt1mdigbTOvcsO9JEd31WOVj3BLqH5FGzcXc2eVzitrqJlDI
-0rGfMnVT1Ly+6Zd62vaFd3msKyVmU6Z9/2EsV2cNV0ztJ9uVn9IBsiPvceHNEEm+W1Tt7pe1QXej
-kH43YFtsVCTaWwg9/gr5ck6ioisN0nXeRUkr8lV+0UuPxb61Qj1YOUCCtym6nYQEqVZFiZZEa1Qn
-fdSxh6Ghw64qc5/oVGa3c26jG77oNkbe9zYJuq6/VkM5f2Tg1DtrIanFeSbTz1PRpbuqWm8GL6qL
-uapjOuG4SoMzDam6KlYjuwyIvNEF14mf5s+dTbvLAjP6UeqxaMzQKfwJI2zjCbLwL2j26Ld6ZmSz
-4mL4AFEv3BYuVXuvsvWOBOmNtYuPsaw+YJHfBuyzpJs1v/IcFTdV6/tt5+hFWUfvnIrmpBezG7al
-rS+rcjKpE/hmWEifzGTotyxjFo4A8kxykXZXyIpql8kQdpLXZVIVM7rpJu5MF6omCU6JPfgwMikl
-9iJHrbh0jJVxgV34pDjGcYs429QCL9dtMTWXI1JdTHGf7uYuyi8citJtihF/53KhN5CmdLwIut5N
-BV7e+FzbT9Xk/a0ep/odztd6x3XZ7XBh821V4yWZRFpshzwVl0vejG+Elu6Wq9FgLIYt+Fk7xLnN
-TY7pe0fxJkB5sKjCmra2N01fX6rKblyxbnkaknFSF3WvjUWjGdtfPX3ERS/e+FHp1Qykngczlc20
-W6UYvHEVTd9iVGSfuhrtFrl0yYTJ46A4+dywerpNxQzlDl5H2wxGNhGaomuWsgLfVGB4c9IG4ta4
-Kh+1DPqRpkOIMevDmtSohxeyFt32unFxVBBuTSH7a+I78MshtO/LzrNkUpktTLNaMZopTe3DOPp1
-X/GGmyyAJybD4iuDU/Spado0YY1bTSDDtM1QPpg1n20EpSqZjF8x3pBijn5DTdHFgc5hk3bltMGV
-Q1sIAaUZu5ncZdJtG5I6k86Qe6N8KX7pUNVvoqxwxrPUXUKBOv06DWjcts1AYo4E32RuqL/2SKYX
-rurX2zobRezTJUtwUYlNNHU0sTUfkmhZPJRxrtM3bbFm2x5VzVuFFFSvY17sylS7SxZl3YW1RN/r
-cVl2LZjrXswrlIVsSFwm5kvRljQWWSGSmQ5iJxYaXSJWtvCREpsxZ1MyzJgkrnKZ4U2WmzBqfBUa
-/Es0ivelzD5F2bImXh/qTF+QmKTRFR0mYbBY3qZ0CnGAqGLmdq1Mats1CRFe7ruQZUb3uU2cq6PN
-NDbFtor8x3Wq06TMQKN1LUFneUtN6cZHSlu76UJwiWPTTZTJKz92+YYSNcVQU2UQDLs3jEJ9Jl2a
-G76KW/CVWyS7PXUTN8p2WdzztTY9g6zWcvdbrgcIyVNHtrmHT/syGKw8+twX1aN31Qfh9ZsFh+Yi
-ZOUS46oKJm/knHhUMpPWxQC/GxNeungVBb1MswV6lbwZPqMubR4HPMy50V2EL7qIibgs8RLLHOUb
-XUNSqFr2a+91c9WVWbWlUS23VAa1y/u8vK+zbI6XDrUbnvfvB5a5W1rNYRsatpORaky1VAM8m4a4
-Y/LarSk3Y49/ITSbjFYqh6Bcf1jbcd+2YPK5IMkSLZ0py7RIQh9s3KXuotFDEadYl7GSIDdM0qu+
-5Oq+9HO2DbyvN1GUt/u54PXl0lu9dxq6LQ9ZZddTspjeluxytSXa5n09bqZ6buKxjzCYe7cYIov+
-nRBNu49KZQabTzvfKqjD7XCnKvmxyXER82EtNplIjerKJMO/L93ew3tmluX4flh3CtU48Vk5XnmZ
-9xtKo8p4cZd3ftywtZ0vsn6N+8HtBbue2mqF71LTFlW/RyozaLgt1jlcQtYdL+p2Lt/pNbd7xgTa
-T3rNRlPNuIM0D4VdzFJF9k/h8Ge9+ZfGL63L7J8Dir9//K+bv6Ye32C2f//+MOL4909vxse2H9rH
-VzcPvnu1Bf/+Nvg4fucApfz9EoACf0IrBwDj2Q/fYSn/gJb8MVP5h4fPoJRnKNZTbIQCIvv3cOQ7
-JOUvHPUP/PUATxw+/yeUQtTrA+DBlCBIQFY74CXnoRT+mgjNJRgxwPEIOnT5bySF0tcSciRGSAqN
-GNHyR5AU/gxH4QDzUAV4DWAzhGLF9AFneYKj0Circ5K1iwFXgBi5wryr3Q1DzZrLbAW/3D6RzAng
-5ntyjFGFgRShDGMCfD0l5yOZDgXEJoOLbuFf57LAkEcABojYu4zpdv3yMj32HXuMIyYVcAhlIT/I
-8Sk95OqiXUoonUOE6vseAKr3wYkcIM2/9X2Cq+dUBFUguAMeJQQRUiJ5eP5EiOO66gwNdWcUicZk
-6f0YS8r6zctUxDNe/qRCCXw9VpoQcgR5NWnnU0WrDqJyrjfpEHEoWObyV+haQuIKHd2+TO97rjgC
-K0MKQGcoqSVAyk+5KvEKANysWjO0mm2ho5+3gAlg8+NUKJcSQEbwEY6OuMKDcnmL0tbkzJJPyIVq
-3/t5TV6m8r3s+GFYySVYO9iBAi98yksbSmR7qVszF8zK2OoZyq+i5XwwjV6azuAw2fcv03xu6wd9
-cahROYFqBByWHMY6T2nqmgZfjUtrmlCTSxQFnoxdkd+gQYkz7J0gBSEGHEpzKok4Ng3iK9RUQwGk
-ytGbUdfr1rvBQwtelTB2e8nWT0gSkGXGiAQxSghBz7nigK2pqK5aM7ou3w9QoV8IiBPXrKH6zdQ2
-8uJleies8Ck9iZ7TW/pmbcQI9Noar/6iwqmPNvko3Bk6p0TICdaYA54MYfrIDlMoaBfXAP4Fbb0d
-4zxf8yXp3bD+SrMxnCF2SohcCgXzWIoUV4fnTwKGDq1QXb4Eky2kSIaxJbdWiDTmTC2JmBWLXxbi
-SeYUlYKAn3Ehjlx5ZEOqekeg9CsHZrjOycb1RJrMrdkZfz5FSiBGJXgz5pIcJRQccV5EMwoGMMoy
-6Ukpbrt8JUZXACC/zNUheD+dAYCDiaekjhxsXKVvOwxc8bV5Y63MdqpYwkeJKdRJrAgfWzX88jLJ
-U9b4lOR3gnTRDF0oCNIiKKfalG9h/SI7484nqWAmlODsMFA5ssVOe+ggItsa7/RwVzTQAUWqpm/+
-G7yAsYMzCwZDniPPSnnKgoU20zRd5QzAx2LrxkacyY2nTF0oyqD6wVoCVvLc1FvovVsXRDBRC4h0
-rHRZXJaiSn+vfGffa4hX/RnnOmmBSkA41PCNjB1RzCNbtk7QAD2QFLtyHD5zxn6DYYfc/LgAJWKI
-HDKXIvJwkCdeLDiy2cQhZNg0kvFUdQpgN9yfcSh8POpSSkBgZ4pqIQ6J5Cji2ki5oeR1awKFNrGr
-6RTz1eYb7322q6eGQrPAd2laFDvKYawEvWsNnTxi9kwU+d4sBbiOQIRw/K0cec6vdhXghiNkGZiR
-lOJt3THb7S0dqu6MBvHBjZ57NlASUOsQqjjHx6XH3GXK4rlpjXUwsUMlGbchePq+GdubTETzZdv5
-ZtMWDTYU6Mcwf7Ix6KDHvd4PSxTOlELfRxoYhsIsFApuwhCnR24/LVAfReMcjEdqombKdCUM6aeM
-JhPKCOA+7Sjuu6Gv5jPa/17mQJnA5F8pTb8vjxZC52rAkClm2sDor8mLeKVDfUazJ/l7QuXIxJbR
-Q6cYIGhPFo/JAMOPeApptKsYYOn6c5NP4YdDHPAFCgbBCYmRPordSk41hYoyGLqoNo70zOKR9fUZ
-6X0ffICKgJUIJSiG9usoz9aASxWd7IMpMi3uG7WEDS26fIeGMv+td+26fTkinJIjmOxhT4eDnxxH
-hLRoVldyyEgin5hPxqCiK5KiLFaq6m7IuGhAVDOoAs/weY7uEZ9iyOYAsEkwZVW3V/nUNHtvh/Um
-H6L2CsBHFqMix2fC3ynhHqpNBKt+XDJ6FP5mr6pQtjUI12H+Sx8N87Ahesx3U60R4M911H96WbyH
-b3weFvSh86UUWiBIi8e14ADAT827LJgx7epEhNAmtMpHE9Xzj5edUEpDBSMoR4BH8iOPKNgKc3/B
-vFmmodygYgXguOc/XkxrftiygCZfkQM68Dyi1kvXNIwsMAuTftrRglWmyOVbFAoYtbXojHWeiCXP
-qB2s6Em+mjIiullAtEKuTHFMHQBicUradTljGYf65EhPUnKJDtbBAL84ql/Aj11pLewmlCPqLq2K
-ql1TV+iyqbjaeCnG9/MURQUAfJOdftwVYO8UYBGor6Ehp0dMymJWa9FD9l+jXr+D6Tp5gxEZYg9D
-tn3TijWHrYqUn+H4hGUe1iYhQxApwG6OEgT0JKKneIJSFKeD8VSXxuPcGofG6Mdjtf7WK2OofjWk
-x+daVL5bOgZLADDCbcYrMYRhX9Gew4hFk4s+lb01ZeiGM2I9oVKAOAB3gEIEhhXkYFtPbKe1gayw
-Cg3xGgbXGYDVTiWTa7pLDjOx25k1uamVhjEBzELPkP7ObA9JVzBKYNUHUgY/0ihPp9qHABEly5U3
-BNV0C1jMePODsQWoAPqgDz0ZlFvHsaVNZ9pOK9js6nrcwOQ1XxNoccsL6mV9/TKtUxxBdIHyE/aX
-YAZ/VKEWzDHHPQxoC13P3oQhWn8dI1LKM6bynVUeeGKUgsoAGRDHQcytuVcTgrEUbC8sSecXdoXK
-odoHWGw6E1tOkZKH7UQqDolWHsXLfkrrpqkqIBVgRAKwR5TAGtRn26DlTHF4SnhQC4ELYNjjwPIo
-uIRKWTcT703LkNu0EdS6drJh88MqOqQZSI0gPFiyOmpju0xaDeMyCGF8hcG76KwJTaV+XEFQUB/w
-PKChyDH6uuDMkxzmKLCyAkshHgLVpplV/jYN2fr5ZYZOKIgCSskZZBzAovlRhJKkChZGct6wMKQw
-Wu+7uKBjHgMkcvUypRMKekbp8PxJqKibJaTrknujxfhRyZpuapL6M/Z2yIzPUoyGogM6Soh/EHcB
-S35OBPczjJpx1MD8rUHXIZ/Du4pOzV5nnK2mmeZ59zJXmJyiiAnRlDEMVI8sfA1lXk4BKLJMgwAD
-DMPnuobZkh5JaSxP7UU9j9lmcRy2hFAgv0dLdAk7bn5r6VTcv3ycU0IGRQoOUDrCgN0/5z+ry2pQ
-KVgOrAesSeSjfAMQweOPE5Gwq8kkh+4TIslzIiJMq+s8h+0z1xLY1JtyWIvrkPbijB+c0qbUDGAj
-oiF+6IPxPjEZmH/XiC5gnHVezzCbp8LAYHyLOYy0+mg5Q+2U7JSA0YeSDO47HJcIw9yJuRobb2TP
-06tiXMLeQxRNflx4CgAPBjUQ1JHHwLYsZUuXDCJi3lXtdTPYagOjf3cGjj3BC4gNmiiIiKCoY8kV
-dRMV2tlDnSrtbTlpFmPH7Y9CRTBoQoBAQNiA3kbRg/6e6EetY9RHB9svHK1uqmUmiU9rdSbmfo90
-HMjAIIpLmKVA53Zg9gmZSqwNR5VsTD6k7jpaFN3iUF42E9dGoPFWTfzeRyjdBCvTK8C7L4X2/kx+
-OZQTR5EF/BvDnjIHtEUdFwJrQIPusxIKATESvOln29V3bOZovObDNNF4nmBReN+OmpyDaU+4AXQD
-MPQjVHAos47cIGosR0OlG7NUOS1iiwTssnh3TWGjIR66FP79wzYKyYcABk0pjMiOs/ZA5FytCKII
-s7CvCEsX7VZW6zlPOBz7uUQxqBQQMrCgb3cUnqsVMOdsbiWoVViXxaWSzX6pV7mHdWR7xoS+lyCQ
-UhTKROg/CDpuqCBWCtRykGBTcBclS1MGBZuBFn/QHeVf7VRN6Rk/P8T9Y+7A8w5II4QvBuPYZ0Zr
-i8Bh5xMWFH1dwZKqDvxjGKb1tzDIMsG4Jr8BDDJfeUubi6ol3a8vq/B7c8UUABQCnQ5UkhDVnpOv
-6oCycRoag8o2S0ohv5at/JXXAFDBPlplBnauqvw+5BwoQtMK0zRAWemRl3aTyx2BjRFTRwSa1jAM
-F+Aq9RlNftdwaMwY4LfgCOSQe47KPJL3lLOmb0ybR+0aw2af+yWsS8US2Ltld6EYV2cKZQEzkmUJ
-y8cvi/WEzcIeEpSzUAMCenQ8qG5X2NCoJVwkiMo0bHlWLH2sU2zfN11L8zPETgQ+GJVAqywFbPRB
-9DtilpKoYFOPwPFFdwdxsXiPU10kI2thBZh1lr8raAWt8pxOXb8laZpKE3Vd+GBbVvsz/dYJycM8
-FpYBFJTXh4sezy2KlHCfdA0TBPtgwV3Hof9tElDP12jWplzS4qZTH3HI7A+nMhACjNEBOYPFAC6O
-7ApVuuTBgyXzhZVN3GcpXXd6xK47I+5Tuj1cHNGAJAGUzQ7Pn6aZus5TWHFoTNYN6YdxyancLFjD
-YpBjgzxTN54ipgG2AgRSI/jnSJo9I8RGPWxwwp0CdOlxM9xOtYySUTTT+5dt9kTwEwcSCAaKEoZ9
-9DlfOGV8kTXwBRc20q95j5cPqpfjrqjL8gIGmvbTy/ROsAYYPay3wGUfomBV4Dm9kkWuGpYG4noj
-VRJZGGC2LSz8NvDOj6tMwcgZUiKwBmjxkW04Ufms6/PG6IW1GVySGIYUxn413WNSAxb4MmMnYqqC
-moodohw6AI7PGcvnWpTZENUG1uHyOG1sl5sowOAvTlVHvvZLO6JdgFxzpnM6RRfgRiBJvy2THNnK
-0E+4hBs4QHeqAcGZB8duyQKDxrZ29sPUsOZajTY6U9ydUCMsKEAJIKH4gv84codRjnCRJ8og1PWA
-EqQ1eLkvQhNL2YkzoeWEhSqIcxw2gAA1hotkzwW70mmQ41Q1Ju3WNS6HlewWMaqLoU3zZKqz6AzQ
-coo1aKsP45PDvTR1xFqYZBZmBXuZTcfEnkQrSaqMN/ercuUZCz1Y4FEZoKCKglmDhL0tSJDPWWMi
-kD5b0tqgzJW3rAX4CO5r2O3LlnmSCuRdTjhMA/W3RPIkdKHKw3osh2gScrgNFVKkrmxkpx/GwjAM
-HQGRUADiciIPrfATKp2F0ZtYPFAp+Sxj2GwrlwsGN8XgShNXKJwJkaesAhCqQx8DRQU73DZ8Sg6h
-VbSDg7gV9f27sV/fVk2AC29QTxkZ8nBGUaeoHe7BwwoVwMTQ1z2n5usuF9SDc7dLyC5r19JtV2Ry
-j+bZX63TOpzh7oTKICIDEq2RBJr8KEoWksA+P2yfmWn0cL9stYiMSdbg9FwVccLYgcQBGAOMliF9
-OMgTrc2eYds78ON5HGWVVLA7kMiiUc44l7bvXjbEE1IEIcJoEpYUtIbx9HNi6Yznus9UbYS2vE7g
-OOFL3TK4updGAOQC8s/sj0dHyNiAlkJNAtPh47S9NqqaLdwfM/no0riIsoQd1s7hMmC0YWkLd8tm
-PCUvs3lKplBU8wMEfcCZDmJ4IlPb55GvIgY1ZldeEpgmbsoKri8WjJwD2M9ROuSGJ5SEh7Uw2Aqq
-jR96uE4KobovN/VSjD52hQdVvszYiVSj5WEweqhNIKccMVb1rSpth2FRfF773brw6G4VqU4C78Im
-mvUCt1Jd+um/QVQcwgq4A3RLR0TbSk/YKVqbbgIhOlgF+VAt4oMVdbtFItDtBPfIztA80Z5B4Ieq
-Gu51wdoCO5Jrp9amyylczYVOCZsMLrhoP5efltTm8L9wodWvvEJwPzNC7Z5Mc3Um2HxfSx+mQhBC
-oaKGu9LHzo8YrNLTEm6GDnLGb+G6yGJK22YPURqGm1VF6aZLQ3cT+e5M5jv43/N0dDBX8BSoowFQ
-+D+cfdlu3TjT7RMR0EANvJW0B0/xEMexc0M4kyRKpCaKIvn0/9p9zkV7O4jR30UDDXTS3JLIYlWt
-oc6vI6UpazX6kwWH4PIWkEa9E7GI7v/+Qd9HAVSdGfqQoJWhj3Z+v5pMrW0bQRuEhLr5VvvGNJWG
-P47aU26Hb3pN6te/r/j+hZ7qXLTUICKPAMuexZ1GS9JAMAZxgG7lVkytSu4Y+PV1MQNW2ScxRIqZ
-qiHW4SMXH7EW/rT6P1l8mNDslGe/PaSGDEEbUqShwTg2fZURHEz07odmK9nWt2HRKu63arTB2B3R
-LA5//f3p3weJGHcICOGAJeIIndK366dAJJAmI0hEtouhWYhfu5Fuh6jJ8/1/XgktUnSGAOX802B/
-uxJqh4j5Hrek4ixTlfL55grWAdPfpyZxzQfh6P0pjbGPQJg90d0QGM5e7CJIJ6xecJ1A5f0TF0jV
-baKDGIijA6fVcKilm17GDao+4WL69PeHfX9YsDpa6TmS7yxEQ+zsYdcUAuQFq4M5Jq7CMQ0KKMSj
-/3wkT6vkAPqB9oBiepYI4ITkYGlD2YrWNrsUjn4yuSUX/8Oj5NHp1IPtyc55NQu4fgSsNLzIzY93
-IKVzBxA6MB9xwf5w8tHcjtCqzBiog+dwEvDTRG5qhSA+oEnFJnDqWShryLAze5nnmvznlBR86uAE
-dmSQLLxjhC115Ibp9Img1ol3vcn7Twn6XjtZW3r391f4p70I5mXw/xqW/5hf/PsmlqINUG853PnZ
-tlwEYqIlmgmyitzWX4zLHFxOwNvvk1mML9Agjx8chT/EGKRxeKXoOoEQf84NTvrOgPqB5JvbmkTF
-hI7iHc37DH1Mm82PUUQSCMxpOz3StnbzBw//Pi9AhgWtxAk2zimMOt4ehYH4EZByD1wNMtoXfIwW
-4uIIh7FcoUdfQHXsuoea2OR/CDhYGPwCfGSEnfPev25biOUMigCI0ZaS4BdemNw3z2G2dh/krmfH
-HSePgdETZigAEMOR2b19Rm4aJRl1bRVsS1KF+Uk7OhjxQQQ9b+r9/2Xgg4IuIg79ea0GKxgZtHHc
-VgIYhWb9Wpnan7TrgpRTugSfgCeqyy4md9xyu5+Adt7zVf/H7fzuZ5wFNzoGm0ZyC0nhPMvCJtl8
-QGK4HYZMxlXH/G5IY13gNKPxBjLj7u+H6ezG+md1EPzAWAnRSUUH5+27nod2aEW2tlVe1+tlMqVu
-B0242Q+t+Qhm+NNn/fdSp3P97wzax5lLpGmrlbF2p+M+ryK7DB981rPA988DsVNjOEc2h8Ln7IAQ
-03RJ00LRyds52y4DsGB5ubixmy9iB3X852zU/D9mc6dFwaTHaYSYKUA6e5bExo5OczKwutp4U98k
-oDdVp87VB8nqHx4tQz8vggwCepzsPFVeIRbhBA2milmXy6s17OPuqGOZRUfowhZogLIREf/vG+Qs
-4PzzaIAuT0wtrI1i5O1XG3jGm9bRtpI2EBwA8LhCAJ35ZQvnorOZZaXOG7Md6nUC2v73xd9tGeD5
-2PvgRYBsj1h7diXPRmeUcEXLZNL1MZi5K1MQXz9Y5Syi0xRd9CBCGgWYNgYWfLbK2rcQsAxRCAmv
-q03p4n64FZNlOwJHmN3icFtLNap9HPn6g3D+7vhh6RzgM/hwEeAUehbqmBgC3gkZl2EwNOFdlIxm
-emq1jggtwHFZ9Ado1J/Ww7nAnY9cDnT1szPYeNpDGT3C2qSjpjjZFVXQF/YnCexc/f3b/WEp9O4Z
-WvggOOEcnj3aCEXX3IFSU3JUHTs+KQ9xt04Q0qb5gw94lhGcPiBYEIDY8U+W4HJ6u0cFvHxCu254
-qiUYrhquxgPhXpYRyeoHbYDx820VpZA2voaFx/bBR3x3Lk/LAxpBUgfmDnbq2+Ujwhhy4CYqsUnz
-A/E6Kmg6ozEdkBj5wRB8UNW9PxUxMiy8Vmwe5Ivh2Ucca9txwRHWor6jx66H7HmCa8gHL/X9U71Z
-JTo7FR2LGZm6mJdA9LOyztOh7C2Yd2HD7o2Jkw/izJ+WQ3f2RM6GkALP9/YlJgq9UxhT1BWCWKDE
-fqSza5uySfq4X4tcURepndN9S/d/36d/epsxlICgwYJAiQbW24UbtBrB4Y9IGedD+gLnp+dpWP4j
-HQgfCbJakKLR0QEChBP/dpF+cD0MTAJaOjzOC7xVVAUUY/ygA/f+USCACFJ04FDJIBc/e4fCGF5v
-gokqioD6JHk77Ejbhhf/9YVhlVOPCJAoGlPnralliLdmzAmM22iEzAyS130bLB/th/fhI0VIRIkL
-iSYQ1/T03/+VLaBVz108wUSAGDfALCXA9baF4mg5wPq/P9C7K+7EaEJOFaN4gVjo/Iqbh5PKtm1h
-SgCp2A/frfIxSWoYHYjEVks+kMsaTdQP9vufng9MiBj4LWgBkL6+fb7Z4wXXE96iaBt4knFQ2ZdI
-ZTDrCbcPTvKflsKJwv2CegV9kbNtkfSNaSH9AoLjY307NoMsB5OHL7DYMv/5MJ3Ue+AgoaN+auud
-7fPAT60b17yDR44fDmzpf89x+hH14P33wn44GW2ixXTaI2fxdonh8EKhbMUGzNyXdfC+8oQ219C9
-LjcBjLZulCfzR9jY+8P1dtWzOMFTN0CyxdsqDo0/mrHVh2Ex0fHve/F9LgJQEx00XJuQoAPffLst
-EuvabiIoSghs7+5kt8JeK7OqlHSMrsJGcFm0G0zRaKP569+X/tMD4hJDZRshBwLR+u3S1i8jIdai
-Hkph2pauUXfd6eCjTtIfV0FTG+g+ur2Qkb1dJRErGE88aeEnZsw+HuG4Ek7hR33d91seNQ0CYXyy
-aAAWd1ZUDVkAoyHdiCpYPV8PAywbo70XcyePk4y0/iAknrb1v7q5eAwsB0EKnBpQRaGafPtQBlZm
-0+SpqLif6KHuJn+vkravxHzqVbHVsA+2yR+OALp+oOCc+uZIj8++VaMpJSbbRJVnyDa0DoFZZWTI
-jyhU9N6AV35tsmWRu79vkT+8VsRjkG6waoo78+zjaXJKviYj4JKSZ/tECX/BYRSUFAOK+Y9E8394
-qUj+U0ByOHioqs5eKlOBy1g9iWrRuoapC3gOMAnKwAYq2xRWoccO5kjyP4flk/sp2li44OBHce5b
-SrNtW5Z1lZUCGFqit8Qf003HRx8P5sffX+YfTgKAKxxzNIoB554zqPSaAQVojKzAo89KE5qk7D37
-+b8sgk40+hyQgp2XwwF8xcDn07ICAXrbNSoIKgXbmQ9u0Hf7Au0TXGPA/dCzORFd3+5/i+IN4KIY
-KmjLp/sebfcqWObt0Lgw/fr3B3oXILHfkxMghiwRcp5zdpua1XwiV0+VGJL4kYOZxS9a7yByrQY+
-B6zCzb3lTUm3ceq+iQ0+mx9sEUCo7z4d6idQJZEgn5ggENO/fV6Ucx1En920c3Brgw6c+LiP+jv4
-3y11V6aSLhJ+oa30PSugn1wEPO1yGaRdGQK649OOtUEow88wTnTNa9uBi0Evtj4fyVMDM8JRf+Wu
-E0ocM2IW8lNJQXheEticElG0nVGd2AVw1+Vx2ThlpqDSBnCvOGgm5vjR2JGRoUybZjv9eRhxxi9w
-AJX6d6iDcfvqI5/Gn2aZzfLn1FG9ltHq2nAnyNBOJ981LeTlOor2MshEKgCOwdby2TZKAyBXaz2L
-bB/RVq2lCzuzsQIIWz7fBP3JLUHETZ8/ob0T0au0Nkvwky3QPn2BV18TCzjwwm1UlXgzMqtMT8QK
-8z4zWH45zkJqGLquavscOpJCLjlowTn864a8K4XTbP5iaTyL23lICMzxGONoEOJZhuRl6t0a+yqe
-Npslx3nytY932ghLdNkHPaPZcW4Wsh20BNWqWJDz22YXujaHmFayickCVmY8qIaGx+5hWH2ofvaj
-SqP2oGFJ83VaUM6aqp+HkXwCX3bgnzS8qEB2XsOlRaFiFvzUFMyS53CtA4haY6+U/zymIzitrIZ1
-xM4uwaTLNUt6cb+cfGhkRWKysq8Jd9nybVznvllhwEbV+nkZBJquhVGinxuUspyFxyaOtH1IW6s7
-VBG1XyfglSIgVBR9NK/+awrPqvpLCzO9iezhILCZ/qJfzdrcZ806GlNANpPT+23L4KNc6L7enChP
-qCxy7Naldvg6Z1Dso+5SI9NP3sUbt0ULE1pyny9x3f+guLGjupQE5lYL7H9nEeVA/INk/TykTZD8
-iryHEyya0svUBGVTm0w0JRxv53Ap3TrBq7qq2bDBI0zjILNHwZ0EZx3Oi7k/uDpR6iVPukB0BfgS
-jcPd0q/Z9g2x0kRBoVfa+btpzUGDPJCFuSUuIqHmpC67WsfrXLS5j/ivZVZRgq3M0wWyBbjUhcFz
-Tp1foFmnFqZkZS3I5F7GhvnwcotG6r9QBcfUzzHjWj1C3Wr7KmGcbCVkET4r8kBzVZmhdcGNzGsO
-wT+a8f6pJ2CP6GpYUyw+b1N27ZxI6ZOGcbHf53xABII18Lo0MMPmQ1iT4+R6IK+FmqhzL4pKHNS9
-DBxsGoqsCzwoIkoQNQdX8RzJkZUnCJwFVaPhCmt2QZOjDVj4qAMWcLUSKDlZGRq5+p9JQ4BiVbxZ
-wAIqwsEFA92DIqTg1raExLuwEIFX2wsYlkTA+s7jOa6jqCZgqcLnB7Tkwg153b0m02zHtszqwAcP
-aTPCPAGqHcdhX+s1KDIrPOvGZP0hhRMNfFOjmsG18cSHWJbLLOwnWGh3Q5D088Ws+2ZcD7OFNHgp
-DYqCLK3GOOXJtYpFKld4F7WNai40orUARzpkeixieNgkZUQJ7PzgGr3lY3ThY4nw9YX3iVvXB9XF
-U8d2i2LZFn6Z+YDaB9kd7KrFCZMk2Y3V3tqrHKShJdqNtadbsTG3hrtlcbAFqhiBs9+dFJObjhP8
-PFoBRqEeYDSMuSob+5nLCJjHXguX/tZju2VXsI5cgm9ZGy3Do8ygyAfrD2QlEA8hJB1+wvou4EVk
-kC2Um22NuQrSMeOPDgXy+hToYe4PfV+n0dWSw4+qRPgKvmdawuCohe/jxcx9f9gSHsIkYpvqsEjr
-rb5JedTcMigP9lHPulvgaiPwHpmxJXnM20R2O7SbZhvBi7kZmtt0NBvEu2M8UfIcxeh9/8AztfGz
-TsWCtsBKCDvgZwFygAHr6krwEPr4ALp10F8tTvGkSmFSTstOsGh6jtcoJ0FB4Dw4XpOkY/1D1LX9
-dB3iBuZ3E22tu0a8G589DV3zVCs28R+Zb3N5LzqSZ/d6Cjx7BhdoGvbLQNqsasLRuANyVacLYxVI
-o7uJSP5rYEs434G22sq9rVvLvmPLDifL5BB0l/s5jeDgyjgVKYSFM97DbvBmjn+11KA7DffeOcKu
-xh4J7H0SS8BTRDmdflbOT/4SjsUU0n5qed898TrXgTrSbUmXbB8kc23Do0WhwG3pt1zMv03utuAX
-jLgntRWNDulKykUTGn2PZmvXGAp6WBP7CgoNs/QlnJBgmFgw1rRwWt0G+FmLYm7iyS5l6tSkfmWr
-DIK+GPJpgVq2qSPNXicqgvEpa6mEz2c6YKM3BZhhHu7T3eDiBMyUcJVaIZDmdj7kuYGNdAfcY7pp
-YQUcFyDKwDIoHyziOagHy/oiwQudC2io2hWhMezCsgMPBBzLcCAAkuzQglYUdC3Nn2wN4PSJb0T+
-rNUocnQre3MyRBzDp5CgY1bG2ItxmU31LH8sq88fQPDCjc1k0Nj7VG0wP8T54tddEzeqRPSZnvMQ
-wC8uWNO9LCD1PPRuED/TNtHyOA42vh+3Lb2H8LTW/1wLL3UezhY6xyW9VNvUrJ+RKeRoSTcJk4fJ
-w9ziAEMTrndwI6W2jAc2J0e/BKC1gO4rn4Yww8dynsBn0gVhhd5oExTNCMeDEkQ82BEkU9+LvUgT
-fo3qxsG9Ufb+tSW4vy9GHU10NzbLBgq21nI3T2G3T3MX0j0NVH1A8QHXkNF1YwBSG5+aapRqCGAy
-CQv0GejFethwvb3E4GL25cRxx5RJZ/BRWtfDGciA1apLN29rd7G0JnMFNTm4Y3CLYzUchOxmYGVP
-FntZw/bCFUKo7NjJWVtY1mx5WAUE11ARnpYq1yHqwPkIV07LORxSUsU2siFIdnXzgHAXfV3iAS71
-kWPLFyqy+ktSWw7r75zdhzPsT/BGCAn2TTsARwqyOcB5GAQ7GXYuSFZhHDOm1yOXtrsf4Ci+HCIK
-O/YLC8PacL/GOrJfOijNp4pOGWkLkSwbYKABWzNdmKQ77vJgKAX+zu3pO6AT7rrBlJrzKCqRowwZ
-DOeRi4CXCPfQAj8R1uCpWqNXtiXyqo4HD6vxDC+qgCpHx4eW+Amqct+Kb/AhD9uy3Xqyj6H8TvBr
-FShFSTIq0P4kXF9R7Mi9oD3+FW1Y5OB1l6umiEVYP82dEPxIa75FRYZMBRQMkbOhZGE/3nZ9mjf7
-LBLwtGHLmup9PCwBIH3mO5iW+2VwZWPA7C1IEjYUR18Gyc6vcnzYskUmn2VXi7DcUiI0DD2zcSm6
-ZrL2JsnqEVLrOmZ1qeotC6sB33P8hBkE0RFGtjK5GOLecvwlQpFdZmvoixjKIFPoTCOYLb6l/V5J
-Q24jUKuG7+HQuYLkiJnFlNq1rpp6wv827mD2vTPMIONLszapwRRX2RXrRUYPyHFzshbwqu9+dT62
-2y84MC/Psh9xn4imbeNKLYzNe+3rAM8SLqpEtkRh/biB7nHJ7Zw8RYlb8kvFoQMom9jUDx4TNIJi
-BPP+yhqO5NJsG5I840cWVelAYR8L4ykG28XGtnduiqJvC2XNddsPkhYaIyY0giETbam4QWDcfEi/
-zFHgvpGh46wghrbhAwyuYVmQgOIgn7t5MuiNdYte1SccS+dhtmhx86UcptTwsd+yR78SWLsEQ9Re
-DTBVZeUAi0kk/BiJUVd13eTxEZ8qMXu/NtuCrarYg4HcROy4bTUvamDUzbHdyJTuO1B1usJAxpTt
-ueZoB3vCZVM0gw2f6UZOhCioOcUeTchlx2IDNii3DT/4yATwIUrqWh4I8unxayNi2NbC47Ytl3pF
-7AKykXUYhgCJpDzO0LveofcW9RXwIxNeTBlcz+GKiZoF5yttiTnASdOKo6L5PF4hV0HV1uGzCNj7
-Mfx/4A6dLLAQp5DDQ8DSfAWsL39Foa9/NuOw/YT9S/O61V1/jYEQut3HqNLvvFi7R8Ux+KEKsKGe
-11gFyyHoYvU4dyRAzJShj/eZTXskBQHHlIcECUV8SEMbdhdxL5dH4OxJ7UvU+6jevFbxwwyNndtB
-gTRWcJ1PcRcQ3FolaLzwx+I9zVskgwoFqunj9A6oPMwpPMRMbA+OfjDvYQCe2S9Csby70LRDOqxN
-kGEUh8E9VCytivVuhF9dW6SENC+ihnK+AGktkI9iddtSGTnx+IBQPNyARMEh8Y19CtnNytKCegGv
-ABAp2O9gjuzvQBP2e6EJKlsj+OTKNVgTgJb5gvsMBDvMnKGhjHY8QXkO3svJMNKGcnrdtg1Kl7rB
-BI5iYT7+AbAENRDGlnRIkcn8JefZ8F0qR+LLGOr0QxikeVuinT1P8OJAF3gP5Uo3liLh4J40zRQ+
-mYEbHJfB199SNW6fUkydeWXakfs1jtZ7RtjWHUZkPKBP6gSq4kwCdNq1Qkz7jWL0xo6FNucFpg24
-m23qbbDv6Wa/Z7Ak7YqEOP1DxPBJgNOLitOK2yg79MFsAjRuav+6BNRAKj/myh5Nt8Tft42uGTQ9
-bngdETwwtGXNxU0kouB3tMrtkyHog+/jaUlfTd2LxyaBSwYkjf1yicE0SJESgCmmcOD4mGMPEq6r
-pq2Vv+0UkO9qsSJCfHPuczto2LIsg++bW9FOFLCpNOpX2C+zKzfHum6HMTh9D+Zmv14RaccZBYKb
-ftcp5d9cPNb3K67wu7Rv9Eujk1wWBm/tByb3zFdWTiFyfYVvXsCDxYZl3xHkgX3fnGS7dAFtIaAO
-w09Qb66f2IwyvBC206iqXHMqE/KkvQsjadV+DNoEHfkQjkZ7szizFmJqk+wA5DJ8STEaJ4U/yUJu
-6ZzguEeQXWZoVKGGryxk7XNBM5uhKgWTIAfaRBzbbbGFhKOzdrj0wHzpfotQ2O+iSQP21FTrA8Z+
-rBIu5VKnJfzZMdRjXTJsMm4oveVT3jyBedE/btGKPhAKv3Up4pFNsPeHAwOGJKS5fej6OvllBtbf
-bEu71JdwkY/pjuVIYvazlbkuu/WEqAQ8rC/CKev13lrGHnGnD21lklZdCSi89cU89Om3wcTkxgri
-k32YN83XGgnregnze/bQMO4stI8YjXDqsSS8dM007fLQZt1xCqkSZU1H+jOHXz1IQIr3V7DQ9k90
-W0ddzsmSKlgeObIVDl/mIAFFbntjGv/Ma+vsNaJFIvcs6qKdpLneygmUCaSzY43ijuPh8XYcc88o
-uuPHpIvrz90MoW/R6imJipogB6iizgW/+1bIK8j9TiEc3at0P5t2zEqoaPQdxvUYmPfC2wEvwG9p
-6SHLuoWvW2zLZvSpKgzGVkwwyacY+0N6GlwkZsNjMogg4AUptywrcJ7pDyB8/Esw0uUrBZ3+G2AC
-h9E1q7AlfMvZ1xyO8z/RCezv5nWU30Xi44sBjzmXQMlR/lqgRHDLAOcfPLiN8YtYLX1+Mud32FGY
-MrPteBCbqAgpn/BmETPQB4mS5aGHuQeK/QisCETPbLozqFK3Aka+IrwaHUm+GbckN1kq5te+7ejX
-OAOEViyYS/K9W+A8Vdge/c9ykUMqEfZEHxUzhly8AmFGkrw2rL72yWTnwuEl3sA1OmghrbLr9bjW
-SFKCcA0rx7N+gKxrImnhUHe8EFCzXvI2pfjd0QhJCIgbw4GOgneFMzNmAqSQlaL49+0wHbgk2w3P
-Tw7UKaBYjRlBUVaXSzPk6w5Zk1MlXbx4Bk2f30VrusFLHfURxjPUp6xtomY4qhSehIUZ02wo6xiC
-/ct8dvNrZBx9TD2jiN3Eq/tB6fxrUsehu2Bd3T2OWgw/NCjWN7CPGNy+TVtmiwEuGM+BRSO1iHAD
-Q/zfTuFDbxSuAI7RPj1CbJrdWxVkX9d4RCkHFjF9aozB1bENDqqfdO5sf6kDEV/1C4pk5L7xsFax
-CjFoJh9gTYeagaMgzSnMnBZkLdfSYwZbMdIeg4twxNPvhGx9vWumDeZHAhVx2dddd6ti1BPoAwFT
-PvQTF9ezh1HCgWPSy0W+dNmvWlJ1Cf46spjeIMUIdW4f0VnOpgo0ZL6VNid5U+XJCAJ9j4YY7DKh
-m79pATb92HrN0r3WQ7RPUoOMXmnh2zKa5+UlmDZ2l4LcB669giUJhrvJfi4Z/B+vAGVisgWAt/Zz
-LTs9lqNWUQ9TVoPcK4dxVFzouJafV0ayrcTYkBhW+jS01zSvHcNVqNuHHE68WSFH3WI8Qb6Ge3zj
-0SNzg9RZRgt5AbkIcneI3qMFkxCS5bqHOm47dkCJHjOyzc0lnCNxOTZIq5sCsYgcWRNYcwjqMcuq
-GdO/VJHUCDIUzbJLHvb+dtH9xHbeNt2VU25OUIAlLi4YJhjctluKW01lNWDMfp3Vsc0AFO08mIfP
-CR/968QsJv/gG3bXq9VRWLFtwebuOy6/atKN35nsaV2myFB+AGRwNyLbMKAGNbP6pK0j/V0AKwZd
-P7ARTeDKDrGGBTxf2/kljJ1E2tGudP1EeVSnVa7yyX3vPAmWQnUap4DkGl8hQKqOynCJu/hwIgBA
-4tzO7EeatLPaTfPit5cNk8M+5wAOj84EDQ6ON+vzIDf2Q2LQXrPPQ6WeYJ5Ov64DpjCUW0zkS4CR
-HbQIUHF/8ZgBBeOllA37cE6xS1m6bv2OLCvLd3blY3uc0eteikjR0F/XPUPO4lEWf07pgvZiaCM4
-A8RoYPdVO3aY9Ae70sHuMDwCA+xAQZKfOwvjBNine0UwvaOxL5oKpKFRFqpsJ3v8mGowE5a2+ZQt
-VeCdvUHyPKGWdb2bSomOXruDOl9ixhgwoVfiTJrXP3p/aim4YJruc0HyfBfBrgfJxja5rfRtotCZ
-ylYdlMRZj+E6bpzHcgCm/TtyWQDrX3yHNjombBu/TXyF0ynP1iku0WNGWeOyeEWnh6TDeLnQiPSw
-6YxjdIdgrocu8Tw2slTeJ3er2LprE5BNVVZvKIVqD9pe2VgMUiuaWY/bPoqQY4ABU4MGLEc5Y5QG
-xH0PYl6jAH/cDJ/CWCBvc8IHcu/R9aVlqtr0XvZgDRTWrSM6bp3MPsGWLs4KPabrTwjiMRkHzZBg
-rFJ85rGSM8HMnRkjVO4wpQUT2dAo6YKDAWt3qxILh070oVk+Y+tE9KbnfHkAqCJR27tBhafw3b+2
-lq4I0/Bww19vkU0XhIfmMfKU3Y7SansAXV/cLarGMJcEHhH3msHAEZ7eGq7vKt0iwFVhsyITCJYo
-JPuVoWX0JBtRg+MhahOWw6Baf9PRDqUaZkhipA1mtSV2N3oC807S+62/auc8PM7jqE0xAv9/bLCr
-TmOweoyl6aDSrhGMWxyoFlwZzDoE3QuFaJrUh7WOc1/BnHgElImBWXWRw3icl+nK7StVvQ4ODarU
-C/RU49sh29LfTczoirhVY8Lfgg2UFUnf+2CPWTidr2YemcctIZJgtlGLYUMzwngGEKbNZDnKEYRv
-B28sDF4EbOY3tHnBh+0+bfBQS0rgtNuEbH/LbwASzV84KHIBAH+0QuBnu3l0/UINIKDdJk8wq24B
-fzTEtJ6iD2n/nTStR1MSMzAfORD6cSczgvFqBPXBHbMCmRPURRgyGQSLR5/Z9d0FxkFB16stYJki
-gTODqjJkrnO5AuPD5CDuBxQAliZzmYiRfmZziLoaA1u6B0A+IVoYU7giEVrXrtBdDkzKZXq8W1uk
-vBU8ubsL2TXIMUxNzGluU2O+R9wFPfK9bbwWnezDi0hz8jh7Gt+D+4tRPYnmDB3WQM3zTgLtu/FD
-ggZYUyf6yz8gQ8EMG39F62xvieL6ifBh6ndsnsSvJO5wnY7G+u+bI/Nt7FTzaxpg4YHiAPMbR6dS
-hCA+RE+mp/DsNeg+HbNoiH7wFSEPj4o9BlzUYyiTVfO3TBE05r03cNxa86aHJBlWLvBrE8kO9xy9
-BYK2PKBU9WMZ14l7BkmafFNAJnCRsQbD3fo1JOIGjqXAk2o9mc+jyxsHvr/H6IMxyuZfcwDPFmTr
-6S8CI8egRDGaf4qiTaDTO9vlC7ESmXWj1+CmF6dIY5uG3ytcn7rcdGiuAI5AfQsic0YwJmwJ0xub
-eEz+UU729zZ0yHexpLqNLElhbWhw3+WZQbCaszR4mHIlpquFZ5EFwCRNUtWYcFijkwEbmOM6UVhl
-JXBYSSodKvcbb+gUrJBqduWIdupTuDVolnYrqq0ioWh71LAmSY64BEP0tSUHEB55Odx3J6eBPVOR
-u0bYixXKD6T3RZqT4TcnktJS2WZCKWzi4UFYtmwYcwSnkT2jCqYvkW3D+xkpSFCmYPncLUj/Z4QD
-zFe6zCAfWaGMt8GMJLu2cIDncsSsWcQ6yJNMm7kLCkXgrzwRghYyXKkssUncs1kFeaxDMbeAguf5
-VXUc3VqDqSVdsVoz3qWwJ/0x4+a5Rac5vINn7xDdTeDCc7TsZIfxGyeE2AoVzl85On/BQcRuvZP/
-x9l5LUWuLGv4iRQhb25l2kHTNDAMcKOAMfLe6+nPp1kXZxAEHbP32rHWGOiipKqsrMzfiFKTXfl6
-O2PlxfbSN5AR6f/FwiJ6vOgNe1nTkMsrZmRFoHka3BGB2IZveUJtFhJlzYVWqJOENhHOlbcybNjO
-q9u+9gIfRzb7P7fMbJJJKupU1M+JlCQVjzogVyhAg76JCY1pL28Ixc6EiaPmmYVo/G4VcbpTp65v
-rkpT58iZ4NxIjtFr4yt1cEN1GkDIWx3p23AfqcDjl2MOTcyyLBTSvyKgbocMjew7lHXnp3jspef/
-HCx7HAWvIL0Xv3RjoPCM0DOCqzEt4O9davTGf16VPAej2meNwCdnNVbBO0U1Us2pElP7Td9Do9sB
-imBpFmdwrnK14ZqFcLz4g9oJZfGcoNZj5wT8+nqqM/FbKqiVjLnZrEVY8aW4ysmiTzPeCKn/umjJ
-FXfJoExvI0iuZyaESwuXjTT3DNghuqNWfdNuB/TTDxR8xMEuWEL3ZEv46AWKL4hOYc6Csp2kVnkW
-tTx6BKUavnTUZp+R85TCLX3q7LGKI+1XjePlaJP0iNT86c29lUWlHkfLrAY8tTAw+wFwvJxt2Y8R
-AcCNQk32YpIO3/M5qLWDHOZ+7bagQVjIEDt/sx/HiuphRZ846tOJFA/kTeXpiRCWXlNH6lWD2gTt
-pjFXf/lKRiVAKkzfDetBHzZGNIMmjDpNFLgxFEITHAMtzpgznQHBGVmv06boOvxtM97dIZcKkV4y
-hMxfSTm05zKfSWrxkvQ1Z6JcrXharo2xgxOZIl7Nflr7NsJE2rMgj3SE8sCU203MBfbOSHCxdCxN
-EKZ9VIfyA3BYlAFwSyQ3MAo0XIpWojoTLHmAje1neUpzpUwJ7kN+L9S0xzilcfywZ6k0zmKj98Fm
-ENrsxSjJjpwop1htp0KA5Z4op+VDW43aTzgX1GdwSCsMu25zyBdP/zn5KdMkz9dJrUaCrSQ+1aY+
-0IwTWN0ycU3O4ZlWu1kRlAStg17Xow6xCTBwSbd+WhnxlUz4oPIcVq3kYYoUPcRJMFHu0QYh8gpw
-SSrlPJmyctnqsyNPHehhKZmTR3hdemZn6FkE/7nQ6bk8tzZHJD2OjpPmV4OIrurS8ZEO+pBhlEZ3
-VD/oyeIB6dNuuw95lI/lPEMyHmMrKnAaJPY5fSiHSA7nRVVuKAkFt0246HOkgy49CmLYfYfvwfbL
-Ox8AypSVY+OGqolfcSCUQDH+GI/9Z9UNToAAqRo5jS75/626s1zGE1aKKDEgbgI4Et3EhktspFct
-3kCZpGzTFt03TgPD99SRS4StJpO1yXFji6+1afB12xzFETPnHmUiJ80pqO7+GG6XWhV+zwkpOP5G
-RrcvJFIi1wQDpd7NSdpdT6pYRNdkZ/r1UIoGhpJ/DLM1LQNUQ+ZAtUaSeql2s14WKMBgwrxIfmrF
-cz91TKRSouCccen6PnIngOLzx+QaI2H/W2IG5QSbcsaqlMI/bQBavfVVWZKmbDJq6omTYrvWQZ9V
-6hupG4ofQipo0dUo69oO9nX3Q8dr1RPlsKtuKN3T82ohRU4EpUr/bfVZ9HOit/orpfr6qJY60Am/
-RNHHUZKA7A0fvCRzo75UTy1wDxBi9GDRUeqnkZZDrybOJCNDjujmUL8acUEQ7EKq5ZwkrVE7cRJh
-cxcPBku/NctcxR+1UR8toEevYSqNj2JlmJ2dYYT5miMSLblx2Atn8okZhErFD2+Y2TdV7erHZCxE
-yyZWSzEcKHAnIMfUmqRlCsoIySNMu7m7zU2Li2ZRUWpAQZ4yV2nUpi11o/qqSa36TRGN7ozjI83n
-xuybH7IY5OQjXIJKvH6zep8xQVI6v1OuIlJSPAkxIC/ArKBbjdingjBtXwKyYOtn5ZazMHwz1EFr
-kZeeZgWdpyrSXVXAK9n1eYCSAyzXYK/6rAPcg5UI2DKaYfTPSwBb9hKTIa3wglW7xlbqOjcpd9KR
-S8pHBKbSn8nY1wUo/Dk95SmZpzf1QUlbi/Zu5lpxr44bjGSrp2rUs8qZDKxjbXA8WCjOPgcMvXFz
-fCkTMXnlQgCPO8qE+UGWJhHWilAND2owxXfy1EsUjaSBLhzHR1E64DXoTKdmW5z61q9uMlVWvtU5
-N/0zZSdFdSqQVy8TzLrnoJiy+0ZPSLFBgMdgwiJfeQy1qYCBP0XKjUCbO9wVeVC9hn2xIBC5gyT2
-gIxbu+3EPBHsvsN/GxxUF9NOopn4oOuAWuIQmUt7qPL2Vw/h4kXnChqQbyjsT4UkgWyCHpflFTqu
-tg5W2sE3qZUAE5V0dBZXjZB2hVYMPOcoQ37a7jpZOo/KMOK0rFklpUs1fgVRxyVkavufI8jizA6b
-ZRU3jRoVu7lM8qeChjAL2kpHjFMpDIg2vQPMoik6UYrC1zI8hm2ZG06tyjXn8MA3bapQ7ULsPUKK
-46koTOlOzXyAQ00wtueg8YFYxAvQ3lbVIcSDXu6EJ+7m6UnRKHXz5GPhVNZtcAudBvFcX8rVvSy1
-1IDrBaLEhtM0BCKTojNdg6LaI0XF8lkMBlnzDDGlLtvXkXQDZjLXHXglFK64r+l0pWPJmBziLOAN
-Uq/8PHVYxLhCpfDCw5ZWsssWgOURgNh7EkIFc20lnMTdINB+J4YH46tZav6DRhbDc9KF7k1SZrr8
-KHhG2MxI2sRFXRjCR8mPNP+AJOtwyisUYzZsBZRbgOZxVhYapnt0YPsqIHNXaupNWalzVExFfS2o
-xBbbaIM2cdtUrWZb0Cf/BN+iv+tls33r1VatdxKaIVd5SiuezK3waUuq2it1vIHwZ9TBDkt1I6QW
-GxVbcahA9oyqUF4x1QZoA47hoTNBufoVsX4YAQ33TSNm+u9SDVNcZOs+f13CA7c0eh5oeZNJ7A1/
-zJA1pF/6XJmDBN8hVIKcE0owKc9Qo7hJa8gFwGN0/2Y2Uhz9ZgpxYBHCuehxfi6CkpRIjQ6zllPB
-Ln1w6hQwQH9sKmFKbhKr4PDMqmyQWT61ckg0ek5o3ohFyh1KT+7Edox/DMVsvOBDjr2pFiri92au
-uBRhtOp/V8cQtE0gi3AMg070Scv1XvnOKoyvgeL/GPHhrRwlL8n2jIj83JhNGUXIPBV3sVyCZxpn
-mpwE7LgKvdgkZbd7gZuoHdOuA2xkDfIeUE5oYsKc4s2k54LymgOGI1opHMNx3mOH3lRsCQr/1m0j
-l8ptSQU6d/1BGZ4rmVOTxacOb3KO3ZAdJ7F+1Tdgv+wce+LHYaJdRk1q0I5wsAdWOODK0OsA9tVo
-Q2ELbGdGQhdDryXxwIurwWrgNfyQWGMAkG0BIBYajkPbvuojAq6fP9eQSJ8GpSlucjEalV2cluIm
-F8ZW3RJcq8Qx2qINVVATlASxA6KekPaHJKf/KS2dRDB1pm3AKO13GGFn9BuySG+IQDLFXoxSIDqg
-lU97u1cS9hMvwa/BMbWaTuOjx5h8iHA0axTK40dIZVQP8jHRDbxlavC5lCWoVnBuhK3Xl0aqbHAK
-oqQdd0r9VMTy8AvP31BHkYuOsxu3U3VvWJKQXgP0ja5iokXmGMNyq6LHzA8BXCYKMHxW6yd0SIUr
-WIu0sY15iF/VUB1+0eNj1DppEsulbpWap1rNKAjjcDhzH0D/lq5rbmr1d3hwpXYVakX0DdBB21I+
-xyEeyEwkgBkZobIkTl2CwNoFlNSaa+i0zbEHaN45JuWuGQvdqYzCE73WUX4AYTG/kXj14OFHQ/Wb
-xzZIoIJ4NRJcxl6glf+KyvfwNAbK2G3pyZuFa3ErBmPRCahDcr+muB0Ys/BsIYmGbJepWzdhl1gh
-aLDQJLkuivuGNj7AKjES3wTgEbk7R4nme4BDLKBRXE0zV23ACNHpXjaA2k2IFcq52VeOyZmik2Eb
-IM3o9FkPbVGZ57lTBpFm5cw0YShXW5C2w3Hum5ny20xkcGmMdHcBoOmO/pCUVNQ0zeQxQh5BcTvM
-slH9AQVIkplkE7XiRiPk1FLCpd8EGCIBGWvbFlyKECa0GASWDf1bZByTcsbmuqK2HCFSRILrFKJM
-y5AWXK5vkB0r0WZCSs3cULlPOJsUmdacCowczbh65rqc171M0wqz1nuSx6H3QhRUD4jJSFRYxFwQ
-uBw3LN9hFFFVqOJs8u1kIrzTR6Tgs0cVnMs0gBMDbNccS69aIifwhzEvp0Y79cnoZkqv/gznnBgo
-RLjR2IKSUaO1YjDAdkewvqvTKv0GMFEpPW7142MfhFm4F0i86W1EpXI2AhmFrVEqWZGtnrcSXUNJ
-Og4kN69V3Jv3yAVbgI9wK/K91JqhdM6K3N7UZiS/hIVsaG4cj+J+1oKiPNVWUZ+HKddEsBsmCPZi
-Se0zX0lqRxU7UGFk5ALM61xvvudhyj03RhaUIA+I03epjKtnwgE9JDhmQHKVPBUEwG9Cd0uYmntH
-iRMwjmWMotFQ/TkH1Nbq7UIs2iOhkT4xOCL/CSZGuptQVh1dAA+0B4H5VM8T/LjGrQC8VQd8U8Tf
-wZibylYUqPE5lAlwwR5EHQdJgotgetKgcP1E/bz9mQVyM5BQJ8EjGrv9eQrrnhOm1IPXqp2m34EB
-zG6T1FbyZnFI157OxqITUcVmhQRNbIALnUg5HVY8zW41FNg3sBhI/Lh6Jz+o0eevRWlEmMIjDf9I
-F5cazdC007EoBusV7RfQPHSMtYouwBwDWVYE82caZ/NbxN2KWUkpmLYuM3rViaNYa5d2ntY7YmSk
-LxHarhj3SDN0e5VKHV3PaOF0NL0FWDQvZvzDIQHx8gPadodmmOTWFg150NgHqhCCMoqD2jNLC9g1
-ZwuWSmagzoFDQ7a6wXlMnFxD1MVrLcgxG4ikIS225I/J96ogKpPEAT3q5JLQD+Ax+wHcNL6F19qC
-M4zkTPBAhPu3LfEpdEjzJa5pUdHdy2DFv5X0bh40vOBfVU7H66xIlbs4VdT8XMVDh9SOFfXTTjb7
-8b4JmwYZ1LlWkAEq09bfToUS33Wl0uAXP0yQViZxptpI7oJo6iybielxSxJ0L1ILrotjU+m1K7fs
-Gi9oo5H4aA11vs/VUe6g4w6qaVFb1YgPmtLy1yF0nh9lNJeCg9ZagaJBLE3xm1kAnNgikdH7x547
-DoAuw+/vRnBzv1SuBrxqaRFzyQNq7b4aAiebQMAAb2jF9G2oR//BJ9P/iSjUUmadxkElEJADelBx
-lGf4ICA9MuhBz1U0cpDXrWRtq3RI6LLCEMp2I/jOO+4qJcbGsdwAn9cgBw3SXElOk8JEtBNZTlMQ
-JhRJXN+HJkMeaRi31KbJNjVYAVdxDfzOjbCYNGkedBxPgGuUR3mqorfRBNmLb7xBlgv7r66cSjT9
-2zxWwRmR+ZPk0nYNk02hZPq9kMkAeTpEQ27xnMcWvTL9brChv4FmKg2xeEiMaHoxO12612loiZ7k
-z6LghpZFcwJvqCBykjojNU0FJT9LZmve4d5YPItCowFYKopAdoiHlA9xh8uvoaQJObzmWnlFTx7A
-J3DcbI8He9p7ErrvrcPPIz74cJ4P8zwUYEQooP5skih4lqmmgaitxiyiE8sSs2UlEyaQgv2CuwTg
-BjgACPx3P59C1QWRNNOGN8xyC8Ke71TA1hWce3TfSI6B5Nudgk6aF9StcdPGmjASqlNJo/YXx091
-mUQPlp9Yt7QNqbgMvj8LS4FrLGxTF6C2jJFKuj8R2V5JGrhqyKAs7baA7GBDrPLf9JBSxaaxqlh1
-J7AQFjivdjqos56hdSEuJ0wsVmnkqX1IWTYF0aF4UmYap+XeqRFUunnfFE1QO37XU9tDv0m+bvpZ
-/RYkRDEbgcsIByKuJRuzLklnEG+ufw8Q/q6jKmtlt69F+uWRCauAJ82CdLS2ClK7nyfhCQIi73ic
-kEQ3o1l6UEYDqZYK3KVMaYwUzR6SQoZ4k+TWuU38WbO5rIckDb4ksSFEWfg2RMr8zY/6TgIQvtSZ
-EYPrXtW4USpnHqjDODMOFP6iKzjRcKNmdJtNZSAAn+VabU+KIR2hi9U3phUAODakjMw+UI0Wsyir
-HEYiPe15uZlo9c5jMvgbgKJqsEulxjoLeYiKhmXRsb9S+oFuBu3wxvUJ+w0UC876vRyrlmA3LV7K
-bV4L3EVb2u4el9U8hoYYF8VZniRgAWDGGkg0vki/C45c51VjOJVuLY6S6pgzFGhnFLvutVcGYfCG
-rpbijRVaCXsqtHQyLQCoM/C5IIhdiZJg9HMMKMx43SxIvZMVEOBJzKYEyIVVydEB/TErOw59ZN5q
-UZJWrtLPKTStAozdCcoPTe0OngIPo1Kyn1KSS81mCmd/dKeRktUmCEmMXYmnWLszQZzcIqZLxYNN
-S0GiKiT7d1FlkEtUWF8IAD17kpCJvforzUcM1SN4H3dFO6HwstgAHDFEaJ/AzKo0IYtGP1YafWdH
-macSaLFZxmgxqr4E8pbIZQs0Um4kXwLyMlJJBYk3AMt2U/hDPwu/nL4VqRSfVFDp4gIYpHZMNdbg
-IlqUv02/5/KnAji7m6keknHFGg2b1kjFFzK+oXW4ouSkoH1tnqRSqaStr5rzSyAM4hGKaS9eQSZT
-fg6apCzFmRR4Jl5CwZ7CcDjTHxXzE+QCRQLDr3QhbXYMDhxAQOwoY4zFc4jpQeIUqsgL60VRe+ia
-mrZy1em0dxOxsfaTELTDduB938+c4ONOpZqxj6menFulp4aExll3DSCCU7IAfXJDdsBxkYpN0dtz
-QxFja0ZVTQFLhk1wT00yJQUpehm8VJ6YZz0rAMNy3ASnKgVJbPc85e8g1PvTctEDiiOm8MEEoWhu
-4Un6P5KSCrLTKyM3DHU0U2AiWKo8W+HEZg7KcDLAZ6WUK7IYYV0PNTz1R0qxDWVYuQwfQjVvufmK
-VvWMzpCeUmTL0x+BVNWgIPyEkhJs7rQEk56XD1IBAoAgC/5C1dA8tqMGU3KXXTy9WJM+9+TxCliQ
-gVKtBgqHtBGctJreqRFcBoculP6mmbVx5gxqlE3hB/S5Wbq1J7ZBTYpfl0rpLNF52sgxxR0vHtv0
-tdHMGWBkaGanBYM6ueFYjUcyl7zRdwEd7ckLVcmskJarhGPTc2rukqJQ9iY1Edk2EZjnCl+MpXRq
-IAP+rH1xPumwRVt7AFjR7dqZ+tst3DMfbVPBKHg2oaoVHi5erXE9t3paPnIvEB4Fi8IobaBSBJ+v
-x2S57VBKz2k+qyI5INejH1YQ94LN9QuMoi9BmtqWFajx7wauoRYtFyvXCBIKpTFwtgFFeABA0fQN
-dGmP34YFdWmjlHB57KKb8KL9mnG9aAn8LW6AeQDSn8g1iIicUYVckbtTadKsCuAPDWFVfhG6wre7
-pOq2RjKMt4KQIvYq+AGvru3cNOmk7dfDrwnfy/B4tULHN5GxpQv2nmsNh7Vuga1kNtQrrkMpUOZu
-J4ISVGB3lid6FJY9a2pwVY8psOCvB1+7imEwx+iyKNJ1VPRFP+X96PiE6Rqtu9xOfI5cr5Z8NlKG
-LaCXcKuIgDVRRQtgZtM/j7hRwRH1khy0CUkMBe9Kb58u/ERr7vn6J1pJrAB49qs643UEhUocpoXp
-xoElO6RKjxWpMIGHXngNG81L20FD38uctnlOBUAeAqDhEyUH8CTWhSe1lgD482NhYrio3krKB2Wx
-aiRCdypX4jwLKLfCnQsAdqRUI5Om0Av366ew1oZYRlsUPoxF3RRMzEompRzUHJt3kCDAgc03NTIU
-4HHQpUgLR218w+hXviCi89kyRHJP0rVlDUraSvoCgGRTJA19eOiA8q0OzIQ0VwKL24rjHvSctS1z
-uNuFov+b/cNicaiDNNaXFcj40moFmgUMRPAvtPsQwoNyRfk3Kr9lKmfBnkoQre2vH+3Hib4fb7W+
-Jl2AmFKWEA9zceBGO0zHiXGvwGMoYMWr1q3MqrqztDTYfD3yx5XNyIjPaIgaG/hRLT/ZX5JPzaQV
-UqSysnFIEg8B2FYO3rL4R62WP88Tk0CWDYwMijjvR2HoSLEqdrQySO1BW6BvZiYdaMoP9wZ46wvr
-5uO+QH2b8EH3mIYgb/P9cKZq+VYmsFLrltOspTTsUHH8DrlG2n39+D7uCRWdDQM3cto96Psuj/ev
-xweVq67HiLPBr+RqTwYDFwv6cOQA8ISVXFPOvWC7/umICkJMMOChJqzVCyVu2FXWsefLUBh++BOF
-LquNl0piHSa3qDWaF3RGPlshWCeYECFM5J/W6uIDjhBqsXQDAPVzX7Hmsind0mj6/H9YilgQoQkv
-qSpvbfUsI8DkZBQ8y7kyKrDOrQXmaKwujPLZ80OuXAI8hQsKmPj3b2wwwOkmIaO0IAR0qIXWvItD
-ufZGaqx08KmFfb1EPluMlmiBHiAtI5qtdphe1FowmcsSkXrrPOQIgzhjEBiC16UkNRciyVqkaNlp
-lmKIPEUV1Yi1TUlhdSk5MMzjWgqy14iGHvjQBOjKXF6bTb5YEgtt//j1FD8JXxwMiJBJxEqcnuX3
-z3T2zVnRAInaaArA6JQMf9tM1FuVLN5UqW9ShVDUraoAeLww3U/eJiKwdJvRZCK4qKtEpZejIjQr
-dnrjd+azDPE65iyW+h1mZd0mgB/tfT3VT3bDkpBhzaJIHEnr0NIMVgvGLqWXBTzU1VC23HSCcsmV
-/JO3aMgouukSKkVIP6+mhVxNEOfLnvPlRBpBvSdNvFWaRhI3Ui6CRo5icTpJ4H/DCwHt05E5CKCw
-YRaIXvr7V+mD+x/bDI+E2Oy4R0OG8V2/YW9QJGmkN2I7YNcBKqd/YeBPtgnjiWQXiF2Db1t+sL8i
-aQ3l3YBhyoNNyvHQ5GLvoQQrnC0qKBci2idzRP5PwcCErbLYhb8fqkpFeR60DHY+3D9XqIGWjVoN
-8TaigXQugSk/JZJ1Sa/4kwlaizY8/kEaFRRx9U4hTKPB3LNJIgkBHbEGjgS1xd8GIiyFf16kFpgP
-C5cNbG8QwXw/wRjSOfUkJugjCORaLTimodIu6b193AqL44KIyaqG4pu+lgQUexMXjwofGAEBgVMy
-JOD5wri/kIp9Msqijcc/RE8k9Ffhs4OvkuWaRTPaACNaSrkGWifU/3lbk0Wz5WQ0FGUR9bP3T2wU
-w34kfQdkAWgkO9WI6xRuUQvtpf31yXQIzBJq9iKHHCvh/UB0lNQgp35qzwPKpFEm1w6AxQuKwx+j
-4h9LUfSysIgn/VnNRiZhGcacIifTTQ4Ez2jyogb8RznC+vdgWJfT878uOcR4MWsEoq4t1iqruBEB
-66Z+QMasKCVXttAsN+U0ju7Xo3wyMcMkLqoih5vOPe/90xvQbw3qpOIqblW0DNPQuMZMptmYRhc6
-5RhcMuf5fDyuABiZkt+tVfF7WewMg7oOEAShof+HnSjdVT+AaROLcXHuxlr58fUUP1kgTBEbM04Z
-NP8/XL3Rx4e1woOcwjyCuVvQXSja+d/XO5o8FMY0ZYm61kpo2Gp0OO6QDuwuFf1bc4Tw1MTJdMG9
-8mNeQClK4ygxOCuhxK/2rq+HyE0t8pkK1nYgtVFlgTUz3APZt7bWYMLBTYKRFl7TZtuvH+Mnb450
-C71ADa9CiVrK+5XSR2JUVRiW2IWuBk9QgLQnqHlqs0kLZDtsPQFStPl6yI/HCsYUPMqlk8PpuT60
-w0HOrQEXbdtX8nmrgcp6SQU6kteCzPX81ofBK9lFFVLP/XrgT5aMiaynyQY02X9rrVl8L0lg0Ru0
-e9SqbmJNzeymLId/zmOZnoXupQzhCsnv1flVlCNcfhPgl5Wa+RZeo4/Im5AbbIU0zbQLC/SzpcPR
-TDVweaKA5t6/v07BEgucKvdSc4y2aHuBrUsjAVV634iP6BFOR42i3VYhuX7498dp8BhxGzFZPtqy
-tP7KRIyI2nWga6D/ATPdSmg+eQWaihfuqJ8tUEPmTkwOqXFVXeXMaD6VCorzIJP1xLAbAAsvyoiq
-J/jbagdPpNn9D7PiKo3QLdceQvX7Wc3IqRRQBFmdalFGLiz3UgfmhUjWhdX46cS45S/JB/82V3d9
-lKmAhaLQgIKLD4cAZ2AaJk1hjekuyTSxuZth/lyqhH0y6GKSwr2Hh8kRvjoYZhmYcjnDs5lwbKNH
-BYVrAgdfoGsTZJn79aP8mMmxOLihatxTORWUVWzJhgSWLbI6UKJayEVONI9V+gT3y6hGGOLTIF+6
-1f3xRXlfD14sU7hZmTxXsofV2xszKwx0WhO2xbbLvKhvxeMwoiBmRW2+801aR1JUNdsQZCQegALt
-KTuYDBqCGRp5F5buJ/HGQviEkK7oxPZ1ehkOIDNxhyrA1tSBh5EuEL4Apfivn/Lnc/5rmOU1/LUP
-Y71Ne9HH/caf51G3624R18IqUtWcTLHak5aFwl4c6K+ZKYq1ZUorGuFyE1eeWLzgU/XZ+uKN/2es
-QGRY7dYCMTnfUJlyAHbcUUGr/lLqKgESJgaHvuGO9vXkP3vEFL85Szg5F1O393NX9RlvCmQZbUNT
-KnTXYBAZUzZcmNVnC9nASFxCHF/hXS6z/usJgwxW07HjnoCEXvXsxwF9xEoOXjHevpQKfDoh7lyL
-QjnYXnH1AFFHBiAgkXDUmIi7fg0ikEZNeCHh+HQUSCUEHmofxO/3E4LX5JcytqnYBAeRuUGmSO1c
-blowoL9+P589Oex7OFopvFN8WKXxNcm9CamVgYRW3Agg012j6I1zCWP4/n8ZCuFna0ms8QB/P6es
-GZvWEnhJ5diWJ9NvQzqcJjBe0ERD/O1/GAy3K0pwpNjS+haOnE2IOjQJb08DZtN1LcaXIMTdvk2z
-zddDffauSNE4AJFj5oRfzQsMk6o3GaUbRdGyM1IW5o1u9uaFWLV8yjpwIpJsLOUhToi1FnOe9voU
-zay7vAE3aXdgRfcEx+ExpEK1KTvYPl9P67OVQbEPiCJoJXpYq+NPaSGNZzqtM/S0cieeocfVMSZh
-5PXhhZf1cW5US1QWBQcflYz13AZVstIGTPXCpq63oV+dC7M+AJXTd2Id9Rcm9sloJrrL2Cfg+bLA
-zd6vw6FTBNzGaa9rg6AfgswSHrB2grojdfMtEn3+hXzz4/qgsi5hnEMeIcN0Xe3lSNQB7AsFpHZ6
-7M+lNE/U3OTh7uvX9ekouByyjSll0PN8PytB6PVxRp0JRBsKrGof1DdAOC95Kn3y7JZciEYLlwOK
-zsvf/xVoKdfDjjLB1ef91N9Kkr9AJmD9HtRs0L/LlZ/+/udpsQQpMsmo1dPhWU1L0dM6CkKuBCiM
-kaxn8s8oN/7Ro5rCAvcBlbBEQOfwWKeUsoDYRD73XO8KBRXdBu0Yqstq7gDFgKAm8s4u7OaPb4u4
-rmG/yZ2SFHPdEKz6EgZOb4HnS6vu2phj/yh2gzL8c3SHUiEaOJcbRHfZXEV3MwPvAwAkQRmjLbws
-yX7NC9Ss1uNLNlgfJqQrEjdwQ+SKLONevtpUKP3WQidCRJSqKXrOCqH0kjb85/o8o3A1JZ1YzBKY
-0PvlBxAUtLeB3HANDbeyk9xECmeYhkQ59l0JbC9uLEB08OTZ/ChdVhf7ZJ/Ncwkb3MiJIHQc3/8E
-KTedhfALeqlOwcpEtRJeq5GW/ev5z3GyeGxxMHMyExrfDyMiD9+pSxkPWpjpWsrwKwdkvPt6by25
-9rsjhYrnYhey9MKt5f/vB6mjvKnbRn/p4AiXhXDWo10mGptCkm0cb0hwIH3h13BhTX6oLiyjQjai
-rKsugkGrdwiWELXeUX8Zu4MVmtdZ78mF76R67M7z09cTXA9F7Vik+4BJDhVXGNCr4BGhKzEDDYUV
-rI/BDWonvtMNWX8loLfuiTo8NSp7off1oOsV8mdQevz0NGVSjHVpL0Z1SBuKMbTR70jO8ANSbzYn
-0/16lPXp/N8oJjmvoizGeqv9RhM6QA6YqYXQnAZAJcJSikVFyYFXfgkw8clgi1kIPDQ63lhkrKJ+
-XRTYlGkLGjH0GWsozTsONE7MsfX/ceEzr3dDrRa+pvu+MVcMBTdxgMSQ+VvEVf41ZVtGofKDNwZ1
-NSLJKi52nRSCvEedkSCjbQe6xjTbZmPz9Tv6uBLozsKCIE5RbaI+8n5/wTiYY02HnOhHZckttglR
-WEz/NfLS+Xk3ymoXcyFBE2Dk8oggqG+jm/UsJtLz1zP5uAAoRyDNijnH0m0yVm9lTIVWDmak1DAt
-0n9KI3oOKQTdRVfCuGSV9Gfp/h2WSDAYjBIB3RL6S2uHugGNBHXq6WLRRUdFhpxRcDhKm+tayKob
-wLfFptW7bof4q+yMUSzvUclNL8TGD++OOzKeJxLoLXPhcK5mnFUorGeh8WRFMAAqZBadUU8uZVOf
-DgLCg2dKx0YX14Mg+4KMcPCcTFVmeUqlaIccrzpr+09vb0HEqFyEaKEwEP4nq1jRpelohfo42Jjh
-hSCXS/MbuilQSNU4vHDHW83ov6HIcrFqpYeNneH7Ja/4RpTkJLe2nkH+bpig26WCdClIiO/HoaFL
-c4vHpiq8IE7JdXOBP5IEKZTOV/vT5rRzNxvb3lwdNxvX3Rwdfn90+bfrOvaOX7nHq83e3vM1xyO/
-Pbguf7dzD/ydd+CXfPVmvz+5O/72yDfv+VLH2fNpm63NR/Lxy5dsCr5//7A57fd8ms3H2d7y15v9
-xnnhS/gRbGf5E37NbzzbdnbOjnH5Wj7xdnvi469cl4964U/2nu15fOKTe7T3+wd77zl8j+d5juc4
-zvJlHt/P5y0f5lzziyMz4Se6W4bf7pzDo3dYvtQ77G3PuXFcfs2sd9uCyTv8dBtvd+04m/1xs/yg
-/GxbvvPOeeVTd3zp4eZ+t7tfHhMPavlu93jM7GXYe4c//noN/ilc/v+u/vDG1o2aLK4bFdjS+bg5
-vew3D0zKc16d3cG5vzDSn2LPVyOtgnvb1KncsjY27vnp7RTYJ9t7vnFE+8I4yrJtvhpnlV00VVPC
-X2YcXtHT/u6O9+zwvHklu6uje+U4F7r9qzrix0e4upH7UlvFKKmfj+7LA6uF9/T1OwLhcmFKy7b7
-63oHPhv+EepIx/PV5mpZ0Jvjn3/47+llw944sVaPL8fNy/FU2Wyc48sL79K+3rKw9nfb/Xa79bbb
-a/uGFXZwrnYs5+fr6z/L8dp2bna8b3Ye28J1zleOzf70Dmfn6orVd9hdCOEXF8Jyqv01G1XE0jLm
-eblP7gP7hid2aVX/Sfe/WgOreIfUDiRGhrjavJwCj23Jdj8tG57Hdsf/9vaWXy27OrCZ4eH3Di1P
-+7e72+1+D/b5/tIS+dMR/+oHWh8pranE2bIoT/uH08b5vdtH9ma7WR76cUOMc++PS5jkxfAiPJsY
-6Cy/dU+bB/dhf3d0nwpi29Z+unrb8AFM5bS1tw+3PY/PJYrc7besO+/AOi/t/2PvvJYjR7I0/Spl
-dY8aaDE23RcQIcmgJjPzBkaV0FrjbfZZ9sX2A6t6OhnMYXTtbM3VWltbpWCkBxwujh//z/95h8fY
-3t3wql1Xtt0rBsQ3y77zDqwkK9feuN4V69DufFlgPh+qbwfkz57zKLZKCmFUJEYqC/a5/YU1t7f5
-3l/XK/v695WZx2MR3TvufsWX8Fh3P/8Gylsc8tlXOAq8ZqwNp2Hp6i8s7+f0wvmyrp3fuBeus99u
-Wa0335gtLNas+OwSa8+rWF5XK/qcrWez7ALuF17O6pu7vbhgwWbcXFwHtv3AKFrxTtglvB2z8Aur
-9s5+W8u26+3F9vp1G9iv18s/+nR78S2yb2f7KbC3LHasQxfX/Pb1ldHImr9xDjessfz3anPj3Wy+
-Oyz5mxv7ll1ktO3AXjNVH84Oh4fDbuPdbXebl5srdgrniu3A8bwb1348YyPaXO3dG6ao7e12Z6zZ
-uw1d79Krb93Mk3+nu9lcaZG9ZXPOvny+dzbegan+9oP3N/zxsijcuPurL18YiM7LiTfy+epF5PZ+
-voNVKgSDLYZdcs//Gbvrc5ctj6lvO+7u903OOTEOQNV9umgCs3vfbNIbRl/QLG3SHecXzH+m2tLq
-sntXNrPIflr2epZL5sXW5gdZHVbXy67Mi+bF86trPrC1DwQEK361fHa7XR/47+aGTnN3ztVbYEO3
-rpZdkxl1YOZu38KFzW7HhFyG+moZgxerZTkN7Q1DiO5ntV65rMf75TW6my/nRDru5sLlM5+/gGV3
-+OeE0N+CPxQ5bzEmZPJjgehcFLh75iEF0KGMMS5GNWeKOJ/SUR1XVfzeDKKPhYnMLYJ29JqxM+yR
-NQlUN/ZavYnHajrD3Lc7aF2grUPuMSi4HzX8MSirHxLYdvjXdMFWw07PIdI+df46Ohu9fR0dhcZy
-MiJP+eGa2MxlnI1x8CqmMbUbNUn3Iy5TqwjLgfPPO/hNrn/cw1QvyMTzaCpJWb4faqqaQeSYCK/D
-uL7tqLnG0VRZz36ygSSx0Yr6WxcN3zoJqqHq3+Ra92VEGDiRjKvaZAsu6NT10bLMHn0h8ismeRZL
-prrhWMRN5StmKSbkIlGqLeU1w5Y/2eUN4rNLLM3zZJVEcyZfY9UbPc8RkJATIvKfdL6u64qIghwd
-K57I7zvEr2e5w5W9t1Hsg1bQi8KlrKt0qzBOT0z0n4zud00dRROVNMnhtAy7sNWFbcKAOCNH2J2I
-wX7eisXRiQKDJUXx/oFq3Eb8PGUOdXMQrmRrFFaljAXo5wPpp62Q7ZZQZqEN0Y/GkQX8KsURl3FU
-xPE3zGqag9AL+vXnrfxscKDAZUpwbYWk7ig4QgcblH2G2U0SSfG6zwiXKdSVAi9Qg/ZMLDHbkruy
-3Cl93N/9+aZNmQGBjlv+OFFwvMmlIcPxQeHO9HyUtOERXJWwxYFHu8ww+8XRVtcvOZKfKtn42LXU
-M5IGR0VOjpMl4f0LFAYUN0IdY6tmqtV5nOTFJrSaUyKYj11rIszi1YmmSN79WEYRilWvi2U22bgl
-XIu69tir5q0/67seYz2s9NuNodYngssldHw/17koljFx4vZbpnLqKLSkLHzgNiSfMATBQ+qLVcJr
-2ZSSEukOzv9liJV2E6CNwTk9vv/8db7f2ZedxZRIJyAzRRWD0vmoaTTN1PgnNG3q1Mkpox97RRlW
-HghKalDb+tSF0M8eVUWnQsEUYlrSGe9f4iTNvhrI2BQ2Ay5U8pjFD2kQ+CvK32I8J4xyAyLiFJb5
-41q2qLRQjlPtw8g5FjGEIKDxq8H22lepkU7EQnATtbFWJban7uf9+dOmuErBmwOLaXbs98+Hf+4M
-RhvvPwydB5kNRExEz7eiPFtJ8Szpm8+b+zAnQCGjcdVVhuwioTzasYURSxtTozBWG7FUE2psR8sE
-nu3nrXwYJEsBIU0sygwNUv0yZ3447lk+J+gZa1D8izOz8YjN49xN9VB7oWTfxKK2jNXV501+6Mej
-Jo/7McWXwQQ05eDAUbqSmrzGhtS6WZX2Jx7uQxe+VUeiPCW6Qk6oH+0L4TyFIk6VkRNMVbfFQi5z
-KNnOT4yLj61w3YQ4Ev0ZWypInfddiNl7HxsV5jFW0mheFfYzRpr6vP68145nF7ELs4p5xSiXTQzi
-37dCwbwEihMBcuf74vVo9bAsg247KUZvw4Ucr/tiOpEx/NAkPUY+eammW4rpjlPxqWQoo9JQ3xo1
-teSOYGU0xypa4VLC8PLCMtvFRnhqvc8fdHn9P66Y3FWSnqTI5m1Ok5N8/6DpOHS9mMDnbFeR3TmD
-V6yVc9k9deN0lBjSWTTet3O05xAtdnqV0k7pfrvPXZBo9svu8vHzh3lLE3/2NMr7pxn1JsSQgVbk
-NTpPG8SaJx1w33PB0jmahyLK3tf2DqqRPT183vbxncCHJ1wG7o9zu05StV5Ip8JGdQaH2kT72Tg3
-dn92Xz3uyWXC/9DOmObYdOW0o1756wq3o3vqzHb+iXFxvHsft3K0veCSFKfC8jTzCmSbg5+zkzvl
-ibn84Zx03MoyJ354FiWqJTVe3td55T0lzu2rtn68vzkFNJeW1/7ZsDhadqkvSycpopnKoxrIwRbK
-vscD/WJ2jDts1bcnRsIylj9r7mjJtQCJs3zQ3OA84cVvP+f27rtzc3+imZ8sGD9O3eM7k6zJGwOH
-9uWpMCZ1uMNzQDk6pqu7j+uvjXuHheOpF3ZiuTiuSyd1V1rh0mbvcrBjgkXew2w/3x1C+7JxHzkT
-2KEdn9hYTr2/45pHBe80OV3e3+Q8zStxDajUa1bhIdr6drru7BMd+z5r/mGtko9WkUTF2gLXh+Uh
-Qyfjf6qNETvp+VPj/3hvPhr+x0pqVYAQGSIos5dCQ7v3qVAt6m7XJ8apZzo1Vo4WDdOIGzNfJpqp
-fen8TQTCopRh0OYJDnGndIBHacePHXi0eMSmIGv4wP7egekF+CzXWIHmde4iN3LJKk8sxKL9/dRT
-HqXTPzZ8tJ4MQQbiqaJh5UbeNffFodopT/4lt8DQUMrH6TbfRRfKpXZ7YsSc6t6jBSZox0gvlhGj
-MGYwxGJ89huiPMe3Daf0ci9wTcd09BOL9Idky/EAOlppJjlP0maZGOjCVtFGcm8zh8Sqb5d0b7GS
-7ZP7+M8WAHRa1FYuJgaU171fsZvEzHJxGbKVBwKT+aG4FpGD6lj7zIGsfNVcAhpZ12v1zNqe6OWf
-ras/tn3Uy9j8TSm6FWIVd/D0+3QVrobV5CarZitvTuXMfvZKkXmgJaHWAa3i0YEghh8ST3XZ2DVQ
-HlHCFAXXUHV67fLajeerzx/teCFYLs6oY5IRRlJ7iZb0fa/qbST7YarOjqC0ygrbSmAiUh2Bvp3m
-E0u4erQ50RQFN+gvKQ03DexK3zeVmrI+yj1AUx/zoH1h5TllWkp6Yg097r2lFRVhEaeBxcTkOK+i
-ShM8pgYXyhazlAu8wI1d3aeNI05ydhGXWXZHhbl0+ad7kQwOxyqCdrRp+jJ+fogmCvyr6qYEoQ0H
-vPSwy2dNVdvsCopQemosLkvYj3s8D8gZjsQN9ZEaVfFH8wBIYj1bhjA5Rt7nloMlWXOHJy/WlrVW
-KMltKvUtPvyZUQ42goNGsLGszi7TePLvtTZvC3yd+r7fVpkuXyHyrUA/1lFp2qUIzvLzfvkQfCOF
-Q7KEBgGVuaUgKXrfMSpss7w1DNjiUt+DghPSYGI1BCUQumOj+xSw6Fo/xivA8/1jjSDsOWiswHQl
-RFvzKi4V/ZTx0HF8uXwlhfGB6ggHfvCS77+SgHdmJErl6EC+SuA/KLINIyz7ih5Dw0i27M3dVMps
-u1E/nlg1P042hZdG1QD5YDL0bzfMPwwTDPaFYaJo16lb81uFpvauxRPyAiP0U8U7P2lpKXDWUUeS
-VUBi/f4hg2YhEVvyjMtxrKNwpQTdLaYYE3fkQ6+fv+SP85oUJjkv3JwooRWPlZKBIY5ZgcOoY+BQ
-6LX1CHezCk6cUT8ccnhtmF0oVMqg62MLWJ74h74LuJxQ4rnrHV8IfXsE9G7HWaDYDKhsF3Vz4Rmp
-n3qyGKvniCzTVy2bpBMr2Mepx3dADr0UkaP+P860TXM/BEXF7DJBbOheUPjCjZqIlGpYLRaFW6gS
-OOz96d5d1jHqrlFgS2Tq3z93poWZUqQ+/kdNgTHhpCarLDOUzZ9vhZqz5bIAKSgGJu9bCYaeu6kp
-7nHfA7OOQSXwh2IS/3T/qaLCg0hk1hZ50tHUSyYlMVr0uk40lPl5qjaSGwmYAg6YurtZN/qrP/tU
-i5SWQhduQBg56tGYkSexSWe5BdszR8EuLoR564PKO3FI+LigmLKGlQYPxZXbh1oQzFi40pvMxjGE
-KHdFEVvCFHbORjQ1wTMzbcCwf2z6rS80fyjl/+15/Pfgtbj8fdlv/v4f/P65wINzUfMf/fbv59Fz
-zbv/3v7H8rH//LH3H/r7Rf9at139+sv5Y9n8suryl8c2KvLjz7z7J2jpj2/iPraP737j5W3UTlfd
-az1dvzZd2r41x3defvJf/ctfXt/+ldupfP3br48vGb0TNW0dPbe//vFX25e//YqwcslI/duPLfzx
-14fHjE9eR8UvL6+/7B7z16gufvLR18em/duvwOB/W0o/KM1YLsWWXOGvvwyvv/+V+puJ1F9mdCpU
-lr5VA+dF3YZ8TBZ/M7htIp4wSdIqJNl//YWp9vvfKb8hc9fRbGPsjssQufB/fM13L++fL/OXvMsu
-iwiu7N9+XSbZjzs7kdG7BOMy0H5Y4v4vE4zLoP+xleOI76iVvzLiOwpV/qKI76iV/5mI7+ik/t+J
-+N5SG0dv7F3Ed/TGPon4MDA2zTPf6I3vUlI2XyDwKGB4tWY4/ywALKwEH9cZPgGe50sYiPpayj3g
-5yXOwf9yMPiT7fPHYPDDBf1/BoMDhq0+7r3zpH8JKStq7+ogCa4lqEYBDButuk6SoVDPpEyJo/XP
-A8RqytNzSLOULf6/iBKP3u//ZJR4tOP/hVHi0UP+hVEitxzvF7e/JkrUlyX2hyX0L4kSpY9H0Pdh
-4tF8/WeYCDZMoCRkFv29JlTdChQa0ZtPNU/mB7rXAUeArS3ku9+DyEEdlW9KaOqOWDfFBmJotg+L
-QKjs1q81+De5eUqicrzlvEXVP0SXR5cwf1F0eRSH/UXR5dGz/LejS0LID1upqnIMx1aGInEii6P5
-I44WTJuxJilclUHmKNYCsVH1qrmHiFtEXiw1MmyWAtdNR8Fd7TbsFtQ817Qsfwk+Kw9KGI7YKnd6
-+KQ3cWi5Axz6r7OQYysJC2ccHLzuunvOi8J1O1r1A5qQmA9UTbdJrE59nbo+1XFTy61s5WPOz9XT
-JFm1g7FSTaGBaiwAOEyqL0HYRBrlqE35VShg44Jo6ZtbEiJj6IhlIT5UPewDjFj66EYQU/M6LyBg
-OgZA3G0GtAEuRuFP1zBrTczWq06/HRsR4mGUhrjoh2ksyHbWQSTK5gDuY8Nxv0TWMgyJA9UAc+pG
-yvuvci5iTkI2Ld+LccluEyWGRg1JJTO0wxFphaNoZvmlbpvmPo8yQD9q3OWT2+jQydcDxornyjQ0
-JJEVfqwaDGQeppANKqzPMdh3GpdHC6+q6R6saRJBeBpC/FXPC3JpZaWN91aKFbSb42N1nWKd8V0t
-FT9wrawTYUhTlHQfpPUAtnaGn+pOOoD6XZCr4g120lLpzUKIRq5crMxsuRt6yc4HfGRAcmfmFdbX
-PSh6M+he6kSZe3u0MslwQa5IhxxRGhyUsGy/VnjAgiIyha7e13ovNKvF/bw4C4KpXui8rRjDaSz1
-onMWTVt0V/iVKNgh0ojY6dqcm7eEM/IaFuMk2rmiQSSLfQkPVLA60q4FJjrbU2mM2zaHUrmoz6Zz
-S8WJDOyh4QdOVGmT6GlxIapeXyvTc4j9FTh2aIyDE2d9ErtNMkyYnY+hJEH0DvMrDo9GfZAmDjtk
-fBMExi4191P7qCJpyS+5SjMBhUZqB8BHg3o2bK28GvV90la+fKbXZJkgIwiDQ4ltgLl6P89cG2Vh
-kHqRJjQgNiKKMR1Dp2rV8ecorx30HvGdJs5NuHBkDcuNupYU7AR8JAbPo4VPJDkkxQX9o8oMOD8v
-V35jlZ03+J3+kPg6c62vyvqx7v36qU20gew/dAfdHsLBuO8aa5bOunoKn5pRK92+idMbXMylm2Ku
-MM8JUdS9kBstItvHNU70ZCk0D+YwW/Rp2s8Fh+Vgru0A4LsBOKkTz9DHyvyxFYgHESP6knLpQIRu
-JIJTsA2/ZmwCAtDhVgEjS+zEqtLZzifNuizzWGm9eQ4VfZ0HjenNbU2m1DSjQ6PGxRdzLqcXOYvx
-ZUzqaXrM0CuCrUsSnGH7vLZSezbN4j5NI+kBk1pAWzhJR5nXR1o6OoGcZbE74n+4G0VgXod8apRd
-0Yv9tKQUsFoLKaqNXUyzkis1tqZkRVgWXzWFXGk5tJyqOlveWLGaokAUDpOWJhF06wHAh2ApLdcM
-wzRhGqAkrcZgtLKLstBnE65JV+KAmIvwDsJUHEEza6L/KEyKcpeJStgt2A8dlkglhSKBa6taDufE
-4gLLtQ4kkdJ2iJkKeiEg3ksdC3kRRAAdyBS4gipZq5xNnxeK5GBbWKDOSAOb7rLOs6GwDcs3LqpE
-jmYnSI1M3Ji5akBrCHxrvAT9HN1TYBa2q9HQ5nCXAafccHoza5AXg9SB8wR9Hismy5vetsq8Gqeg
-GJ10HI0bs46heeOSn+h2K6udYsc1Bf7QjCa18ay50/cqRcqjw/1afwtRoQGLZA6Et0ZWhekKVj0i
-HCxNdXcQ6gxkDDgK28rKGBp7NPj3LNHN6DRjmZ53Leb0ssK1lmMWcnczqVPJjaA6pfdSV9FLndUC
-OkLJlD2FPPez2NWFv1aAQT5XKOUqF+IquVT8yX2bAtb0mzqNWemFYQLCIU2wF7WnPCEtY3XKnJ5b
-NRwqjIbaqV41Te4b0B6H4NAZXd55Uhkb14ISS8+RhDHASg/9zKLeuwZI1VEcGdpVJRUAh7Havwzk
-AsP9wcqs26qvrcxB8KzFrkrgado4L7WxjTLFehUypU5xxe70Q4Fm8evkjwMbmdkmlvNDZuCPI/dn
-R2zSaO8yQkfx4V+UETqK4P9/Rui/Shf9axkhxEqLm+t/nRFaF9H//l/Nj5mgPz7yj0yQ9htDkasT
-yvvxunurov0jE6Qpvy1ZbDI6Iuo/LEIJ3v+RCZLk3xSq5amd0KgqXmy5/5kJkqzfuFAgpYn7AlaE
-Cu4LfyITRLHZchv2w6GfymiKONlhltsT0k/HRZySGlIXnwS6ExrFAJJqTPxyO7RjzrKrD/4Bj8/R
-WmOZCo5SL5LE8vyhmb+Dy4wHuzGk8EX0k7pca1rcBfvRwrDMFftYiHcJHLDWMcF/NE4u6HN2FaVR
-q1wFo9nPG0Esemvnj0g7Rr1yNCyx1sSc4OPBLJee3ClM4zQMHJOSu5VmlY0ziuNL3JWsJWlX3k2N
-uZCT4uZ1blXxmbgwQoif5Z45KuUmrKA8zJIGvl0e9XatmW27F/FhvcGEpHdHjWUQ1g1qVmuWdWHX
-KsLw1BoqnO/BTGrR6xV0CythLHEpV8Bts4vq9AqsY1nwdJ1UrF3mlvFF71rTevZ1H0sPdSjhwuu1
-EDUr4PBWaAsBPnmsY6Cfz+NsYSAPOuRDwubcIp1fUSf5MmNimTuBr0wL8AWWzBRp8ewCidL3Fdua
-0yvwQQjQq/BKnaQM865U67KHXCigi2ZZV7hipAG0hJHmI/ZvsgiA7MyX9lRB5m8xlQK7XGjFeBvr
-0C2TSS254q1LmYt8/BhqEuOTsA/8iV/mhFYga7NK0y85ZvAjWA/J+U2vKcO6nSL2V7EvrozBWEmp
-ttXLSH+YiGqdpMUrrxcS8TzURiBD3Ig2UAnJuTTE990k1imBY2XaoR8KTjEYoZunowSSEwaXsOBJ
-W6F81jP8LhJ42WdRGn8P53Cbqe3VZDBGbVMVAFwNdiu2hxJYnfyS6aR1MI4r76y4fjGyuE32QJfH
-2VEyuPCOyYhfW3qht2cy4PfJVeICvEcJll2yhyJJr8NiaBT6KRluezHkacsmaHZVYj0L9GywsoBa
-+Z5k5dZN2rXBE2Rk/PhbpYp9+K7dc5EoTjHlq7oHJT7rLyFUK8/M4ye5plI/0PEZCqNq1WnhvgYq
-k6Jtc8xSzbew6G+bVCztFka3U+rf6ya+ToUy3g+S+b3gahwysGpXcooErl011QSNg5uSoRNv50La
-N4Q3o2l6kMzXaQqASagKmPXEuaIP17OLLGhgIZDvvgnPsD2+EoigV5GUB/kaKCR+pbkxWvuqlcVz
-c+qrzEUzfBi7fq/oyn2nJhcpFFZGvBEjpBnMfqWqabRrq5bARcit+FJP5y9WrDxmTZmUjp8l8bUQ
-6A+jPubES4FS3RoQG7+nUsspLEWcy6BR9JU8KV8pjmTvFvyy38m6XrwEy2lgy8k1ClcZHLT8Lcg6
-ULGCZTLR7FCfKXPUXU5mNrtlVgnbIBj13G0Grey2YyZF3igvgMTrrp39ct9Jc/hUkIPH4XwKVM3N
-FlfMIFkrFVHHNiiMKbcphAYVnZlZhEtNAudrN4Com9szIVQT3G16c4oPkzok6jpC/G7tobYkvDhN
-qsmclCkQbUDHMkRouGYgLn1JLp1yxrPNseos2dRigGQFIKe1g/OuH5SqMcHg5lOWJyjLBx8n0Dwf
-b4nck/JxGH35a5EF4+1UmdwIdxMEBl5cpevOUMrCHl7rBPMxF4Zb8qf8qZpoMHBFa2JVCTBRN7AT
-bFhbisjH0yjQhgzWkmn2uleAFwq2htWqcGViYO24hkxWVK01P4lLV1VLcRP0EAXwPoT/s6UehbUv
-EZSiulDwnOVQrgy9fwELly8txrqfOfC+WIOGoJSp7+iUUl4rQti266a2zoHfOUZpZitRCCCkLndw
-JQe/Vsj1dVTj8qhXXfe1D9MLScwe0IVclkNxlga1tngKXYRy267yWYvsAZszJ9PHZ52yiivcQYR1
-0KuVW+sV5yhReuUw2K9nodBWWuETOetJ/E2sFN2eoiJYZbk/giKRL0t/uF1QkG6Ucqiy2jbaJm0x
-XwJANtdCJLfexOW2WxbjIQrrbm3GGVzBQoA0qhrwKUiLXfQz8zSs2/oCkbsJlNoyDlqSmU7fpfk5
-Q9dfp1EYe36ixqssncczKdJyl0PAlQQHwsE8sHcjvsQWa6sveRkrXqMr0Y4T/eDJVdmtZysczmYI
-kmtTyeR1p02P8VDdV7kUOIOvHxqM2+yKZMNuCAbxJhFLV1b00E3l8i4vUhErn2LeKLqp7DU+6HR+
-EK10DbdLXSQELgx2kZAhvpIa87vUmXtRoUSm4qs4El5N3+agC1wWOUTFMOpcvQyzO0J+SLw+j+7r
-NRavcp2v07ATr8pSiFfmPE/eHOEaFArPAXtCavs6mMA8GQ4hqKmmy0HgNb5JAoJICAcs7dD047CP
-MhEQVOkL9hDpMcfxONsgVYpB20dRc5OKWXzZcdx+xn4Rbju1ndBoGy71vHkio8L2qW3CTB4Pb/NB
-KgN98MgzxV+p2khCGyVSvZIwK52d2eyVTV3E2RczMnTKckaMMJnKc7vqhhahgo8JylcOdu0e6Qoo
-1SHIMXg0oazdSHqQ3ytjkn2p4SY6Pq6TX0GyRbFtjqO5Bq6nXLFzVKMNdrB6ZQylw07Jo3bbFWJ3
-r+Tx8NK31cQlCBmS4lFlxWXISsFVKM3SJYUSeeeCfvM9KwH8Pc2F2DjTPL8KViFemrOe7jS5Etb1
-OAnnOhGX6U5BWd4kpGgSTw0Rf+zyQBo0INpq6xmRr3BcZbHKEB/KfqkfEtjz9wpSCR3+5CX+I353
-J1R1IXOQDOHBeX0Y6W4014PhTa3sJ7YcB4X8nFDupLpmHEY3JEkYvOREMDUa8y3qiKrBNzkTr8Ef
-Sk+4HaUrNjvZ5Vwl1o42dMhNoGoZbqNM7U0WWtlj2+ul4pZzHVSbqktLLLuSqXOMypS+NklJsiHg
-5LydLKvyDD+rD6RB5NjGJSW5GrFGfRJZ62rWnKmN+Z791K56NRav+igp9kRDYuZOxqhdtBCnQcKr
-M3WIRtmIT4kBnG9raZMP1BSH0JrIQ7AWNmtPTA4odEF8J1kQvAymSMA0aFZbuIubZL9KKQzcQYjE
-oSroWZYjk/g4mozZoQhRdg0hVaCVZkYWXaXy/Kw14ZcZRaHTq90u7dONH8702QyRYUu6ouLGni1b
-JUPjgonZ6+J8qYSEUyLU4ckYnhoRHK9dEQgzr6bYJcDx2MAOnTaDaleVjKWdnCELbUKYuRL6mPUd
-QAz7fEJ6BnyrqMBHN4V2WHHhRihT1EtAhzqpHjx1QN2xQ8Fpekndjvx7uuI0QX7ZVB0o9KkeCQJJ
-tuEobtkqQYKN8kWxW8J64MpUozC1SScKOsTsmSwntVddPzvWGOVAUmUVLqupwTQjTC2ts7CKq/i+
-TgKjuspnq61uwK9H00ovrNodFbOFT4vOEZnsIA9k2bKOFEq+xp4XukyrTneJhi6xVag2eInDBjig
-GXt5Nat2VnTGQxdkRmHD9WnbS8FUlkOCopTJhqRYJtmcNKqHvh+6clVljfCS+COdMeXZbHCYCMVi
-VYWYn7kVBusv5LXvtVg3tqy96kVlzfplqg+y+ayi2Ar3o1p2D6oaleumL9pHU6v0akVWVPFtvNX8
-C4ha+le58bVDC2iV7HvhHzpfman3hXsl7MCNJKGnmgnp0BmxgE/IAAvlPJKyBnCyNWXpRVBGgQUe
-IhPO/CSQXpQiKpw6El6H2NTsjpIpn6R2gx2X0tf508BTvpRKqn5LrMy/tirLdINp1M/Laaz3ee53
-s1tZ/dKF1XMkWMPBInNJ1jErtpHEySTTRmNVmiwmcWY9kTzq1mPZabuYPPumQirqKmMJ3oGKyYnY
-r52EnRhEwoVVp+qGzXzYkc80V7BkzqqiI/xN6J5SmUjqA//yhDEa+dYWpUUVR5vbXNXM52zI2muO
-upo7lSoQ0ZG0GVuXvteqVMagvNIdIbPYgqLC3Mdxlp1hxU5pLAaO7Y2pdpkrVGUuOarCbGxYuG8n
-ojc3qQaTNH+ddh78V4k0f9nUcEI1NLut4p/PltDavSBmmwk89X4mV3xrTEazschq2VVmoCarAXLy
-xDFp4moGNTmamYOlbeAkZRtzUhNY01WlibzJkkLXR1HrqKQIrwuuNG4UHucWga0c2F1G9VkvqMYZ
-ylCYs3k8bmapym7nWET1GA59teFdihutMe8ptoQWOcqF24RRci6bkGVTfzZsOaXYsJHmrcQ3POSW
-YKzZdRRqbXQpuRKirNxWQS+5OeEH1XWQyY24Fc6MvDA2MRbbmxLKtJcDdV9XWCRCI80YlpkkZ7ep
-VRT3VqCmW7G30N9rZV08dXEyXysAZ9dRrhFNEnS4jdgpF0IXdDs0LMLB7IX23A/y1Kv9ktGvNflF
-0JTWc2TIpmvEs7JNtL762jUT4UmQD16jhIXbDUbNHVQYszK1WWOHhlSsjdLAe0Vm389QDangcXte
-hNUnrxymzcZO265ZayoU1XbQlXVBh22yKprXfWQNa87YsReYLVLTMN3FVmPt005U3Mhvqh1gLCrC
-paDam5MRrSzDTx1hSHMPw7JpG8uAEvRQrNGwUngsFum32kh8L8uDwFkcl9cBAYvXRpPmjZlfKe4c
-y8ZGt+ruiaTH5Ji9r3AHEI+j19TqIvXydTfXSg49bViErimF2UYKu+uQAv+LKfXHFaBJLbHFzCqe
-zDwSPbWZx7UwxdSP6HO9oVJR37RWnt2YLLX3KOHNbYqq9lnq5HzdVFbgRZYo8xCtsDJLWbyNteCu
-zdTobCDvco5MKN7IvfA1Rk1917SY/HMUEHjv8W0t664whDOvojG8TjZbdMqso0bOssMue4NXsUwO
-VdVzcqhiE1wOg69tGkUctsypwCmDJiJyH/T9KJsPvthqhKc5F3BtmK75lL+VooSdQlrAWHK6KtRW
-2QBBSx/AqfMvqxpZIxH4KVQrqzw3rKraDoUeuFHWHfj4fQjXwsm0wroDGbjOFmySNGpfRlSIXmpO
-+bWK+fx1I87QV8vS4Yv5Gx1fZ08ijUy5J/XOwfg4x+GDIArGlrCwdFS5L7dpFX7RpD7fNWCgt9ps
-PQ91t08DictCrZQ9rQNlg+v+bM9dF7tBYzwRKL9qdUmYMyVXslqGa7aadR6L1VWVaamL1nPC+Luc
-CZpM4YLDh3IJ63C4LGXEIeB+LM7/qumJkLVIWvV3nKevmWnxatB9EgnTUyK29Vo3QvArA7uxqCO0
-jPv4zDTC2Z0H7SoQh1d5LPWzyRyUTSWmX5vJWs1hkzohatB1WgMdLtSFI1EFITXJ9aUux2hhJX+l
-xRX9CrnsQidz5VgZyZxBNM+AbAxuq0iN18AnP+vlOvYSKyAGDsv0gnujhLKc7qoYi+miURCalkZT
-rhiRm0xgExGk8atZ5d+SQQxdLEfih7yUFY8NzbgbmF2bRpi+hCWr9DjBu570oNtnnXnei9kK722Z
-STbw4/+HvTNrktRI0/VfOTbXBxkOznYxN0BE7vtWWTdY1gbOjrPz688TqdGoKjSnZeqWemzG+kZW
-pqrMiCDA/fN3NTLjpB22DKCtfqDowN77IIixmj33ti/HOKsgdLZ8ud1asTckMRKmoKA2lcWFKuwh
-HNLqY2u0xjMK3BtFnEFIm2wSIYX8LPrlUElegVGlEyV/a4VPovE/5M4KnKFgTfODXt0yvCuEQAIh
-xFpGmKPNa4qfiijb0ot+rpZQQ4NGXZ7ewjy9Kqd7LOGNTurWO/fNAbgtz70wwOjLWSm4LoLtrHXs
-syYz8ji3uN4G70lky7wvl3rvMeqFsyAtwjTViysbCFzV39cTDv3ELPMoZYmJxq53kb+aaj9X6V1h
-5cCOZkr7rG8toTOOJ+162P1U+1zVS7ob6uRyctY9Wm8dWW13ooztJmggnOgrek0Pjebt2n2goC9g
-Ye3v3EVCQ4tkeV6g/k7TDvgyCyaIWWJ6X7FOfEmt9rroAnnqVAFHvRz3QqXux7Z+Uxtf+WpeSD2C
-xI0GU2edq5Bs2DzS41K+poLjhabekITQveu1XezXApe+GvbgQk1U5jMW26B5BBW/YYRb8X3hMy/m
-LN0PTnDWevVXozOg1qcWUmmVek/gRhG1xpJGdplddYIY1Ull57X2z83KkGd6yAmU0QwNMw3CO+rl
-KcpTeXdjHAJRvdwRbOabwhokhiFyrCTYu2POv0n1U5JK9rHgcml0vxuRQcRJut53A6e2bkseKQc/
-r5Ly2mRqODMMQ3NE3jYusPWBVfpjiSk6Euvw2NEywBEa38qUcjlQh3fRUC86GmBy4y5tzjqY/XVO
-XjK/ecr7hYRn1Sw7d86epKrt6NDtya293nVBYJ+tSXPujo11wrSb3ww5AbzFdgZgd7Fa5WW6NA9Z
-Y9Ppbl9MAMxR47O916DP5bajhOMs95uzoCv2aVBclh7j3JI6YZGnZqg2NqcKqKHMge1Ngphn6VJ1
-VnphhutBICsgcPhMrlkZDoW3k4C4dePcmnR9nsxpAZzg+DczxcSgPCeCXpnYcrZ9Ovk6SnTyLWG5
-i5LSP0tUR0BCW4mo44SSh07SldxAa35upOpia7xvMwf8aMvyCp3yEHW1rq76jCFIGrE1CO7Y5syi
-8MIBy8naPK4LfdZOzgUuAB26VvVta/T5sJi3Miivha4+Fr3tXKVBku1BXFkmetAswVSV92SM+Kl3
-Mnn2NdhVvxN19ZGQjNOx+rqWM+2wy2k3ba/5an6sII5tZ7nYFnvPz/lnup0e7NxnAu/Lp9oLLk1c
-EsG6XcHuv2Z1ExET/qhle0rUahemvsEDipCGP6nr1nev8sHKrtMye/C8aQrTJL8c8+EBmQTYbpaK
-+jH1tHVKkGmyM6z1OevUJ7cL3Diz6J2bzVI/jDM52ZDpfXOWv5/kVmfKrViSEO7vOdbW/ikyj/TL
-6tEbH6naKu9ygp3dvSHkkO3z2lMLBzcN6jebrvXqB9mBaFjT5dPM/25C/1D/eI/WK7PjPqn9E29J
-+PHO7aGVJ1+UpzqYQL18anR3Jqfh7HYou9SPUMaM2YVkqc5e1CDSUBnqFJo1CfMiK55ZMn3rcaKP
-t4pd6qPpbibu/oHyibmI+75CIpBxkPAbBvNqLk9ULrd4yCRmXpW0FIGL/Kkayi2Ig5mY7Y61mAe/
-9+V5hwMXaUY9jVUT+2Pryre0GFI67jY/e1gEh6oUIHmJ2ooyCb66Wn4mbt8Yw8DlqXwwg2xYrgw4
-hLN5dvVZkSuFkGXwvTO0DZ79s1nqX/r4H/Xx1t9kQw/6+BP9VqOR/9L8n4ex/J4YRV1/+OlfiNHg
-J/ItSCPiZERZK1nD/ymRd7yfMBMFB98Lynlcg6h7fyFGLe8ndAP8nIUCnuowCeH9i0Tetn8Cj6Hi
-3qS9guAmTDN/gBh9F+n/wIu6VJbAzHpYgXAtiuOEdP6yYFwout1gE1HUpS1I+Lw1UHqbjVf7dio3
-CIXIrWRPU5Cr0MShT/BhcUogncpkxxuEWvWDFaCWRohkg8NujZPqt7HXhr7dkt4seuwohI5ku62y
-1+yNgccM5NlcIuh89ntzBp1yJmdWV6anpFOeiq0r0aCJUk+MDJ4xgW/UVW4kSGAsijMRInlOnXyc
-65rDZDoug75gchZDiP6s98E8zBG3NzJo/lvXtXfl4Ce+lqRP6dirU+NioeVz3nMcTqYYLJ/fqIJB
-X/r5qECz7Gy9LSt7/rZVhPxH9uCrl6JpPB9ZkAB7MZIm8CO8W+a5Nu0hiYveS29WStlytqfA/WyS
-Q9PtqzwrgGRKFTwgwnGfk0brZ5UMzcNapQ0Dg1eaCLvQaJHY7eYPuSu6G8/rnCuuOp653JzE2Sh0
-keztVtcf80I3T8kK2MmRQulP9oYxLmxqnX0bhkFzit+obqEv45A+QkuZ5jxO9VUJ3b2wFRBC/qbs
-TMKieWbypbNrfbeZduseTiLGuBuWtKJiY1HtrZ9qq4i6ZYb2KBOZXBY+gAxlcs36nDsL2HMZsBlH
-hpuPHmUjVpFdGIoiHz6+ZV/LJJie9eT51PAi2rTihI/2kA/N4O+dxbReWlFwIlqaLFp06eKvpFLk
-0oQRhkdclvFidddBggJLUmg8yIgH1l0OUo008hs1yPTS7GFIa5mMu9Hs9AtCOgWsZHPKy9zyxeGc
-dqXYZVxI7SmpEEtx2g6NYUzB99j5K6iAsryk2QEXWGUVWIIHt0rLSGU2EL+u/PumSVjQ9ZiZt7Va
-t7ua82S66+ZlmE4Zhc0v9AkJVFdjs0A2bYTV9x73HrJVXyMMEpVztaalC7TdiAR5aDcjJ8v6V6Mr
-mONIDRQfSJOrDtXLzTKH5bhA3pFL1Z6Nk11SidCs8sGdvfXGk9V62Qc5aK8hiupBDQFAzDJUygtl
-4wHpmJVwMDZjIO9C5RbbV+pRaeJIC9P4OHrD9JIWbDGh14/FY00t7UMDHIaiq3CTK9kWDQq82bBI
-RsjqSiK57EsRIvrq90J7HZI8VRdjyGxS3rtTPX2y+sFe4xyi5oZ6qu01MRkMSD5c6sfSdO27WU+W
-iIu5tK6d3GNA2JJ6YddekaVGyrLSTz6Chs/EXsnb3DWXNWwM2Mh46AAswr6bmXis1k1OLUaJpwpk
-8LEXU0Wd2TJWH7rcAE82tC5e8kQuZQT9tb4xeNC7NOMY/Tyxk9JdBCCKmDXpnHOsgMzUowCPQ+no
-mq8VhV0fAg5o227wNnE9bg415h2pkpEyfOp6bB9aOoRhXlNC/ibr3ECYzD1CGBKO2t5Cf5uNqH71
-4kKTZMLY5qgz1fyJObhjbO47NIyg67qOq7ZtbR6Rub3kOvofGRuDD5WwBxYuoxiW3ZC2y7ObztYj
-5YxJj0ggb6+rsq6ryOhgWUJjzLtlp0npKqNyCHh+W/7JPU1owLst7VO3JF5zxAxK7RoxrMghm595
-u+B9GN63pdTNcgJTEai4FO08RZkc1AEXnDZifDy/PXHbqbMwFW9oFDYlbBSw66G8ZbRzJusUSv96
-yB0DCFyVwI+yzfMPmjyqxyApgttKWZzi5iTZDDCuGdyBc7hlhouSW0Mlq1u/QZW2r6aV2VzDBptN
-CE+TfHIPnbqMp13Os46SNAizcTioXdyqiuDHSfECnCjVThIIV4alZ0h7JyrfuxGIEhAxyHE7I54i
-ZWYn/ciP/S2zLvtpk09poQ+kgHbVBbPnuO19jQ0zFMDX32bbdy9VVw1WDN/lebHyLZsYHkstU+QM
-HWvEtK3GBwL35usWF66IfbWJR3vxOFZ0BZKM0HJSZvOZSsMpSpGL3w1FsjFyqyJLdkki6MlYTct4
-mpW9PXGQG0VkiXGhs8a3xjfS1+wugk9fdbRB6yRhp1BU0MHYtrfwaW2Yt0PLyrRshh3awrBPa7N/
-rIpG80TZXTjVxsTKKCrFrC69YYunoJ2XnZjbDTUKEmuGysG29mZjyfQU1Di4M2rouygALrIu7GlW
-z2KbRhDcYV37nXRnFANWfjhj83QHN0MNJxSng2H2OzsL6vwMS27T3G3F6rQRcCYEs+/0b06HpADz
-EQvMrq079Mps5y7TLOB5gpZpHN8mezbm3Txqke/Z7DnCOQvbWWSr2YA3LdBqxq0aDRpgwOs/boAV
-5Q17kch3IwztFFXNIDHr+iur0Bx0ljovIYSqq3lS/i2gLnZXG4V5yj9ccuvG3GqU1+NmTlyczq6+
-iIJdaL9mW7LE6yIyixOnkw0x4mH66CVn8yz2xl7Oj3kJ2xlWZWuI0APAvVedB6La5Wi0o22YqKBa
-C119LeulnSKV1sE98qqBCsBtra5IMxw+JAPJVdHa9O5V59AXGtkbZciRTyScQNGdiPtpbEAEDKQF
-1yIRbRcu6YrRWcw0dsSl6ZRfmqRdn7TDZtc6fm6izV0TBcY9em/cA+03n+R0sjoKIe+3EQ0vb9CB
-fR2YJz72w4AOdeqmGqXWpP0b0dqdOEmkv31Mjdm8YvKczAuS0ewvsyNs6iGpaO7CrszTs0Ta2Qak
-Y9Y3K7eeiIhiGNGzoqLiy8wqHjpvgZHM1koiwZAmX+CEwO+RYQ94CB8Di2dx8OwawuyfOqugJHnm
-JnigbHQhLAy3wbUY7RKBhs6mu8GGuIyEX46XfavAw5tElNeemkEhSrNvpnDtSGCMC9fIXnzVaaRC
-/eildzOE8xcG6vnBqvupjQqYTubTuvDvYJpTLg4FaDddWVGcNHH9D5qz6WZe20xH+DdQzRlG099C
-fyefi7bdNuRni0HA4+Kz9/VDWr4GGft3mLbZ6u0Sq0zZYHOvL3dM+/IzpLJfh4TYZ4+ZrIcqSs2g
-e3Vo/yp5dmt2CdFpESZJ4fvh4s6sDXQMO3zLjZgeu6WqKsBjhZEjhfkdY8tY+2/B6m5EFRV2q6J5
-WrnYTiqQq7S0hN9L1eNJQGbofnJ87d21dV/fqrX2bxOzzxOuXArXzk2udyZK6o1citYG72OVX/dW
-bjv4XJahfPPKztx2W1tXxt6g4CSI6w02qkKA1oLTcZx+CWD2qv1i2RT9cYz1uxPRdMbVbAG67FIk
-WWXoDymrs1+mYwcbuLTipqf85kuxeU0RyV7wr6uyGk9B6PszkstnarnBST9sRdHkUeDNCQCn4VEG
-2Xu5PFk3J7OiqvLTHonLkutIdsV8u65SzvscrfwIgWUZgOQOQ35atibBPG5uGBAorXgt641aHTwl
-Rv45SAlsDkcDX0qY0Hbsn7SdNLMXD5Q+iF1VpLPPtzDU+cNsS7TgU5oK2i83t0ifRo9XjDVCRMHI
-nQqJFGRDQ1kGzs81ov86S39/lnaQu/wtZfHtV12/VZ/QD/5wiP75x/7jEG0FPyENJkqHPBjkGPSS
-/+chWoqfbKS+h/wbesV+OERjThdkAR+MvjYgEX/89QyNttin1OUQscFKRtLMH7KZv0dl/CotdnhZ
-pMW/9sMcR+T85b0MP/qCf/t+jg3c5h+vojg48f7WRz6yZP75jQi/V/HiHaUf/QMVL79XVHKcKMsa
-/z+4qOQ4EBUl9t/VWPN7VQWMtdxDn9/uFXarf/838X8L8NL/nVUFv3sDHfla/5yuiN/tDPGPzDn/
-6gz5qztDDp78v7FqHkw33z8RffePljj9XkOPf9gqvnsGq/+hDT1HuWi/2fKO4+L/cFsVoPjvfHdH
-O96/SuD+u0vgjlIjiMczv+9jPc6l+6f0sXpHKz109fDn97HKo1f5x/pYf7zx6ac+JA7+2sd6PC/8
-nSWph6Xv16Xxt69yNCz82a2v3/exHr3U+Pf1sTrvhZo/fiRKOQQnl0OHBSzg0WoPT0abhuS0anUw
-C7GVecWMxWgzXog0qJ8N1ZB9n6UyNfag/tPVYE3WEHfAaQi2h3J9pnOkWKK5INyRvPrReSONfxG7
-IVHI2ol7dytsMu40oGfKXIgP3+iWk2Vb5jyGxIYa55ScV3fZIkH2vXpN0JX6rqzRTptNF5cBvbr0
-jZNkEfW+j6Z6FHhdONMXDpqEeax3FZrM01Xgcd9p9yD4GZNOipOgtPrnmbbl7NyyEKiDQNIFvIzb
-/KXxa9IyZrxva1hv1UFavWABC2djAA2hPcVb8bWhrDSNcXm2e7tqrhCioFfaMkTppDLMtBnbTrbO
-+95XcIADDOUBUE4RdLmus2axRN6qY0M75oD2ZANsU5gAn5AheklYYfSEJ3KlhYfCTRTqIkOXemcZ
-XfABK0732mgIkZgqp2ajLNcuSPf1iha/TxbIq6UwZisi2LET4ZDZRFQUhZ9lsV0WwZfNHE2oirbB
-w1+TUlCF6wLudQoOX5lAPVtVXHVg68SFGCvSHaiT/I7mbmFA5pjuN9dtxbcq76B/GI7X4IquUV/u
-1tFSRoz8L7gecD/ap2WjAqQsju02uzFv9U2J+gxtfFHJt9pK24fes8pX8Izyk64df4097U9jDDiW
-5+HkmvnVKiQ6N5khhnyaqgZFkltLemUHfynIpFic7ls9TFPNJw1m+o8tWavdAQV70MW0uFiYDu+g
-LprsMp8X/IjZuNlTrOFePxZ+UCAsa6o53ppCEtGXCi6L4v41dj0ZFiAnwVy+juNkrREhLP3V5JvQ
-bGlXFWVotzKIE6Mk3RwkL90FpR2Up1U7FS8BAnYVV3xdW6QbfzAjwrtBMRWl5/BadhE8VH3T6v3q
-b7re6U4pHEPc8F+R+ftXVZ5aoO61D+2DpRORfonzpTjts2J5JWYSLQ4oQ3VJRdVqxA5a/28Y4FIZ
-cisM9bV00sA6K/p5LCNAyOmO+qDgcynmgayWTc1D6KuhujfQExePy8Q9sqPR23haYMMhZJoJv9bm
-G3ddCuO8M2zsEYVTV/Ue5pns2MAZiErseIrW0DWxDTTqIGm3+9XiWTRhIyM40OTKtirUj2WVrjnm
-K6sswtUwQA8zKTE1aO1ztcSQI34jqnQM7WWs70w8PxPe/3rKTnXv9fpytAen2uUE/5txsgg722so
-uzkkRSYwsbp6pCFsVtA+JH4VvOSmsj4DRfsbomine0CTMtbXmkwN/IHdXONotRbrdEiS2t1hGh31
-XkmjREdY1GZITErRnfqLsj52TeIXUDmk4OCo3upL7QUez/00mvf1RqRgGPRjDtXiVs7TAFUW4LYp
-Id/nxaufevqabMTuclWnkHwr/hm/1sheRoUbeGZN2ULDLkpsMwC/cbtkYxf3i4Sxx5JlATwvnQqi
-stbUHJszUu1EYKQ0a12jowFjR31YN6gZDAJ7PgVduyxQSBrVfZOp5HFsSokjuOKb2NoNUB1sHitG
-78+Yz1K70GS8UbmyRjxRwJRuW6fnGV/8N6tNhovEWNGfSXNbHtvWdL8s/UhAsEiC4QxuPyDRpFPp
-YzDZ6mPWmN2z9mYHc0C6Gl86N53ejELSAZT5pv0guwMeTwqJ+gw+TRIEsibjyeSRfMsKSJydowvr
-qiw00HAvkgqD5oSCPHRc1Tx5i59BR/iyJ/LFTbGyqnx8TVinrHBM5+o50/b8OFQj2tFlG9r7zKth
-bMu8Q70hS8TheH6z62kajQ1Hppk74VJpX+/dElHb0qHV3WcJRrEdFyBo9y2C7gy6IUiecFcnZInn
-hf8VuV31gGdawNphGyGYwkzwpaqunU+1sabjKc8Pm5YaZXKtgtb6CiDdjxhcEvS/70rPeeQpPyvS
-wnkyqMJzEFWaLrEbuIrPCTWXVTiRVPpSp1wjrns3Xqd543ZnCRK/Rx/Rx+FqNnKNZOWiZEyDNne5
-UNIneaY1JBqLsr1YC7v70GdohtkzFvj+pu3VEjkoLexQlv2EkNXvkotDVGl3btArhlIXgz7alBzB
-pmPDL8XYjDcilom1kqjHp6WI0MWglTd8J/X2LpHBz56wDo4ARAzJdTFW9UXLmomKsRt1ElujGvGO
-OfJDL+Z8gj9wcAg6llu8zbC53CWZyF56k7cWKbPKTrapwTU6bV3/xVBb2YWuXpI5nvJ6ZKHB0DGj
-5qsGfEsSnjWEfuHzkZbC89MNBl98h4DhMwuPY53RxrTuqrFF8mPWmQlnnAfGp59tsubSmgJXWA/7
-4AjM9YXL7UbnUSlx/lSsNBi/3lV5ssaAP8sS8xaONuz5lHOP90YWsEfPhlFl5D8T1HMiBL4N/OKt
-U+4yONp03xR9WZ+nIPcUruD9q2OkL9kjCS/kW7dNH3wzAsQKl/yq7DH3MTlF3mA041UeqOxGS/zr
-YRVoB8J/tZrhhOaArIy3ytHLDlMe0gb25RRiuphK0rEtrAYwe3rDhjdVtcsD37vWae9YfX+fosS9
-EcOKfzIv0/JyCQRpRRYU5MO65EOyt5pWPCXcSGI/z3m7YBl9CZqc3DmjtvmQ2qqLz16L8i5emi17
-WlNVPTXTVtyQRWDfwQW3xBF10wnckuHHZZOxPxSb/ZWMAr7yweysO98g6xePkQ3dnlqJeoDfKsZo
-CpSLN7PmVmkT5ZfxKrLkY97Cdu+JYsjPvXWdsD809VDuKjnOxJi1rggi6GK0oKQDJUjHoZULhBkm
-oWOIWpiU1qyCj/ULT3/AKMKeueWYgCKPh4/MApq0MOaVWG22njsvZPqwX5O17a7d0UlulrXhrusP
-0QyzaSGJ79f5K2aW+XEl0hnzsDEh1V2LOsHYw11/mfuauJzRLL6MhWmnseEmza3pahw1LspjnhAT
-NxZ7+qj+YKmVDLhq1MkRA2LSZEfkyREU0o1oUzPvQ6AKAtJshiFc1L9XC/abY8zhRch7ZuCHFXDN
-Y7yFDnrErOw+bIHBzu5s59zGpA+tqBWb9TtV8i8G6QcGKeB0+/+PpgnfMkW31M/Jx+/xxs7hB/6D
-OrK9n0gfhuJh/KO+QB4g0F8iit2fHCoGHOYPwseRWnIM/EV/6f/k2IQQmhQe2rYnTYvf+Iv+UvhQ
-TtzLpk0QtsOp7w8F0xzdL9jf6MsikAbPN9JM57iFZyzLJcCtPId2OWYRPmD/aRnmOcJTkz18d11u
-fz54/q2opveXIoGHegqLesPj46jNglzUNgOyW+k+JJ1fxmNpiN/JlT9CC94/0Pe1vEe0zF9Vy3uU
-TfnfXct7BCkwpVp/VS3vMa51iDDMvb+ylvc9Zv47oOPwnf/Qy8vT8j3I/F/38pI0MPY7nPV9H8/H
-7bw6HY1mV09SWLs/fJf/UJx79E104u8qzv0vHtsfXuXoE//5TcAIiQ8wErDVUc6vxjL0F3T0Hm2O
-f1FH7xEx/c/s6D36gPU/r6P3aKn6izp6jy7tn9LRexSpxnP/Y0fv0TX9taM3IDWc8EwxDv3Vb5t6
-ha+QiE99kXN+KNx/uK/36G0QWfTX9vUeFofvOLV/Tl/v0Yv+I329P8pHGHv4Wh1b4A/FF8J0crTi
-/NrXu2x2McY+8rb7P7u09/gh+ftKe48oocMkSNPMr12wR8v2n9EFG9jHe8XhRemxogyMYRFP39Hl
-FNNardLGNGPNWA7OqfDVokfMRqn312q0mvmamCaSShq08SDKHY605GwghiB4zJO1wkuY97m4D2iq
-MePUn4LmNPfnbHgos2Gr8CRXk4FRgrSfV98pTETfAY5G43RJvW6+aKwlAdooR2/+WA9yQpU9EHq2
-3RI15+ZDRADb1n01+oAAW7x5xB1cUVWLbUJrQIfzIh3sEZfiRE3LjcRAX+97XXNWPeR7dNbFdMDi
-ryyP0+ZVRiphuxsrSZqEg4i8B5bfivaU7Az3m1P6WY1TCGPsDiehYUUuuA2BZIQCIgnX1jzcprnR
-ra9tRuzGeREokn4Cp0zWSwkamT7YlBmoMCjXoCYqukMWnfmZWnfEIWRt1KPqe3OChERkU9p4guih
-2l4rhZeESOlMElbnjV29IyB4MXc4Vzw3RmyY1FgqAPueRwtdcuiNU8b1U1AGJD4roPit0Nuzo8tt
-PrHIg5ThKAP1KTBcYnjXYe1umtHlAum58y6HTaHv1tg0CUExDIKnAgKIyfpwPHPnE6sjoyrAkH1v
-4T8dPjEE9ZkZ5+OSzffiEDnZ7bq1HAmLrYFA19ca4CrL9hxYk/ZbZ47ZGb3Cy3g9z5ODgL5eu9dJ
-A9CETeNXH+dOJl8KAA+Jg6aqRHy4SxSmjXn8POMIzDETbFjhU46j8mLzCAkC5JDO9eL4uEYcgvLv
-4IVQ/zZpK9urLEkqrnewGnuylFPoB3+u8V+3gsC/BQEqamviLr+1eBLJOx6Fh1EYQ/2buejgQYpV
-lJE2ZULws0MuftRj6iCciyNPEzZzud35FulXJ16d4YIOkjz5rJZeNrBliTdimtCAGx0xwefgh8PT
-Icl5jketChEDdhrPM8eZh3KQiu+rkvZLy01IOMmqDu7N1kufuwSf1UF/XjynSo0ZbQHEhUSDlar5
-sliRIZvV6hzCAyfvxFmH2QxRnJdPdHhPZTR4RnadODqQoUdbUY2tyeNb7OtDDDzm1azZDb2xlSfk
-JK4PiH7JLrPadHj0PdgFcOtmSTCD6u2lU17zlbb6qYpZeWF0FunjJKkCx36e22IwQ7s2qzNU6Q4B
-zaLiMuZk6V21nSYaFKAMF2opyCcMR1N559vUkkAjTTTkIT18LNCUxcHV4BBP9UkgFu7G7Z2Vat4Z
-KhJuYKtsqbCuywOJ5Ru2yuLxndsiiL3FjO8WcF5Fssqr/J0JM95ZMcB0GDJZOZis4bO6V/tAofnv
-bJpRaZg1IiWF3iUSpzt5f4Q9hPmBiOvfOTlCicH+CFSFq+OwDW8XvHN44zufh6EObi+v/Xneq3fO
-z3zn/zD8wwXKd15QHCjCzMjqGzKh4A2Xdw6x9Wz4xOadW1zeecb2nXNcD/Rj2okxApnCwDLztrLz
-FoDsueLmESdGvx7cUWLaZpJCCGIDvILj9A50J8QUzOfwzoL6soOoIS4AdpRgzbqLUwXmjLb8wKCK
-NYVNZY3Kqru1UbCsBPJMeTwnVrucdO9MbPbOyq7vDG3mkakeuraexW45kLiNs6jszMTzR9ZpK5fn
-bmpgfMd39jej1u+qDGYj2QNmww+33lY9D0VlvFgDaXMh2aVlCm5/wMeWd6xszStws37KNjfEytPe
-WmDcaewcQLZakU5tDABva2KAwXXveByLSoPVHpn1I4Go89cZK/LV/I7irQdAr6JjS7IfAfWZ76jf
-9I4AQmW51/47Lmi+Y4SUFoMX9tOgP3A1QBE95XInlO/oYvOONNbvqKNRpEjZsVObQUTuKshkhq+y
-3PnviGVt0YMdrmteQkwZiZOeBok/Rj1PYH9SO32aXgf5UF3LDq9h5HpBY4ct7O995lLhgYi+xhCe
-jGmriTMx1uzUTMyhveysTX9wnc4u92OlVvr6ygOU3i9d+mWEaaT4NK2tPPL7nEzZHmZUnZDJL6gg
-8Bc2uF6YWENTVtFHHEdqJpt3zbJQldPw5SCmx6qwTM5NYQhMjw2LRBmPJiFqsW+1QKc93QVs6uaQ
-vZCSMQaRlY4e5LrtYOtxZ/ooSZK18wdh5cVXQViWFRH5xYY+DjOt8aZWK4r/9sB72WjSY7mydJ5q
-d0Pzj8jkCZq9kZGk7q3ANVMNyY7Hjj4L2hiHeBlTWK5VkKYTzq7PX5K7kn3M8tX5unjCIMBpGHII
-f6kzEVdb4awXU9MXzm5oNdbCIbFkeT4Gq72G7JL1B0u7uH/BxC3/lLx+LaKm7oftce2N4JG1qLJB
-UxXJMomxEboxmPZnIAODlmJ7OYTtYcAjJ8IN7GtmB+VF2iK0jsQdYmgmy3N2iTP33SlAGKuwUQ9r
-c6pNo8flTsIyP447/15vhwCV3uk0iHyhtkdNJvXXSeeENMvDE7SlfSZOtLUO2D1Vfsjgacf+TrL1
-EfKAhmyN0sYF6x9K1/raJmsg9xZGM0E/QlrhkZVZ+sV3Hcclf25MbtBCJOV+skmGjXqMAhiCxOIS
-TNTi4R9BkPGD8I6hV0hoeEp1YmKIsQbzdFpabHRsff71rNZUnKV8J/ne6S3zhECc+kRmE1FHluUs
-n23V4ZcsCDzhWafzwYhpkvbcUDiS5VwamW7DyUIIwNvzFvaDJCM7oCgxM/fSO0SrOitVyDVFoOyc
-86wjf5Rpd65kZRNPZjKshaTueZIU50NRBPYr68nVxMihLxDVJwvDFbHVXcrlwghaPRN6RyxtO9UK
-r6tpGgnLQUeQYFYkVXtTLZwa9in+kjm2zb7o3vhd1bILNOEbsWMu04ECJTllr7UI+JV1WX9aDIu8
-II9UCxLWmnEWPCgGDSVhNfVieNn0yiVK6ro/gWgd3zosr4+Ut9G8pWGUSEfQY5BeQTzW8wnOWC+9
-oHgkQTfh1Kl7bi6W+jK0lsSMKTcT1443h5uNvZqU5kSaEakpvUVoNJQzjnVBbNdSkfmgC48A3aZ2
-vwVNIotT0c+1IqUyr2qmyT5NCJArtg9Na9uXi+u0t037/7g7k+XGkTRbv0q/gJdhdABbEhxEap5D
-G5gUocA8D+7A098PzMq+Wbmotrq725u0tIhMUSQB+D+c8x0cRdQ/usuPbEULN0wmAJbhuiWHJsHW
-MVx3QM0OZ7LDjrcPrPOQDOk5N/LunOqSx7dX+B4QuaY2qRmjwb+TRqO2VtBbR1UlQQ40sLJeUnzr
-OAA7L33PnEY91JIHGHbCyfi59L2J7EdM/udisrsJ+RLsVzhSdRf2g55UKA2LHaWZJNYDsTjV6kpW
-3llOcfLcV1TMGKqW7gzTJsk2oln63TKp3N+kqQshyKlEZ20jTrGrKcvjp3SS3nc0iOExmQrvYVki
-8wmtSbllSI3/S2KY5PshkvY9Ijz0VE3m8E12SWlhy8kcChdSZ2/F2LBYtzo3qbDEVskz7MUJMFZW
-fWCugXoeyQRSYsLOUfIYieUN7yH9GGftvHlaTMTsGGqxDtKCxHSYAx/7fKtSuH5N095Hdc09KLki
-ufZXvGi/NL7YcWaPZ9w97ofK0+C7XLmklmx9945YNBglfSTqIuwS3EkspXN10qUeHtgDy2obJU3y
-4Ua6bzZ5aaWPCwUGmTRlypHvivmZFXLMX10wqmmDEIZ3O4BYTSk54ltlGROrTPIhMAa3hrtsh6nh
-b3G2IH8xyPjQoSjBGwdOp28JsMUxV+I9nXdOFdCPUI15Dz071nSj68hosJeOE2kQRNL4ENW8Yd7B
-/JYegqMp4+jBjsgDLyAXhv9etF9poQgpHvgvP7N5sc990KXf2TTNAc7iBLN4r5bACN0q8b1tCx2c
-5XxgdU9483XBg8fuf5X1XLyNAj0GccK+x48YWudA+wPfF9ub9Ti4PnyFclRAAqq8Ut5WZAFJRGNs
-GI9pOhGAbXvw4eJ+WvmqcZ0Uu3yYsnoH0hLMmY+1ftikfe/0Rwxr+slLzfwR76H+bnsWiTb5Kt7O
-G9rptcQZGl2M6Y9j3vFZjUUQ07jmlpesZm3/5GUBV5YhmgQUft7MCdADnrJidOZyO06gFjH7V/5P
-IaykvS4Nr3gb2tKzOFn78sssFlCgZdd5n6ApjOTg2DHfaN3V9o/FMPvskFDmeKHKCxPs6OiW3k4Y
-bmtx7GpQy0jF7Jssd7PXPrZ5CKasR72jSBAM7bm6q9sJVGx75bNyckIY3PNB+xEGuiYT3VPB3Xyi
-UgtsoDmSX7ejBohD5c7F0wxll8z5fpweY8h56V7nee9umzSVN/Styc9Odv3bhD2FA4G0HiMsnbbB
-1xhZE8esKLjIzXTqwiAWxccc5LDJ0tTLYFikZfarmCrJbt/1VlYX5s0sTLoiSFkdF7E+dZmd5bsU
-rP9PLL1Oy9lvevGxlDZvv42j6SEnMRDOmrlWokaXTR8gtpt0l1Zy/uInL592VnTBBvAbodQr/wfd
-WSP64uDVWV5vg0H48V0qzJXdaIFb30zlCBw/KWX63Pj0oCEO4O5n3TopPTrhKTUGShpgaoUytfcu
-3FZS4/N48raLMXgn/J5qupa6jehGS+AFPMXJgjhmSB1wcTpB9ikG7f0SeYlAbyqM/EG2hqTr05X9
-w+8t4R9bp/UmgpKSKd+4MO1OrHFlQD5Tibe48mv+CSazzE9xIlwvbJrRlzsNz+sF6KA+z7AvubYT
-iCrdfmjHDIRAvcyr2VWnM7c9sq1JM3DImvio+8z/AcrYf8sBRrzbXV08mmO75MiLoBKCJEuHFAFc
-mahtkgbtL2UpqsG0KwZYeUslwRbNlP4b24hAPcywj0hmR9+3dXVHs1cHhmzCWnfzmcmF6nc50pTH
-ObPEI+nKDjS4vkdqmZDw9C5nUqxxG/s8QoSyiFEjAhuSt1fcj2PqdruYgKN4q/14cneFY9bf1ZI6
-v6OoZVI0TAC94abN012O7R3oEV3ZErrLIm6HxmGgUqKFO1j0WCClLGCpfBtIsoB5oXkIcUWIKswo
-WLJtrYUTH2SwGLCIe3Sum0hZALyglMVv2ANjI1xYpIKlZ3Y177sS/hEipzIztzSSawXpRMLdxkIX
-zZ5zTurNpDoLvpfsg1+kLLX0hYNn/Zi73sp2TTplX27jJhltycryrJwkheApSVSy8/xFRXwnnaY1
-2syA/M0ttN2ts1LC2kkVYRQpxcjGiIPuSsZdCzCZWc7IwCuZzggk4SfQSHU/vVpEnzZZFw/c0Fax
-NoPyA9gxCiNv6oIfNlCamdkTjOZNK+boN7zp6A1lEZXukCIYwqmMP7UoExzyc+mbYcBYi+J/UJxu
-kUzN0AHgeTN33GbrfIcxou8a1WsZFOqHFigmN04/GDGfZkWiWlINoP2SuvwsqE/uidxjypG4KJlB
-vQBvAX1B7t5kajvaT001wEqk85p55GYxshPO4mtnmMa42lqJZdnQH0vpfl/2eP+RtuGu+a6ehu77
-eyBk+e/Jyv+Szfz/cRpzgCLlLyvONe/5n2qGP9KYnz4r/mTLH3dp9a9Khz/+1z9RU+gSgEX9aZEl
-1v2/pQ5k8Pikk4HnRQVBGI/LxP9PqYNFdI/L/pY0dNcyLnKG/5Y6rMZbmi9JRg/tBjnj1n+Emvqb
-wl9C7XclawXfZxR+8QX/dW1CUpjq+xGtZeUAbcyYVj5LBUx1sevp518+of9Z6sBTnZcKIG4h9wFm
-8/ed6TB6jLoTBm4mb3g7mZO7Bb726//lRdBukHyN0if420bGAMbvexB/GW9GapdUhhFWhGCc//2r
-uBczx1+267wZlr80y3x4xBcZF/fxX9ZNIsgNgg+MGfok2CrG9roPtSjm23qJG+/GIcSj3DYX3pXd
-wB8KlwsHi7NuZWINRBNv+g7QzS8G3JwU217QTtlbghy0oLO2vaLcUouXyb2lbBXw1HeZysaOn+6Z
-mmgezd3KZYA+6+qj42jhhU4PA3Fj01PMIUI+89uKmRVVqZp+FbEdk+nTkG6ybWWU2dtJlwtJC3E5
-4IHQC/hyV9DLb4h5E787Wdc39WhK5I4JxQmDgWz8dqSbIglmaEpAY+GqJ03Vy3ReudYLp3AEQCJf
-aeoRMLatXqIu3S5eaSqGEmPG/Ir1AIM+I+PMGC01IjJVfhoC8jawEIyVlaLVlBKV78zjeGsazvC7
-JViA6QVAs3q7gM54da3MVRtLS+vnYDjOyRYNHGA9WdknP5+n+GSOgAxSo0cW3Agv7VCU8zw81/FU
-3RpeJjPQ/J77SYyIR4SmZRIRMUMmmrYQm1AlEjIyKf6cBM4K6qS3lTKvrkGcIEpuSRV3IFgszNdS
-vxv9Yyqkzq8ZYHLgAbrvedAjUyJyozWotRk4uh9JqRm4WFp3D9VgpcaxdW0+Z4NETBu62jLfGG3Z
-vUbkbEJQAL3/rEm3+6qIxPW5EDRQCHCe4CvyvGjM7dhTR5xNWbHOGUDBOefc1A4fgedk35EZRy9R
-XqtnGy3sgEJ4SoeFN9zMDpM7nxG4BZT0kRFy/WEZWXbvlkuvOc5k8Zrkfvth+X1lbC3oX3cVjNso
-jBtTvuZGWd0gsh7OVZn6eF3sapx3UeyNd5E7B/OxSQb/3U4D+dV10IU2KPcZuYH7qq9d+NA3Zi35
-JsYm75+DuMqfpj7wruqqHBRYULd7D2JSWcPEm2nFzFrMR5HPRM1aOuk+3N5Hq05wDSUpWHW6v5hL
-93NS1Bpcrk2XHIoooveYPXqEjSuW9LOO7Y4sC2KRUFuXRb1i+TOcEoYBAGbrdhh7KFuXGJKpQJs7
-d0NS0mN1FDW+HvVDnJDysDWtoobhsljQfRdCG/8oMz97SMkPU+3JX0h6oyMAKpBD4NLEu07SD+b7
-BTcZO5Y3NiYU2WMuF41CVLYNLF4LWtg8qv6haPuFkfpChhg0rGUNgQHoNm7qzBxo4UVsnqXWxp12
-aZi4IJeh3QK4qpl1l0X3o/dFH7FBzOafUrChod1flwZ0Xvgz6lzEV8BOI4J8HPDatL2iiXYK2BWJ
-vGTF1Bt4/yjYV3QSO7/BR9I8QDpjCmGyCFIiqCgKp1lcEWJmMuUCafowNPX6rTNUzViylTOZqXgQ
-0pPVBhVrP8asL4nwZ7kvxz42NwiO4a4bk14W6EBjNWy5jCiYhtpuVUgOB3AUr8+G8ZBLlT+1EM5D
-LCZE2sSRCZy9t9ra3o7+PJC9BruaUFUGr3i1xCKXtc0n/dPJdfIG2c3UoZ+ndnqIfZgnBIya0jrU
-WQXNxHNAWPEYm+sfRrLe/jni1y7kVvRfGCgOxi4FXyaYdKf9sKOYWuElVies1dPAOLkTdCduhCT4
-mryUmESRaHpvxtq788relrtuiephxwYxgZbCsiHESxI4W7tHD7bVsUqz7VLU1rtd+gSImtFiiBBl
-BEx3WP+EeTEnmKjwUMI8mP7gPyZMQH4wZXVlyAwlBsAux0QCG7NeQad5BxxtFOZq6exPNxWMfx0m
-olcdAMhpZ7qa+8CKCOky/do6+WLKp03U5MmvPk/jH9ak+bpHMDcpI8uWCD3LLgXw5HwdWfSATfNN
-nwXWW1FYyR2lMcPoNjEtSLMrgwu1PayyIDVYqQQrwsy/0MxY5FYR+L7OE2B/V+LZUNjJvYP/Sodm
-MzWP6ycCI1e60bU3WQD25gIZeHShqJFJRlPI3rq55V+DPnRjkGs6t/SrSkn/I1phZbIt3hS8q9H0
-P5YV2VZc6G1r7VKF4kJ1S7MZwls6afU11OXKfbsw4PK44NksaCxoYr2i+BldiHExjorTaJHiHBJb
-R0MoYW5Rn3fgyLbDip1z+8a89S8sumLF0vkXQF3f4dZh0AS3zlsRdvj35nkzXsh20wq56ycxtrty
-Rd+lvFSBWNvJ39oZXwLGiJgsnwsxD8Rm9GxfMHpNKo64eWDrJUvRFJvqwtzLL/w9iP7GA2O66gtP
-RwFPN8KuMF+ofc6F4JeLybpVyWjD9VsRf0tSVM8EWcP9m1cEYDW1UNl6TEZhao3OniV8eoVhI8cE
-sMIDjQtIcDJFty8veEHGuaAGlwt2MLZHlPhypRGifIXYVK6MQkB5+bPI2C5glxumN6XT+NPxmSZz
-ihvLNzBKFnrgON12XbTQs6gLEhF0JI/nzFHlU3eBJsqVn0grv9y1K1ORswq8IkmuzVVTVgCjpW0o
-tUkvMEbVVNa7l7p49PKV1qhXbqNzQTimhe+eele5N0u99NGmu+AeJ49ZHqyqccVA+h32gJUN2Vww
-keUFGcnwFnqk0cORvCAlRQtdUrqV+EnrCnKyYGnDRWu3bIZWH9h1fQFURhdYZXwBV1oXiGWqRyws
-zsq2JIGueAtW3qVeyZdj7HRvyHUmdPosqJOVkEk/nN+5F2ymzfH0pC8wTX0Ba8YrY3O54DYZsMpr
-dYFwViuPs17JnEWS2pCQGQnuoQlaTyUjdCtsL0BPlXbqNVspnx2h0TE3zAr/9AwXlReUP6CgVUqK
-OQlXKyv0gg1t7FRc00gDE80nlsvQMG14ixfcqIaNPe2EI1vA/DZE0mhlk841kLINy870M7elPgeK
-+DGUGRHBisskwJvKC+rUdXNY0dVKQLWWFYbKAqr9Qs0CIjVdaakc29XHaOZZtM9XmipJdmYEODR2
-b6asg6yu4a6Sl0D837jSWPGKAGZlj0uC5kprbWPPfaUU8Z8I1cULtVzArnkwyJ/6gnvNVvKrLe2e
-tGIq+RMHrE9YGo9xrqByltRWKz22UsoX26St1G9jtvR9cAHNJhfmrNeMlLsXFK2KVizt/9BD/L3z
-sjAqrgZk07IMm5X1vwrWNLOcCmsoERW5aB/IXgzYGnTqkMymfPv3L/U31Il0JMYr8m08tKpg5KT9
-NzEeY50O6VLZhmyv7WcgiTWSEbZIH60voCb23pzw1akZDUnhOC35JY07/y7nlglo7lrNq+kRe4my
-IG/Ms92xBAdiusZHOZVhnjV5Os+NNfpGyPdqfY/dtMh14dpcDanp3Wr8Wr9Nz+gfAseZP1xXYaJ0
-tFtXLNfy4FOPtv4wUyWZZzbafxhKnEaStdFXpYrySdlWz5ZT0R9tLp/LfzTOuEl/dnVf/x7+l44y
-+NKDfzvKuGGA0f/X4bv7TPu/Wjb++T/+6dkI/gEkz1uBXibFExD1/zvIMP/B9RsA7HJhEvxh5/hz
-kGE6/7BsC6kdF7pPts2KQvnTs2FZ/8Df8Sfsy5UQuv8DZjb8sH8FufDqgeNzM6ElZF+PXPJvNp9J
-s32fK8ciwjaw7n0XziQBHNPG7ef61iqsDwYq0KDTZGfS9VJpGpRpg7W1WOFX3mh+tosKaAnSeN94
-jHBVPGF6F+TZgngstz5L/Z2tMmJ7cueZMDM4gBihb7n50us44/Cyh4LgTdLHtqhUsp0Re9gctVXQ
-2PZHAorv2x4nZk3kwkSS8J712mM7q0Pvx/lmItsF72z3llNx7uYptlAgsfVrO7qPtHX7l2YOuuuB
-9JqdaFR6haucWbPuXlo/6c/C6JyfrhsRsNVVJI3xsodcrERX+KKfjF6cJ9Zw9JKdK/dp4/5i7UdZ
-x1zXcAeJUU5qYs+H2tqadTMfmTTDmVbqRyOK5kozFb3P0piCFk8fJn3LP9QUPrekMdzFwit3Ugvz
-UKy9gxORfjDB2gxhImOEngIR8yE2r3hMn/qoU/thDrI7VkwW5jN29hziguYU0HVO/hY1hPOgReUS
-YYWRr03y/BnCrf2Y9bVJZGW1J4cAfLTVq13sYQNsu8oORdXuMsLwTonf3U5QjJGBYcDvl+XFWPt8
-Aj8QB+iO+Le5r65Suea8dIQbV1nmPtZqKJhL4wQLAsoVE0j0bsnV4zKwWnIYle/wLlYnmoCrydEO
-Xp1mCQhPiE85urA3cyEuV7TsEiU+ym5TtszZzRYf6kjdGVpj9NVlI/LGYWwffSFeXcPZKSn1vjL0
-Y9nM9zH6na2foqlwKEaZ1FvoikaDmppoW38ef/i6ehOFPFS2fnMiloXLQB8cxImxXabupHQ7XbUu
-DVXSu91RB0V01QLdxOOnSKXC+Enb1XQdYRAOyN3RPPjB8GbzGs+JcCAllBBjKVHuR6EDNhCuevaS
-prvGZP9R5vMLZILXJuh/58uCXrGbDk0d3KK11PmDq8X4G9Rt311pysFgYzbmwKq+dht91c+MmXYj
-WVveOStn/UHaig8INojqW6fqDWRejLFywk2j8m70i6xo0Inm/usg8EhmWzk3M7KPpHNYO7G0vmvc
-vlg25WJ21cb17WBBE8KIFGUm670doU4+MIFkjOVLldvwKbLOaj2+CzMxNvXME2S/uOgCwom9pt4g
-z7WcmzwKyruqbuLmllKChfsOu2fjWyHT0rzd2ympErsShzqXBz8//YXCJ1qT2ZYh3uVV2bwiCpEP
-emRdHiakweK19YRA3FIi5NxYIKR/lMqb4lPgE9oRD47nHSCZLqdIiEqE66yPaBa2f+O+LeqW263t
-Sm73nMxooONqSDeeDaP7KlcAPUI6o+gZsnUQhXJuiQggoMR4lJPHdzPYuN+3XtM2Vgjcs7L3uYOi
-5piylnWhlCqLBqP19cLaLuhTZrGqHY0AQGw0yg1qQHKpACEHw1EApnBDr7Rlt7eSyGn3S+SZwDwr
-JnI7ksWCbO/ICSGsb4gsJVeDYSz6TDIuNu6A/9aYUCGFOmpqUlCbyn3pWWQmtJcz87kCruocxsXQ
-tmfgzcwJTG/RXWgzzSHaKGEXjW2/f8M1HJu/M/KUq83Y+cnD5MGQ3ARmqcGfj6gNrwovD/ptFDf+
-cIv1GfxDHw/LcDOjGxG3XUCICEvoMZ7vA6P3h2ehowqYd+laR2jsfMG15ZL+nEek3TEpS42AtCtB
-WI7laPVJuCLU9t6JHvMg4QOpg3QOdiQdzQuffjdPjKQ62/2JXNq5D5JIfYLlmD8dpdxoJ1N7ApxQ
-LA6BwpytwRYTbmodaC8n+6w8cOf7NHAa94iZPWsfmAF6+a5hWDKTUejSjPv2iC87i139NEo93KHV
-svYAV6dj4S5nQyTZOR+6hoSmoXpw4/Y2zQzkjqQChIny9J5BTH0XSwPpUGCoOyaf0WbxS+a6Mw30
-dkrUpxlnyyGR6a2GUo6MI0GMl/bGNXCLZleV+sqQ3GxVVAxbEMZAkXUcGi3Rwm3f9DeGwXBqMdER
-Sm+kbGRmTANmbaGmRIemI3XKzonHzvXY7Ka6fCri6SG2nYjCr2SkixIyhY/Almwd5+QvnVHk5FD2
-zrFEL7lRzYrloN2W4E24Sw6QKOjWZHMiRpVZcrC4V3UsbsnFXM65KA7dOsycoEpE1U2CS/5mLNrj
-OLHnI+FiMxT17w4yBLMqorISYd6nAcMxIwMq0TNlDL1C2uE4RDwT6vtovUJLNMaLTTRgKpjLw1vG
-3w9c/LaGmotJOyJlj5Fl3ti0lu57GyvjVPcq4XRc1QAe0ISqkTf4jqcwsqiXgUsfrbneCbM8ysW0
-j50a+m+5uFsYK3nY5IU6JigJaxAwog7lyNGcNd7bMFbPnWkMVzMXROgIdonsJYMNIaVfRMbnQ+jq
-6ZEkHybqkgpp3g2CoSInVcXcsEG2HTrTyBODTdU5U3N1GAF7P7mdn7IJhgHCBr43O8gZ6INSFDt+
-4b61l0VuggpmOUgHXMbtFJvDGeO9bey9yzqYJcsU78gbJ+O0h4cDpx4nQPSAIUCCH48YiW8wQYAZ
-RyZ1SIN62dWJ9KYzmjBSwSCkZ6QJ1cNT5kWDsZ9SBNnIblhlK6qvZl9A0nHvh6Sd03BM5zwI+7Jt
-qnM5q/lYazKKWcl7fmUf02QxzZPjxPDlVW4V7OTX9TxAZzb1vq9Ee1T0MHymk+UOV2PfJvOhGflB
-V80fYoCsyp3pRyWS0gUEcFELZFmH9o+U9TK6Si7igoWpTnaa0bOYLD0KDl+Esml6dNo1ItVfF9bn
-cWhzJh2r+pwSBHLu20Jy10oVceK0R3Lay/6mED1BZq2dVsW9ZHs73hs9HCnmnnBloh2L8/Fx9Ntc
-bLAGVQ+B0S3LTqF3bB9map4f6yrNuaulNy/bzHcmBkcVoeK0XVXsMaRx3eFA6536d1nrUcx1yUiH
-GUHToDqkomqO/BbEldaJ8pMraaSERSpKg3o/eCqNjV2+imAy1lxUDUOAKi0OhuSlLOd8CRsFSWAn
-BqYljwh6f7gk3B/ZMR7TCRk2j8h2j4DngBauO4pxrWl7DiEvyKGlJ4wNpnR8TkF04W0xfwaJ+MpT
-0htRJBBZgAJP+NscPscTFBJ+TYZwOxBuL2qQp9owdtRtIcmq3r62AcQrA3hD2TdHnA6wVoYgfskY
-b/pme2NKFAg1Mex0AOV06EybLX8RbSX3yV4KJ7hyjCIg+rU6jW39LHuWAJPi+iE0+DhGIkQhfNd3
-rnrgA35LMqIztV3cGX5+GloJTkohoBy89jTrKjtGo3tFSXQX22bzg8eYvnUH/zlKk6dRVPvRdnZu
-UQy7rq/ezcwkqaKvo30tWe21w2vRNvd9MB4Tq/oq/LpEB5Y+kcvwkGBn2DpRqz+g2v/wuUMn9Dyn
-2Rjao8nV5xKZRmCuvTezBmUm0suNyJcvU0U3Res+DYDtN7Y33WD2RelDEOY1qQroqOy1IpLBm9Ma
-aEPr+vcyxUMYuSa9CmQl7albj9NlMoPDMJU3shcPRZm9Ll5/a89MRxm2n2RU/GxGNLRlH4sN8d/J
-wU6GaKPa+j1dcEwIViFo4wsi2RnYfk1j9zQa3qO5zMk2jqebxAmO9FL7nuzGUTM1ZGHekHLvXS9V
-TzGKdcSbh1t2mQ9ew1DNVs19FrgPru/shT28Ms4h6NDqA27RpdvaI/z+2R/eOaopkRVZaMJEmxH7
-B0rd9zoe9u3ccojXLIFaZPyzUjt7ak5WNahDtqqgsqD5FVlud4Ds9dlFJEckiIX64LTEkN9ojRiG
-QTRqYveXDijKG+grNhoqu1y+posCrirMg5MW7xnNEGdLM/lnZ5BvxtIu34YU03XkpC/BQkib6uUW
-HR4ZE0R0k6u2hVu1i9uILEQiqEvjXJFvv+mr6F5JvDCVvGYpsKe+3DH6nV7ncbxeGn2f01jdtp73
-5BQDMXaOZfCoZxOaddq/SsE6bT3L9z5IdQpnl3wSp0VY5TrqNSV9IewnIh/BDtCWxYh63TK6T9q6
-2aL2EWFAQvk5QqK7m4mAbtftUA5iyprvfbu5zyNiY8DOY2dLm5+LwHuVjlJdc9g0G0/P7GG0Bl2G
-AfCKn2HF28BmPzw73MNlmn0HLawVwljqkx6ilnibYNwvo9sNB2e0CRpXkwlJidN2LN8IjVlNDXmP
-ttpRU3TnjHPvwMYZqKLu6OJ0vWcWmo5XAkUmwb8kbR8p07MmHDozaQ95OvXZjrbHYdBeW5kRX5G4
-M8ldrNrC3td+j11BIOMlcLLvkHEuwYwW0ib5nchQ9IVrRDTqUH/MZpN9Vi/OPXGBcmuVlsiudetP
-BB+XsX6edGT9YIet1PUEcMsImcun54wcrIBWaCSzB4h+7y/b0eskBVs3B6c8q5YPpNSxvVUMYBqe
-CXO2w8hAhG7c1bwroSQ7f4Evx0AYRRJO1UzdtYtWMzla9DE3JGfQ8ASqpCQnqJmSlm16/SuKmuk0
-0lghRK9kfkWKOomf5lBUZ9H09m87ttvnKl5Sfy+IUKWo1cFV0Tc0no02Pt1ieY8dOyOFZ4CnVtdB
-cqot5U97jXQbrF3bnwY/urek/Tqk+ozy4xY5cFOG3WAZN6WnA3bGynT3rSNIdGT0CLJqpZjZhH15
-AY1PhhcwRgeLcJaeHhfi6n60tgXPhWIaWb8iP1Sjear0cu+g78KOiIw1kddWT8xzy4lZ2uPBDuxX
-my7wnHhIm+uUACtFjnlBytEsys+BzfqxxzvFQpEYl7YvbxEoU1u6LQGypvU6FD28pUX+4hy61Y6+
-hiD1pGFoRVfoL9jTuXYkPo2gCp4iEmSilbwzxPuiHx+ZbEXXGZpRnhYiV89xjQNrp8RESncZ5cTA
-orBcV39Fi1xE1nK4Xge1h8XxMla4bER4P7Xq8jOGghsjmfd1hqXF4i7Gk9ciqf3VG8OttUrAiewe
-2HdRsqn6ZgimPcu4r8ya+2tVAwIiCuJHlhrxgf0lKd3KS3gyWnsOo58l4wFKDwJZt/GS8cTyrUfa
-Rxr/hHkHHK7Avqmr+Z1h0reI2VhzWhufjlufUmOqH7QuwSXywDxwPC/VU5a3lHy+am15Xzsj/WRc
-rqUXrCFxpiUPuk3egU/aGLWHCJ4Vb/Z5QRDF7IhgeKWSUiw2MKbtjM5iXwHcBT5VTsQo/pxyZRfV
-ArIedSi3vxN7FHSZ2SYPnN2x3nZwg/ZqceQeH2e2EGTGcgPBjD2/VaUNQbEb+g6jVSE501XvYwLJ
-S8UNHTuJ6m46Ekj6xw7NMvmtnSCWnkE87DQ8usgDJZ6I4GdbBd77nKyDOLLZxG41KVRbxMvUrfHc
-rGWmnfDY0X7eGTsyMzkpeluor4Z0OXHCLgPqLJCYADVYfGKusSmYk1E/sRAczqaS+T2GOu932hot
-KnsS1EtGitTqBK6SN2T8rG3mcQSlFdOhLMbmxfMTtfOIwGvmHqcitt8rbxy/S0x3WwLT1D4acRGd
-2JS1W0s1uw4Bb3BKtD8tR2nFnf2QzVKX3P2ruYThYM5KHgVWdlKBmFVoFrqPz730m+YwULD+YiGG
-nbA0/Pk3LLws2AWWwc5wyHMVHPqMJ+2tknV1yjRW2KuhcrCZVJd8y9w20LgsIxHJ597JaVnylgny
-TkgODfTwRpoxiWkYtqWl7cenpgBLuyOCjQdv3A/RHVw3ibTRwExluL5+ZxERvCRza2z7CBDkkOEP
-IppI3xYoXV5Tiot6sbsrIy2ZLDHj+XYii2vSiN3sU3myONR82TH2L+m8TEjG2XlghNq0Lj0DKSbB
-k50ny5E7IQiYRvHahBAxetnCXvP09VCL1d+T2VFc3uDF1OZTjyez3/OMqdq7XKVGeiTGHpnxpGle
-rnIr6rPPpTPaJ9pBlpI0ru1yX/SK1HCd1fG6poxn99mdDJBrXWcQhdWlrl6OeYNr6Bo0YlYwufOc
-F9UZVfVIEdxUD7Y/p91LNttufDVEs6ngEaLViHdOShuPegwb3m5Y6qlirV0F+OWsjGX4tS8jPgNV
-jdQLEWC35FjVBCShrxd59sxbIaTHC+je96ZBUOJuDJw4eSj6ukM3lOv8R2TrCvdGZwjzt2u25VfK
-d/Obdtsk+A1ZWUTwWh0S4z1wZZJBX32Ncda2B8QL6AHiweB3VKRuMhxK7Ni4i4pq+HIEmUg7wRXD
-MLIfyvPKx/X3bYv1lK+OFC/it2v810js8eMAfyIysDIH+yniBDLvKfU6FCKT3V3HIpi8PbdJK8JR
-Ff2qKDDQW3guVvid51TLFl7uIneRbycPdD+pZPSVGPZm6czV+TFLa9lRHse/+siOEMiL0g5OPNhI
-oGY0t/CEGCIeaj1ekPV3LtJh55Bzhukxkr2+DZwiuRphPCVo8r21fx+xXeJdzTK5Q0BoTCGjQjId
-I8/W+cHjzvo/7J3Jct1ItmW/CGEAHIADwwJuy14kxUYTGBsJfevo/6asxvUV+WO1wFDEoxiRkkXV
-rF6a5SxSxL24gPvxc/Ze+wJVVx5dTgYS05OUwMYH3kyIs1ExOA9mH8tHxAzWNWsEVaCsNdb6RlL+
-d/EGHEHKXo/Yg9lG8jy0UYwto+0vlqpZzqNhFte5ncw7xJDODh1wcuEO4th0nXk3k99XUDMfGBii
-waDv+ZlRtQNCcqZMWpI6vEhFA4ZUuaSjL7Xr50tTnlfGkB3cun2Kjbrf6TpYysomSWxmyb1gTD35
-IZ4AnHYh7D4OuhdtmFgnrqWRBE5cueYuXwtnPDbFDOeP0zRqaD2YQZ1uINPeElwaBmOv8kdoqaiP
-WcMPk5Ez1627a+W2h7Jxry1afC8EK956Mj+xdXb2nJpk0+umc1N27hkoyfN2ICwqr+a99FC3tInc
-Rlm07BBPRncMgF+HknBulGDGiSSnnnloms7+mHAvfEbOdu63zHBo7NjOf3KFujZ56d5PDJFkWj8d
-NW5V/a//jS6VfF700z+EC33/t9+njab72yqJtlxmZ45uo5P/c9pIuJBLNBC2gjWI15UIfP8cNsrf
-XI9AIhdttMfKLfkwfw4bySRiNmgw/15xTeDl/smw0TT5U+/J6DZ6acN1HNeyxEoR+YgUzPFXDiHV
-dkD4Hi3vMJydp0TrO7XXqa4A8Xq87RztrMyE3RgtZ5khGkC3DCQ54aYrP9mi3k73c+eJiKg1h3hp
-y5vJbjQZqlWdxAuiz7R4rNigyWXrIAe2dZMV0dFO4+60W7wpWuv9ufOJ5TUrLELUb3sr19oCtVJZ
-P3Vod9kBPCHGbWLFFbHvOsPPWWrWJ4WQIwr6SEXP2CNL2y/BmEaB4AUqt6a+qHtS69zpVC7NCAE4
-YgjqckBQEEYYRtBYTuYnTcY4LZjEVkAtc8+knM7QQMMxNpblgBVzSC+5Cm6fuafJwom8TfGXTsDA
-s/N+TNuIVjXD4xtzWSxGoBjxjPQWfXEUBnHXyovSWzJvL21ovV+m1c1A0zgtdppVaUu/KTmtGYhE
-tapsNyOTq3mfIvBsN+6YxY+oX9AUjfxFP5k1kQYjjp9i2xnIZyGC2zdL6UHfMIxKD/0+FSWR8Jod
-FX7SCXyTuZZ2foimYp9ZTXWju0v+wLhDB747596jYyb5M4e8cqZfpTMgst+GAX3JTSXRr7Y26y9I
-bxvDGQ3NFA8lLIjeouRT4XXXMVWYh8x58pzMfGrjkKmWMZkxno5KAaCNp0Fz/a5hVwnWdukX3XBh
-MDuJpWL2wXWOwQw3Oo6NUaWXFMfmKyOVEDucJfp2C/SbXl/TOaPNmRtVK5vKOh/JB9vsAgOxmbub
-YjU8xmaNSQnpMbMGWt3Jp+Rt1EINj2Zy1jrtrkOO1GIRG7DJ0pJ1L2RbzcxlW4NoxLmU5amZo7UK
-4IQyxSmbbrxO8dOkB70QxhfKcjjmFuRbThhtDmlEq3g4CCVdx0J1Z2KdiqHBV36t5vSToN/Kz+BW
-rkd9ljJWclXXtj7TBAJo67ehkyoTXd9B2QHB7SEsTHcCIzQ5ij28hSgqsUZH0mAEP0sMdoBWVkd9
-4wCE8ae3WVe+oEzBXpZZ3QZHmFsBBE7sRwj8erpPzZGiFFp8PoGrH+I6OlYOTiow0V2/oGofx2QL
-jWH4NvY9IpqC8uGeMF3+CtRK+1utiEXbpnbJqCvuh/yptjnX+Ph1eL6g4HVXlcTC59fMeM813Z2k
-P8bRAhwkH5aKjiI2fp876V6EHmnZW8abzLgj3bVeo7mvVjN3adzIRmQ3BHSvzY05fu6UtxhnVuXJ
-u4a4VjbgDIkNt7pTz33Dnp2GTjNwyHadew9jWb9tMSbyrM1oe0CJgMJg2Fkmz/SwqSsaXH7Kn5NK
-evRZU7qBaFzTz0ZTdyeLW7GK/Vyd9Bf+E6u8YQmBE0bAtXpbat9ZKVJz0tK55ZLtYAS6gX+/oIEz
-f+15rXFn/fxiH7lPOEIc07KJp4NNzSbyQSMicuJx3cFKAo2Q2w1Hsa+ww7tN0eS/ItuuhqEft4gP
-l1q/97vv5YXADRabaUqCO0xtPaIFtnEuim0TaphDOZrar15jZTTcs/LY9jHpkpFEoR0j1UeiZzjb
-n3/3v1BA1w+EBQdrDDsqd/3HDxTTdtWLgejuiMiKI5nJpLDLptz8/Cp/83Oy0ZrgdkE6Ccv4wBrF
-kIodVCEFTBTEjImqkkUIP8CVESvr0nO75lhAkf7Fd3v7s+8MOTY7JLWCBQLW4aqYf378ckQq1R77
-qvKHDWWo7/nJ9n7xXz5fxP6V2jyNPvpfPw3+8Xf94aIfNHyuTJVb5lzUtR/68JCgF6/xrthlttFM
-9xcX+/jofvyG68/77nmyNBgUNByYlZc6jZYwpwRv+5Mhk98Rxpjzoq/V3zi11uzGHx7dj5daP8q7
-SxWqhCKz3sxmi/UiaPww8PwqIBxi87R/VJvPox/94rH5C6/04zU/vJm4glE/F28/YBzgYg8sH0Vo
-gArmV1daf5WfPSofXkyiKfPZQKXMt7M3ejCeKP+OMcHlEsjPOJ6OP39GjF9d7oP4UogyN1dRtD8H
-z8tO3+tBtgXWf5EcITHsf/nbfVx2Pt7HD++fN8WMINb7OAbPvA3+S+mffAtu7n7+rdYP/e/vofOm
-xXv3hHCgSnNtvcqyo7oI2q0doOb81S/18+/i6B8AhCJpDQtwhfLPm+1zFtx+tfdPdzffZaD/9nH/
-1Xf5sHRMOaSjuuQq1qdwj0etvEv98iT81Qr1UZ744w/j6B8WC6/Ncqtdb5l2AB8UwF73X+S5PFGH
-n/805q8u9GGhmBhkor/jQuYelyFLobY1LhreI2NTBfa29Fv/tPVPep9hzP3Pr238fJHi7PbjyjFD
-2s/V+rAzotglB2NzC7ve/4o/xGfguKOX+qvb+vO16i9w96ibEodzgfIFS7/tW7xdw4FNN8BeFCBh
-2UYbxHXBrzbTD+F2zocNx3kLmnr3BkjL6B30Wor7+uWu3BCi7b+eXOEV/hOb/ncr8brq/ew9+7B4
-jCigNLdZv92NeaLuqovmRDyHV6gkMKfXT/MtmKFLcWXf/uK66yrxs+t+WEXwxaGSUFyX4Osgv6zO
-w43cAY4LPsPS2HzDM8dTpPvffrV8/eK6b7vEu7uaT2M/6BnX7XYIIYNxW+3FOWK2Xz01f3cdAzkM
-kSS2pNPw4fupzC1QX3KdZks2Ct9RbDyuaAXeaREAa/ikrsoAzcDeOvOOv7i3f7eqvbv2RyN00uB/
-Io+O77gZt85dvoOYsZs32U4dzUP4e9XwH437u3QB463K/PO9+otb/38UT0uFyv2HZtXbv/neb7Kd
-32gJ6bpO5apLjiH8ZN8TCaT4jZxqy3CMVRBvv/2n7w0n8zeTtGrTc3GUmCRerybxP/pNyOUx1Vue
-xbHGktjR/0m7iQyZH19H4dpcXuDRlwKPvis+lCzWiJZpdu1m0zkFkKZeZdqyLclBMh8zYZvFoZ8I
-IqLcTtp2qgO8fXXIhBkZavVFh1DIc9Y0xK+rVut2WZxGzSZrsWJ9o/HdJU9GE9knjVcP4jwu1y67
-jjSzvnTiURmnxH8305WG5TA6Tq1BFliN6Bgf1lRrZBPp4waMkXPdmatNyarHbF8p1eHlHAEl+b3t
-zhJRedPGX0q0oto1QUieb02RZm6jqq8ZT6pKylO4dvoXreor/kgcGz4Sue4QeX26ybLSqF+lzogr
-m7H33iY60DHm72aS3NrprCM6THv0hFhcOJicQSthDO8sq0BgyDjr7umBTLcLvfsOTCjH/3mv1Z1h
-XZRpT+t9ntv4eXAEugG9b7rj0NpdsY4uCOapQto7fhryjfFUeUv7EC0Cz6ka0QuIYYnvcYwz2Y/L
-RoO0hRMw2nRROh8EkTDMEhcMQEviZ2GY8lPISrlxccsMsu/6607oxYUaIUpZanoopbGOijvs02NL
-K85mGoIHWUzpI3lENoYbaT4TkGJ9hXLiXGt2h0gVGNFywkPbH1oMi4Bch8YIBNrOi6gp0zN78fLL
-eDDaM7Mo2z1z7HqbmtLyoypqN4kj0OGkg3sPFixDTDGLkhGl238uKoGwWLL1bAQz3p2AoOaHHDQO
-oYB5YDL8vmnJRwo412c03QHnLITS7BY3LTZg4ejcp7WhTqTsvvVImuG5qrbZdXzoXcxU83OGXdq3
-5dRfx5GVnLbYJh9nVfdaQE8/XR+BMiQpsbFjYgQlt8PPpRzOVsQRnIO0vWpDRgf0SMVJ5iCj7fW4
-6TaJEuU1rNbylZ7g+Bwzwrjhrpn3WoJVe2OEdncCG2u6Tgyhngcca4+jHbmovnpV9v46XDtg4cXO
-rVvGQM6b6pVPtlD50Jsg7u4w7BrkvOVOIoujKmq7Q2iFiUFg/x7AxWaBKRyUGmhFbGzwL6aj1eny
-Og/NoDc+8YHWsGMm38N8SbLJMe/oKEr6Y6VWMJtMexU/W2brbo0+aoLRwgIe1vQB86xwvjVGFx/i
-OJKnMkJXmjp1caOWBjTQWKCh463vedpyWwzXhbuI7gzOo1Xs5wn3/HGqsrA5X7X+4YEknx55lJcN
-mfo0JiAMPrWdCrG62Oa8YJU3QknQ30RD7rRKGxVv9YFWjOE3Yzvdq0lrUAWmuvbYqCZpLz1nGexH
-SfE7B20aR+aZXTli2vSZBlUAM8FoqiO6Zid+kXFrmn2Ads0coUWiSmG+mjnisqtmNGqBjhkNpBqU
-CbusH6txmsMjEKa4PCe5srPw6WgF+UB4xOIazHTeby1Zx7darWFrRIQJaGww9VzdpI0NLWORS9/c
-y6gw9N0ssLa1XVavLEFjrsA3oxVryyqNUC6YMWZpnZ5dHoByQJGXlLypAV1seExRYsRBlw2zBZW0
-XGxUupWlNVdmp9LL1KmSogtQWoTiaShdjYb7pIt4vBDeFCaQCYQMg6anox21SNSUUU2b1HJQCyMr
-a+3pDEtd3W7Q8DM8Hk1n0q9GUaMcqTysE8T20WVtiU0LUPmqvQuu37qwJcMPJHpTd5GOuuKFz1w7
-1wKj12Y73cyDpp+Bh1xH6bFOe5Swp4U+06Zgcl2fK0//MnS0nqOmHy4h6+nJzp48d9iMmE92ZYRP
-BW3DqIvNmE+F2Fn5mh829oT+nSFMSVA+MMvopqtITWgp9LLyEBT2zF7udOaf6MR12vT8hdw1zqJ4
-qIaDMgYp7uikrivqG7AL9pwTnVWGhwRL5yfJN24ToawSg6ZNXzzgBdOjWnvMSR5lCUS0MUyHJxSy
-RUpmou6WV7NI6vQqImgAj8akxCWm4ZJETT2dCWsz+NAs3DOz0AvGFu3jwvoanTQ5nv37yLXq5lQf
-5CwOCPTQizvFHD8JuAnwmgaIzmf64pUrdMOwHeA4CgrPuIkQY7q3dNZ49gINrIOEuzea6XBaWJoj
-oVoRi9ifWHktxquUPlh/jFFvldcCE1YBUxBF9hfDnOMqGJIxodOZ9cUwH1PkWvYluAOo3M5ANmLh
-W+xDgWLUy5TIc7+CMMsfF1iPm3zRnrIQrZAXLeogkSVsYlXKKyfNl+Qlk1Ef38eLHXVHb6yYQOVq
-bTH6epxEXXRN2F6XkIEm6BtDnUuaGy1EdvagRtAtCD1Twoj8CZkhHX63YXaLzSCPTpak9V4yAfgB
-MwKBj9Om9uB+bIknDFdm3IwA2qATnQap3pfVJhHx8lzMMz1dbDvV59FmSzhX2TITh5iOyzAeTXcy
-m8dpYs3BoFfVZf1Jn6f5nLxG9dgitETYGfde+5Wy58alqe1snEZW15I8wL1lgtwxols8h+147Ge2
-ufarPcTCDIaFXx3KY47dS9fTbWjM/bHgbeJ5tCCUgZRM0+YZZAccBiebk+XGQYFDzCpSpMRcrVDu
-/LnS0D37wkUDAA3CwrO/aaCnMMUwS9FChOy7BR5vkdaFnzZ11YFT8Gp5w6KuwocWg43w8Zf1chfT
-tiPDj+Begy1gnnQNfj465/YOpVvJ9uuiVuHPOtFi0GLTbeFiefbqarpDwCqV2la9tgKIS0NP1VE1
-tPnp2gLUucjghdgePsa429XjmPXbpIEAv+/Bgj2ksYs6kzFoYVyU6OOvGar2KdqYPpSt3LW6WV/W
-JeTIFxF5WXpI0BFkBBNOKj7NpTNHp+3cyuIGfkAHQRVycfdZs8JB3sURC+0BDdKaCxl27mmtz0lE
-mman28cUZMohW8AiH6U14EbE3ESMgE+AYlLt7AIkyy72+BE3JgiECw/q32s6MeiwzKa8HyGe3GKX
-h3jeiPJg9+TneWRi4KfUy+fEQ9I+EdiHNoCsv+G1mbusDLROd/rzoREGlWLp8mgQrDvTkPKKZvzW
-SdFU+2XChAAdZGhx4qwjqcrGBeRC2GhaZ18rvZ93iSYWhKuW1xjSrxukWvTom9BBsx4tTehh/yKv
-4dxCSaVxaLTtdjoBmz8IYM5icHnCtHEY7I0nF3XKdptcO5kQmobhAXnjykCx7ehSOspmEoC6b3RM
-4CNsf4KURdwhAJPkY46AXVlblDhd+sVMbbCIv6Or/nMefH8e1HX6JD85D+ZPUfXhOPj2T/4wO9u/
-GbYpJSMF23Jd06Xv+P04KFwMzdig+b8D/+J0w0ntD/0BogXDWf3MHBWkgaWfU9of50FD/82C2EY4
-nWGsAXbePzoQGusneN+fIf/d8RycUUAw5Jp396Fn2UbQacKI4iU1RmsfVpocbzr8CrgjO9d8mBDB
-5dsO8KR5wTwaEWprwSvzxdybIa/D4mBkmnkFgoUMxB6HIeR73Qca032dif68cVYB2k08uOTigjHT
-0BT3zs2EKxDsaUQx1VUoJn1EDtmp5sXEvgpiMyu/ARkpt62CTLTXGzc8iwcnqm5F0VnX/dzLdHUC
-TYyHm0El915h1HJHvqk+7gzCDLBBWRqFh1WjSN46HDgCEkO4WCa9u3kgnJateg169tbMZ+Sz+gSs
-KI1Ou4FQEo6M5EMz9kPCw5Bamsc869vywn6Lk8a6Lr811BWETK95045wFCyI2MTkbCUKenQ9rymq
-WUVQtdlSfLDmGu75sCZZa0YbR8HMR0Qd0aZVi4go827itwjsuBNF6osqAb0Ujitxsu4dK9kg0c7u
-p1q5+WHprdHcjSGUK61e87alHmMoJRhEnQ/9AATdWsO5u7ec7sREL7E1ojW/GwSLYIuvm5xjtkvE
-98Ah5EuC8GwgMHQiA7xa48AxcyE0heNDSnizBoaDqyqSbYkVk8WuWzPFB7NuvvVvSeO4wQnaHN8S
-yO23NHKOqSSTj2tIeft7Xrke9kgsPPxFVGZN/qygbj6SPlDfRPiXn4Chkn0+rDHoAM3Izyje0tFj
-dm5xYC/0Lhoy3zCA8hesrcTj4J33dPMNf/Zs/ZuoM+db7LEd+u4ax14OqkcjDhStDczSzbJz9ktl
-72xgtfQB3xI1Rp1a0p/fkja6NXSjkCnKi6q0QcHX1N43pTeSEoxhZ3xwvXGZjxiimmVNlKGQjLI1
-dBfKNPLhwtEQKkoy6ZeTiXqkOeT0zJnvR5Z2n0ujp1LXofYGiU6k+XryST4tEuHfEjHr92F5Ga8y
-JRfcRyRcmadmi7rQ92SNB4c1xb7tZIlMuKJuKnw5ZNaLYBtafNuRab/VeRuwfsW2yA90J0kZIiEH
-OUOtVU0f5L2WgdZSRYLZ0u5X4xQsanvvNBGlQYn19r4DLgoPO3FruFu21hj7d6vh33SdPzTxWVxY
-UywwCo6J0lmXazfqXRN2yjXyWBZe8koNzit8uRhLAHfO11rp+D+/1se53/eLOYyMTV4nJF0/Xmys
-XMqFwcqxDRXlRrK0agFsTHXWakVzMYcc1jqn7w8u0CBOZql5jIAS/D4z+Ue74n8HsOnaw2Rc9JOt
-sXiq//U/3zdKv/+T71ujRWMT1YThISOgH+msG8/3rdG2VmWeaRHNyh4IuZSe+vet0fqNiTz/k2yQ
-LLOmyxP3587Ihsp/WQkhjmOvj8E/aZWuT8t/zS0gmeLBB0ViWNKkMEQi+OPTJLSoTKnQIANGRHbs
-49Tj9FPy0aqt5YDSoIAvjXlDVDcoOp3T2/Cr5/nHl2f9BGgCmSHzLKN+MD4mGgOdDPusQ71nN2SR
-g0VqxvAwQ/X4wnkifIgJnIg3cJWNBzutknQvNBUVBGM1yVbNYgzZo9Eb7luWgfKYssmqAPtD+Pzu
-V/2bV3ydAf54nyyWaXwYEkm1Bcrgx/ukY0Nq57zhnKfp5TVVsnOL7Dr9xUJCzfPDdSANIZG0UWOa
-qJ8Mwbry43XQDbIpRcjLOYODV5eGKpEtKOm80Ol0fQXKM8KtZTjA1/CT3bANTped6Vi3Ls2OJqjc
-hPiBFE3SvNWU5gBSh07aXtbZ7DFDBR4ldhGSRPdMI7XIuAqJg7HOEzeazBurMmaAhYk2ez7/97Q/
-RkYllq1eTXFz4qSDvtyRfrWYO0Z51T1VXymCOcoaTlhZLNCgQYPDvkxCQDAuOlq1Sq9b59NoxIMX
-kF/SlKcTxPQB6X62oFlSBLDvXBi6zk6fstzbZLaguQPrGu+BJUr+a+WoYrycU2thJAk0JrsaMC2g
-sndLqWK/IweN5pbBBF+d0CuW4V1Z5pMMcmfBrsGWGkLTHkD0IaahVU1UTjdtQH2EyWGp5roETUh8
-xDHK0rbg+AKMIEgU6eq0XUpQhBgt4mqvtZXeBgli7eSorB677Qh08pwHts4Dt16tbO0okZWApx5X
-Ur0yH4o0qhFJe7qFtVnSe8Gwx6a3sUc3ffDWQ+g2zb0C2c84z+Z5BOMAmYMqFjNo5eJcNHGk3Sdw
-/YrVWdRR0yzw87fZzJRxa6VdUyG3BM/mk1OGWL5ADKZ2Zjvq7V3peY131MbUTDcL+Mo2aKxUr+8i
-JEjdRT/BKfTTrrVuna7NrS32X807yGXQnWOuLa59HMNiMvyud+r5S7GUXXHL01+PGxyA7ue6FWZ1
-BMwzAusji7nfCtNtXm1YGidFZuAwjaFKtnvcgihuMgTIzXmi2YTLz2HcW9TMU45doRw02JKGZSVX
-hVQQFpQzJT3+C4PdPJNEH/gVaNPOT4cWWSa+AHFrWpZNezWkNbDRs8Ry76bIsIq7cNSK16isCQVo
-rHzAMDiQZQMQYw4DERoapoeRagY+S5lDuekX9zo0qvghNW3nRS8aHRhLXKdgdctxOuhiibWLsXGc
-Hoxk3Dy4RgTjVokhe1RF2VznIDlenYShx4G+g/hEM8H5FFc69oI1F/Exco12CkxDEesSeXK6YUg2
-80oobD/73ss8fT8ibGi2ugR5iJfNa+3Dgh+en9RVxV1FgNM3Wn/asW0Z1mDWwp0J+LUjt4Jw8Ijs
-C4Vlb0dJol0YcwaRwLAn+4kWD8GBKmVD8tGKNta2jtV4YEbSFdt29aI67mwANcRdsu+6iKQUUthq
-HefiPCYbPTYBxAxdVm1aE0rmnnCS4VHkwPcCnIILINhs4Ack06NOg0EDEQcylk7YETIKR3SLLIN8
-q+rQI18mmcZhg5BYTSeR3ucQWdNSHrKiJZRsLEbo77q2ZsIZ66WCvjJppJVGH1oBzSyH/KDJ5BFU
-fRRfT91i3itRMWYwZ099tlIZfbajKfwWm673CcUqXW5absOy80QnPsvKfiAbKXnO9Da6r/C0Ea8l
-7Rn/nCbZ3apI0aG2wtAZD7Kekou+i1O50Zd4GfehoJAmH0PpaE6gEzU44+w+2o1RZT/ja4EuX6R9
-emvQqNb2ecdMxBdduZjbXoyMcVRkU3XijoyiHUgE/Fg0V2KsvbMt7wx38sa9TAqCdLCiItQdI0Gs
-HSoQ2FhWDXnBRkf6Qvhi9xr1hlH7GKmyEyC+y7M2LMmjq+VJtJ+gRL14wzi+MDIAgzI2RKEP9PB9
-RG7mWetpxWaZZH81e3VzDwPg2WyihFk9W86jiQk9jMbrAczpi2wbeRy1Kt7TQRHXnr10r3PbitFv
-plliT9Mr7c4EP/qYDV3s4dv2qpInIGoeRzzka1eVo6xZNdEXIj8m4BJhD31U9KZ6Luc4z7fMTuen
-uFBkWpRjtotax7jJ0gYVrseEMBNp8pkTMCcS8nVDiBCLWT3UYA0qf+EqFx0vJyIYnFLml9mpOieA
-XzmMh9G14hkSb599dVKTWabLkRdBGr1edHCyzYoNEZzjynKM8qslSarV+oUN3xeJKG8yCFPNrg1x
-3hOfRsIEGuz8jlgBBL59Dtxno3lYuHmCI+ty9ET9KtgzNHq9afnq0XqPyTTMBvfEwLHMsM1VHKc7
-3Zsvq3joZ/z7ZqSfFJrhXk9panhHvHfeZVaHHUd2CfKJUw4/dTArybFhsTm3nQsamE9JEYEk8MSa
-4Lk4XiyCOiLPFESHi566XeL2aw9mpKAHXKUPnaXXug8PMWU0m6RXvZ5CIIw0o/O2kbcM9w6ULJZQ
-eFk1YFyxwjmYOX0KY8ct6HbWg8H4QzfLs0zm+C3dTlIKVvmUfmICpFCt6J73yEOVV/8XMov/DgcI
-zxCU1P/+/MCMFV8QDp/d11eQgvn7k8Tv//aPg4T8DWmEcCVOTvE9/uD7QcKixwYskKaWjjDcpZr+
-8yChGfZvWLuYJaHx1QkTkO80FwYqDmAolJtYfNbzh/VPThIWB4/3NTK9PYQfSDdw+PDfVjfSj7Wr
-NbcL2xecCFQP67ttOKP5MsGaj0/HYRib17osPHnBwHkPvuksdO39UlFMCnVaRCbdHRtsipx5GfPH
-VuLct/SjHrmnRQP6raqugUBg9Ey2Y0LcWta8tFNFhQWPFOzbV+WmJ0UYbwat+DTWXkO1WAa20SIs
-dnZgf9oNdvldLeyd7o2PzEf2lCN3xAbDTXCv8PWedRGVQy+WDTmHV31tf4qZKLaxtxvGYl8yyPe9
-VmMZA3ZhJngnsfM7if7VzsIbuouH0sWqV/b6vjO9x5Eew5waJ+ZcfxW9dUOP/KKz0y1Oib2S4G+y
-+WCGObyl6WiYagd6+0SuScLKkftS1I/EVWOtscMT7swJIZe7+etYn3fOrZnJraGh1Ovv8k4iWaFN
-IpZ2XxIKA28qyFCPuF5xwEO9Lz18hdEqexDZzp77z6Uen4IUhANAM80iZAzmbwrL34q/CKINHeuE
-VKON5XJq0NQuS/Rtg59TT/pdyTISjd/m+fOS9huK+ADk9jFqrE1LLF3lzSfSYuzQxUfwU75DrFC1
-PLmrCsIQfj9UR6uxP0XpgypnqGXLEdQNLSNMXYAKcoDB0XWtj0E73kfJtEvsat/yc8oLEnvYUiVz
-MiQRVHPTcC69PHDArLYkRfFdexkBaVyH7mJfm+2BgShBgI/teAKpd1uoy35+hfcQ6ON1H9/F3c2c
-fdNUt6tku5PiSwwBK0tPtPzajIOm8w6LpgCshycO0GCMFlv6AxIWngf0droxQTeSAflIcMA+zPJD
-4cizCaXAEBFtmYZAAOx4p0L3EgvpAVnMESndfRbXV9FiX8/JeEjGMTCSdJN4/IJdeBdG9ibvygsV
-xucw+feGsPeTTjbGUNs7Q7lH3qhjnsAtIMvOzdu9mtsLDjSUkfkO4t2e3idTGQAXquj44fRLjLDn
-yRTzrTIeUt09HT3mtURO1GZ3koFFDhaHCiUSEziXJijNfDvP4jVx011s490flnZreNNZYS2HhkqV
-kRMGnzUpA57sPp/Cy1yIE/zae8sJg2KIIkKL4ocm4QwDniY0oIoTA3CICfrZw0WVjIHijR6JOwQ+
-D9HY3wsa7iDPIUyyAly3ceH6Uc1+5Tans17v4S7w9iX3c2PKI1joI7S0lyZWPN7K2c5O8WQ2I8DK
-lvitVOmCzbcCCpzbN243v1S2Frg5LKA0lgH9irsFqwpTKsIq1r5G39tBE1mhvAfF3ACIsjMXfIjb
-mN0XjQMF6IBlPLhIPvYMgqmxOrWFUVHv3NbLj2VtDkGROBRQiMNMfUgvisZ9LZfsFip0HhQNgYeU
-jvHG6tNjpQEGRsNM0Dee7WezHZJdOHbDdVovtwhwmVtmzelEiBPtczxXY3zHyrNrI3M7AuiKnGxj
-ew/C/lTdZW2+yYlA6VygJg5ljkmyCLIMOqQIDqqu2mkwEopIbWkLB4wuSEEZdqpwcFF7xjdqt5Te
-vjgOybKFaac2yJUCbsMhmoYjp6fz0bS3Cb0galniELCuW4t302rGKaADhd3POuUAR2k+5n6YTOYG
-b8qjNKtzOBXnSWcfUgULD6lGVS7fqJYoNtLB9NvG2QgbHWy5vJYK05rtHel9AGksr5yEOifJy5sR
-FoAziqNbtLeaG+4Btt7nnUfFzfkkMqjX9YNBulvnZBdK9ri12zYotMlkQagOnCj3g6wPy7y4cA7d
-l3TuzoyoOJ1M9zlPjE/Q188jxhxTCr4K3TOwqkcbnsvWy0kjcKL4UqvgXNGG9+DU0lu2B9Jkt8A8
-vPOytRexaXPthrnwub3aFN/2+n/URv3/HahMUfJzl/P5U/tUxv/6Xz/4m7//qz+KHwNRqXB1XdhY
-/4W3ThH/q/hZixdLFzrRGuKtwfrHgBHQMg1SWqUWvzztRZOu3p9tVP03k5rHgijCByT/8f+hjUrb
-jm7sOmNc/w4zy4/yaLpKfHLeQ79NiQVC95QkD80yF2yPdWhdNRmHN5SUcVcSngo65/dq+t86Mj6K
-69fr26sqW4Ir5416Myi9m0AIU8sscH2Mexx1ZRlWxgGVHNbBanNi1VRs32RIEkH3hCN7nxmGoVzp
-Tc1nWLFl/YuW7o895bebgUacbrKrewb3dvVbvPswZk7Jiw2aGBSaWAFQou55dGZtg4Dc8/M5zM6V
-e4eENj55Vzn/H/LOo0luJE3Tf2Vs72hzaMBsZw8IkZLJTGrmBUaySGjAIRwO4NfvA9bMTkZkdISx
-rmutq63o4Q4Xn3jFxRrtf41LR8SF+II+67FCvMAozsV9oIncGTrHZkhie7kKRxMNwfMDHZas/x6I
-SJddZduWSx3+cIJVXed0+2pqnb2KP45zbvu72QzjO/yOlH+hJnxqMC5FAIHrvl8b4QerORBrpwZF
-mQj1HnEr6Vk/6BrrkNHDt+j8vF4Vn0P4pOswLo0K+hhrEfzFhzNjx4Wizbx85CX/ysHTfiQjHK+K
-uiwpIwHePT/eial5FAcpvoAHC0yxJhQvxisdhLfUjKa11/jB1sCxcNN1CZ4+/D1//smCtUPHVUGV
-M7RIg14OlXmrG+WADn+IpjIV9EkpZA6X2ib8rjFFOT8xnz/tf7oFvzcISgcrkN1H/ZqmxuFoIHS8
-MkHGMDJxgN1ghsNjb7STLvDm6q2/BmA94qqFmnnBZ+3UuKR7DEnbzwPrcDguHRyzBI7BuLruVTSp
-zHmwZoEha52lH/XqLxWMqfH2/GxPfEZ0JUhO6WSRnq6X88u1Hf0RTrRBxYZtSjRac8qRKoKdTV33
-wtVyYofSM3MQq7e58OEZHA612Fr5pGOEjmiV0/pdrKvZG4Nr1cX5VteJ8bcMyb+9WE9NLYCxQDIr
-yJOPx2u1n4ARC6lF9453Y1Hz3FaU6t8tAfJZ51dx/enHeyawoXWzhvQKjxEqOIdYQ4JXDblQVj6s
-fRaAr6QT/2AUWBGuhcGoFx7zhQRqXAhDcJu0eYnrZ0yCkBqpfnN+lJPLBsVrJWDwBK9Fh5c7ood2
-2yFGzihUj/0NnOByvnZyZBLQVAxEe+GKPLUr0Bdx0FMhQXJ4yg+GEwgVdQgFrhtweD8OyxPF9VV1
-nhTap9Jw4UOdGg0GS4AZg3AsZ63vvJycrPvcs1Gog1HWJrd11tn7vkj8GzFN8m7Ri7owuxMbgxuZ
-00ymyZjuCm16cUsCyMeGh65jpEcpVbSkwhq3SWPGl9jZJ74aQ9CLDULurldekJN0TIzeOcfTiETF
-tspCtfULOopAX+Pu/fktcmIVWUTHtLxVfob61OGs4smcalQGa1y7U9Sx+TntD/xd3BjvG6pcUTk6
-6Z/fjrzY7HkEDYgUnfX2fLGQSxOgLzmhUJ2PWYygW7J16OjRZHDJd2LKJNNk6gsvwak1NQkL1yDT
-InQ9er3TASe5yiAH9Pvy1rLiYldWKLMWDvWu8wt6Iuri+f6fkY4Yep4UKug8FjQcQ43GbG7bn7iv
-yXRqPzc7ikNe9Q6QT23ucj26lzbPiacn9Lm8QBO45gr5O1xcEDoBRlMmxgnTgpIyDvOPCyDfbev2
-7W4Vm6G+lcWfz8/55KDees1wPIARHA3aVaFGsRkWTq9Z1Cwsi4/V7H1MvbrbC6+197pPnQtjrut4
-dE+vDwE36JpwvGZCBgupuw3KiVagGSVpfYtbVPmZamL+o6ns6tmt8MtzMRi5sfRUXbh8Xn9ldtEK
-tiTCJnU5vgwEel5oKoPFUP5kPimL+liZdsk3cOnqzRIYuKXHbf8GrdILL+HrW2jdvpwcl7eQKvRR
-aIEVLRjCqa6jGEj3W7hWlN3s3Ho6/0Ff3wq2TywB5gXSHv91/RUvjuhI3zfLoJfAIFPpc4KFebpF
-4qep9048Nc+DcpNv50d8vaAMEwKQwI4HpNmxAW46VEYq6MaCA81wS2yz2n0M1YIgeVc49FhtWnN+
-nYjVFxAnkQvXw6nRf0f15iquAnjtaL4G0o5Q9lFeBApXbn1crVBvdREZ34BvzDCorONF43OD+vu1
-hmHw8/zsX19PNm+KWF9NHjKSx8PxvTbLCJu5NKyJ8hD/+lZIR19ZoOH3fzwS+l+WzRwZkET+cCRy
-CbrLJa8minJ+va2XAMmdsKCuvPdohaUXFvb1KaVVQlpBnEhfA/Dv4XCobRb5NPQ8L1bZ/sWDAvqT
-0rZZxNixDnVzlVRz+1VqX14hD+l8Oj/ZddkO7whG9+AeEIxDQwyOHjeQE16h8FqMUjSc7kzpicjN
-a+uPj+Q6CoUNAmG8nFb82MvDwgkJsiLURIwYkELLdLDymYybfzCVACCEw1j4Uh1NpXccD+kfBvH0
-Ih+hq8QwYZBnTC9cbCdOPrgElLWp1/gE20dRFWxjF9MYUB+JcCAFtGCrsC1JbjoAFLdBMBh/HKIC
-x4O5HPCB4ET4Rzu/T7CVaNdPZBi5vSvHoHxwgXnsgLs6j+eX8NRexKwTRV7LIbA/Dk8rFIbJv2Zi
-AF/3NyJH95HiQrW1gNDcyL4Tt609oNLe5fR9MBK6cBRO3DGEdSwp8FTAtMHRHeOWxVh2gmA8XjnE
-IGTC9tEJSnC5YvK7D5ZluFCKnKz9gCrq3F2Y/PqnHx0FHNDWSpttB9TZjkZHeU5CGsDoylwa8ZWP
-kXlRbXEYNypNEOpL46J4lxgTQqbnV/3E1cbAIVgt4DUUB4827pBlfYuJNSUxs+0hmIJrwukq/WL6
-qnh/fiianEezpDgJ5R0Mpb/W4Fz7+CiCduf8wToO+gUoY0tBH3qtGVLMyGarta5S38bRt7SooO+z
-YEBaPyhw7932dihRJZ0L86s/BDj8efXYLPvMaoOf9SznepOD8up2i0QEtEzWbGas0u4mGYV0Nh5W
-pUTnwH9Xl+QMrwZfQG/Ilgk7ZnxtUQk3ulr6+O0i3gdGJHV/9QuAhEiZssKColftG7q0vr8FP+ZK
-4BtV8VdejRDRpRymYJe3moYajq/8sbnwp2+tl5U/hF2DSQCMjxlCXkxLsan6fvWiVpZNN2cERrct
-kkDf4+ad+XemLwAtgfQpzL3jYHTReWOJm73hYPhUEK8nu27o5Dszn0E2jHOXvJ+dBeQbnpri+zA4
-YAs9rA0zJJJ90KBz6LW3Rja7iv6VWT47AAOBLBJW4EqdzfmtKOcJi9FwqO8Xr/YekJDDQBcOMIwJ
-gyfAjXDAQQPeLrJV1HdwsWJKBnOfKrTyt1NrwOgMkqYtt8D9hlsxuG229UkRaHvOiX4aSMIGmpGq
-XaIpKGsslvAi8SM8RJvvIpDwz4Q5VHLPAxsPm9SS8L6QTnREBLF8eir90Xd3Nlgw1KmMsJFbnTU4
-6WoaWtA+Qp8EL1TDU1rGBvbi6ODdZZLQn9je5h5pK1M9IMNvyW0P0gRElavEh6r2BnouuaTdmBr9
-l65BJ9hB8hWHIpXlWD7HFcRwO43NHzlWRu52HGdt7QIXWycE8nPEhWE6d9Meli4U/UIUoC29FT6X
-4YaC2VovQfD7U0xwhCRk0eNADnNhO5n1hPdPOuMIDN93aFFSX/eH03ZussGK2/iaNgW8ReQGkU5v
-F/xzIBcnePXUFfLumzaTi9oRs9KObrIx+4zBd55vx6QKjS1GRgpZ+0lOWHeVbfBUtU6Kj4gy2udY
-UnQHb9gvD4UDBwnBdhdiuqV9F+ZlGIcfKmy7cLoY8RzbV0tb2BGSm+1dMC9Y/KZLqFHVzXTbbkJo
-PTgmdHP/Ad2DEYlSb1I/5JK2cPqxlH1eKj/9wG5gGZBh35d+LqYvIBaSEBv6PsTDqZ0c66ao7Bh/
-inREUF4nuuu/aaAD+hdicrbcuJ6rjagETwpZ2cefY4tRlCyvxro3xZcK87FvvcSVBJCaTOXDqBKj
-eCchfxZXtbv0K8sdzj5hBfoDm9KMG0QKfG1STjcW29g2JR4jt201zdP16MrMvhutLEmRUZ07Z7No
-2c9fEqGzx7T2kXJPsOODlGJWqJSrTgSfNaof5s4ZK7CZiyfK5dqg2iZwW+v8t+gqu97bIa/ND61M
-f0tTQ2G6BoVqddtOTVb3JghgQXxJ0DAtdihpp83jUItQIDEdt38N01DZW5EvJdmLESj7Z8suAgZQ
-uvH8PABSiqlYpngtsaoewITcsMK7zDH7bzN/Xb/Fs66u3sayDNUbWD72QJvRjVfJ5drFPA7Lr6CA
-dLRop7zJuQH9qOSeAmyC6/obUIQT8qwVEecb7XrlcJVNjoPHi2rFZ2MexzgKqRuX0cwGb28TyI3D
-FbQqB1fkGg/jrVG0xtvBhTm1Q1hyxDIHAwdUyXQGgksBbh42i/DSZNstM519DN8wD+u9xnxspWwf
-U68fMU0BCzRsgA6mmF1gKrOHr4QBQJlWbfaVLnuePoQaaW3+xjyQOxNYsX3NEwlSUg+hqd+qGIbw
-N/QtbBskAnZgoCmdutn0U66M+wHF+l8AG1fV+axfhacLVUMqDanCPSESnfV33oCWBCKpfPu9Ci39
-y8FzAcHoaqz8bTHHuMf3ZeznN4kw8x9iGWUGC0gI9Qmangw2ZVijJU/7R4uoAjvt3yEzvgqtSDkb
-11k1he8sFMvjyBoXGwu9jl4NHmNiSreuBLsN8BJMXxSU1ljehVWICSUFKS+8gTldffWR1uVuyFtF
-dDI0XXk1zdY4bIfQ8D/XBlW+LSIVNQZ2vSu++8OqY5WpWd508YJguwvYNyq8MP8JsG7+jJVg8saL
-8WYPhar2VhkWb80SttSNVyn8feoetQEacrO17PsmA89aqXwcHvxK489Y49ZuYYVUTy4FjHkW+wmb
-gHEDwV1By3JrpCAlCgRQ8QTaDKuT10iPfMyd5qa1IG+DgyrDbGO5lTvvShvx3YdKjFV1bSoeUBTg
-s8Dfec6w3Op+LIprfxq0sc0WFPCiPjbw1M7wGUHUvaz4Niir2/GuqQxUYbtyykqIV40dXKnAA4Xe
-T7gd7M0CQNjNCPkNeytnPQ0NjxHe7jLF18EZ4MXdUNpw3us0G3xU8D3NbnSWJea2xMYx6l0G2wwI
-zyM7bmYIZcFdKe/6uY7dLZ4UCtFlN+MS7+gePqiaCGMjRTvkEHNbkgQTGY+fSLeYbzxf4kkOudKT
-OwtkwaPJueju02Eq3/agY60tSq0ScYgE98jtOIkSWz43tOdonmOIZ61a5OcmF9ZTFcyEGSmuE++0
-7QCkXyA2YzRrZ9hgZEliq43CAecXvQ8f3a+EkhBCtVhLgS+xy/R9hYXUVT54k9jAbsFhyTHb6QmI
-eFnsR0OK1UvWyvyNMZL2c9jH6d4BDA8AftLJr9Tx0285LANoJRwsBAaqkrZGmQRdvePqcvF15Gov
-o5T2prriDc6f4D5kWGcNnvfWd6WXb+W4quFWrgyfUbbBLQGTyewT1iFdxw8eMWbxhlY/ypyiJEod
-A3Yq7CuwCjJbXQeC2H3EqsS9z6RVfNFK+98HSELJ1s5U+pXdayabzA3qW7waAXa1rmqLDVFJue4g
-Y8aK15wTG4WetnnQZocX6ZQIGZGml8+drMB+q6HrfyCtIdqdCix/t1ijV28mf1E8M4IfE8HPGAGl
-l93HWqr6V2l2zm1m2TGCL4gfYYxpTKOzgWqW/EgbEOKRlhwaGAkxght5K0bwE1762UCMg2sxi9ED
-6JJBe9uKIGK+t007u1FV1o9bOaf42FvQLyrinZq9JUuv/dAvgT1eS1N05SbEch74jCTJfpgWPyXy
-KkC/bLSiRolzSdGNN26V1C1hWIr0vqglQr3GkoOzsVLHgkGPSHJer1LBI+akuAIFMDHGib1kjyO+
-Owgq2LtYpsgraVr4ckNnl2zFQGgj3xm6I/RcnAUPB2q75bulW3BLMsSIKcKIiIB9Tbuo+9Jj0RJu
-69j3Mbw1rNUZycwBGLqiE+G2HAkYeDPG/JvRpavqEpCtYbcEyClRV1T8sU1YB9d+kxthZGERiLOZ
-uTi/El0yjq5iz3ywbINKcg5UD80PANdwUE0nw+d1TIF6GTPw5C3+M/zpY20jwcQFMWVXPk/fx6E3
-MThuO4KOTRKnjX2N/Vzu7DNzIMpp2gzLZYx/pxBp8nboEKXt4k+pExgtQCen+tjMY0no6duLcVfV
-qedu02Bu38W9ny4RXIW62zh1BwmGtwJPgaG3amxpPS+4hxXsSHBVKS4V0ut8sQkcSJRRay7Dqlsd
-tMFtEGbBT+I7TtwYW8TjoKvlB0gtxRDh7Ogj+5Jizgo2MXtvLxlEJxq/WO5WY+hERuav/iNDD4+o
-6+cArSb8Sn6hdBLiiwTgdAcLxX5X9OPyZlGl/jRLV87cXkZ1HSxV0m2wgWT9vCrMcRWJrWCPfL1n
-3YxmEt5NTcqP8JLA+hWIXqb4chbptHFRDENKDBom7AiMUYdNgiNbujFCao/E/S7K8ygjFH+5lTWO
-XHlFJjetH2PuBv0txx9vqFJ7W/slCjCGaa06WkHPX2lKDIaxmZTqahk1GjtF3fYZWEOHLRbzyzFt
-mFMPCfVpddkCV37dLB4grEKLWW+0NrDzYfPb+OFJlGYcLj3+bIwbrcgylwRpnU5hONJNKrzXOkd0
-xk9cNjRaLfgNIcS1/iylpu+i7xg4CZFl3uP9y7YsDF4cAklHf9ALuiGP2NO41TW+VyDz8mFu3+ee
-wtaohpZFNwkBE0zCktTzyQ56/bPzV4uiMuQHUgkkUxmpsmIoaAkG1lUfv8W7zfkopprMpUHMjJQB
-qwqEDpHwhpFcTszHTpAlAfTZlhQSWv0zF+s6Nu4Ex6pPRIilR+qtfkhOR6JDXJU+5ZW9mET7SFJF
-dTbqnyJx+JMw4DPnm6bCq/qmzkNGsJcBayVeu/C+q3Tl3/tzzXSIc8P7nGtg4KXWcNay0vX8HaH1
-eg4H7Y57LO6C/YxhSLobpGn+8jAp/n6+7nBU2cEhHpg1ZSVanhTMfzNVXxYAMRPtBmn7FacNZGNU
-xuizXYskhuacx+iVAFUiIXPQJplKNMXOD/67NvyisvP36Gsp14HtGHrWUWXHg0HTdpWBUj36TtyG
-c7IlGbKIiwPMyxG0bpXTkec1ya5kRbZ1HsxXNS4EO0tj6JPObvfZsNlDF37XWik897vWVXvRQ6hF
-67lU02uKGXOb7jozRkmmCutph3nCr6wGHsX+NjIRdT4VdnOIa3ypufK6aiQfa73hy/lfdFSJ+nuh
-fmuJr6qItKsOf1A7Yaqg8Pgh2yVJBraoE5zJyrUN2Ddec6Hcd1SK+j0aJU02BHXU3/Tgg+lL7cCz
-MaFTzbkbfHcyn5AqhnLlR9nkTt9jDAIvlG5PbUMfrAvFPW8Foh2VUmuM6JqiRxYOq0Tr0UMkJsJU
-MNglg5huoJeEV7JO1aaxvQvAk9cDU1C0zZUPwT/NY9Tb7BluiYYA6WSNqiLl1PnNDKboDroq99OE
-wh2qTC2spjK5UFw8KumyyIcjH33SALImLDqagN04N+kWg8QxfOAimN6GbQU2V8cLj22L+KP8WDmd
-Nd6MaY8b9PmNtS7s4U7nV4BwhMQB2Ray2+HG6me3IeDmBJa8oaSsufV2XmRzc36U1xuKUeCPsJk8
-QGHi6PMydGaHLecJatxw65q84kFl3gat1u992/Iv7KbXS0tzk21kUmugZ24f1W25gN2wtZnUwv/7
-bKhVE7No1ZVfaFQ1DSTPIwPYfOQOCky0+lMth/XL+txpiOKj/Q8O4nBNocjjbw+VnIuL9BVn9h5O
-CBeVyM3rP19XYmkY7ytSDITH4UgyLLpuymjlxq3V3pR5YiJxvVonBr5B/twVvv/wD0bEf0fgNADZ
-ftVffXkzmljttGS4uJunhv4Rz4aBGFkOzc/t0gKJyDm4gLg4tUFBktDUWcG73nHzSAOQcRo74Sru
-FM96uMhebqXfj/WF83hyINB2KC3AAeZ4Hs5s9VFtq5G1XFp8dOthIGCepvbCKKdOAt1aExAhoDBT
-HPXAtR8MS5EyCqaX7mpQEy7XeWp1uwk69mOfGupC8+T1y4FcHUAc4MuED3SID6cFcd9N5mDdIuYY
-Pul6aW00VxLf2Ck4edWF6+SoVfP7UkPKBJQR3XCHO/VwtCbEew4gFVsfAP23DCY3JbKCtGiR90GP
-9iMMymH8dH5PnrjDea1MpB+4wG0axIeDLnGw2HAZ6whn9XTPJ47huMyoOiBc2JZx8CC5+68cbB2L
-C9M98TV9wMI4nQI+tWjNHY5MZbRJMQxfay0q+GrBO8fLRZnjdbdQOUvstN6dn+qJTbreaCDVaDvy
-Sdcf9CIwQQJ3cJ2U6mdlGyBENFw0ZWANf36UE1/RtxAU8eg7B8CvjzZpOMdJXq9njiqKOREuFz2i
-GT315f1qhMH3zMX81pyhOVy40E6OzDvkmLxHdHKPAsI4yGdKvEBEKOWSYEy2FUO642xEM8ig7zwt
-1RBp0x3jCwOfOCaMJwh56PUx5aMv2dGi8AfFwKti521fi3HnTYbxFEpHXbjRTswRlNWq8sNthpTk
-0fPQlsJatIs5V0OPbGt0hn01uRBuWFXbepIoGOFKGF4C35yY4O/WOHBKgODWqtb2cue4slZhOK7M
-a7PHgqNLEpjZdnyViGm5cCpObNIQjbQQkBEoQPsYupDDpu/UwgTj0nJWot+E8aN7Ccb0epQVcCJo
-m6KLAy7kaKuIkcpc1gKLwzhLYQhaYDqZ5uOF+PDEKERHJv/g9gRBcHR9osAqqSeHK/2/yyJ0iV3M
-vNJLzgYnRiH5obXOEw5txT36OJQGx4ksB3rTTCvlbYdOCma8nYH+8PmTfWogwlya+QBd2QlHJ9se
-HSehPL4aw6FOkFVWt2nS6fn8IK9vRVTyeG6wjqcQzH8ebjXoNKjI0u+iOuiiPBDa2byjlcDsplpZ
-uwIbqPnr+SFPzAukF5U58FfcGr89Ml7ci1ntAUIqCaZtm2S5SwO5l3i7b8+PcmJiCHQR+iDj43jO
-8SgaUH5C/g/AJEQ6uClT/x4sXb8PfGqcckouYRNPj7dStX8zAY4fttESyofMXEdIDdMMNcou8QE/
-JSFNdZE3T2rq7B/np3hyIVdUN68MkIdVuergmqjQtLdXaOKc1tkWBk6yLZth+eNnDKwESE/XBaQe
-APg8HIXaK3XriQdGlSJ+DCYUcvu8mC+QedZ9dpjbMIrLUwKRCOXG8OiGiD109qDZoJMI0n+f4rW8
-sfNRv4fgFF6FOvA3RZFM7dbq0Z4/v4wnvhzhFljyVXsS5+SjCY64E7cteK2o8Zzky4r3+LKo0On3
-ZUM9L/IK2JL780O+flZA5/DByAdgjEByO1zTVFto8WE2HcV2vVy5iEM/l4bCptywqBk8xs1om5Rk
-U1os5wc+sWUgN6weCVz2cAKOjjs0IALYZgB1kQ7GQ+6i5tFLqR/Pj/L6/WJ6sPAgZ5keC3Y0vUZO
-vgoDRT2/DOorGpaAIsAC+hyFsqzcCxv01NZZn2awXawoCPPDxVQ8apDxwYJgyJld5Z6ztnUyw9m4
-9DUhdSbzG5dO2RUdlPnD+YmeWk6fZQRsFbB93HUhXlxlfoZ0feK5KP8tLi2vyg93zWx6m/OjnNqg
-+GgQM3NESFWPlpNunITxx6eqkPyM+tpAK20CpzoXTns9Gd4lh6STsyKT9yko8TYcx1fL0jdNr4Dm
-xE6DIvzgDBLubpqJ/sJufCVuyHyAGZKDEH3w78dQuWyaizhPbSTPlhjNpQ7gDqpaaLuX1645l/VO
-FeiGCyysA4o+jUQDArBuNFeA3C78lhOLvELHSIdYY172o0+5WIntyQWA4AyOfUMLUY7zPrcgOftJ
-VW3Pf9FjABkPLZuGzBU24VoNOAaQVbqAz75asOdmnMDer6o4p4sUuwi3pHCDMC+acpwxS+l29R1K
-se1nsyWPi4rRqvDq7Aq3/mHKxZyuy8lwU4AiXFZ3vjUCcIlJrS6csWPG6e8fjHChRZwvgNkdE4mm
-KkwTT0DqDjnM1S4bB/FGT6V9BUy8vo4DNPrMrO2vUqwlIFoYrUWzbfZNpG2Vpy4ciNO/Bgoa+r4e
-T8bxvsm9oRwFzc8oxoOA1VCrlhggLcfdoEk+vHWr1LgRUP4BHrT0Y8tqiYxxDgAh5uLPYLl/r8yL
-33KU0abAtHPwv00Ebi/ZQZ0s8am0LiWTp7Yn+wUCKpUq7psjVlAzZyJGzQoO6tCiZtWF/U+7a4s3
-Yy+S27En8zu/Q0/cAURoHkeS9xik/Pr/v7jZHG8RDUQdQKyu3e46YwHEOlf6wtqth+ro1WeUle1K
-ksWnPDp0E/jKclJkH0BI2q9xjjxG21rJN9jNlwKMkxMik1udTTFRPbaXW6V4KxrnVDukX2zjjmZR
-N1p/yEn+vRmw3l5VW6movAbfokQpMX7BJUAlWbCv8aNRW/I3RAvPf59TKxfwuvKN4DhR0jj8Ph0p
-QwC/k4EQeN/DK8i3fjP6TzJN7Pf/ZCiXAu0arsNEORyq6qcePA4fSU6DfIumPdiSIujGFbut84//
-YDBIWxT2CNyRNzoczKlg8HgWYTTkt3Sv1ACbCPTLdgSosj8/1KkdQeDHswpjkbjhaPPpsnFQm6Qg
-ZNtu9VSILHjwgvGSLempg4tagL8WnXhgjgPbuhw92pXsuxr0rIgUql/AhTL9KaXutZcqLrbnp3Vq
-Z1BChH7m4LwFh+dwBe0BFxyEaohJGuT/86USH7scLAPZQnrhY72eGzUYiAKr6jD1kWMyjXaw++kr
-ABc4xXVXadw+NUF3C/TOuxZdNl6Y2InRAoD7EIVCghN4HocT0wop2GHV7QRT6d2uYNEPoJjyXWqq
-5TFu0/hCFPt6f3jcfshtE5yQ5ltH42UwyhzTaICT+G3yVZoL0Bzb0u/Of66To0Ad4RiTwnnH95Jh
-jN60tIziy6T45oxJ95BWaXHhxTyxdmuARfeIlIPX+2iv0wRYEhkA5KrHeXw08TCSEQ5Y7a1Tae+z
-1cblrz+eFlsQqgqM2d/Ns8OPZXslrlQpiQYEfFKAyvoL06A/JAJz25JlOFxLXOge/cijwNgyVCzr
-ZSRpbGwbymVcGdSsnRpJ1aQdIsE3u7COr78W9zr4+pBMlbj1+FlsR5Cw80ivD3Fgde8vefxGKG3r
-P77dffTbfOjhPrc7Wffh6gUoCY5BiPd8ag9oxxfVz0XiltZ5+X/5H/5bxvurCXlArXyOE4m3tSbe
-hyMlQH0NJVo0dds5+1o1htwVQ3qp6v860GcYMl7iCcTn4P0cDeMjaNEGiL4TuGobYx/sFOw7PevC
-Rt9fluMu70Oj2InWldMVtKBwfKKbSmBcm+3FTtypOa9XCDk/twldv8M5l+RSWVPyY2Z8yZoIRnd6
-j1NBdaGkcWIY4nuPjckF6cGiPBxGzLQxnbVQ2Pg62Ia2/lnbIrn+fc7+SFLo/wdhRUQZLGLef6+s
-+B5Fof94/KbKQ12hv/+2/9YVcv71G5LBx8cuUtBs+3+6Qq79LxIJNidkeHIcgp0Xoorhv0gxeHbW
-+5l3zuZ2/W9dIcv9FwdolWHENx4Nb9q6/+d/H5y+/uh//0etqkfk04f+P//X8ZZZHwH+ECi/v21V
-XtWFkBmwp8oyNnbQeF/TAlWhpi/+8MVZNYOoliCoQdeIwOconiuBa6IHSkl5Lu3yaygaRMamWl7o
-nPxd1H8Z3FPgoqZHdkZrfVVSPzrzo2MXnsrCdFsnSx5sOs+ppp2eLO9nMavg46Dt4hlQUY8Kbt5Q
-PekXKEWJbfbo6gW5/hHkk3LuwjEpwH8bRfJmlQB/LhBuxsrYCuM3QULv5KqIUwfdXgdS2TNCNoXa
-6l55nxzkfcen3DbL8FYRw5SPOCla4r6V4Mm2YEaRWyd8sJ/haBRvV+UHuTdxJJGfWqtMC38TSm2q
-77osxZ3Qg7ozKoWDpGulyo6YV0zJ3JgH0k6FNVYUTI16zjorFRsEIcevIkdDflN2MFgQUsQgdLS0
-50VJN6AlnSC7cD/KcG4jYeWhsdMg56YtrDb9nNcrsLqYk865rxD2BhiBatsQqcCfv3jjpPF9DFP0
-nJohxg1Q0J5q6RCAANpgwLYKxkG7+JnIbr4PmhwfExMfGDeKu8WYNmODu+CuBmiKDx+k2YC2eTrJ
-SOLoBbsiQWaFCNVS91mRkN/Tc0bbpZ1A2YOGDJsoFfU8b4S5IN5QhOo9Hn/Zr0EpfTugjv+5oHaF
-4KH00ItMCuE8kODBErG9/qlHwTmNFP2bu0G1Wb9d4mxBujcYinCzxJPGKJqO8dfYyj1kIO1uFcO3
-wp+IwwyY5WWZF0SBzwO4nSVl4s0El+CDtuckvCIjDh/nvpRJVPUl4M/MCg0ZZZWo15b2YkiMN2fz
-h5C5/w4d8wYJ89RPHsCJs4wo5S8den+YwkWTHM3yDfva1puqoGMakUwCmU9gYcldkMnquQDHFgPR
-r5d9Bwez3S5JSCVGdU2MdmLa/OCKqL6P4VChim1Y2Ki0zlx+ytq4AYPcWOo9NdMOh7uhl9+KYSnf
-yDlgx6MgiTxkJfNuF9RTwucxuuoR+GjtIXbog2Ct2rTcT4HuQUYi0gHXIsuZoKimlWYmnPCXH+jp
-W0bNBOByLsSXbgGaVCqgSMCZB7fa50B6ImW3fP2591DQMzS8wGsXFfgpssPQiqOkLQA55jHoJY6U
-6D70lhJ3QTvG7C8fejqfaRJWhLIx4GmBIr6zsnsgfMKdGRFT9RLir8CYgqc5TBBJTIzYuNeeCXgf
-1EnxIcO1DMmnzjCqXZK4fYBmi50L+IPL9E7zSz4Ydqp+kTjLlR9UuPeFZQNZrzvU8dn0euU+to33
-YzQnwMJtov1nsPk9qGjuTkAn4IbfJ4Co4UjVVAmHSQwmUq4ii7e5WurPtcj6dI+l4pBvBVs3BQOY
-+w6XAajPXQzz4z4ZwlpHTrPoj6PhgEvPpjKT21YAQr3KaAgsq1gzgOG4QpycNDgfOCGBs0zIz4oy
-3MjZW25ZWrFtHDgpoguatwqZNnTorwL3gVqdi3hiH9vvBs9HCGDxLLaimbo03ghZ8n2tyRDHQlHW
-CqY0B8ZuxI6zG0y3f/aDIvBv/VmhsMpR+guqZJ9s0zybBdWasObvTpLSBFKfmL8kjethSxxi7LCz
-82A1oNXRRVU7tI9j5rnQTWgvIcTN/XeD8YF2wU5PRb9PQHt/6HWSQycIYv+LyLTwgRuHQIw7TPG+
-1ovXONHQCJy0eqGB2ha9Hj8kXIcLMtwpSM8knoEBOSmYj0hg5tDiMgRqVxdoZkZsZGCzRmCnT21g
-z7dwxjwKi5Qb6p10Fm1ty8qr7uMmXPqbuMRQPtL5UFIOlkn4kBt1O2/myjQ/pKaJ33JfgsreNcia
-v9e0iiSffPb/gvIHE8Bq8vldEnrVz8mTXGNm2hlXwxAvuyCdkEnVhuvRW21wO8GBuAx3k1v10GWQ
-+49q9J8yXLRGpXdz7TnfdTqix8sjXXQrhQCdUR4jFzdRJYC+OkVf39qGn1lvRVayr4FCZt1dZ9ex
-juyuazyw+lXig43GQnO7UtAQ4l0yp8FPdUhuMEyF4Kbh4P+0fZV4d0mfNyW0wR5pzKFP0tUVuoqH
-e5Ii0K7QIE1c8Ypl2o0ouFM8lp1lQ4FLCqxEAeo+L1O2agmhggydwHdznth21u8zxELTK4ibAmMT
-Sh9b4qU5vC79UkCBGNNk2PmZRDMKN48SltwCUyqqc3ycN0DqsrvezUGmN0YIkBwPE4UniB1bX0WA
-DOo1SHXa7nbdOsmN8KvZ3mgv1h8C5H01t0pP3Rt8LtXs0R4tYLHByPr7mbOCzVU1fV+KhWZ38htW
-IirlfARsrKor7LCn70lfe9V1n7nTci0UBD0OTM4uaxKw5MDmZwp7Njejwis1KaPATlB396Y2fNZ+
-MTV75YSF/r/sncly5Ei6nV+lTXuUYR4W2gQQExkkk/OwgSWHBOAYHXAADjz9/SJvS8rKulKptjIt
-uq26spOMAXC4/+ec7yScklNz39I0ldLShdvbQSdCMeJhWG4bM+2GnQbDQNEA0VQiRF6BiMxz4ey1
-n0tCFiWtjjpht4Lvnli1+xh6TQbEn1rR3exC/+ezWbjKKZdbin1pn7vThnFYLL6Vntuh/Gkmb+2O
-f07DaPUJFjseJ+Uon7LYgqO1AGmnZjOZRmO4N+Bcx3jT+fiFmuZl19oOca9zo1mxx+A/f5Ve0FxH
-RQ3l1iHDdmezUrogjkkz7OHKh8NhFQ3M5qxtHAlbZBbhTUZShFqz5ZwcG1Q3rhSI42+DfVyFxmGa
-p77hYZ8N0UUh2NocLaoDCgCyqekzpw15gIzV2bso5970CKoXzXAce4MPErtHG/sEYsm9jrjh027W
-MLrrThs7sU5NdhBFYXmJl5HF3A5LZrZb2fjtMywxi1G60Rgnc3BMIx6w5IMJn7OFAnNdlFTeWev0
-3PZ9mh4zVXItLVhLs42cIBLsWACI47gUqr2HlSnlPiNjnVFx0i0ZG5rGza9NZ+71JajZyb0wjfNl
-PJxtabcD2eHq2EJ4718oae7jaTbkA1kC0grtMI/pnmZ4dSREfn4RLbfSsa1MIjwMXLh+TTqT7WQa
-aNtJKIpeo0MnoURdOoVhPTaRtssLrkDfYOZH5Htjd2lob3Hc+W9YJMRnOaqGWNVcl3IvxsBYN9Sv
-+LT3GBVBDq2nPnEqUV8b2mnOTy8TSDndOu5FY5BIYrxJhLtPSb3iZM1NtLtRdc9pSMpxswZci+y9
-wp62TX4DoT7TLvxkwCl/b9iG/Zqts34XTAi5pN2F9bsXfpklKwMlyrqly0XaN5I7juZY0g+laXEh
-N9rkAs80LN4NQAeupIDuCR5m4yzvyxXAb9wI32B3Skbpkc91/prLioIh+t2bi5Z0BakaS4uXaljZ
-PxSeNAl64J0no1GHzjMcDeFvlF+xlKVDEULHKVqcwDCK3WMY6IXoRb2uxE09OwK7OAVsKKehV3cB
-pz8W0TGN2KE67Wckw3M/kqJkMTSpwGD+QJR1Y2eL/tEG5RIkKUq4jNNIGkO8BFn1heCKZsSBozd3
-QBHyj66fiL2RmqeIqsI2CLV+moutzKp63OTrMPxgzGKQ4TOq6jnytWBmTTv3lSTr423H1V+/ZWL2
-n9ZVEQySXV0PG48s96PMTVse+MZde7M0rtots2f0W8M4p1/70vFeU+LroB6kBSFBUbW+oc2hp84W
-/DqLfGD0l6z2XR2n+ZA9kIXy1a2WITo7dZZkhZUPMGOnVI+HdZpE8+5QK3IKyCG+cT3nr+swGV5M
-6MzMyPrMBRoM/o6Rj9JwSdqBktTEfRvqw+U8hihsVscrWS12BjIlQbPB56PWDd4ieg91ySiTWzP9
-nFZWWvJibXO7hK1zymirX2O7CqsJ1EspHfZQ9DDtFFU67mE2svWqn/Kx2U2lqT4D+jJpUM5KGlic
-waYI0RR4v+JJ4ChkVc5GAN62S2XzvABpDKhpZq/VluG+bM/XBEYKr9k6ejQ8dpEO0cShZ567hW0t
-LgMZDinV0dP8IbRlXQ2VkRs7FawOJ5J+BhhKpQCbvJ56J39bkvp6IyzCYujO7njXz3kb/o0H5XcP
-A18B9xykJKI9HJf/Yl2rCp+AOO8vo4Jkihfe/Y2QOtoaOBtZHzkS1k3X7Bx7zf5mzG2dz+F/Oqfz
-u9HfOOIyrHWhJ/15ThWJ1kxLElJxsejmpZZgdPnICdTxKeEf7UBq27SucbQiLFmcE8AdYIftPEAK
-SubUNagwqFhe77t5tU7SW9aPTpX+p+GQGCJF67HftOY1fR6oWLaTX4Y83/7zZf46Mfld7Th/cIzo
-UXaBPzGD+G3Ilq/0tqZGZ8eYITjszGvIPcqxwxvX/p//KuR6xj9nCZbEzXnG/osk2lVm3pcYJrjP
-pnybymZNNCCfpIxk/zdj5v/iK8GCwKiJ/yCw/u48F6SrLT3OvKvBbC/ztOn2RrrWsW0E2Z2a6o6I
-z0ideK2dE77iv/Pv/K4W8KEy9YCei1WISzL4TWy2jSgCmpXbbB+ycG+scEbIt7LEmobDebY1b//P
-X+J/NfayCA1A7mEk6/8+kSK7jQ2Eum5Wh9I9lGSyt7LI1d98qH99V/yCX37Lb5dKiYBlQARJ484w
-A3aXfhtX580GHWa30+R4fzPD/0s/ys9hHtxa5t4Oh+7fxW2vgb5ahH6WqMUprr1Ke7fd0rIBCRpK
-SsJN2Vm2frf8tEwPeWlZ+1HAR0hKyQSHadk6PLN8sW9jj1gVh5pMZJWMw2i3hwUsoCDJ1oEw4Ir1
-uFV7ZT1ovQ4PQCLStwLirPib9/OXACBzD3J/kNcxBED6/l3tM+go8vJC5Mm6SoqF+6ZdfCClYXnl
-VKV4y8dVnmv3qk/HSx3IHwTv6jg3RyqvpACKCZKyDiDWpGxjkqLv3fd/eBWdE0SoQOhALj1Fv/vt
-ncUFQNNGGWtSnl1RUCcT5rzW31xFP2HOf1ou+TVQrG3PtlDD8Zb+eRngS4LSA1Y5ifQS1pd0G9Im
-5nhTN2xMWZZmvLYkSs9jwel9Vdp7bLWdV5xPZfPQemr+XgQk6v/my/nLtX1+UTj6MG1hLAp/9/UR
-kyIolWZF4vcfdToCE+76bjkoEF9FvNb/9JO2CBoyEcV0h0SKGvbnj4CdUOAaacN5iQUCqZdEOYGc
-f0tT/0ja+H+/LeGn1fV/L2tcfacsat+3w9D+67P91/1Y/VoZhSn7bCj4t7zhmX9AOmeqj4ZwlinO
-Yt6/axO8EOUjOsc1cX7ymDz/rf9ZmxDwZ+w60DS5HczAtX+RN9w/TJ8YApEuk1kEQtY/kTcwVpzF
-hV/vHhMq3U8wHTco0mbw292TOgCKUoftc19BOjsXKDmPA2P7cWdB3ehxT/fj1zTL5UWMAJ7MsOEA
-E43SOnb2rOM2aKx70kE6ObfYHppZUFnids8W1KiPrA9Lqp1Gdc0uGba8zqYjoJSZKSE1bbe5S6vc
-hhEGjvqoACsWmPACinSy3hb2gmwl8RtrUTfPOmryXacEJMKyRPXHl7dpcoRzmLauuXdQDx9dm3HX
-BoTZsJtH9pY7M8iosozGIXi2G8XTsglWdRrHonwlCBVZm6kW66HIZfsZ0r50acgueKWuLUhYbO7a
-KOIw5a6NfjibIB6HqYiuGShyUPIhcp21J8I0s2VcujJAf2aGWbTEbTI/nsE/vZfZGO4xjhmXfrm4
-N7IuxVULe/jVtB0xHrOVoTNEGGn4L4McmdxMkcP4FtLF3OiwSMjyOq+Uy6c37lTqh3qY7MfR8En8
-t4rRg5lqMvazmPnEwnnNPqFjZM6mcHV7gjNzbo2tRqL9As4Pwz/nTC3ABn+eVekH05izz5YeTLrW
-q4VBDuKXvJ9VCMKHpvX3uVjGfAcriS6hPHLXy3kOoQdkyrM4uevzDBFXIjH8EqtY0uZ8HoPJPxWW
-Xd7XjooEs3kr+0wdCHPxQkHDsh06RBbasVJwe6bhzhdzZwEJmHLnlS12ehP+HCicndLfsA0gz06Z
-gEQUVANs6hEOFV9kxli9KgDUNN3z4sE1EmSO4dHQqvFNRaBEthVo6YvF9bosJrs/JGVjtbcpY7uP
-GR4VMfPzwMXQVqyG+qMwqhs8+guN8WFrHZAtRLfJXLM+WjzEb8LKyZ9GO1D7lg77R+oYKfRQnOxA
-XPVWEHtG2o3Y/8b0CDTBue4trz35RRfc5hRiUXWrvww3PXdCzuJZhyNdVjSgx7SpR6+ddP3HdLag
-W9EgJB8H8BjQ4I3quZhdJz8yf+UbSuXsb7VrNSfflsYbz7fIOJh0a1L3rpommc1mpVA+c8OrtuFC
-NUuPMQCGLfF9hl8S3rQeY4R5WqcqcZ1xfHEABt3kBY1XvM9KrLR3uS5DSwt+g02jByAS2oBvyGkA
-iKhAWFS000KUuDA9GgUYd7pC7IIyFMHFQN3oPvTPXDtzRCK8NJmuwyIwVRgcZ9+j6KhBx/FDw8CI
-Gem9FcEeukp91eh75sYpvuIOOkcE/f4b2VHFSxQeLD1dN+PFStnvVjSeEJvJFdl2rWzBrdz57vd+
-1RVECNEOAE6k5erbrnbcTyAIcCtUtUYJeq71iKkw3It6rvbr6gH5K0MKGNXA/8UrvK3A0nMfAAYI
-NjP56pqfh3b5YMJTusX43209P/3hzYGfU2Baj/ll93PIzNWXZt9IVNXWVqKnvrWqOd8MOgVygQMv
-3PPY4L6E5ONld3NzZv+FQTHMoDxa57WdQ1aKsgnOYx2b23QH4YO5T6pDQIQwzQbK3qYy+wy1B3jG
-Q10Ld6s3cUgry9IowVLiXzieYUjVAcC1f6xDsz6pNtziqn01zLagTGxIP6aAme5mMoejX7S3plpD
-phX5S1HlTYLstxXIFptVuB+tYolPo7X5zAldI0WlxZWXt+J6nuoDo6JqO6nlSeXh42IEF/0YXC/F
-cDHWFqi56lTn4WeYMbKyxKl1+ttoKvJNkDOkdzSOM220t5ViHw/W+lZqseu79TnNnI9ypI+D+PVW
-Z/qWTzrYMfkRcWH59cMwud6zNDJ4LgVcVDvvWqAV65KAE0R7Mcf70Kl3M2juuO/Kj0BHl6E2fVrq
-6i31sq/+EqHhgGaq7Dt/sB6D3paIusOBUdgNbJZL2otvKqPa913zAu31qsinK4Dt75lpn/xoRNHj
-FWNes7boajuVLncm33/gjYI/UjfEA5NJqlNFKfe33o526Rp+b2weSBJAz8YunfcJwmbniu6i6BbB
-wwSb/opsyh3AzLBrqpNBC+NiuB+lJ14aWSZDFt5bCrt9ZD/M4JxitgAlhcdIXFALjhTMvoYtQCyE
-pTPyAHYOw7lioaw0KHY8dyDHqAgQeWFTHdNa/UcwBNbRNPyOnu5JoyWFCARRBJGmjD5bQLCHVhpP
-RId4IPQYLiEkMIRsxRD+BLac8mh9Ul613nGGn3cZp0wIQTw9sLhyFTc8BENooOiesg/BFRYRsEAJ
-Cs1dEXSpgXt2ZmEezFWF+1pRuzwlblO0h0G7Brp5/i3nHt55WRa95I3bH/tRwi4JrR/ZmHUJNqz1
-OVNhtpsCxLQVH0A/1PahU2EoELPT/mDlJJQ7b0y/ACGRECiCCSjyFFxX3WRsTdb7JplyiCOFw26F
-cPi0o43oVIXeeGzPWpQ2y3cdOUcj1E9G0Re7IMpyzH5Ffws07rZhPWZmLX4YozElvAK6DZvhPcRF
-EgNKrHZ1OXhbjBBI9T2dkhsx27SHL9EbrgMort2EUIEZ+Dgv1hh3tbLeM2bIcbW6J2eqL43espPO
-8u5TsqvH2lRvYIwqcE0Eh3mcV9Y3pX2Fqd+jP0ndZbnc2V5hxlPuDtcqzT2IEyUVj0t/LDqqNhAD
-7hCdDsJmCS/pH0DDLcykcrPy0LKLIw6pD52Tih13uEcc0/IvBr87TYZ5bRTqqayKT9NhkpQBKjx0
-YXZvlt2DnS/bemrcjS1FNMQ+3zPF4Wp4MsqBUkxl+nu7gtjoLOVHFrjv3dQDoo26l2A09iFvb5PP
-0N3YK7Lsu/quXoz0m7Zmta8lo09HpEgSitKuYW4+a2EfwZLxl9Blx1M7r9O2rdSPzKr29ViO9+ge
-iOsWHBV3Hd98ZO2jX7XrF5Kjl/ThmFM2yXRspMt3Yv47NnExN9TFT++TFu9siaplW67qygnLemuF
-RXSAjChvsjy3rmmu1wfdjXaSI3exRJPGQt3R/p5T7ZOWoOuI/45vBD+De8P8VFFQbx0jXI6QzU74
-Xd4o08AEM6xRLChDp5CSouGmLdyNF46QX2ZWEzOi4Df0Xx2jpF4mW2/LNmuTISou5FzgttCLu5XU
-zCa8BQBi1XDdhuGBJQa1M3Lv7VTfAFnskJTlXasy58igr90yPtxmfi7iRZnAcNPhvk3zIycH75F6
-np3pjIecye+GPVXMlg1Zv75oFu/7NFtf/ppdskBPcGSZvjsZK6WwHHwRVMfku0WJ2MBYscF/ZW4k
-ye8E4xz8nFS/GHogkzMB9nFENx790EkpIaUCcVmtTbCmwbHUw40zGBVsCxdZ7uxinPbMnfeGtb4O
-AZahCIrXl5KetfXPTLm1Uq+hPVe3gRJffFbXEReosN1TV8hyRw+WPLen0RHisS2PHCFiai6/Iltd
-R/24q4vlEljhU9csxYbqm4l+kWaAA8MTNcxf7Lz/rG36r5F9kNY4H+vB4fUwGdk1VVBcdHb0lvWe
-3qsyPS1GGwFhmL5C2syS9dyG1dWoAYbC1Vp7eCaqAfqmA4bSW9nhWSIFULJKnvviR2q4n2m9vmAi
-3gKRXB9tnxbuQG7zPiC9wcRlt9a62hsVBZq+xRM+88a9aPKjs8J3hbObXurVOVdOZ+tG0BW/meQZ
-5tU53lba4xWboOzSz7CSIL9CAmYQmWChOJT+0m7I1D3RkEQ8uQVkPjYe3ijXeK5a6e2LJjc3zJ3L
-mI/e3iPvRHE1s4e1zTW6hpXZc0Q7r+pUm23dJlBJih8/7pexRxcL/HMnaXMYDaM9LQMC6SQZ84Yw
-75iIGWlsKRw7buk7eyRuFHJGphdmzuNNc3g51rbHGD2dj1YwWJeiOl+OmKpeFoVAW1QTCPTS3boj
-5QeLUwNisW1U14E27CK9rosAmJ0OwJ+GbXB2Z4y3sKX4n/UaIGC3ZxobHbsG+6FDsLZPXLv1blkN
-/xoCLc+byRKXLHjVvnDFy8rkZzOiOYLHZAMHOjHgGQ/UlE21jk1zabeToDS2KHpkVaNIzMo1v+sC
-egLdUGkirXGf2azUnG/H/aKW2OAj23ay/Gqq9dqNhn4HO/yZJdjaBbaLwupRJ0tAnjrhsq12a8/3
-GSqr27ZljlPCgsMJtoi9U6pvjVCe1tYxWRZXqH+d8m5ZU3GqNX6PRTxVxAyL/LaaVHky7SliZ29Q
-jpFNeuut5UV2brCAoc9K3OngA5caz0e4k551Fgo0E8DArordyIWZKbLsqD9siieanCUFHAfX7m4m
-Y+lhRjRmgE7Pjd3DbE0WlFmeM9Bh2Xmk12vHW/Brc2va5vBo9nl1yEJ+6WQaHw4Pn4tRwiDW7Yxv
-z2zsLa6ubtOmhtjjvasu9UioFxXsDgYl2/Q0tXaTW1nXkzddkt8swKb3b07BjiUP0K9wErx0FK7v
-xymzH3PMHMQ6KTemMtWEyZfNl060vOJR2LmEA+M+z5c7djjrl2CqT+HvhFELtuQVN9K1gzsC3LcZ
-7AqkZkJpuuJBOhgXKgfrYA3Dx6yt6kKt/lOzuANuBADMM7bBJ68QflzJot0XvZfYlIO9qjLj0Fli
-h1oVMGOAst/p0njrGhxluYxi6RUxY5T5K+/gPfuiR1By7FfalzsevOj1c7C4iW2P8GLtZfymPKqk
-12rtDgEQta1bhxMbZQL5beSDWxIDvLvgDC+MzvdIs94yxX4rRx7CSssxoQhx3AR0bbfURGypMEsP
-jXb7m6DHGGdYLY9+0wKkZ9pbHagAzbtOtyO3YiECZwezMdiqfBwhIhX17SQ8uW9LPwcrJ7sfILes
-uE+naCeVPXPdZJ9adzkzAATR2XbfAKK8Sz/47Hsav50mdz9sdzKey7qv5s2cUe0aYemeixIJS3bE
-HVJ8cgViaBIURYdHJLIBhab8O4uDJBpkeYPGSXYgHdCszbKm+zaKToG7jN85sYKLDOvstkQL3qsM
-zGXVYKgM53Zg1CrZVTF9Y5gU5Siro3UbmAZWvODSw093F9DqrHm7u8kJ671fiVeae86o4HS5j1ye
-2n4/DwmABx5yguGMp913pHwe5GcpJBKl9SqNGe5tqe9WOC4txyymUoMNPRpzm98qwsCBnriJ2pMR
-CDZ1rCdWVjXsj8wHJnunpuujlzqTNzbugJS26M7bNnVnPaSyW7e1C2Ac5utqsq3PJsYGc5Wbu7Xs
-sjucPpgjsEIotSkZc4/8cEmVcC2i977RKWfOvutxOvWdzPoDK5YcTh2Yyo1jGMvWNVMnDiK+jnWW
-zHDCis60Q9l0/mBsCfE4A/UCtCBchkJx5u+agHLtITSmYjN2Jj6rPhtY5pdpSFoduOnwxEwkgCrY
-4h24tgpSp1tJ4KVLMqNmotjNAV3B8wpknhtzSNXj6ESDnfhi2oOsl3XiIISzIJ+172R2+mL+ltVM
-8XEaLN3l1COvMQ1aYDWTw+3SeDUslEU91dGubencSvAiwcJnL46XQxSqj07d2tBoM9Z51CdgePUO
-yxiQcJjgy4YAR8k8JfXEpqWYuTu1wi84uvLGtnrwCrxyrUPnAtpB9ionIWnRmxw6pTU/FQ9KHS30
-2GAzgOCppLxOR7tU++gsDJ40JGPx6NBOLS8iNRcHamHDq2AdLYyccHurRPG8FMeoSpn2sTMXD6Y/
-Ua+tUBfj0mUStm3ol8CiLIvI3bJCdlu/sSy67qb0OFvZ8lxbrseNqBfGaQDjJvqKQCUF+9mpcWRY
-zACwBUfY8TbBqPALmE3T3WATrh4m387E3iOF1h4iRi3gzkKI9UcGYkUixJxArLb2UF1T/6KcCBRj
-t/BKfzs1qe4TmG+A1vuu6kzsunougAMv21ZOtA7A5bq0wzT2ib6bY3gRtKN56PWEEddvl+yEKWt5
-Exlj3H2fm8vFUIC+Triix70Xyo/QE8eOEgstmIW0/sKF7+1Sx9+bqr63jeYCqWs3CuyVyn7K8+IT
-xf/QmwY2A/tkLuGFKLpi0w886qym2gdiekPyOcp6TkZdfffb4Tls/GdW83vH44FmrK0VO96aGJWJ
-ECTqJQaXExtnC/kE4XRq3xgX3nlTcYJttAvHD9UXb/kSfAzWctGD5z56fTiZB7w/7anqrF4el7aT
-uDkojQw7mX9Tcx+Zl7McgOZ6JIJbGEKx2Q53OhjZhaupeinrgqsiGw1QVFydJcBfnEHR5Cc8HgoP
-mrLKPf82x5gN4nb0sxi3MCTcrsUr84Djx/8mDS6wBJvWkh+pPOHv1DM2/thgoyYe4aO91yJb7kWQ
-qx8T7pvgwusEG+B5MEAK9bl8Zlwyf3Tu4Mk416vgfNdx721m3nd+mKeywhfqtKV5iCxqI+J57Ysm
-UcrRz260lsE2n1q3TCpLryfFe6ZwPSy1fbFEiyEOEgDUTD0F2V70ccrE9oHRbNnzXgwr6/CG/SRJ
-H9JUo4LGzOh3tzAPVwnNW9l3u81TDA6egzwgZVZnV0ZumRB7/YVzaT9FY0ApmWl+ihKZGRXTsvJH
-han1OLK2Giertoi8S55p5X96Q/6/Dvavr0YBND9+/vf/ZhMNI+T2f6WD/VkA+/n3/pcAZsNvOBNx
-bDI5roeV5d8CmG/9AbUJ0YmotHkOpeBp+B8CWPDHmXZJMu3c5w0V5Rf9ywr/QKemCpaIsI9JxrX+
-if4V/Owh+5P85dv4B8FTQbbDsXKW4X71kDiaAAiGmzBeQ8SX/UQ7DTjmKBtuYQZ7/sE2sZFvFr1m
-ryPijrlh2IwVPcLjvyQruHR8ckuTr0nYtEaYTL2Znxq8+m0yBxNwsDR1iu9zZ9d+Ag52LfckO7Dv
-YvzR3sVkyyoH2LCqI/M0p97SVjl8SIfepI07MQ08+iztD6zrzbeBk912GOgcI7VQp++M/fIDjHnr
-rVRZ9Eian2dM6M+2BKtchYo9i/aONFwFGIynxdlhjB4532P3sOOumYzXoZqiQ8SDC6vwfCbbkNTv
-X1Or0w/ZPLY/7NAYvi1dSRKk7ha4/YpA1m29sABziozKq27NsA9HvhrpH0l7yfnAilpOpLI0znN1
-pzuCFzZ/pGQ+NMuI2dwFaUTNziIXKtjL1GVN1BmbBADRtn9LNxMRAGEwFU48sVSMnJxJ4KTH4wDw
-3m8WoN1d1yUl3OAHYfd5vVeQeaa4LVnms2J0n6MZCsVW92YlLrxBTz4YXs0ccDYW72jIYLmZySn3
-u6Cblqd+icoXSnkmRJoly+5lYOlnoUY4QKz903sUccLeDHCkbryopuoxaz3KO2iQJ9cwK58/5FTU
-d4xEFE5+YzWzp8qdZJ4MsnTpR7aH6B4tKjDZqDlVQEJlsl1CCv4qY2dgThfn5WDwXQU6f8BVUv+Q
-Vj7qWKAyYZ4qDYefakTDjxx7OE0tTjddSywzEqJzwXMyIkr0bmUSczXBqq7eKdmpGy6CSO6KMSOh
-Ck18xFVP3QEmTi3xJ3bhmVwzqVZYqIg5eSa2IQpCDyaFDpN1kd1EXtu5u74QICd7P19whDd2jQqb
-1kGMWNwt24Vew/vGyu3niJzoWxXZ2C0C7DKY2vmO6IDvC+d8E4wZhnA3nbC+ypzAE7ul6GqYRbvG
-Lfvdz0nXo5ekqrfE1vNk73MonyXIavZVB7/WSl8KixjRJrPzSe3mLujRSesGH8ngRJxoeIz6+T7F
-1PHl11L4W2W37gf0+/C+hGbzQNPB9Eo0pQ3iPuutK3AkjPbc/Mu1Oh7E7ngjwqIQ1D5woKy6NrH7
-Lsy3s1vK56GuGXhprKAh7abFQt5lWfoHdynyEppqXRU4Ltv0laqd4lkOw3zSmfUo2F0SBwmbF+rG
-otu80BLlE8/gHZun/nsGa56FgcIEbhLLFLeGQ8wDiP04huQKXNIFnAVJAPP9kztqWSLfh7LhrnMI
-6WK6HcOSUJeFGsDkLO8+K1MQIMoMKzrlIqUMq+tnk80bW4ZqXwVpGm5S4QU3tsOom06LBnMu6ZtU
-7HWQI5qSq6m5ljpB9bCZhfyslfAKXE4KZfm5DLzwQWfnvo2q9Mxj20fLUxtMqTiYdh/uc0TWO3cM
-JTAp+KUbuZg9o9/QKup4WUDr9vwbKxF1J4vdJI3owcwRChJOmt3XatKBTTy8taI4SO31I7BSfRkV
-86y2pq+bZ9qJqzRpgWpU34x5DbhW3Nx7h1hq5ftQonswFKNEZEcUw3TpDw2VecB9I5pjEa6K3Z7N
-xD794TrFLBgpMz1T1LyZKmBLfF2uCMzjJYVjmVcneVNhVYRUaGJRD5NMVlSo4MQgKrCAE3zhVF0t
-uA3TNEtsInC4/iJP9JdmUKTLZjXT6Fi7c8Dk97ySxX5Up5/2zDEr7sOlsncl9ScYwdexIz9U5dq9
-9Gl2GOPFZLVLpq4J6SRxce5rLO8lTk3jXHvllyCJ0floJpGrOe/xRmjCeHoKOJm7efO0RqAKWNnD
-sdpKpucMKiuCXRwmhteQYU2wmRjyE2cyh/7ZMjB3xyGjj6+R5FsZO11Q2/HsDMF4akK3PetAuixB
-T/qYEWhFa+XOXUovO1WVlRHRItjRUeRp+caGgIF2QT04gUjqFLQHA2OBoW9oZ7vYehQbPmiDA0Vi
-K8ucjsvgEB3IrKZ5WR2g1hcA1ah3yymEwHMQ9GoT0C2vEpf2uWEf1LIn11OUnUpqTpT4mq2WCCAx
-nqGKW/Q8wlO2j/4q+HhkbASVQ4USJz/Op4Ee7+pKnd+1Y3c0jOhe+rsg4C1sKqvBSpAtDm1qdBXI
-ftuourYwyHmtySehnRfQCAMUdZku13Nfp1YC29jIN+sAzWXj0JA9x0atVgLkHoUFYxcqlxYyPqCt
-6+nUApqVgbUn/tPqYqmJt2LdMvLLlRQW8a25UUfRlgSy+tVnSJ+W9tnVEjF32hLzwr4/FEHbJ4E/
-Zp/CmEh/ta1DickwjizJUJ/4b3Tc6o7rRL/3toXg3w75M5j/+r6eSUjt2Blnd94SMQ6x6KX+YqgS
-hJveTtEqHIvnNnVvjNQNllhMD+OQ5hvFyIWpkkzFc0pecNicFxAWIFfbjDgb0j9MztV0P7v2Gu25
-5u3bcJpIGhEBrprdTIKA1Wm1vQsrF/OwFzOgmrjyeutWeNSp2C2Rro23UFyRhB0BTpqdKLIwhEUR
-RRdQCMErJy1kDANqpDl554jiKJhID/7Uv/Ck5bt2eR72mzXFUojVXoVXog+pyiBwJb6bwiFgIvTP
-sFJXU9KCMyu8llowyYNtXF/VLdSXEe99ypNwMafhMTfs8slfXAcT+rwWh9Fv0u8NeOeGcbBlX7eL
-S3JMm16/D3tSNPHSLOp6nVW7xKr18F3KpmWP1addhivbajRfTVvXL01oyS/KaZwvl18XbdI2xCWV
-4hO+qQT7DmeeoudVD4uLvJOpZ1Dq4Q8ZRt2PwCisk7a90NhVBLXPK0NmXhfNGF7SHt49SCMn8ETR
-djUACBVInWvG0X9gm8u0rHTar1C2/Y+JcxKGLj1YNFKSGXsv2pL7wVwLugSthquCiF1Kb0lf+3yC
-ypRG+332VXBRW5RqbJUB/eE/2DuT5MiR7YruRXOUAXC0A00CEUEy2CT7bgLLhglHD0cP7EYL0Cq0
-MR1EVklkJEVaavwnv7GyLGSgcX/+3r3n8kUW7mPUqKxjglM335xBb+3jaE7zJ4/h8sVQ1iVTLMui
-K5kbtfXd8DVGhk3m02aiAW+KjYcR6JZgMsaWdsXAjO3bcO9GSQLsynZau7rnH+qnEcgedzUyhbqw
-KrevAsdcYvqcSSt+RqxMjJHaavQvtC4x5FeO/tNOgZSd1+48JeTTwGfV1k1JoYVrZ5nFV0ZjGiug
-lTDyC9rwP9JRUKxhb8h2lZ0Z2G5CnMqNWYnLSnq4/+CnWS+zRdthhd5y+GYWCqpSkibOad/YHTAT
-v4zvh6liieHgbJ8DhcPGN8I53LgQR+Wm05esnKyvLPLs0oITvj374alGB6WjazZqt1ZTqxsLOVgS
-gM3JqyOQhfFZip/3qUYk/8hKXF7giR3FcUKvZUtXs10iRTOV0qadMIzgz8MJXKJotbOEfJtwLrN+
-R7fPMc11GdJvTtdYQIhsO9Hrwq+8B8ZQXhHAsxx/MvVJn0Y6sQh/qZyaoNbQMwedVre0X9mZRkyA
-6SJAGyWfm562OI6iovfO6XJjJmpoIg7n+JDI2CzGRSeURksoTY+JCpuCWxKsxMIqeWlZj7fegBR7
-m3SifiwTE8NRsbxxbmrhZtrH0+DVWswvZRifJl7C6ujiFuWcwr8N4UJDJ4CwEIJ2CrfXTt1KZ+Vz
-QTZ9taRF0owwuXSdNsQ8RVjFvS81LXOY6bkkcIi/WRqhMJCCYCxnMobjuhaMLFFVjQ9UZvnXHERc
-tW3w31xreRXSJqsJ37L0IXyQucVWYXaR76OpEFWyRi7WEPGGMFOjCcG4JjD6MnMDMjvzGyxZ0gqw
-+5mcoyLRNhsiWMTTSGglAjU1EybneU0zHQlaIucD1CnGlA1DKJiOXS3XWajSp6nSaz1YzBwZ3v9l
-9CLnPn1qUIuSjqUG4KfCTvlhdDbpPw4VDb1gsE3jMvQHy9u2c+h7ayWl/QzSvh6OBEOY9LyOG+dK
-hD7FZJIgbCvs3Llgn9W/TMwMbxevea0ow/GDZ6jzQj8hH0AvO249VAYOQ4xrCdlY9s4fuYMPiq0O
-I7rfRvJFjqZ+W+D56MjxIWeFZdvqf7A1e/TR1OxeNRVN7WCUnfUdT4qUQckX8n2oqOORkcZWterd
-ZNLPI3eIr8ne66iEu5juXc7J8EgjB1IGXkH04Qn9qXkbVS4d45gIMWNTVPqAg9mxO8Yy0Tx7p1jQ
-XH3rMW2TrNmaS0hYGetfSNGCH1kskgKn92drbUfxSLFhDXxTqiYbaRWjqnxoW47SKwPHuVgrUgYZ
-kBviGTMpLk9MFhq0sL6PnmIoFS5PT1cNGalqrHdMyTsUPKXLYkRQ1LOPyUYjWgu05cqaPDC5DTD2
-+nSME87RhGYC4chh3HKw4nDYohjFGbZOsZ0O3HKcX/06HqA7BniUHDqUXbOkJdGGy9a6msvpCDw1
-gUqNsNhYZsnHRXe2EKcj3X9t589s4as2nen+xs5Ijq/h9jxeGI3JqVXksmP5n80zQvKwv2emLU61
-zgXTXeL7/5p5yFUYejc9Gqk4nouTlJv2tz7+Xz201z00G1b4Rz20y6/1f/3Hm+7Zrz/xDx3HQest
-8KHptoHviKSd/+meIR/H9GFCcRG6gwXEoUX2d/fM/IsDIU043bIIprG8hSD/DxzH/8ujR2NAfLL5
-74WpesDC+QM2DvHtFK14LhyMUZD/3QOEWU8EV7SMzZGXIZKaWjQXREW0m1d35B0/2YGR4tdVBF1E
-C+4lLoeDBl0ZNvhyBd5MwrWgQXTYB+tizJ6xuap1nPraJxktB9Ynrgdfjrvn6QtDiMPd24ZgZnDE
-9EevXnW1TxYfBA/g172x+vhXvXcVYeNWWbJVeUwHv8roPAzcOvsrBzjzAd51fkJtM39ikPv93tk6
-EEAbJwrOEPsQeFWTliBbl3J5TC3pBtJHnUYUjG3D+/AnolsNhqe3H/+yA//fcv8Y7oG10z2yEn7D
-evqY2aucCHG0gYWJnVsRc40sBiqb53zy8965FBQvTBJ8Ggv//8D1wvBaL5GGcSnqrRVr1LytCE1k
-ZJtnn6DD3rmTDn4MuEncRh7bwVthV07haUWOpjZukhPSvJ1jx07aM9J1/C9DXbq/KGJvOFSvXZTv
-vB9vrsc3/LotPbWINDGgEt9WGIgBciOstE3SO/En13nvFlIf4Ic3+Xl4G99eB1HYPMWlrQCDK9kH
-STIn07qNu/mZWFT1ycXeu4n7iDIdPwXu44OL4cp0OKrBWIomM113fW1eSAe2s215E0oTVFZ//Cou
-8wOXOcNinXSWm/zKH9pbHVrUGFGbkXUI8fwEe3/LESMC//nn37ODYVeQcECkjWv+dqlYG0l941JS
-z6EBh/Y2btrokxd+uUGvhhXLt/XmKsvTfP2DZreqG0SLnCnKLxJk0pGXTuoeZKF1tvQr79EjPf75
-PXz9w5Zn+uqShmbbqTZSNE+01NetmTkXTYKd2yek8/bjSy336LdfZ+DwAAAo8FEdfM5MSiVMLPRQ
-FV6Py7SskB96hfizTJJf95CXnY8ZzbV7aJUL7dBS0qfzUTY5HdWxdLZxXzpHH/+W9151RI9szMtu
-6/vs3K9vW+27iIqVQ3+lJsYm8Pws3WVOHv7Mq0be+qxX7Scf13tfMreO5dDn38ib+PaKiSYBfDqg
-HJn5O0dZ3z0x0v5mKs4zH/+09x4TASg6HGoHI9ShYQyzp4wGOvUrGYLdGfLGW6Pcaj/5oA6J4jwn
-9EJLAg5DQDYScUDclJoXd5ld0E4WtYCxDwHMpi29Yf4TUcqXYlU59lEYpik5Au1AeG3PFGTWLfnJ
-KvL778U3bDm6aeJnX16ftzeWI53e9z27jIG7xEEabsnmRIou/4zybyyL+tsPgCtR8OkmsTw2prK3
-VxqbyJPGSOOC0V6603FubZWqxG3Z1+eRo427mhyYDZx6A0luB3JtSjn9u0FrtP5JN2nqk1Lo9+Vm
-cSDyRfpgUXSCDt7+fcDQEDbcj2iAdI7xSLj8nBzddogwnumRCdGt7p3rpmvzz2Dn714ZWyLVK5Z7
-Coq3V576yp8jxaozSJyJXZTRoMYdRXJFRN/lqUwGtf7Tt5rf+uqKBx/sZAoOwAZ7E4oO0Ihlkgac
-RYs/fpe4Cg+YG+e4IC0PruLRTBNUlKimJ7pvGlPkoLcwY338W35ffLiKg+8UdAVyXvtgKShKM0wb
-l9ivFMTWNW1HtRFLCJneZQjh43refny9954Wr+xy5rD5TvYW01d7BImmM/G7bEtOMlhkyStPOzVD
-4CX4pJpzs5/8do31s/ksQO6z63pv3xKa46NSpaVWNGvr02QoyxMCw+fzhGbWKWAUeshpYnyy/L13
-c5dqE1onBby1oEdfr+xjBfcPFw43F1zSIzHbY7eBL4mutfDJdJdE9D18fHt/X9l9m88Q9LBFZY3l
-/+0VOxENhd1EqIvCplg7SgEeyoF/aQVejY8v9ftaRylNBQOWHxSpfRg+xcx6TgeHnsw0MEvS0xk7
-FD6gT4rp966yxA1yBPXQfliH60pkOs3osH4wyQkRYsVQmAjkrefpz5+V/fpCB0t3MTEosUyEx5pb
-0QxLmXvDBrhC2bcYaD4L/ltet7fL93KuJgKPtwNj7x7r8uoz4DvGXydn5rYY73bS0/IjJtz6rsxt
-b1O5DrOwAb3WKp9QW3zyyb/zKYCWBxhDfc2BXBx8CoDU0Ja07P6z1vo3mbLNLwZ9tqAybcXA1pkT
-MkfDz4J+3nkzIeRwUKbCJvjDNN++mZxJnFYY9OBsA29eJXzC440EWbaOfvLjN/O9H7g/KyO6IVvo
-EBHtVc3UWFFFQSXL/tTpVHeC0djexZZvHreh2zK7VzAnP77qO4+UFgd9BwoRwr4PEwkQyJlz23JV
-0dFqxWAHl2+Iy2Znl6K7GJfI8sLDGqXwbn5y6d8+kmXTpY4zmdcuCqWDJ0q2eFEpxYoSIShcmXoh
-tvRi+vOPf+BvT5Cr2AueYglqAqFzsLbUIRORYeadneMW8kqzgCo44mbHTIWLT7JF3vtFrC6Un+Cc
-ueDBtVJ01bFdtdjjYA0i/+60+bnXTDro/4/fRDALj4zOACfAt29lPCeVNzDJ4K1Mp3VTTdYpXnjk
-oGPXfLLzvXf7XN5/BNH7jfbgUu0iNmLWx6UUomjaHtq6mqcnJkzT8cc/6r2bRy3EJ2AsrJfDPVbl
-HjISE9V8ben4PTVqXTlItfnjqyzbDJ8XN09f4BJvNrcmcqWvFl1DZjN90Z1mITVgD/j4Ku/cNQrq
-pZ/HNYhxOFg2JgO1ftIgth3snuKShWqDwz65ClU0P/0/LrUsF769kJPs5a/yak12TSC9WpRWRKN3
-4bZN2yZI0ZQFtEQ+wWu/84AgdvzvlQ7qAtg7KmQOCebU6e8x3YgNpuDqk/dt+Ze82WKYLNCe5DKI
-JgnJPrhzBiaPvCQCA/1dCTk7GRW4haE88XF8QZ4bxvHo4/tnLP/G366IepOwM2SXkK/e3sBZZUlG
-oBKoisjnBiJPW49FAWjX7zGdSDuUOEz6aINg2T8qdGX+1CZt19hFtZVi+ENSOm1Mfj+4FFrh9GdB
-q7z920QFbD8v5M1BJo16u9KSDS2Cl49/83tPEs2qCXyV06d9eJOdRQbQVIB4R/DhzPuHBElyA8X4
-D2Pk9r+G4AraRgQ9LDSYt78mtFJCZCdeziLBd0bsmrPSB21LQO8xJMnpk6/uvZ/lEX7geyCSSLI4
-WKu6sSHfsC/xj7Z2eJr2kzqpWEXXf37zPBoeCG/Yt5zDxrabIc+bIlbEpMnrs7KTOexeEf9pBUlW
-G/MNMg05dtDMObhzGBi0FGLMUqe68iLDHovJi5nfH/8WrkKvkl2Lw9RhS8Wbe63Vlnc/jQXSkWnE
-sx0W3idr7u+djuXHgEGzkSATn7JvC7xaoxCDIiPJXaLnujA+0yZPbA2VweO0/ZWj9xfeYF9DSAs3
-SrrhKf3uneNX1Sf7y2/1FX8JAhPJIbCXiOPDQgCAWMc8F3fx7PSmsWlH2RSXaJT1/szuBiwF4+Bn
-8QmyewSsH9/mdxY1inSPUQvRH5RZB5uORqyZ3uU+2Ng8ESmAMmdaD1V8Jiy4tQiT+M+PL/jOl8Dm
-w+qxJBdx0w+/BNMdc8R6rGmLlHloBHLgfP7sS/h9lzN4pHTIeIMWBfxBuUPPORprl8fqyDjCt+qW
-J1MxuyeMbD8LA/z9DnIpj9gLXN3ID6yDXY61Ege1zR0sUxtt1VQuIQf6LI07H9n4DznkQ/jJd778
-7d/uC0tYPMdf+ICMKA/5ZjJV9hgpQSxxkWtry1f2veqG+Zvq3GxtGIX5jTbICDZFlMd5bTbPHz/C
-319XQnIoDIj8AaHFBPLt0pkXSo96ROornVjfdYbrMKvdZ7ugQaX8Il911mdV5e8vzXJFDq1M0+iy
-Hp77myFOYtPADAYrcBFWdN0xn8pnqYLvvDS2zjx3KcL2ZK63v6uewdagdClRcIYKQkY6tYEfGvKW
-PC+RfPIdePvzy+unSHPNY7TMmJiCh4Cjg9to9ESlN2IivzC3Mu24Y7l+wWWjLVqhpLkZUbQaq9E3
-J38zjd5UnZkTYqkjynvIUEzKSuIWkOOh+eb7yVdSS8wzZn9aj+LARd1QFE3Zn0CfytIjINVhvRs8
-LHZbTzRTeTwUTQW+O0lDseOlnqJdOAxNdjKn0ijXbmtE8hhrn7SPl2FSd9QovysupZU1GAvSMHW3
-RgrIJ/DAx3vrUYXGU8XmkwZ1Rspz0AykMqAR7NEBpk4h2musb1hRXa/B3tEgQsvWXhlFBm47MEbh
-qTeEpTj28nScFhdcogXsAOmPHFJ8FJiDS62j42+cdxbafzAUqkc+q3iaGN9Y2vq126QtfKxmUU8l
-JiDqyBtRMjpN1EP+DjOOBxN97Rj8RFnXGPv6pD5eQPLjESrrKCJ0CaliUJvoK1dD11ED6Lqr439z
-IIfwV4CVdCRjuBRrfxDgfsvISV8AoiM0mnMYhl1FJbe2ZG7oqwYdB77bcB7yI8ZjJo8Q5Qjok6GM
-gZvrvtUHmqSRse1pDAKE6v042nXu6NrUsMMSJgEjFvpLl+Y9XKdZA88Z1ZEH6KjKjYDQBcfZLAJm
-4hgcQXqTybdfbrq+jIkxyfMaB/lq9gRi97ngdq5mQxJNZ+XR0j2zJ6AAkQZDMUAPEzVEs4yxS6wJ
-Wh0C1+oiwdDbIPT1kPT1xypz1C3+QShaoohJgDBKYxjAA0Vtv+YAHZ90w6hNZ4WitbRuwNihHS0m
-FL6+V8QPsdL783ywWvzXSTZP25jQHRrYGWLP1s8Bs5dl3OXrxBRhs2BLrF2ClP6nq6b6bkqz/qec
-kaNj6p1JK0fl6eLkTX2IYtBN1KZFGfkd5yo+Stqy2bNjT5zcy8L0L+bUKC9SUlDE0VQLkLHSavMs
-QOqH9ihj2+cgZ3vFbjYJw4Sj7MqnjlohAjM/uN8mL8keBwyHSLND+xJ+aTutpMMzXCF0HzkC4BFA
-cW8MlxYd1nLtGWFdr7APJPdp6bvTOrMr/xngQT8HBbwgUilbx/kCjxvLYem0yRUJTBM2zAlACgoh
-2062le81xaace8wYduigN+vzNl4yS1z5dQTa9dOeex32BVCXs7DviHeu5Zjgr0hceC+DgJm+tQ0F
-y4CXA+9L6wBQQS5dHGGlKeRNb0CYXblJY8a4AwlTWTGrFT9jP6dlhVAfaa9Wqg7Oh7sg2fBoNNeZ
-N+l8zYZmXjl2pB5igUxx1RFjjPLeMPJqoyKMAGucvtAU9ESLzDVfSgZQA1XdmdCi4rJoPafaxLqG
-rF9LNOMcdLv+Ahkd85Oa67p+dCA2jl+pxO0cym/SRlvSn+Jhp+W5qs40O/WRMadxps6MpLTDS2UR
-mXwW6W31OFvGJO+jwlfwt1qQ0jemKvJ+yxPy3CuFXNU8tsIqJYRULwZn18Za3WOZyWEJZLoTzqdF
-b5rjWuFA63Z16dvDGsgobHIsHfw+7CBOZJyw6Yz1Ua3PkbNNlSvDI6XlIUrIcCAEActouNYFvKSt
-m0HMCxoEkkyK0Lv53zpEvzjp2R+16Dg0oDRcEYVsWjstoVrf+qGFe2Ycu2I+8WFOVZfSZeLzuLwI
-4iW2enxCPJfaTKKVXg36eJVSIBYPeC3S5KaYUDnu2AEs+vzWGGbpfRjhxQAY4uOgInYnYXODoGHX
-0Wgcj+VQhUCSBi+pf4adF2XXs21l4pRkF+CDq0GPWTmVnSbp5eR5JAWXXp8OXxBlinA7EPYRITV0
-EMlHveBHlaaVQUqxono0z5uwrgrMtznadBg7lXNFaAB6OX4tCzHFiumvlFlWPqpVWVDbJm35YKWw
-YbaTIH7oPu2iSIHS2EvI6e3RbJRR2p1DSu7Mm5HTh4neH/i0d1anei+2GVUgMSyWn9dfZq9h8Nun
-uTZuKi8OSSLgzqmg48h0Gwl3/KK7Q3UjQnBnNE1J1l2VeeN8d4yGymUIbdqoCz8WnxxCgqdZzHAt
-IyAFV37r1tOKQh67B1+gWZwRG9kba434sDzIbUO7TGjtaygJO5ABU2ziLVtS6x+kxoxw0y5Hvw1B
-W9FFpqnkQtJi1KEVlMlj7mYhCaUY215G/vQcGAhE6dA7RFUEoxVGKWcRhfjKWsS3NFqy+nxuXBzh
-/cR5ORBuxQyYvbojd0Ib/S9TghnwpNAM77rMzEjfQdDrCD3Q/emL3RMzvCRdsUi7Vdp7O8xhsACn
-Jil+WEUaggwsCvUjmSLrCxlYBjpL/GDOuuxn21zZQ5nfy8J0KhITVPmY1UmntvBLy5tSs2OxIkCx
-ZCrkR9ml4U4jnIsO9CY6pLkhsDs2wjlwEzMvA7ft0heEJ3IKkszrB0q6snWCuIEe92xnVYMkeorU
-hR8WOBdMLe5GLDeui8yVgvCOwy7qWEgk5g0wCehCqdxTXPwozUDZmBDDRAr+iSCEsSETU0XPaLNJ
-p2dRmU+deaqeLA4+pIvl5GYFYsrqp9kztHvc/S764FkA2gjtuf3RG63A7KHGH0OVyu+0QDAWCgih
-eEVjKxhkpP0U7dBd0tTIvrU9yzhIGBsqRjVrw/dJ9P53X0NMfcQji59guc3f6qFMd1AgDbRTltf8
-8Oex/M7wRxIJM5nE2VP2gIpO7BiWILArhcV/9IcjnTCV+ziapLHkLuAXGptS0zZpXHrQGsWQ8ZK0
-6Es30vOQzJuhcLWjIumS23gobQuFf2l/a1q7i7ZFIiJcCJ0PulgTA1WL1yksTiaVr7tmvgWmOwyd
-4djyY1MGEsAfXDw9SmERzWQpoMpNYJKxX2X+CgvXlG8YCGb986BPGY6gmGww0KyTMxiXkiEGDzGc
-PAJ1kiapvoA4l4DUp7TsgzYMAQ5lJMC7a8xpSGQdH+POykpcqh+n6Myv6P3z00iUhEq5bgN+aTZx
-0R3hiRNyZc5x8qzwcQ5rQf8cPC3joK1tY/vfZHme4rmNPAK/rIz/KYCpEycSO/2zSIzovsYMEB5b
-ERgVPpBwOM26cXgA/uiXgW9k1Zc0czwJSihBHMBq6rRbUTY6Zzw8+P6qnBvMKLInNw9tsQGOTjJ3
-sjdzl1fXdtLpq2R2pHeVpxGez8HRknaVjy6GTTIZnMtO48ac2G5U0b2OhB8FlpG4T2OESw8Mi2ZX
-F/jOzOOS6Cn7pBTZGPLHNYvEDbcz0Pxz4iLWC2wXRh2Ck7It2572BWdW2K1dOTQ7A2qmhR3IWehG
-5M+uhDmW0I7gWTzJSLnGWqQwdOG95QjdO599d+24MUVQWBTuKYlRLg4IGoswQ3U5ZkGCqPFra5E9
-se392pxXspEzEyC/SF8mWwGTolCMrsSou18tzSA1CYFpOKxBuzePcxtZeFAKW2+3iYxjwSkgbS+g
-40WPgyl9Co450m/ylPWYLWNiqSLlo7cDNRclL5tdq3CFn8O+l6N01Rqer31We0V6VYQICANJztH1
-7EZUv5WmxtOxD/kL9VmUpKgnWvnQz5UP/6S0gFyiIfJR0MoxvpyUaT6P8Yg8YByxWbW6iFi+8WPG
-QRH2kCqG2bDualOfnomSRvmdur3AJuNr+H4A1ZH8EXbLmjoKohwDs/f1s9FzlIy/g3Wr0BpQnMpV
-MXngXi2rYXecuxDMEMbB6EeBuRG/hvRMaEM8IH9rOQVAvbTPhmzNncyvORyr7ynuCFr3JZyX7VQ5
-TXPsuxlgFMcrEnBVXSKoWOo6m7ZwehlTOM1kXs96H3F8mMbO27qgW0/4We3PzBTqwZiN/MtUJliT
-5tYtX/RCn795jYuHGNmeRQqjdB2YPkkVbUoa0HyNJuoGtvHRijZNXPtXBvatW7OdWRyoNGJrjXTS
-vq2JUboP28QgHweIxpU+NWD2RFjmx35b59k5UNiwDrqq1y6qlFMsZCsjPpky34uO08nh3JlMFcUk
-RhjdCeAGGrtQoFhc5bO1vBpe61wOcnTvIH4INzDJZHnp9WS46crWf4ApLyXjmqY/XUJ6iOwqLPfG
-jKvxp5MumTppGzpXPbX7+TSMC+TP5HPtTG2Ugc5Z6A43BQq1lGHA1bjP+YoBqr7MspmvexAlDQjf
-cHpAb9uKwDfT/iYjoeLZzP1hXHt63J94c1h7O3bAySN2KzUhinBoLI8arWTbmquEpWhuUxhrXhFi
-yDdxN90mc5qoY9jL9KXbChkqTlU/wUUbx70Hs7ILH8NpVNeRRb4geuweV/6EOHdipzHDMPCcupih
-F5hgTJdefh14fCoR72cybrNa+s+mX8RYR+Uk2uNRxv4ZUrBKfsvwRjtbWJtLk8DLimuEyiiN0ibG
-DkS3DiBuDa122HiK/vMGiY1vdwz0mXz4U+Ax6e/nLgBqQMwD4p2UcvxEhW74g3I4Gc61uevq4xGf
-VX0kNMdWN9TTvs6gs02cLUpRy8RzriNnB0QoSXcgCOuhG7qU7oCPjgaTrqT1CTYQC6uxt7NyHMfa
-ai0uVwzcGF552TC/ZnsjrM8rkayzvUFWTxez7Lw3zqZ7Ey1tfwy1xd5c2zhl4ZxiW2IrRRlrd2fm
-3pLblSGoPndx6up7065NlNtDt7fypjn5rszCcfhSaae30xBh+433FuDCrakPiTbO7529SVglzbSk
-zC3mYZJlKJOnvanYQv34POytxu7edtwtDmRypuaMiMvFmGzsTcr+3rCc7M3Lam9k7hK3VwFMhPAH
-hGWsztkv23NShCfz3gzt743Rxi+TtAFKLOAILnA2Lz7qxuwwepUx0wI2GPZzvNZ/W69lY8zCUwE4
-qr1PWyPzMW3ugH9h6N73EP9lQXljQUFs9qq1uv7afv37H198zV/+/d+woHz9r//89vWtC2X/h/52
-oQjrL4ZUTEEIs6BVuJhG/mG4CO8vMrvhqNG7pw9FWsz/uFA0vCtwMV2mlMhREaUsY/im7Fr57/+m
-eX8JHanKoqdn4oASzv8TH4rYp6+/amMi8bAIUABSjzjER6G/9G5fTVDSkHeuyFSGBETW95WRJc+1
-0UW3VjdgfvfTVmtPsD+H92WlOz+iLJpuczOhwhZV2J5G1Vj+dKsi2s1VK5utnrjGxP5osPnpkJTJ
-Iw1DCKpThf56laJyyYJ+ND26JV166WljZ61l6Y90NKo6/jYWJS3IocPcjFO7LuWmDY0cROcUqieE
-atFTw1mOo6ebmSxfdPzwSIuwwyNGEuGwDkWa4ao1cVMW3f4QjL8xY//TaN55ZbPA/xNJF7If3eIO
-bFwHOtPxgA0OAETvyD5MIHGkuq2vRN/p12KeMAdnsFaWEOFZXkwLvGXtjrH5rPOpq2NGv9Qq0tKy
-yymLh3rbhGHhbGZzNI8V4ceYEVFqIT0o6q5gHNWqGz00PAawOMO/+17uP1Akqht4+AKHcz5jf59a
-A1Kx5dXWDXMYaz5SuZ7SlBygx65yQkbJ0UtT58QxuvnS1MvhKTdVhbG7UM45iLb4K6d0lEVCDyfo
-0eil5a5qSuuOtMcpXisX7AeUvrYZYMOlRAEKN081xkUe1D2OLTQPEr/KL/S2cOmWRiElTDHrG/xE
-E1bpzLGeYruTGreb4GJYq342B0ibSdByDLxFQTirkWNoFHM80qzCuC0tlCUrlwMLxNAW2nkHcE1f
-ZfMIcicaos67r+gmw6qLzPInBEglj5NaM0DcF7rzyPSt7U7MaMif0qztBAK02D/BsDhGQT9P4YND
-aBYZb5qRkpfJmJtKHwe3e+RqHIvXXmQmvHZZCPojLGxq/JIa0OCoOoYPsGuIHCI2MxIBp1btzm2b
-+IomiAVboo41giWbETBP3dgc1Zs2b1wAGEtZPKWaddT5YXVaTGOsbWo9jblJczNqFNlueo0GWNEM
-iCZHO51Kj2ZjBU7TXrUiiesTZYiSuWQNvQichzWculYhQ9rQo/sNG+MsjywxE7/oVH0F3jrKFHzV
-bCGJwpjIH4ysHB7GyBaXqNdlvsILjhWzb5r2nFNn+Oh6xfSzIriWNLw6z92ND07JDtCYUY8lJmEj
-7EFtc8dDAg45VgOQm1lNsFgZUGTVdon1ftYyrM0AA4b0LpuxQK1mN81uKIR6tbYJaXyhB22a275u
-+suwDVv+fwS+1o+7xt46lAQAFzTDvIRvJ9tthdz/UuTx+IjRH8pj5+tMoXw06uKEEmRoUWkiPd3I
-NiKxz+7ABvH6uFG7Vtkw7bQmpaAY4H2Q80vbwmRmUgBr8mLXuByA7H5vCjl+FznJkevIabXvKofr
-kOM610e6XUh6YxAYGgXotdnUw5VBJxClggnR/yjNaFIGdIFAvuu+P4ug9jntr+fatMuNmQ0SF3Hh
-T+26Jn/vavR792dD8glgEVm434o+VSWG2bSK1x2H0XiViRzMDmY1D1iC3UYxPyjPxart9fZ0GvKa
-hMYiFORwDHZdbUyHotqnslbrgmfxjOs8nYI8KcqdSjgZrWP67aTcJ+QCro2eqQ+dIjoqIy2fyxov
-KwGJwLvvImv0WV2ZBXH6IFqBBjd92fSYHsC5HsbZEyEPxgVwAzzwLDkc57OSRwjcHlngCildfVmk
-Glhbn8M6RLuSL6IYJhrC2agS6NZSJdlpY5rGlaNZ4qcF54MugTZPESEMuXMFMhNUY6mP7YDSXaQv
-Jk2CH5oTMS4uM9HyQhsmcA8bYOG9O0Wxu+XoXpFg4/cjE+w+EdYRuynZd5ZgSrqG52KRfKOPcLj7
-vGrBOQLf2GmuCk9F1iBIgveJzYHeRUKmDsRGXI6yJ+djBPb0OFrqNCSY1D7vItfXYYRoCUlfQqUx
-VuzSggyFXG9aIRKYboGNuerEiozuopbMnHhFDfHQq5y+k0DiU+yk7mLJp81mb7MoJQ9LKKM+ifSO
-vpsvwvFYUxHFHydh80VxErhYwNQ8BA3Q5rFU1XBs6zQEj1JiePiSY8eAAZ9BHrEb3X2pobxPTLKG
-8I4sZUcGcUfsyZZbD0a6Lbqo2dqZJPE2r71621d6Yq8wgNOTq+nHXEwSU/+mzxJGRT6P9WqYW7oY
-4zjm9BvUcNuyhN6bs1B8O4nRPtWgsHck6MBKdkZP0kyf+vLO7ytkk7UR5sg3UljeHGYc4zyCoyQ3
-jd7FX11rDu8qZnJoHkj2/C6QddMcT6R1E6YW9y1u+v4rwRTaD+UOyIH+VX3W8ff2TSGJuo9a7P+G
-CF7HS5bW1+LHy5KldVHW7cs7f/6fQlT8RUIViZLo4C04+Itu42+YIIWojZTcx2j1659grPgHJsif
-QreG1hBFKHbYva3mn0LU+YtykZGOj8WNChLzzZ8UogeaCA6cAm8oB69FSAvN+0CdBhmTrNvGee4W
-bHepXeHWzMFMlwYta5fA3go0PUDZXy/S/2kVPZBC/Loq91mnSge6tmSMvS5+tc5mADQ6z2O386V3
-lvcbs+QQ6iTEAj6+ejiXvyrq165U01l+wttKW8cOZANKJAGJ7MHlL/Oq0jZ73U4RE7DslOUEBmNf
-LhABlmibfqki1JDbR7qB7HJDakrrBs2+5JD78gOgrvS/+PuyhCie+KpNTe1u2Jct876EYf4dPlT7
-wkbbFzk0uLIhaMY2zQJnXwiNNXvlkbkvkFxiWduNvS+cuqWGamnyRUG6VFbJvsgylnqrzMu+OwEi
-4TyK0qSPXO6LM0qq8me5L9mGuh68+1EqoQIO35R1Fqk9V86+2Cv2hV+41IBAICgH4StQGpKFRZlo
-7UvGfl8+YqYtGCwZHRqceqkwl64KSF5l6xvID/naA07iLNBZUqPNpUQ1vX5aAN+RwAALJpFVPwcN
-vrEYGUJOjuCenkJ8cY2VLsjJhdJiTfZuIIP4VE9GMrZB8NAB9KGiX8SQqNieEnGB9pkqhzPHtVVF
-j02kSQXJNyFjgQhe0ayFQ/vgv9k7s+TIkXNLb+VuAGWY4TDrp0AgRpLBmUm+wJgkE/PoABzAnnoV
-vbH+QFWZqqolu633qyellBkMRgCOfzjnO8wmNQiCc5crsZFdFzE1jnr6AA1BFPR+UqRdAg8MZwoN
-I4q7bSnmed41+tTJvWFTJlIYjFRjtWEM/f0iSm2P7L/WLnZSeJ9TSnwBgtC5H3YDzhhwgpCM4rO1
-9mRHq/XIsLEXUf+oB5F9tWgTJzYdWeOGJsZgbG0VixEor5WXrEoGInp8eqltMWg+Tnkn7Uh7TBO1
-M62uyi89genst3n+MAGKKub2VDQ86Y12yeo9y5aG6MnWqbKTxiyZOKnFTvuWXWeSVnftqDJGHcaY
-fODhwY+c9XoT7SCkUqolbpnxEQKKPNTE1DD+5RIDC23zimbq5gxe57587+N+9Y71mXdDoFj2SP6u
-8veppcwT/J2Fz3wUOrRHI81+setBHCDMuSKEZYgzUq1Zhw/h4EXW0W5FZmwwAslkD2Opf0zg6zo7
-rx2HM7Vk76+fGitvBkXaVe+aWrYdAS4WINCXnnAdyES3raGadwpm0oZ4AON1Xsj3eB+tub+fWGw+
-19OcfEAAGq767zJP40JbAfa4C4N4rQQHZw2WMF0iB1glrAWj8V08zt+FJLPokr/+XWAa86KmDWkO
-FJ5E1JrOfpK48jfGWpsyW+zvi++ClZaH5s6c8ucWrBftIpUt2jit34pWTR/jd+XLuvW2yD3K4aZi
-e7ZhlkqZ7MGwAVy2Vs8ZidXrexnpEuLvArtLZt8hw4gApI2TYNcC+47IFTS3TXGOSnj6AVnQux1Y
-Ufe7Za3j8WoYGQX3Wt5H36W+6Q7917DW/4syDXOHqcv/8mB/wsx37PyBBRyInLHO8ydacZoJxVbk
-lWDCvNlZOG3d0Ifu32PbXNuQAmriU/rdnNTfjcpUcL+y3IOkHpKVRzMzOtb8iwSniF1E2l87322P
-tywx69+1G9LXvqhaO6Tlu1mKp4jGqQWIRxNlIhDdIpgEfwgywvvpfrdccu2+IOqXwHFqr4lC+d2g
-MaWnWZsVcEQ6DWFrZ7adNHTp2tv9T0Hz94IGloCPPPXfFzS36fvwf/73n2uY3//JH0gX/TfL0wnu
-NVnsoK1YM6t/r2Hs74mZAe8Kf4xuwJH6Zw1j/uYhs2SsTaAuPlzjT7M0QydjVOALXL3sq6fiP2K6
-INL++xPeQIvMNM/wkDtivv7bE16CzvbdykbeUHA9Hxc7EjeLLJN625iQNWOsinmQT479VPopUUlA
-fDn5nNyrES3OkfvUW7aEusauFpuFaLVipzGfuZBnAUhMX5MnI/S3xaaM4FwFBYoEe8c8xvzSKnSe
-h3QyrDmwelhgpK478s4QEXFuY0XWJPM69Hew0CIddCrxFr8qPRdfAzOkRxIu4Ja3kExRfwonuW/g
-dLEPFTyBGHzYS31gOav0jZmJvj0MM0VOOJuCrR25oz8NJ0s9mIi1fVOaPQdEHqX8c093NMmGn6g8
-TVv8z97z1rwFUaMaWSQoU2LB+uWRoOYORVwRm+IwED3F6E7ERLenlT1vnL5yi1MyejjIlnosnBCE
-vzufTbMAugjTDo2HnuTLBs1/3G57J3G/tEUlb6Mr+iicDMEaX3Fw54HB1IvuPV26l1k0QxRaWgdH
-faGntIOE1Ikny4uqW2uuh+KgHBfUFSFyFBpSmdP9Cmg3ttXggW7Tp0yYASOx/CtjlvPggJaHU6BJ
-OuhI17z1JCJILCB3JHnp1IgdSIqMaQD0VSCgFdcpLKpVUbBpptG5sBkc6aFV1H8WZUaUDUvxHPHg
-Uk+PSWqDTBsMAM3QH2MTWDs1m9iQAmZdMjfOSStqIgIeTTe35Kab2jWd1CbHoifWKdqmFdkwu8Zc
-uh/SaseGkM1WTw6DQ/zc3tZsMhU5Jo2K/a/l3LvoVGF0ti4PdUda5U3H4yq+WZmZci8iMfB8b7z4
-EMesxE27KT50xJSfCl4mShcjid78UQO6qFXp8J5pwgVPK+tiCDQjSh+ceorZNmUc4eyiW/POqCVs
-gJWwOblFVbFAneGAE+wx7plaNHuXGdldMy75pcWz/zTXS/LkNiVDMdRe+QeBslWyaTobg30hf0wq
-o3YbhsYzyJgzjad5Xo1LUZ6qB+UbdbpheVxcmf3sclmiP7pI5aCOk/Q35oHrgCe2UB0yc8/E+rdJ
-TL6izZD6MRs3nXXtRi+dbgoT/GRr7I1ZE8b2HViOmxj1UYWA7FIJqx2uq9KZTfilMmGFN5sKORLJ
-odoZLMF0GIGee9eCHBN4i/mpH1yDa2oU2oM3JAlSQYjcFHTEUL67ZKldUqvLhxA5ZnlXGxW2SQhy
-1sW2+0kRUEJSBrIc4rkOyEeQwGlgUXnSFQ0QYh3OKfnAEC3VroDEOsPbrNQ2Jo5e7vMJacVGs6bE
-COxevKo5F1sofepV7/JuuUbkpo/BsHQ5sX6GXR9abhTOh9JpLm2t6fq2z+B3o8O09efVZE2XQbMw
-niFFw7NkI2e9u5phUy8IXx39yoXZmsraehTKwA9E1Fp8O08GuFxvKPhKdAPQeGC7LaMfJuzWlWMO
-iAunifn8xm399sUk/6ym2szJk6zmqDACClOataxpGAA5ump/icUl6IzwFqjcyRTbduh4MnpxRMKz
-vGg9zjkyiVgAD50nh5DR04JKu8U4eJcL5ebHxmcqdEBR7VyzwGiXEFA7f712xfCs5bMmw5ngomub
-0Y0T1l1VXttpUWQhOZvlU9+kC1RImevT3tVUdoyh6TH/G9k2aFo/mqFlFsuPrBitt6IrynkbpVHx
-kTBkUaHXjzQbXZPMV0k3xNbOlq3xWhsuaBzTz+WzbQ8ety7zfD1ITFRjmwxy9+tcxNFZEqTxqMda
-9pCtTluUyugeN04doWOstKE8o9RNQPrh66D9qrzpLobeqgdDpg3XFNhN8wNGY3JdkyWcrMlpbbYn
-sbYlQC1L/Tc344EQLn6H4AKxF2I0O7Hkoc+a1kM2qqYHZ+SmoX1ERUgx58FtNo1Zv2d+gFYX8Yvs
-HgakwXuISopRWeVya/jITucQJ2j7CY52XUcLtUUcmtS3MaT1nAhK3+q3Jn0z8MzZUiyYyyG9zuw8
-Yh8wLMgTeOf9j36kIuS+8My3ue9A9yGGMx51ERW3njtn41aPaPM2xtJ5F92YThqhqPwiy8w8eJ3F
-xltnLJms516CbI25rvFjcEvxooxyxRGzH4NhXnnEUEHRTm/jAURNyJJrOMEGJDaqhvmN4ja2WxtZ
-yMyk3yWwV4TIzBCujEsUq82IUcnZlFXtvHL9+8UpU5G8Q2ozkw5gIADCPBzRhY7TLA9J1k9V4LRm
-1e2NVkIqHW1pcS9Lj8Fxnxgq35N2Um8Rm5dk70wTNxCGEefLLxxJZJg7kR6tVx7k6wKpw7s2DOMr
-5mHGwlmG0A9pY10UO8Kz6mIvsMNey3hAT93anv1i1aWOfMt1+KZmxM0NxQiMTVJ8sCpy46KKIxWV
-PYJHxW1sGtTW5FJxvRsHr1NkHcZROS4hOShWHwjaL+QBPnVGDRbFXEMPNMGuQWue+RpddLy5b7xk
-bBrEtutyAlGnXHe/bKTNMwjQRy/O6jeO/pZHg50OHx2SKdDiopCPokN4HrSm1bBGWnylB968MA/I
-B7M9l4uRWRtzdOx4V/iIXYLUj/xHUjCdaWOw9QH8vy5hgziWyw1xKzUBYYPWvvEMR1NPUpC4S+ta
-tQCS10JoiEk/2OLBSnmGI2x9WZTNWUNvMg+hV41Oz+a949k2J9OsbWp0Dqj7a9KeQCUV2ms963Yc
-1KtzgyVEJdttrWICgHzZqHlLrBH419EpM7klEzmPN45sVsh2l4AcVi6fZcBiMrsl3rHbxS4n/Ba+
-TDftuF8ISeadZ6BfnZFDZmzoXLAyRMaHjJD584jNiU1mVk9dYHl9/5IkmvwxJlF9W1Qu8NrJGfRH
-aXTGFLjMpJst/CVM+mYxk4CX5LjphqHvz3hTcUo4TqwfNTH0d6WhueN2yqROzioMEVSGSIa3ndGS
-yTzZkiMSKqG6a3LdYqIg9E6c3a4hRUCSntTsKM+op4SZ1z+dBUziZka8sqaRuVDeE7NeegbbxnhX
-tUrBBKWujbdetLgndDHIR0i8WYHBuhoiQDe9sSPn0/YDw1TJTPjCYl4vWB3IUE7HxgmWOG0nwPiV
-e4M0pbqC+6Awc0xNdsr5ieRv+7BwN6VpFG+LxmFLZTWzaGCtmGwdRWgvASacSBsGJvpPMp2NMhjm
-Ln5IRug+m7bvmnsJrT8OWQwWCPUyI6d3tUk0ZpaTGTuEapBI/FHE3lkQaXClFwVQbNnW5l7HuIDz
-I/cyVMGmM+cAssWSbhYyGPFauEv+YXGkvJfwlOy9ZeiDhiyoUWINbq64TKIy/6zKzMHXiQTfw08z
-tNe9QbV06Bb0xJtuTJxfUUQlisSsarwQLgXneLJMhBuOTWPvpwGmSJDAROyY0MmeJMFBpzjOEkAY
-edyiw9YY3h7R3qsuXPSJIyoxW/E1pv2g7ywHOG7QT6b+qns5MFzSggVyd9Enb4lgyrNzKHeLnaFF
-ZR8QpN6Y+3RsY2Ru6cCcxJOLjQ6gK+XPRBbGL0kUBLl/U0Q4ObdpHDEqYJDHsjTqbWJDcCQQLzG2
-8I2U33yhkksVBhe34f5nZQNnTQwDW/CmGn56uaARGjQ9l0HtGOVPh6UjEm2sRk91lREWOnnKszeI
-pLj+Eru0eCcs8tqTwaXXBaBpCpjpZUt6MzWfT1yDJm7cQlGgcIhMXAk4NLm5YLDxshw53d6Me8/d
-1DWTg22GV4cnYtq61t1A5BRf5thrOycaqr0tTZ1E07TPdv/5VOHSfFUPfff11V+/N/9r1fd81A17
-6zjpv/Gl//zTZfzqSJv5+i/+ovwvBouf731aV3//N395CZCnv0uGVnHMX/4A9x8/zd3Azur+Sw7F
-P35c/FWvf/P/9//8XW7zODfIbd4/6fm2oP/+n8kC4ieWFv9+svDw1cVp85f1yEog4t/8sR5xf7NA
-OFKsQ2EyHHPFdf1zPWLafKMsKAyorQBi/jla8H9z1lE+qwvG+fgaPeQ9f6xHDOM3lCNMA1DpgFBg
-yvCfrEdWFc5fdgdAMhzbMBhX8FoYYP66OxizxhftNDKLzktsWV3+ii7u9U+fyb/YUPx3P4OP58/7
-Cbv3l8yBDrOJUlgZ8SyTEAF19N8YJ5EV/YvfBcu+x6/h2abtrFOUP+1BAGNEK3WeFTPHLtkmiV8z
-MXEr7bOqRfk2dA3+qBRG4iuLBHeVLSvZ7YuJxm2LrdGoSBEpB+1AtmFZX2ezmQBNIArihym6OSM8
-p8h/UXUaM0jsjPpycg39XlWjJVhntoVXvcKdF/ExRiWzoDhp6/ZKsf8vg8p3EAOSD6+1xl5j8woo
-T7R6FZAAnL94bczZmRkda5qZxtE/qISM3g3vBTEJXvd2CKKI+JCN4XhERHYJOP2DYZV9t4HTlw2h
-bbU14w1jsT8atLc0U17V0PnDiX/EjUIgqMUTWAcw69XmeeSzIxmaJvhTjzMCKHSKq7AjKO4u0xfC
-7Hu9pe4pPWPoAtwe2gtyB1bBeErAjyJGrpYTTVfPkmQskUsnOejQzaBJJA5DjeNo6/tqmY9jmqkf
-tY+CImghtT6QmpwdTWfqC3J7Fv8aTqzbBspInJFqRJTHscnJNywtaT0bdF6I+R1B6nE1StImZ+jq
-767E3Uis7EsiahTvjZ+mpE/X75hv+kcDTVVM56ZPD1JqS7HH5ZWwryCjV23EDE4wREgHC74cuRs2
-0tOSG4cfXgQKZvyTPfdMogS17Z6BlQMGeJ7VTTK0sbqyhCwdnJnpkOyUPuTPKUZOqhJmFs/9nAKl
-N2Zaqw1nuPUy4TLIOffT/MHEIfgckYuNmn4Gtb+lzq2vxphohByJ8HKy+kh7aUq/4HqdpE1KpK37
-uBZJHtjIsi8ysIrFcmerJSdBVNkdXbpTOglbPpjmW0JDwNJLz/IfZKkN7/GAgywwGNdBvB9G+9fi
-+hG1YWNgCoJyV2l0qUnM8y2WQC3kQO3R92WfXAEkShky1XSVBgXznXKExDBlpO7N7JHUjY5hie1z
-hN5+bTwYBQbToA0fwJgRYPzP8+VfPl8ISuRk//fPl8f6453HXSX/Mrz+x7/6Y3jt/EZpxFLYM7Dc
-89849X5/wjg6E2omhNCJWEGzbOdg/mMB7/yGoJDHDxQC5J6rYf9PTxjrN2Ak+vofD4AzuJX/5Alj
-Asn868EMUk43VmoLiX68nPN3FEI8WTjZGkaltTNXp9oSJKXkzH13uJj6nRnHy3GyyYfhxhS5RoiO
-Fj+BU3MuamSLGcnODj2Ozn2T08OgCa3wWydfIi4XXHumOJVejx7J1Vr3rDfOyljkcApLjOk7PVXj
-Dx0kzqXuypYZgMXJ7ozaR+ob6h1z465unNvZG/Uj5Mv63MaG/zSV8Q+Dgfgb6eftI4rO6N4mSOCG
-sFjj1Y7N4ZXg7O62EISdxtHnQLjKldmWHUmXidgRzlB/jpHJ6LXA0babsFZffOnJLTtS65yNjAB1
-jRQYNSIQ7AiB2noZkWwbxx+MS4G986AGN7+1Js4Pl/iWoGdQvouGARN0Frk3URMtm7iZMRYXfXeX
-VG+egSiKrBXMTkz3N2T6eNsmx2KPaZA5bjYx49XTl06ncSwsFT/NgjM3YSWC3a4sT2yxjm4xX+qU
-icWC2XOvdIf83GTOyeimlWA54ttb5WUYm6ZsKclI9yxeeByPWTTUYTGNI7PBwfUIWOBckrXRBvUQ
-eaEXpeTFWBbBVaGHZav4yFuxzhqxlBzYfHeU/dOcXRZcafNq2oo0omOlqz33uVJnmeTlhVQzgvKs
-3D/EBmt8p+Xj2c7jXO0aIapdXdn5TjfyhoN7yNuO/7Uc3pE9F/e04bG+qWw3hKqWHYRHW5NPKCrV
-cJVnH0b3E8vixhTLjpil+YDd/9VW8mUBOM8u5Nle0n0eVfs2cnEyf9V28stP89PIaNTLjS89Lp+G
-bG3wsLoXrnVM/eoYIxd2Le26zPUdbKibuY7v+7w8g0g6t2VyIEJF3hjc41uzlngt0HS2p1QU7a4l
-Um/r2Gz154chTU0iy2btbkADuyokG0IqMMtUj1lCf1IwOQ3HTFybmleFkva6FdXBixhtZSzjOz3k
-Qbahd9hP5viKsXyvWrEzx59DZN9pDrFB7r2dvETzmzExaxDRGKGA7ANr6q2dm/bxzWJ4IdfhXq/y
-7VLWO1XgEVtHxttpvJOui2fJJ8N5cPaDheF3IL9tTl8wyR2cvAl70d64LkK8bp0fra/hQMgtegzC
-JpbFXwvewMRrtok3H6OGsfxQG3t6+XHb+tlT21jZzoriRxyHV0Mxd4Fuk3Ze5DZdn3ZrYyksHP+p
-T8UTlRLvPKr1MNWag9Hr13bzlZJqNC5Q7kuXIUWLj42wRGopVk16mLNg2XhMbWFR7JVVIAvW9beq
-9otrNyOzxkY8uPHki+GnoaUq5tDaAXF0MPo+/m0Xsv1i/poZqe8TuMa2c9fr8Sd37QveJGBbQRv7
-l9K+XnJCphx5H+vx07Qm6TEjw8RZaReZY4tLh+rdKLQ8GOIK59aU3ScQNgKGz5dIN68jgb9Yx8S3
-0WJxGxnpx5SxaJCuurWq4W5ynFcibl4c8nXAxGtXS1Y8EFhwFk1fhGYl7/S+eMV1yPWZX9erI8Ws
-jnTd4RCbVRDXZG6PvfEzVvJDdf3zAK8CDTLIz7LQ2Lt57ziezgZpjyA2ntukfRIpFSaFy1tUsdRR
-YJd6ByHALMXdIKY9gUE7lQ4XFu8BMtv2tp5AF7RJtlO4o2X9wXbu4OXc34vUz25/m1jLtqrfpmrc
-MTu/Qjgc5NoPaxLB0C0WI9flPYo4ctxs7w/TxgLwzAU64C42yHdsbhLfOCyI/CnQ30ZVzu891lWz
-hD6RPzXRWecY1PXh1+z2vxA9Mx7FXj57a4ZrNP9ivHXXFCViMC6DpevPUfEpORfYyL9FLXYBy0fs
-ot3yPOKaTc4acDUnwpppO4wdfZwEWqwFRt+WgdNYd21EQGyqyx1L2pe5VLewFHeYUp+EOwWgM36S
-BRXWvpGz+GvxP2kMdWa1s6Qa2bWOweKMvwbWRtmiPwPiu2GRdgtz4jgtVIFFDsOkYeA4jIAqdJXk
-x0y27joOVgEYmK3SKnzbqOkC2qyW+QdeYdSuTzFwBRxTh7IkkAgY+Cchao+TLj89TI7nMsvxLvrk
-xY9tw3QjOvbuXsN5kSKX7hzoauw1sd6nrtpFKzU/XY5ORbAbanY1XMdZ8wlwTPE/Z1dTa/Mhl+Ak
-8FBu/BSUCIwuOECqv0nn+jktm2NvRyG5mhpSdV3j2kvFxSy5EvQaWDXzb9Z2L1Mp+xfd7dNfDIQh
-SCDMZ30oD0pHhz7Xnb7XGyzZLUd90ObTDYfMh5EWlzwytDsEJKFMWGl40j57+OMCF1a3JZ0Lj3KE
-ftyrjc2WXBav7fLpdGVIaOpmHB5Qi51rIq+jrn0QqYWQ1/jIEr3aVeywD1ABUNp/sI/ouBDJV3fQ
-l2nWtovIl7Da7tSWk31RIBAOSr7hdGlnBxCfsSJlx03XQ5pRtH7dNPG5oYP121uYqcfOKA7mEu+S
-JApy9zXxqqPuJjvHWghWcqHV3o6FoAOpTsok+5Vo9JF9Vsb1W2g/JO7AJLk4zrEQE2M+av0+2WL7
-PJlRzAokR47D9+ebVA76FjSI0G/Tiohwt9gnfhRYY3KjVx+V3b6CrmWpZRF2FF8NLiFtif1S+y1H
-cbWtSbSUuXpzyaacqCyYbY+QWuqbaAYkKL2DYfabzLdoAxFSewn5s9YZwRs0pnhrQxTqmwXg4EAh
-UP7IC+s4yLnBEHPdrGYVMb7JzD+ztCGpPNp0uYVhx9xVRgRtJL5ynJ9Zbd3qKHtataIpvH1dG3cJ
-l4pl/cIdwcESnxqrDljIjAjWxRKHpRe/lQRhZvqLXLh1JDaWvrh0Jf+KwVrIbBwRKEZkW53YQvPu
-K1wcBmb/TgARkCne6Fw+6iS35cI8TmMaxOxc/KSud9qwxq4v80EKG8mbPYT4xetrakv2k0k84Fkl
-f7acH3kibddYuqTwjbNfedF+atJPpo/zhQi9nRv5u7mVzgk3r9hNlvfhpsU1HSMVLHM8Yh/dY7K0
-WJHySzEnu1I3n23dCDGbX5O7w4koNq0nm2vPICWBr2gwHMESKFI3wme5QqBl1f3qNIqdgBAujFJz
-2d60EPIDb4FL0XXpY2u4RagMOj5tkSwHwCsF+YwFKmDRxA68Zy7JX29iwCctqcqedTDSPVrIfeUY
-P8m8CkczPSrPC7Mm4p3GFzfV3tM0CquBR7w/1meY2QFD1ZukHcu93nk7tkVIGr/B+dNWklbcztY1
-W5ATg4lQwj/H9HOktAtRsm6RboSeuGa1vbWoSoopCXX2dpTMNqCf6BXrV2DUzYMEyGFUuK6ZQex7
-+ysyfpgWVRLbdTbW2oD/F0YO2zcgKStrxFWbLLbD1L5vhhuqWVRfBeBipr79wXDHg8XOLZvZbVlD
-t8sd6VDZwtFckx2RwWgQrcr8uV8pdV19ZS3CDEUxb61M7FI+kHwW49bgQXlw1WPZ/2jmfaPfifl5
-nKMDpDiUMO1uTIpnTYqwH1DUaAgLRpwAII42i7o1Bnhxpf4lbHEAU73aVth25vvEpR9Sr8nk7hdf
-PEsO5lj8MlmnTEV7NEroIuwoyeQ22fg125SS3lY4xMbxsSU22eEC8QcQAgvjt2I6yWzaxnm6MxaX
-Q7glDTvrQwph4GBa6lCaXxvFY+n/yNojE4Mb4rVPAlmqFvuhj66Ok6BIcHxjRkmJottU+brIs1TK
-3okX7bQwYghn2sZOVI19ZATarl/o3vXNdD/wBw1dXrWcUd1sF/x2J/g7ciuLd730Xlcpn5dHZWiP
-3UPFua/IaIRIDE8quWVHWz3Ce5sfkjrauN7F8dkvGizazWrn9vOeu+CYNOVBOp06urAn+Nrj6qtj
-m3yI4WBBkEfhkh3nJuIYIad6ju5l/1yWWYbL4rlPASMZKEcMMg3wFD8SFB/qMHxKBlwAJ7fgzLQ9
-O3UuwkFtsFLKK3aMm9nq9wQzt1z+gsdqHz9xsNy1ur5HqROgj0XWinoLnEVoggLwJ7zX0mgktgiT
-QMWIuX/kGFCQ5vlRIGZe1HImi3o/ArUKhtpGxoQy5mSs+ZJ6E+RWOWEa9gBBVeVu6WHPxz7hdBXs
-ACIzD3330rGRkmQ9ZWMRjgkeP4nCOrlBmNugM1QUE/G9rXn1jQPKZYNIhicUx5b5srBvHmztppYz
-97C/JRYXujb6ajZM7OsQdmNNgsWwGRM1BSayRmLhReDnWdBzngzZWTh8vnqYLWqLLoK4Qv+mjfMr
-L/kaXcxK9s9Be1VTWuz1rNpNCVyjxrnHu3fW/XYDgi7M/PmhTSkflnsYDIRyv7c6y9rqEPFtpfTD
-S1vdKMxED7VPjt7ggIiZnR3J87SVnHBEL4ddPR0NxrGbKl6GL23qOV7qIRwZf6oZl0+tGZvSHfNL
-JNLAmaNXJK7HnuofDdaeeJFtbxAnyCq5OHuTdfYIEcQYroUIieqTSDpyFAbZs+lvg9mRLNhoYok5
-HkAQoIzNsl1H5LAd0l548dmNM4Lia2NqfxboTOzR7kpgY2nlbtWYRe1arpXPcwQqvV+wVCO++YqU
-uIrzfOfHaX4oW1EcssjmCkw0vb/C6+8d+wQxXFhOulYdEmMY4stUDo28g30+kY2sNZ52apR+Ij94
-a3nTLkp7riW+bIpoKvFbbD80tSLEPU4xmWsfLiLsKen4tfsicBgRT+bMolNsLbfYFTy6o/lgcSGF
-TYeXyNL9fVmsSLckohHIMn9kuydMUTFDdaxT1JX89VG5L3DKup8uY4KtCUdma0V98WNBFnXdWVHZ
-vseIJRR0OKBmO3dKbnt4P80FmmQdhy2ZJtqWFJk0DvWqlquczHxmADKeAFvMl7z3OSGnpn4sORyP
-vejqy5CUDDdqqj9rkyvt14S0+3qocJNFjGe+lpJ8js2MhzBwHU4gvSB3GAupe49SPH5Bgd2EEft2
-LseRb3lxsRdLHgRzDKwJbpd5pWv1z1xT7s6pvfumqZKDi/LshKTQBksnqnAckyHMyOQOmXAjXU+b
-8bTE3gSXkQ4WkVTxsxaMYkUCxoa+vj57ap0seaX3pmcFaAUqTPU4lb73lprsgtD98WfoiAxOBKvN
-h7W72kuv8a/0QfFHEMVnMbl0BI45UUSAYknvpCb9K6hZDH1EPSd3YHmwXMm67Y+IdcQNO2H/Br+Y
-uOlJ5Lpach4PUvjpWUWTuPaRlJ8qgMRm5z5i0qlPSTO4B+mCOxEmLVme+595terGuJv1g60y/SDY
-NgTLoj4YdXX3etyrnR1r61uvSMNe4PTqdYFVl4H3Xmhz+6AWHSVknq7vqe/6o5Quf7FreT3mRKGq
-MvSOcuZVa3+MLmzrn+FvJi/SQOIO5IuSff2RsmnFXo1SXCeFTHfesMgDFjxrK52V/qh66uj1ZxIC
-PT0KtD4X/CfyOufbpTpIkzvRVsldY4/y0PZ1HkwFpI7O+9TNhtdVOuE6uRVdyNgW1whjijiI/fW/
-whM51Q0/VsGpvEjf560Uo9rVLqoKYcH7YgCJStNrkzukQmL/j98UkcsZHEvEWMOeVoTmp3SSDNN7
-Yr3GRWS+xgQcsQUaeOH1s0WgygfSZdxaJZ5OJJYixH/DC3fNrVKJzzgQC0pKfQ/7LrrkLW+7diWN
-NP5ziwJFM6hZlxdnKNW+aTQWJCW/mMVV1M7lh4QpEaiWD1hPNZZClr3lU11DJP1P3eeGiEnT3tfo
-pwMJxfOmp7d8zSr9/vti+n4Di44WaInfalRdm7qbivsYNsU+9rVnFfHGv98c9mgR5qXkV1g/IDvh
-VW0czDRu+lb4JYeD59CRMzzM2UGF+P2jSxHh2YKIAmRqWh/tlksx6E3+FbnnYHJ8PoZiSeMd34fb
-8GHXOhYgiRdpb498Pdj636xIb8Pvt8mU/NMe4xcUo7zN0Uf7IvJqKzPlX6kmfvl+c32UEcWOTOme
-W44+yOb9S93qfthzJGDv8EO8Qpw4f6tdXIPrjtX6yfS0WOvnp4R9wgF0W7XVCg78xAKLr2bkc1EL
-skkxsieL41VGafFmyANiJ8pPqFsYY0byoblQGwl54ky0PfZy68WPIUPtMm54rift0/KjZwnfZ+vp
-ndpRotG/MRnc2Kb2jL2BX0zww/TKvhVs4yMRIzWjBtyyxCsOnWz7f/x4kh9OxIc34fdvCTmPVxir
-6GD647vd86IaK9TVls8tPo11D3m1JRaXcNNANBFvxS76I0gtEaKrrnhK6NU28ZdTbq6/4PfLceR8
-v6tuGvyroSpuoKO0+wrqCPiA9UKRjX6QKDYAyPAb1hCgL2Lij8obqxOYnuJepaa1rfpJO2u2EtfC
-6cVem7rqlKua84KwzLvvq1O1y/STjXmHucTSzjJGBxuP/Hz1f8k7j+XIkSyLfhHaADjkNrRmRFBz
-AyOTSWjlgEN9/Ryw2kYsZjHr2bSVWXZmVTIC8Of33XsuS9lzKNCrfz9qK8KLU6lWrTHPYKdKXd49
-v09UKHnj/LOiyEf+hKjBSB0SO+Xirz1yZUKJgNoyLaRfe0+Gh6sN85fHe3h+pdWSXwnxI+GyGuVb
-pmnuTcUfjjRR0+0i2MRYL58UrQA7TFjVU4urlG5qwzgAccHIAduHfnmlv/lWwqtN7WaZva0ZRENZ
-kn2LtWTLEeTc5JRry7avHzzz7tvdxsrKTVOHd5Li3Oq1Ed7UwD2AyW8zRg0yFfacpC6Wk6jcPS62
-v04ujpU73Pu2+YtT0gDXX669xvVXBka/jaoyCNKE84KJ3zzqZ3zQcseDcGxVpb1Ek99hbhoP7cwk
-cgxOtNqVhxDX3xUvV/VQ8Q++7P/6XvcObqnAbd18lpZ2Uky9CTchS1Uf9ERdPb777ONT7tDfWQBI
-MaIvStuwRn5VVL6zYWBL2nzyBruKMnPe4aD+IdV4TENtX4hpYZr9w2CR08fSuOfOKXZS79QKgOo7
-4au57NQueR3XuIp9RsXihpXrVlfxH9Ji5lqrKMOyi1Zu2QzvCcxj8bPRZo3XQZWP0iqmNZeXCRQv
-u+Zb4bkL0YtnSFN7W3mvllOepCX8GyYngl+QJQD3DuhLYYBzjMvad91XuxTj6CLnwEK1qSx8CeOL
-jBKextDfztkIfrzmC72E7LPsMyPRJ+TBdYJV9IXK1r8qtna9Hxy6xrzHvbXRRLYOHH/h4xgHcnjJ
-ZnBYapbR0jGqeoOzNlwWSY2dHeiGIIxPMx/IoJWHqymT1p7hDPCCvo5YHQR0zxwxLN3tvoWOURjD
-OpFg0gZy61JFL101vsEEtFZjz9HgKQZkmdLtiy5GoxjV3HaMB4B1BlkPexnqfCJ9hmd7KNq1F9fG
-CpKuvtOdQCy7qHyRTfXW17GzUlNHXaDmZ9Dd8Qz20rYWircU7GSPK3KZIFfAtiUn3i7bTuCfBfz8
-2KgPI/BWdsXfxgxiF8PVjAAjEXDwsyHdG4TOd5gBYK3p2fCcMXB/dCpI9tok1IrYsraHRElzeQaw
-Lfdak8HSQ9nvvO6BvESGcQ1b6ZikxjYnHAEBZMIGS8E8L1HtJrWGe7aFg7bDfsBKEpO+VltPUFi+
-2fhkByOYo6JRC7CCN8XGsp34aE6qA+GlNa+dUasVKr68AqeVqy7RrPlfILa906Q/aa8bvDU9j3uU
-pJ3KqOz04ooufYvb2D2QZ+ND9iN/4zhc75qKAGXZFf4h5IuNo69z3H0DXnCDyVG8hB5Qtl4yt8Yw
-XLl9DICRFRbAtXQKUKCYz1GsQModmkJLN+Rw+TDs0PgYrLhkUksxIMisrqGrDfUfXqukDGDc7bMm
-EqCftUT/oJeWGD5hifBohxW7r6iN800oHV6iYOugpObutGhspzq3KmZ9OI7uS+JrAXXznn3IIASv
-DNAxhC0rnt0MWPJiVKRBFti6WRWFDHAYHSJa0k3jw6EVdEGXCQrdNEgEk6B8aGwljuTl/EUC6IOE
-IwVsilDtaVBZziRf5Z+VF6UG9xJfP+pYbriWm28YboZvk4X8virhQXhtTtplXlpjOx0spD3l8oUs
-E4MgX8Ekqrf+GG8nY0RssKCGmUJ0e6hgUb8mSsAESMmQvos5gU8BNSxvAI+ST9pm5+NIyyiOz0z/
-ZLkMbv3geGcMS9lWmyr/EVUUm0o5+dW3Z/TFNoR2+P478vY9yHe8vtT9oDNX6XvTOgy4ZULAwXZ7
-MM7dOEzh6p+x1TDjozd53sVKG87KNIVtPrUOWilOkGk9fwTLUuPIRNhm3cMCtN1IYDVU8fHXXgyJ
-Gr5Dw+TdnDbmJQ35oFdl4Lox2m0P481p6bf34la+9cM8knoZQ9o/gzbAjl3qtjbk4FSRQgoLZnyM
-z9ld1sR6oJXkn9kk4IR3hfNBDKl5IBrbPuM8Sk5xHQTn0cnsu55H+Q6Xk7OK6479Dq33086XOoi+
-wkyM7WSSX6eKLmbtZ/bkTSNRbNOUsxNCJI79zn1utLg6EzoKrnLCZxRNiOJhFYcPI1b6Y1DxvdNz
-R270GQsT+u7dhNp2LhS7dCTu1l9FjoCSPo25j+gV21sW1xCgXOU1PjDQKEUgsdWPKbp4FUkj2QXx
-1B8HZmvu3Pm0aexwXEFWzolzJMU2L53gOk0md9tCb05QszHHuG2MeXsyGuMbCVucLCD3VxbADZq+
-6XO9yFGUQYHwiIlO1y4aa/EH0iGevilZ9N0JjmSv4z+E+HoErOKJ5j3OjPxvM4T51nZKrUCAQMdK
-ldXzNobBc88zO9gF0Ee3wPHtV9vW2NjSxB1/Zy78JfC3nvFgldq0LmZePRfY9hvonbnvhxzGFgSd
-5sNw29BdDODWLxjizaOCc4stWgJkDHxbxZsis9OdbRAeb6XFDwinLJZvUManKCy9jNN7Rudbla9O
-ttu5IEpDs9/IlKdirsVw3ygLqk5QSOpu7cdW8tWYASrC2CX1diw795J7HYxXAuDmgtqf9OpGkblK
-kjDE2FeLWdElUxSS1SgYGdue766uzV/7ebqvHD09GrXHMKRkSwijqS0eFk8A8AuNNLsXIP7OGU8w
-nZRl2cT8bwIaAOaLd1GBcq+pVhEmpoXgmVUdyjxj/jnQtGQT/hYRoAW9ZA4ddF8+N21uUq0yzFM5
-X1UwO/etd/GSmoeqGDNt4sQUrCyt37aDSgyMJlboktwikIQ0x/irrY16TJHPBBA0Luh0yvhlb7y7
-v00KVSfDHJt0ZyVH5Dci9e7QNiuiCGl+qund+YYm3n9ikkueBmUkJswAN4SyJXsbcwCfJ98uDpNy
-xSGkPVPqkrO70QNuXIqIORLuEB6IU5IZR06Zrf2RaZ/gXnkXI++na1rPkKFM0TuBGQenPGc1knIX
-2PIVFDWLzoRYE2sEA2wpiAL3HTQaxC6TQEuMKa1YVC3rTK5KlEkQzir2vGqfYFDcxqqsye2V8F9d
-r/rGKXlgunu04CnfwHGitVvhriNsgzgRw1VKOgR2wLPOPccTnxGPG7+sWl3HydRPWaihFkI2b4LJ
-m1/qTupwhenSNV9QaxWDgb2NaW7Dcje7rV6H7rprPfvExce5QdWftmM8YDJSUX2TWWQdu9p1PlyH
-qF49v4xqfx4sPapNJz8VX0OstZuB+eKQ84MGflYEQM263v6MB7s75r2y/uAbkEwYY1s8Ss8cCqLs
-KFw7J86HYe8PQkWrqXHgehdR4g/bvsqKY8UUEKyAqxevFQGbdu0YwXDknRluI2IiCK/0ofQruyt1
-/nqTNborOMLDCs5B81ATWy7XddyPEwDYqHw0pOf+sRv0Mph5xkcHI2I31mEIEsAwmG8D13zBZE9Y
-eGzSUhCSM/2vqsToZ5tsTKSVPgdgWj9o/8a5MoIicL07L7mOp7Jw293Y+eMf2hc9hUgufW6LXNe4
-8uNtB2NqOHiT0OxXFW7jhevKbp/xinia4iBIttXg1w8V3130azvZBtWIN9JPbPcBgZfrwdBViHke
-f0HKUNChHTSSQzZ3SIjOr9d5ZnS8Z0C9fWoxeIahr1gZ5AhfVmGdZzfEKss0PumcEwPrANck2y0x
-tUgDBQshk6Achk8iPfkHr0V1DUVXn0bd6d6a1PxOeY0twd5D6kwymklSPtzQ8Jah5eHG8QH0q8Ee
-51BL9GROiUPJRHuIS4a/RWAM6U4TZGf5LOPr4FvBH8zDHcN2Q3rIk/YeLYe5RgcRnHrtA17R4rEB
-dw9gw94Km/UkuLqzYSjOWYNt37gYZBg+1k732oYPpjV1yGXaHqNTzvaRdeOt04vu0hR9fkcC9Xau
-I8cDNYvlhReoWAcx1YuyjIntikHse8LLP/00zBR5zToTUWnJkdYaroA6vAbYVQGu1M2dYoK11jk0
-uKAG3oo+5jbjB/nOreuMn7cKLiZeNNAUOdmguKqz02D34Rl/BdbbhjNZM/MNLYLhCVEeG4xRYgzJ
-CrhicNdXimDrU9tjuaF/UCyVP73TPOssez7it7EorW3t2UcQbdcUIvTSr0ROeUGAtBoNGoa1ZiQU
-FqF3y7bcGYHprKYR0veQtj9RnvK+r8JPTJMxX3WN50Mnx4JDqge8YLzXhnYXtVHd2qpL76EZBhsr
-z7hRl8El7EdeXJXWvhCABP5RxxLxO7AvWZu57zbgyofBtNyfkFjYJcrSpF8YUcuNpoQEITJ/y+x2
-YVpLbqY7qF1ppP4VYa39tBVf80xvm09bU/UhGAsWxFjBtqEiaK5nlnH2zBIf8wTvRMJI3siwozKz
-sLotAiygRoMPPZAt+VRZTfZJc9MeJGQ80Ebhh+E2H6JkJYA7Z7QI6MZZk1q8lHmZHxNvMNbcn/Dj
-zQEfh3QYOO1tqqonko/bMPV44nrTii8VG6hD1gh59YdILPPIb57atB4PzFsOt3u0pX8UnonD6siE
-hRrkGUSuUr1B8i0yJkHKIlgXhuF+RBRfW9gS1s2ocbxzFFkPMivjNVplvWkz4u1tpI0rQi/wwiaQ
-KZVu2w8O/sET7I/mULWCBPTsbmvLaDxHWtbsWYRNO8stl4EnonA5apbx7CRGcZyyINy3AxYs5BS2
-3mHZxhc3Q6sy82LgWGKTQe4LW4fUsodEFvYGApl/kbnjH4EGxae60phg9CHfq6zyNk7q5qgq4xju
-o6DiN/fmThV5e64xUG+FhuBIZrnuZXZq2HBQZmF0Kn9kp1KR4hMe7TCk+poVLE8WkkK2NUexPfVP
-VVuqU+w5Cd8gR6xKGzeS8Hm/hVx68XqyQl3QIgNzG8wxuy3NNE49SsAiYrq9ZlmO4BR0VXbQ0TZx
-fE3+ybVzWKSBaQFFD2MOu5zc+j5yiNe2Dd0XZCnrvV3VwZfnxv5lyofkU8q83XfCQi2uFQnqmDEN
-155j+EiQkZ7dIe+H3xbXzgP9Au0hHYeqOyH+BQ8CBe1o4UHfemNhvCqvFazG0QeKGumwp10OaRU1
-UMKCY89ZXn91xUSi2RY5ui/OTFYSAnz5X8Gl77URpbelzkO+hd78pXERaFksgaO2rfj4u/AoaonO
-h0Vx72qsF0ruNihyMfeupqy4i0jQVd+8GwO5gAwVvVpaztK3h/9/13GUbsoI42kapi3znmIBgiLF
-tPMr6opZ3jdNH5HXkfof051AdvUYDdrxE6p/T8kNLx5YMtySHSL8VCeYe2+cd2jwkFdaY2lPDdfE
-jd/LF919jBtcdbY+XRt/mJd5Fej8EY3GryFlRHV5HQZIlLXob2kyyI30g3jjMFEtkCTrA54v9yGM
-dG9lKEYZA+sraKgGn2XjettJcw8j+JElTlFMlVXORBOUqynVhmYRsMSA+5/q5koXODP01ms2aeFN
-F00fIPMrvz4OsWUuI7qTliWWbU6qkZLo3rWvwj+AFsRXVOXRI0SO4U/o87GqnORll0crbpoFX1Mm
-7EY3OZpSXtyf4BGHpzSf6kdmKP/Eci67WzoX5F+jcEH0/qy3XfhNPQuDtpeY9WNjo9ASSoYUoXl8
-W3QHrR0JNj6S1uYeHCscVhYHpSIaEVnBP6mk/xNp+v9FiA08Dsb//z1kcC/lZ5x//o+IwT+/598R
-A9v7Fw2QYG5cIDSGA5PvPyMGjvUvz3SB/M3YHJv0zH8mDOx/mTDpXIQrwidk1WZmTcMoMqOmSbAR
-beNPNGCwWP7cBv2bGcRB/e84Gfm//5W1x+Kdf031Xyk2m/ADuzTDtLg0c211f3/9vyW/wiGpGgc9
-EStdjB0rbU3rmeOK96N0PLnisOZwbHw9+Uzcxv1hhoQ/MHR/nXrYOKVnrFqqwxcEeIKl3U0epL46
-gJcamwHciFo3jqmk2ENVFS59yAjyDI0m4800GBax3oxVK1egG8zpjqXuFMFhpQ3rpiLOQpgx8TpP
-RwupHWAmbggt3hvwXi5trb36bsS6FR3u0WpyfCyqacrPLIywoyiJhBagsb8HkZ9CkrOLR8cgdhNR
-sxQs2irUiSXbBRq9yXiMvaBPcTlVbncQejQehnyo3wWA57OJePcgQ1xa2KMhULMiFC3GgTzCPFY3
-8TkPzPSYsxpMVspU/r7iHfpKbNQ5aW1ANZbG7LGIwj74E/aifKqnDCoGnVQEuUxJvbFPKHQ/Sofx
-3jcmB7HF/4kStmRp6Vj7DKlyYbLv8jDAxNNDipV3I7gdkkga09kMGtvji4Z0xa938ZbcUUyuviU/
-z1C7jm2PQAT1chGSQYaBWJ+wGzQdeezQnesGE5VtC/TgD8ze9VLQF7Hza+0dAGJzdvOiopO+Yrst
-Wt5YVoVLXwWp9j6adr3i+uRvudF2yyRFl07Z3Pzp4RS9OHqfzX/ea1vaf/PEAZWURhq1HlqqPXqa
-3vwBoFLNgUYoA34IhUQzWQclpc+sWLLoOFZF2t8nKAibAGWD/+hgQ2lUtrAzTW3p6hOsa+NqzeLA
-WuteM5QkNPA7d7LwXhHo1CovbfcAoiB6EnHrHApYAptGzxBkfLrp3icg8HjpA/0kjdbetkWEJsyD
-uB4m5d+DZHCWAKPIFmt+WODzExOffJql/dZ2s3hnREQbqM17KLU8vtkBFfPgVePnNLbaLfpy/mVE
-kb0B9OvcMi3i8p0MJazCIGNbXIni1jlIoBk3201deuEprDUa6QjP7IsKIhWFXW9QPpMljjavRxM2
-e4yfCNZTzCSC/TI915QCLau0cpiNI/u9MsvuK6bYmvRaYT3EDSIUTgfYenbGw8t+Jb2SXaCTmYUj
-u8BykKtgaqNt3g7yRURVc7d1kInkxFPNQjPWxnNPSj9chyhjP4nWVyWVJ04jzFtHQ5tZ3R1LdNde
-65kUvBwvAr2erAybanjqI1CLi1QJHs5qil77suv/6m1rPWdyDB+KFEAGFwvxruuN9az/zsAkEPe6
-xnI8bGyxxKyCjSMsdGxOqYkZsRzYw9uBPWv2plzja2XnOQ86KKgsuhmzXxsOu0vvsrwMCaj8HSqt
-uEGkqLa/y93KEMNRxx6+qkMdv5bG+wSPgzWs/Wz0PlUz27vMXm1KfBW3qO/dp65uaGHTY7wfzEbV
-mnTWt24NrHNJsgxPDcHQG+1g6GU1Bgmu/khp/O7+L5MEg9O8PZcdERZtKLLPUmPD3MxzHK3VzUrJ
-Xn+xGkhSE8yTcBG08YjxvsThECR/RjxrOOaYDG8iJ7NQNyI4s8zvaJoCdALYhFjEiohvxnV2xiYH
-3BlBBkwJ0APL2HYIVu9FNTlXHTXnNTN0/c73Snumhw7ehDTbr0x64UalXfQU4Uh8lURebyijqYvL
-1yj2rqTCjW2QxPXotTNkY7A3MO/dEzYuko0mlBtAYDCR49cR84RdNuWusPFhCr7z+ybNqDMcpnSN
-wjcTVBjrFgQ55c7thlDyySaKbKjfPrSUIH4IYAQLn/QPNgHY7SpBGmln4hPwE6ZFHY6TJN46XfEH
-ssXw2NkyxckA/ceQz6YmK1YY2nisWalhZwjadjWXXGOtrnIAJEn+5JWtgT8xoIEnoYbgRGMTJq1i
-0s6VNRnQJyT31igFV10k9lJaA1agTvrc3Al/5SDqNtz5u6NVeX6wsNL+LZtt1aUz6Rsa3aZT3Prt
-pRv4xbjJ402Jt+YpDzVj6WdVe8ulMrd8fjWEd7e6JCLDgQd0DFBRHBzYjU27MqZqEdpcmOANo7qJ
-4uH6lCXykf8vr9eqPDpeVpFqrsjm1fNHkrqhvhVcc74FJ/JhcpX2wTLE/2nquWTHdEv7OHFpWsZ5
-651ERMoWkQNtuswe8JVlP4liiMeYXz6VY6C/TtgbQHknD2PY7GExYAfMmVuulVGmnzRJGSsSlHiN
-jdLdZ72pduyMfSJDHWwSen+PE75Uxmm0ZdOYwm+DVdw1q8PqbGCcX1e1GW1VI7Tt5Fon7rlUjlrd
-HCpoPgMiQ2TkSGhjxqNZ1J8oUIPLtItdzWQ7WhlHiS9p6Xqpj4IcJ/tO75pVjp+Fb8UYfmUJmwYP
-JOQih2q991tbbmjIqTc081lvKT+f7wrl9+x1RvhUYZK8MAoEXNr0m1ZP5Gz4sQRap9a5SPStpHZx
-73bC2bI6MVF4p7mDtJA8i5xyUWGEghgwnS4bfGIorjlD03yqWNNK5J7Gee6UG2Cm7G8iTWxGw5h0
-YgYZARsX37trDD3aVYlN2uP25uFnW5o1roCuAveynLLK3dHAEN9E19VHzSB9R04JdbFrkbeLxvuo
-kxaooNkEj3Hs+MuWHOLK6FizBgaZDVOhiI8RPXPm2KfHMKreMy+s3yNdGrjvVb8u+sq+ZazmcBSW
-ybWv1Ihml+UYAIxozd9vOvh2rS8pIBkOEnI4zzrZshsUQJ36NFH24EmnjhtMUPRv+EOKS8z7HOFn
-Gg+hYad78tfqtWs0/WqMofOA+6v/0qbcWQWWsO5h53TrHnPrsnOm1RgWOXqdCrewZ6KzSPuXKhip
-4kkH66SZGa25qW9Ve6kya2OMORcpEL74s7nrd0+TEWMLwa9LpUEUV8cysgAxOe1iBHZ4GDGNLCPs
-gNfMNVvnRAuc2DkmGir6XHscnA/7lx0yEDYpBj0zlybCLEt3CpDoQwuKI3mnBFnOjGg+o8hj6wBm
-hX9oGTkRqIlDSetbNuBl4MlTYRransZaBD+mpT9Db7GoASGdrENILNQoEDfesxCZcBhmEnft2NbR
-qfKl+znMPbuUXU0bz8m9L7vxra0ReR8jPJrd1JbTberIBTIBxhfDab90R4mdIPHKieCoZ6cOCetK
-c/jRW403gGVXCmskS15ZT90hN4sc4581vKLvNs9DBMxtWVPh/Mnfw8Q8nWG1g6kxPMWNaDaDga+U
-6Gt5jI16pgfRQ0KFpi5uOKOwAFCul73GtoxWvtCL19Y0gvXYexxZtEdCGJI0xjXQgjchWeFtnvbO
-ufNqax77sfRHHZnRkE31+5QWrNYZIYha9ibO7MQOWP1GUW28WF7U7I2JHlL6bArcpF526oImODr0
-MFygQAaffku+swX8+51pprmPVdpDISq0YWHXVbACRmGefFZgpKAwM9AuzNB1IA8iDgwgpCGQNGHf
-qEJdvAnclJpMQj0RdnC3wu+GEtVc80BiHOkzP+YHafingco3Hcmhm06pWanVRH7/eZhzqVMfiz8O
-sLKNrY3tn64Fubn51eBZvejbxFAjhJwWNyXIJzw8PFPUGMY/Y6CZTwJznB9kR60qxMXvnzpKD2Aj
-sg0kdrv2TXnkmzMd+Qd9z+Uhzhdycsx1KIS/gsklYpBthv+nSxvxxRZcsXUMq/JjLMh8SYluZQQ2
-1QmIrdeU3vJN2aXazo6C/NFMTP3H5O5C0sxzbhVz996pG4MT2ko5CcrXOvPODDibJGNxyIVn8h+U
-aQZEJpt8R+uY2PJ0FGuKHUFDgT440OiovrKKh3po9eY16PNwk/pkLuKRUwQrHbSuQBvzfebalDnP
-yOuFMYzzBmewM/pQ1HijvVRsW94urJJTEsk0H++bCS/B6GZoe4In74p81fyUQI+OIlbJrmsCOmFt
-sdbj5MWE/xFRWOqoDCobJm7OWszdz6MfXAOvuJbcF9fUQtwDRY2Rbeb3sSDaMPq0wbuPaKsr2wvu
-Waz9dVzt0SRrkrjBJUs1Z4mMy/q3FJKMhju7mGOh8aasnb9DD3BMj4X9kNdtN7s4tGpfDZkiLVjI
-VUX749L3lXOpS5BEBo7YJ4rpmyMu7/Ih6vL0UNl5uCUI1VxjWKbbrg/8e4nwuDFST2zBj/nPtL6P
-ixbiZz30wyEMdO8S0Ba5V+54SvJqgOkJAeRiudI+BFBAj6GdrAFsVnuKQ0tGQSP8IcNq80SaNhO1
-iF7CGSlCgHtZTfipvZFjmsPe4biAMFoltyiHABSBxZLKvrQxnscFo7GpE/Vt7CfGFg/9tqjvOCz8
-g4VxcG2Bvr/nKvOov1VcD2UgCBXavnkzcqfeRt6E5Ns1Y8dLaoz1Z0gnolrxBAwvBN5rJE03TaBR
-ezhNnVG/snOe821grqN13YVU5xbxtNVGaS2I/IWPFg3vCd8+KyHXwYgX5I0l0de6DSp0fssi8ydJ
-5poCKMDRzY9t57PIJJvIfGiOOrGuTUya+jYNeEQ3nj1ZeMyyjEnTHv2XqY7yVe8XveIaVdQXsF0Y
-ZKloefFBf8wxrVT7QRGH/2ty4m4w3WNOUl12tXE7vuS9YMxy7JjUONedY9jV2glmjblSTR/uYr+a
-q5pabEow9qNV1LgjhbZxsYQU6pGIJt7LTZ2sB1Umxikek4n4cqqd9BQ9XxWjsYWRPwLih5THIRaO
-aQribCAx0jgY1bqpXzstxoglFkjvQO7ePSUB7VkaYZZTRPp1XNJ8Na8ZeirE3I5kMzRcArKOaG+N
-T00PF8Ug3OIZ5bCpPI1cexH3D7roHaIMUbzDcj9vw9P534HjXPBm6ap55RpiGg6oJ+ZaX9ZrfLBE
-C5uJ7z8hPEz12TCwdrWA5sps2CmKAfBIFYYkBwymOKg7B584NcgrMw/HGk+lPf1tex51WZvZNWLp
-y3+5zek/kCZLhJOgnevak1nHxbaI4+bLCQNxzCrcSVVXji9MVt6hAzF8bIiV7LuhnB5pEyr2o7Ka
-bZTVVBWgwZ1hFkVffTXwkditCbBMCwkME59wc4pJucu3Od4cvWSngNAk6x0NS95jgBa0EDADH2Mj
-y7cR2vujyk1/nVte22OYSvMjN/xiX4+avy1tXNKo2Kz0QY6Rd6FZeQ8Z+KfWp5RXXcPNygbEP5CK
-V74QT4ULLtOEKPwa6JV+JXyk//SuNA+SNt+1EwoNfQLm/i6JpH2lKrdbCzxa54zBZ+9Hef5D1ZN/
-q4KeF47lGW9aEBFdmgqbOU/hzF/YWun/jOBUyrXK2RWO2qQB7wxp0ClzU10n19YfCOrgOqW9Tp6m
-UuTXwmqGB8eBzbPPNZyjxAR1TM0Uz2MgYczKoQfcE2rB72E9DI+UVKidndjGmQdCHiUFrydfJTam
-lBpPC+PaMuqN7jU0WaVxKZlOTZS333rZRR/kbcdj6eEASPpK52Ymup1bKmOv61yyPSBE3zqw+qtU
-Vf5VRSo/lJj/N2ketrwTu2Dvxj0iFU77A5ghsR+dJN9lUFrvVBlhuktU5O5A9apz5jFQYrwe679m
-1debRnZAL8kdRbtStBPRp5q2Jfzc9kRM2i0pViCqdzJ8u/igtzZ/1LNGPqUm+IIgK/21GQsInO2Y
-nLHKifOgud2j7Vr928gK4KZHVrTHAhLdNE+KozJTesXycq7j6IX/JjQSPIY+Lh0FrGD0Qm+v8iQ7
-e0audsLp9EMWpxY/MRqfGWGDO+hartVCiwhrxwBA5eCCSW37tuW6mRInxiC1kJrJf8hQdls3gOe4
-oFdX+2MTGT/BYMVP4k7FcxzVNSYyrAhGII1veh26e0EWf2fHlbG1U9hVTuAkJ5Nnul44Y1OA0tNQ
-J7V+pkeJ1Lqidbor6jVny0AlN3Rsbu0a9aN9jgPNf3T62rmDMw2euJjqm3Eo6fEe2cpkhcrXijzv
-44QdcMGk2q8j+IQbQuXdxQnVT4La9Fi7NGwtWOhGZyKV02rqIuNNtq7J+QdwKi/onRs83VvTNOes
-nDYM0LGtKYUqELL8U667SSwtTBYxcasjnCl9Gw1p8oazgh0Nr3TCdTT8OTkxQ3/wXBSq/nFsQ33Z
-ijbiTxkGIlUCjG/JhfhKUUt0VjEHYD7rg4rK4YfGCY0XHGfdQ0Sa7c0PB0hZXmbuhqb1HlAKY7Hz
-HGe0F1yiaawKZUx21UbwM/QUMIsf0FlPJ+08H4VVJ/JFXuhmcWJoptTKYjy1NUOSpc9SClGZ49Vb
-Y9EmvmiFibtdqiFPNlVtiGtA6xzfosE2iMFCFVvY7B6QAvXcfHe9MHA2smgxcNXYPQlnlnKX+MhV
-Ol/tdQ+uy3lTkAISivxwxpCtTTxANREELXxqMWod/hvxnhhocqxA4iMnLVmhtkEUS8sZtiB1Gd1c
-A9GscLrZ7B/i1jjjrmbvrYVd2e0InQMQkL2MAARU5ErKcRi+JtNCWJCaqC+MDOxLLWDxS8Za1D7a
-wOSigDpaUiyphi83I44lgznJ9dvpKCKu3Wia0eTtTGFggGlknIfAVFW8NDhLmUexsIHinIZpJ3pc
-SQyoAyDzmHXt7xKVZ6r/G5I2pLC3QvuTXoyftASBfeiCef1KES4b0N5CttSUwaJuljK739AT4TAk
-W8Pf+TgVYW8zEa25xxUry6ujVx4l/optVRxabRjWLvHcOyMI+okJj0jQGUhAWPnXMHKDA+9ddW8m
-7oAahrSx9qoLZSMGgQsteyqUSM6hEg8ADW5QrmCYpToMdh/e2EIvbbmreQ8drCJKT0kLHqDRreLo
-BNoHVh9uiprB9RNwFG/K8D/YO5PkyJE2yV6lpfdIMRgGAxa98dmddOc8biBkMBLzPBiA29Qd+gZ1
-sX6IqL86I+qvLKlli7RILiIlgnSnEzCY6af61HWACNFf+9moSm/M2jXunNbsNrHrvnrRNSPnJ89n
-hMkmufged0G8NyQMvd721QGrHkXZ3uC8tB6Mc+inKt/R8BHsli5STvSVuR694KG3OKCHFg9MJ6Vq
-kI9pPnjN0nc4qfx9ILdyndeD2siGgKiv/RCbedDupjBPOc9QKek1ZGvjMNCMeTELrGLgahuHTd9J
-ZVPyoRqk6IaN2ocJGf41N634eR4Z0xfGEL1Q8xQE235a8KI9lN5iPbpUvzDRiqRmN4W21llVeQm5
-5s64e6mddP38zPKTXvye5z7Ni04c7WpqDh5oeRxvm7Bt93mC4R2FBFAPdws3DsnJr8azqIgYrCq7
-n7DwMDcX7s1cWUznUc9KzjwtUdfr/z4A7hx/a9Bc/+x+B4X+ghr9fxcuyp5H+suk8u8ms8XXv/7v
-Iv5lNvvvX/eP6az/hyKdqqh14/zBHxn2/hsAznX/8ASLoBDOT/joXwBw6g/60CS9aMp3XeRp51cA
-HH9nUW2CZKKUAGj62zz2b+ezzIN/mc8uqDYJaM714Jbyn+VTlfJXMqfXMdaaLZkuLpkvNrHlcQ67
-ZovigNlvUKOJm5tiyoM7V1c2BfTbfDA9fPk0RxWmb76lTj5c0xcG/CtTI8AcOxqOYRE5J9G02V6N
-9RdY8t6DFX70szHfp/50k2kQRlFF7GMK+g9nDi8hGfZOPVfEiGkavXVdKu9z4t7sEgfg+LWetu2o
-/2wt/0XMJjnoQL60U3LtVNG3UR16j/w3CoRdVoe+c+6srN82kbcmCY60djG1fI29eOvU6b5OvdPs
-Vd+6iSB00J+julpRQrAlK3orxxFKS6+oGKYpZTWjutIwSZow2zT2pxAhWou5cRiXNoQNVl3V7pO5
-2HYmDUFJcIwl3Qgdw/cPgNvDVhXsm5ln7fv6mwzn56RtAEFE8tWQjnmsu/mFhG22i5sa5WrYD2W5
-CYdwwFtqN0c1Fel+CKetaNU10e8T7bsPY23d5jER6TyTD8qgfcxVEwzvZG2x0eBIcoz1mU0pKPph
-a1gXx+53EJqPjcw3jMjh0DxNOYTpKR6Ma7/xN7Vd7jsscMpcF2mBKhy8gSsiLxlv6KDlbNMPT7lW
-7ToJ8GOaFokuE8wPD+kBdRup/lKR2mKUXyM7EqA7FgWXQIpl1XkrYpwq9Wze+TyM35GSaPnriS5p
-5xpsJZ33vpmAAI/0N+ylHxEexVUdOh+mcBFuHKzhTN3dfT1K2nM7B4pMl+kd9oDifirjezfcOe4x
-KfRCpC8RKziGrCLyBNfYEPW9P3CuqeNA3spmnF7C1poO/oTzajImzoDhuMvowF5j/jKBdI3BW2UG
-V4Gb2ccByeuK5f6pEvrVqj19aew2PnqRSk+i6BJoGPVjy7DfG/jXTIrbDZOaFLdpyjbSumHJPTSM
-nDigX0s9IgQELVyJMsguacdY30ySYxoP7dauzPe5K/5klshTumADLqf0CZjipcT4yhmWk8GOg1L5
-iDV5HYjxWSuGNI6JtbUkwbdO2UNmoMZ3kgTbOZzUKsFhi4XtDO5hDfh6JbRDkE2jfg9ardmu4PGt
-9n1nL76lQ6vZkEeb3tJsCPO2u3XT9Hups5fSgzVo99j+HK+7TAmTnAqqhQEPzPo29Es9I7Mo0Z6t
-xRzZaDh+rrYPoH0fHOadwFGbe9J7dPV8n/Xw1hAwWVlRfKzaek8BHw5wh1KkXjBG+4AV+yyA2n3N
-buheIhtkf+nYpEJxiFn8ADTcruYs6QmjHMry0Udxlc6IFR0kqlxi0K8YrB5wKvOmwHlI8G1+8MIX
-rKZEQWyZidSaCkawnVvNOmFPm3IBwOR5ZFqYoTkkq7k6BJV/dumG4PLo11h/t3IgX2hzoWPsKpiF
-rjr7c/bSB+3EKVR5PMSN/+qCz+F9CAeeiKf3cynjtSSXvmq7egLros6TQV110vUwyqK82rnIMgeM
-DpiAZxezt8fBCzUieE/DfheBeAsz8xgE37p+wIxLhqA2EwoTsq3TVTt7JEjdjltRz6dKmQeLYQW1
-gikJ3PBIxN3Ur0mz6wYUJ5FV1+hsmHkT8usTmqg+BZm+7mJ0FM8AVokfRTifuVFcQMzv+ybbxyiw
-eRuA/uh3RtQDJRSn1qzJ2tE4DK+S4E42EDrMwrsYpuk6LfVJcNRFCZ8fyqE+F+MHNePXsLUupl++
-jplE3ZtPKmYrn6RXBf6UdZDQNRiPnCaUE68jGd9D72eVUEZ7yF3SgwLD4SrSGUdr9zEqaQ0sTDoj
-FJHaqnjIE/8EDHdTIywwPWBqBc2uZfdnyX6bZuqQqOg5wJ+8JpTABpKWjSZyj4y5nmToPVAquU59
-tzr7NVSlggIdAjmlu3YYVnIq5YrNlU4ORN/vuty9bXKxr9uOuuw0uSHRck3xBAO8F28O1qbRfoSj
-3tfOfEHcfwxL80R7pbGynfFRIQms3KG9FyDn8d2AdmxpAAz9P0eGDHk6XzI7ucdxQB/0RDzb75S5
-T4yTubwDwINbfDNU2TRyn2Qkj/hiHA7RRZukdKVqBS3HS6iReIGAb00p48YsqseBXAvz5KnOseoP
-RAAtLrjhc57q7sw+9jbCK7lR3BA7WdgvUK3IgMLBM00SxjaReU77ZG/unC7eW/1LzCq67qkOOFpN
-cztN/bFB4QgQl4fxu68TnKjgRNDDrztwBY1eQqG9ODGBObkRdyOc/CtPmDfIr2uY/smackcECOQB
-EoB3fYsvAebROpbie9ECmnFq54xVyDmYk/MY0arUp86NDydqpUiemi4Dd1PoE1PbU+eT9iijfF3J
-6qqrg+c5iRjeqWPJLLieKZcuHBqD1GHybX8LP7O9wjGcbg2yDNee6RDZ6OxXK2BQ6TUdxWKcaWw/
-5z6dd0Czt1kcPAZNdA8mp2bOCRcglEgbAJ+FGD9l2D4Txb+dgvQ95Wq2hu++j2GVDROozeks26WZ
-I64uQocdWe+AIqiGMpdJ2eaBHyzfGA34yhZMbiv1W6bm5gLpSe0t3Z48bMUe3VZHJGL/uQd0NtXG
-I6YEwBnI5eccpuh6KEdK1m0lAIV1zXOFZX5kG8ocVZ5dnEG6o0VN9om1t4taXZlRSK6SwWJT9S+1
-vyCZogAJO8qVf5+UwRnTirOrKz7EMfW8HZe72JJBi9el/Y27Zd4Qw72QebgwXSKOrfg15iQuLM9r
-jzT0+C+xUh8tpJZC48NijrESmfWQ96THXb/8sNLAOzsGRyF46/vREptGWMM6oGeHpSDcudQ3rWDR
-CVgRXn6tlWesOX3+2XPsyjNRbL2GeYgxWVfGnD4Q+KAbMhjJZNSPXW5XhzFTP6YWgyTk7LMSPLom
-IT8dqAYGRDf0F9GFyRVEVrw/NoO2MIXR8RN2YhpLhJcd/LqZTOsUj0+hmmCZMAGMjZ7hrBnoDbxd
-vYM/CQXEwRhtuwtWIiY+nXT8xQ8Sww8iiighDvyEFCw4jrQemVKSUtmKBCRDasDWSC0wJOnisdYz
-ucy0d8DtUa2xS+WIE4gc07U3+AvNgi/78Y9LEtin0B2BKkxASuDIAY7BNoG4kFTW209ExkJpKOFZ
-vSzgF8sNt2MQs/m12XLxKeJzCkFJ/HhZ1Ee+ScCnkCYLXGPxl09tYG0Qur9rT6BRtMt3I1o+PtYd
-ZRWMMmN1HuIY7l2f36GlraGZnmA3rZ0Qw0k/+YeOYyrg4zSie2su6bszEuvKsmBEMqd2Txat4NgX
-0G3zmImEaTa35KmfkLGfmXDXXCoJZF00HAx/MNv8uXwXssQQjxWdhMC6nMK99sp7UVtHYnZiI5pY
-7zwzA2vZNw+Gm954RnXyldxX9vKoZ2K5sar6UvnJbrYJizj45WYo12gwb62u7g3bGSg1MvUV3Qrx
-Lp3r6UCuNcQmKB9m27rLsHhslTE+JCK5qKi68fLwLmvTaxdpcgO+OrhyxpboIObzDeE59xuEtP7A
-me0dR6siSQRAkZk0HvICl5Fyg++Mc4HaJSN0QH/aOmHePwiJpyJjo7nPieIfhZnQwTZn+UMg0k+u
-JAQ5lZaEL2Jn0wfkvUIqVc6lNPtNZU7USVXQH3xnB+633tQiWNbdkJ2BQkPBUsvV4kEIHqJ4L5d+
-3DA4EXWLNyjOags2sts48SCvwVQ5m7LHUwInaZ147yqxPxOKEdZUJlMT3JdfOGfzL3yqDtHcNrj4
-DOLuKK6aL17d63XuQ2wiJHtIMe9CT4uAB+fTmhvQYicfRGuhbf8CI2Jk10A9FKujvqncIllrsl/r
-AhzNsDJl7m8wrqjrRbrLQtM+xNGU3JqDqXZGYGa7n7dsPWX3ac4zh6YvJt6dt6CD4EmnkAWuwgVd
-3fQ9t4dVLfd7w7UMmmB8MRyffXcW0H4r3Zbsw8y9ayd2cEOTNoohjEq+PCMOjkmQqMGMx2YbEOSf
-2K1iHYR5l92XOQ68HyvEjzR5WxvtMZ01rwZiDuXNB9oT9jmoEvxePQ+VeHy06axL11j78CoCdIaT
-ZMk3EDLc5LMxH9qmxd6oJ/sprf0lpUN9Nlwz234CUF6dRmrbDsXCGPrhBhwsviP5s/pE2ia6B/wM
-04S25odWqQCfPlttXHUaWpA9YI60W72IjjWCINcpaXGBlXj/cylLNcKm3YIxDVOr99diXkAxFoLl
-j+UqVD2fys+3iJIBiabsm9e0JNyR+E34RWiM9zQRkcWvw+UmshmdtpUWXqq2FPZTrzqj2uRx730Q
-R8XDCNviScSss6BYJCqrzvPM2v1cDKt2/MS0Y63LkLRuKiPwLj/AWEKQPQ3DELnXXf4UxEOw/7Ew
-2s2iAWcD3y/VxMrBbSxfJWpW2BKPeLxMp4nMlmrAtZniogwdvg3Zeb4Cp0rEj8tRquGS53dTPBR5
-XLIdL8Xb4PnQpyvTYDo4MvSPuiIXnAiSgLrKnH+v6xwmCU8xiWV0Kd7eNTPPCTz6gEXaNiVdim8Q
-GG1vSSY3BOUUDGvSe2WlONOzdsnM927diIwnj+HI2I7NWEfrhM/pyoL8S5FUb8xnYPLzgwNsAoWC
-HqTNjFB5YOQYmStFhck6n1PxPtOmdJoGywCfPvUnMVvwQiw15KsqSNUddBfaOshOZa8OkTTEZE5W
-tASKUr9ipTaeVUTTVzPFBut6qZdD/azUsbGM+KYHlMYctra6t5aOJVAlwH5OUlmz4pZOigM9p6q/
-97EbTvtcG+5jLcp2E/LPNmZHweAKn6T/XVmT/jS7yT/1CxGFzsU3BI35Nh4GUkwtZ4I16dnxBTcR
-mLokUfc6kiIBVhZF+6ZMwmMQStuBXiysqw7D5LnKExVvq0Saztaz+mClPCx3MlWVcfCVl1wzdGxa
-fk8S+ElnEyCo7cbZE7jKAH765lo6UX82W2a2YRQG+1ZGVbexqz4DjZ9hdnPN5fmDM2BlZj3s8ITR
-iplU/uechOy/dd74J0/FYCo6VHRSsEMdyR11m+3J1I2+4aYfmdrK6nkQPXmfQo7IXyO6UhImYbHB
-FYM9sUHOlVNhnHq62oFdsGO8zM48n0qUpxM+Bu+Wa246TyNav8mZnzLNaWF4BFIUOfNugfARx+K5
-h6ejKaXpyWdTybrg55vgzu5xuYbDgGoFEIMSAwKUQLYnv/5y6UA/qyH14LFZVctO2kzOZrFgzilC
-L6iqRfNItuVkGU/8b/gNi5T16tIy1W6YZKgvaCaMvi3leC9p5ruPXJ7umZZ6uvaopceIZai7nITE
-CYbK9NB7/kTUXwzV0dJR9RIQqH02osH/WsRJtMHacjFoZmaEvTXB9ezMQfRJUonjBkW1gG/tJqse
-K9xJzQlmhXHuvTh3V7HZtp/BWKTXU2ayMUZQ2BrYrT8Hi9/kPOn4nOFe9paMa219DnbA6YHVbG3N
-jTyalq128+j6Ow+8wpmuSfVdmVjfR5+jsz/RpTMXekCR7NNxbQsP875jOwfQDj62QwrAxGwnJybe
-HCE9AfU018ztZZXngHm1Ere1G4I9x7PfHDgaMObFGntBFqQrni+GnnHtZOHHwPe65uJyGeUEHY1h
-nb9XSYnXZMZMdk3p2jI6SYhVxxYboUkxXvLM+KqEtUWGzTRuA1K/67nyKGUw2YILs9N3ppT5YRLa
-Y07+4jBue+Wjb9ZFU2bn3FW0YM6hQch3mo1t72XqFKNBHbBJfkqDvQ4ByG41mkN+1LnElhCN6k6T
-069XmNfgjlqyug4iD3y2xrIZKbjXmVO0OycPxoc5mNi+ZksuXnn5U2tidTVr0d8ThqxXOMLQDPMp
-wRHtBygEoSPusDkM11Q8A+Msw0+N7+NWAFhkkgjPYj1ALLnEkc1BoJUA/wOGxpu0J4O8bppQbCIW
-UACdqAidnAKeUJIuilQbmF2NYitEMh5qqdsbR8MPnVUxf9XMeg4m+ZCT49gSZ2RvbFrpG+e4Nds/
-wZsTaiGTWnKDVPql1tiGF1HarbBl5HIRPStrCj88O+TjHFmzGhxRNw7uFwssat4cs8QcrrCNdgcW
-BEJ6edBbV8Psx9Ve4kHBbsDp9D2DUJavlVTx7aCLvNrjyIo+k3SJ2skEw2IRLfNMQsE80g0HigbN
-s8P3uZuBjFu+As0fgJlYrkR7PLGWWIdxHO17H6fce2F6k79SVgU+LAv9R8MTOEwafyyvCw/W0kZ1
-vneETAIYtyD2/dx2yobIy3D8mGJO31cSWsGIP/KUyba01hhU7HHXkPdCKZOV+N77EUdjVuep3HWs
-tgz3oXq8M9hOP0qlFw92zgfUTDzPoDTAhcVsPJ6H2pGnOS6Np6FkpNBTrXBvg4JGVcpd9J10TILL
-0AX1BRdLuMVTO5DVAESzJffV0qLgz5a9rokmvE/RoN/CcsofyGMg1XMfPpB04vFHtar1HNGEkPL9
-hLOZGqBSmGx8yQ4Ehv8u9+seE3DsbUe6ops1QFjKKVwCBbdt1nceG86pfA9SJ6UJVrjhOQTkcAfD
-rIJObnrwmyYsxNfam71HMNLBOxAPxuQ4sTbSVNWND5vpUNTZQ5s55lURhdE69nXwAu+P3GRl1XJX
-yay+DlTqY1Tyx1BCzO3qR43etombaGgZGFfjLuqNiEQTxs1DkwnYECms4JvR0uNdYhDuXlGcEj6U
-UZA+wrIYvkbW5RxZcUwwFk9ganl4GKhvM3PvVxYS3sjM0wRLVO6z4IZYdJk0l/lAcXU6ftKHBtJW
-Ef9fj0DWjkDmT9ytVbQ1/NLHReNKEj51X4kvNuLNwa5BnFVZbEMbdAjUYKkYu7uwxUy00uT+n4lT
-ROdhUMZmZHJ7Mn3IgnE7HEXvuKCFqpHWIKe2d1xkJrQkOUOgok3xdjQdTnRNF96anJRiJIPC5g50
-etJIEsJ+hOJBl5xDtbrhodUQOSc0aMUNHOMuxEUaeN+jMqKSYJooG0Aw4dk5NLF54fDbIGsCGeMI
-17tMAooElXid2kV8NWKN2RO5yrYC8DLB4oqHZuVfUZIqKVq1u+KeFBC21cp20OmbhjKTJNHbNCqN
-+9IGK4NpiMoHWsivnMKfgF5Ymy4PH1m/7joDA4ThoqHHznxyU/oKpmTyNjJ2w6+8zZ4mOW0iRuxn
-hg31JlVGc+7txnrTDDOg+mLb6LvAXUW1c6/b6GhU9dan9/40sKL7PHgMGd3hQ9rlBlxkahX1aJ7D
-MrpBBEHzSan6gTSQN+kR5kS6CVz7JSqx4gi6YFsUPQo0d0AY3qpAXTUVbJiJO5amM0DSRTQt8hbG
-SHItRz9picNAvmhkOu9TR8TbpCinedNQQd+EvrszStVenK6ctmCCCBvaHT1HXl6/m5WUO41/49y6
-QUCtLDEaEjyNfZgNF1IezgfxJ9m/6sJVyyplq+AZ4+D8JEl4nnqjAOZgRqq/a6yhePDCztzWFMWs
-0tlJV6U9P+K6vFJMNNaMoziGEVHazpm2r9IheMVWncP3McZ9OvYwsKuZIig7oYuF8zz7VsxwxzAX
-DQ+WJttEFpjAMNHuXbewSwf2MKcY7+zGz8XU7SNMm/dGafZfjH9LtHTmJGOkm31pS49JA43wHAet
-K7wj07mywvbiGibOVNsb1EMzuP1VGqmZneaovilsRru2ltgY2HOu3RJ0Da0IGRDEKt759ux+GiYm
-tlSV2StZOYf+YJGcmgi7t9EKn/1v6r5YdiS30zDMx6yI3J09SYpK8Aznd62TmDA3jH5rShJnufa9
-w0QJy5MRjNauNyzvG8HT7pzXkw9Ao0uRZNLoUXG6+y5GCxm0TXV7zipTbDuQwifHK51rDcobw0ae
-j/tsMekIs4i3UwpNoZ2mBVtIXzncREZOTSLSN4upxA6ObniLlx5ZsJqzLeiX9HYoybASfjVumZdZ
-WzxP/h0wAkzlzEcZnFjVIQsMdzu7iyzidukpiO23EugkCdPeITOro+9J2HjgzLzp3nJaLqSsMiRk
-rcH6qD0+udGqgiMg/HQNmrt5CCfXwAWT8oZKnPlmMlVgaVRP2E1RHMt6dm1EP0QoG4O9xwF0EwQM
-/krhNzcZQ7fFKq8lQwsbnA/GVrI80GqIGhCPi6gBKcxjJCYKrMwQy2xaA8pmR0XPkxw2cHHpdinz
-+TPxM3Ys0mYsgbZ1SMbauIqtKdpKtxBb5fb6CnuHPjL+bAG5s3vNAUIc4M/N76PB0HhkhH8/T9QD
-9NU0Ei5ImkdfFPWO9OeeI3pyReTQYx7lW3vGNz3XbhNgMrUGczsbPZ8IGSTVqbUkEH5SVZXfEZXq
-IAeO6mlqZthBFBNCFLMB+VG2sLRu4KgbeBIeZT76tFKGVvhCVZj34Bq4YFZOD7OwVCq5gZscX5LM
-1kQIfS2PRaDL5me96P/HBcTfur9G/33LFo7CwPGf21JuP5qP4l//5Z9+1b+ZUmzvDyEdzxeWQ+DR
-/CsywLH/cE1FhS3+E/UDGvDvzABCLhTfwgWgD5epnhQWVbH/gAZI9w8qDinF/UdhrvrvmFIca2mD
-/b/MANd2hclhyqd3V3ounIKltPAvzABZUnbPcBg0Z6k4UDngr0mDmgXXpWwkzBXDNY62O2KEquni
-YATWMX0H5uelHzaOVLnmrsVQkmEA4C+VplJCQTsLeHgLhvFevvBWitQIj24ge4HmWdbm4jKlE6jI
-kukbgPFuwRNmzVsjeyp+IFj1FKI6PaOViej+jWOE5lWoW0a7tAkgk7cCe8Q21BWzmbRuKeaJfdXe
-WbGUDRHclo7oXHKWY+1hz8muQdgvvpvTACDiBYiZu6+z6HiKtaUZHBK3cb868Pl3jRnkH5PT0SM/
-YVXlTcD7I2kaZjDcUjwWd7buZoQKcqGY1Tyj58Tp4EGHk0LQLG0azvcT5UHDBhccisPYDLgCysUD
-uHaNOf6YogqUcRoEWPSiaEQp7nUCGYfprf/hdfjOVzKPQI5l2chmsye8yq4Ywxw+dWM6oIey7fXC
-TFNuRDritSjyTjO19NUR+nT6EDDZekRJipsNherybJd2SdS3MxjkNrENCSJs1WdJd96rpIoPowbi
-I0epit9641LiAf5VdVeQdIpzqGP1PCtzpv0dvMNNm/FYWddVod+VXc3Pds6IHKWhJ3pIvOy98Mv6
-Ph4mQWcVpguqafCrdxiynRQ+is8Q+9EAxPbFKzriaFix80QokK6UIZgHb6N7ooy7mhhlwrpqxZ9q
-Huvv5VjHKPth3IOrpS4vV5vRSii7w4ZAPhIa4tSuWZqZRKFQqVXZ+I7eLOLAMyq33R7jxIfVE6jw
-TU1AA+txCj6aICqxDwSqrXdZqbp7tyjmDzht41uEed1YmZ4YLnE15ZfEzvCQRx4mKCxac5Bw9F0G
-pH1AMR+2+1Kz+zc99cnWmABoyRAy2KRTnRlcfJ53LUSeYksw5/mG001/qU1XvuZe6b5DBUEidHXf
-XAtaHa9opmbzHGcOhPEWhuhUaU3rU16htkhW/jvThUi26qEIcF/EnfPg2h44Nzv1hx3zUyLxwi7b
-HaEd/56O5QY/MlxBs6n8PSe7nCI5L+vXrFZFuxZsYen+1VHp7dGUh3ti7ZR2ZJ5o31uhG3dbziPh
-fwMXL6+pOAMilwMJIhxqNsD/Q/3Nq702WA3UG111uJLsbWYSndrNIdN2aHmZXWyzEgooW9gy9fa9
-k1MJNSbDLJnPx3BPg7B/n72ahkdRactcqwBJhchbSkmMZy2Oe52K7qtg+FmA5W1QaYlH2czSw5R8
-HhIX5/9+Toc9O/SIZuZpsq5HVRZ3SUoUeN0GAbWk0czBgWJY+wOnFJdjXZeg5pj/UEhtViYVJLoH
-3txUTFRXtsVTFjrccik1CSLvKow0uYbU8OFkF0Udumsfj/8bIYv2HTw9Z9IhKT77jrK4Vc+pxWIf
-iFhCks8A7kaxtEtuPG7VQw5Lm92wRQowMTsKhpFrGjaIXY/m49W8EcObsDu0qeW8JXEJanXW/Bq3
-IOC6HSc6G85gJCS0caVNslYOphQxd1MHI0u7z7mToYLZgnYaaBPNGRhlEi9stOyF+LfBUt577Z9N
-mDFIR53UiLrEDjZl0tXxtoZwkG+Gyoi+eW3UiJ2NMkWwtR7T7yAWjHYtgVpTG6ZSGIRWOJFQHRcj
-oS8aME7gXez7oPbw0DlxWX6NfeA/DDKzvJVuG8pr83yGcO1IH3BLvlwTxDdHk0y/to/8rKHDtjpm
-wQNdlTDcjAU0hJkE9MsI2AQJwEHRWoNxhslO7jp5rTRttyu7x86FUoZlpoxK2BREm57KhApcajlI
-eoO20gs5WHBODCdncLchW2Giz+PCDBd+uAw0oqxq4MrVGMfDZqF/4SPF69smjB9xGfxAYOQCdkWI
-E/6TgA4jJbesQdVYkQsq2IS/OjgefU9CsUavYA6a3cqAAf/SklnMsUV3ALmou6TfCEYto63OGOwT
-LjSR78PJ4tqGyn3xRzaXm5Cp+luCEc+ClK8AptoVSbo9GgkqNB6c5CvOaved3TWtW3XPRBjHBOR8
-bGqjTE8JQbIn3zGEfTXPwJXJHE8w1SjxrCTRMlATTHinqGN33MTZsfUaLH/Y/v2ZM0tvP4VsaNE8
-ChC5x1Q4ej6kncm0ixRCs0Gio3G2rLi1121ftIjWnVowsmAfYG4Vuj6EFS7Uo9BpjS7GDJfSLhv0
-1qFENdSQJsp0fECxIN3C4qRXlrAdfQNsJzVJJ5f5ezDg5t9MXQm8JMvrMKG6uGVGQxbGPUgXouda
-TD6SCLmrGdOs2QYKirfJ2cOeexeKfWkl931lEX0dMCclq0lQCorkJvHxzHLBqSVacbiJIbkBSGxr
-t9nIrsnqbdjBPN02UMuKY2GPst8J1yR6bRqEUPh1JQNp9G7MgMtEDiVFjtXx7yM3zqmbnyucFJ5V
-RlsL9cbj0rSmB4XvrT8BbOz7fSx4RjUY44JDnhbY4Ubw0Y9joc3vNkLeR8lZT+/LIkRbCOxIwwNH
-QMVE2YnsUzcjPhlEuC8jCn0GSxPDfgadWtHB5U/1VRnX1huk1qVwEUzVGxxExPSmM/19zWYh5n5I
-ivyAJhTcd2lZDSghsg03kIsBpJtzbZL0TkkZpOjCoKPGAhgzEFcWQMhX6rbVBuHSsrICOqOWVsSO
-H1mu4po5xtpqJ/EkkMygkRggPciqFe4ahKPXrINmLG+LxPaCValTLEkm43GSy/BQHniSsZnrWqlu
-o8ChUbL2AnZUnP6IhldKlI9jklUu+x3XLFeyzWgEqeg6AopmiXrcSEX7bFGENS6jnEKUbQZr5CaL
-guHVLvoQdi7OpevaGNVXYKW4/1rZcKGUtmMYDBBSklQRlRwYyWZNJ2wkBu8pGULBcgCbFm9DNJVv
-Q5LwGymSgsf9NPP0ZuosgKkritDivYqVHDdWCrfGCyBSAY6ZXRaYuOJXx+cQao6RU9euGxANBEt8
-ZDX2iXPurasBK0ji6vTBbbEt7pmIMXdwCE5qmhtzgiqgxH/UjYwzIWQtWe6zvg1RVHlQuGSJo/zJ
-pBvX4kovsvg0dvlk/jzv/adUsV+RYhwP2FQ4nmXZC6aMP2Kd/+vxgAOp4wI1SjYJKTJAW+gfrSzI
-pRu0v/3l9HT788zxP8h73RIo6dr/9T//2Uu5lmlz8JUOSEP315dykGTYxfvJRs9Wd1NFZb4uB48+
-qBSU4N+/1PKufzn0wIm1OPosiQBOUvZvhx4x1/FUwaDZVHou936b/dlYbrH9+xdZvsnvL0ILlBAu
-jzVpu7/9PK0FNdru42RT2Wp66tkJMVS2o2vPKNqziCraLmejcVd//6r/7Ef766v+9qMRmcIQENE9
-bpnDfBiquNuX7SAP/81XgVjnOCYgPOELhzPur7+rYIgYxdsTnHHdOhvTy9q9WRJ//ftXMTnn/voR
-/ngZQhmcgz3Joe7Xlym6mAcvPgkU/OrQ+YxoyPsZ25IC3XXttuJS232+i2pFsm4Mxh2MOrwyeK5v
-//6NEAL52/fx211g4xqCpUchZwwkdDU6qtkra1mtFWozz85tSciamS+MUoeqtv/iQvoPv1I+BRej
-EvZQZXtMaX/9FNzZopIlZzvYY37cdlaGgj225X/xYf+H2++3V1l+F38RAgAilzGDiHjjhZgcnNol
-DhH2w65E0tv8/cf5exCGO89XFmlI11IW4Rvnt5+IeoUgiidQ+WiDrHn9yJOAB2mTylNcWvV7Hzmz
-eSzLQryj340b3f0f9s5lqW1kjeOvQs1elNS6L2aqxhaYIUAgIZmQjcoDjqz7/fo2U2c9T5EXOz/Z
-OAebxJmJWczieAeYbqnV3fr6+/4XVPLMKI2VWdgq2mWGCaA5EQjYIQYShGcK7NZFDT3sY5aGHIkk
-QnRMhgMT0l3NK+o7O9WzB8JOyLKmEKJCrVSsHR5P0DQuNUt2KiGQ89HxBD+RfF/5bf8ofbUXFCcN
-3WScwEVuPxBqgJTvLbbeTBMsL0uNT+EB6N/ZL549du5l3JwEQa2OevZ4FU8eu0ctrYd5AYywQU9w
-uZS1U58881kHCeLV/ht6viGOUpgqS1k2ZQ7jYyrqSVccqtiQfT90AHp790NYx7c6ApGneQDjpLRS
-CeU+ioL7Ox2fxe4ubJoky1SwMqTgdjrVux5OK7kGqla1fx3j04H/eZdMQbMK4LqBSx6nddUzuKnu
-fH/Xzx+gqZgWaARdCA7zu9OkG8pMghDK7mUYnWPUIrwI0YdwfqAXKGpQeHh6HDC3RxXxGeIseIyO
-KRqMvlkAp8p4mNzfy/OtmFemzZSHtYZbE8Kl292kJs5XnFoxJkqJZJ28TT2TGMqsqkkdCSxs1NRX
-L/olRbZpWcgJKxGQJMW8IKSoY2VZ/p0rGl+fuw+W21bJXbIrqtbOBTUI2+Q5mBBULXIN0e58uEl0
-yGNBkRmoNdWN/Z133vPpC6NPthXkVYWs2fbOpkVZRZMaOAtj/h5ZuwqNLseUUgtUqMn5PMisC8Ce
-6NHsH/nnC5RuSR+b9GroiryzQCtJV2UFzRPHI8sEwywYqCbWiT4hX4vM+/7OVm/UnVEVbAdCjHuB
-TMy3/ZhtzOAQ8swDJzVHgRsMCYBbltLbXJdNpwFmAivCV5CyLlPRXSryYF8x81P8qTnDzqqiRkMB
-9bzZ6rL+X3V4VnUwxm3qyTNz5tX8aEGgU/VX83jx80/TxbzYLTo8/tNj0UE1j8kOCMsSvKU0KIRE
-M49MWE051pAultfFCMMaebdJWqzUiMUxe9VYARgXum3KTP9NzcE8tnRqFBQJVFszdLbSf1JzUOHN
-bi9dm1hGh6XLzDANWTV2VpLW1U1V+Ch5GVWDv6OJYRVIpSEvH/om1f0Jp5/lDPIjcHScdLo/VvIB
-mjDCeUOFtJgUSgu2Rkde4YNa+/W8D+rSdYa0RA2NYm//4GGA1+JHZDSRQ6hvAN0YxTk9Be38CTwJ
-7VPFln3TkySMXnWoRKBZgveCcDBbdd9hkTy0qOxKYEJUEjtYLhiQ65eDAIlaV2j4Tf2+xYR66afi
-SnH96M4l1V4YhgXPR6tHWmvbYtTZ4oMCfXXom3eNYUr6iaL14fUQtIQ0Mqe/8yEgPc/RKko40vaq
-ajqcM9PzQilHbFbW+h+7NohzRzXi6FKSDVgNIhrIA8K7K/Jp3cgVboRdhK2SXgE9QeawxpiuKwVa
-TZ1bvZGXpjQXeY49cUPxuHAYugyR1LK8zrqMk6/ZYGQ2I+fmhQ6ZXu8SN3e1n2SljeSskTf1K0V1
-I/1UDuPqtvUslGZbtw2hxifgQ2AqIJVVKjI5u9JExPY8RuYJawnFDz4NxLPtNNN1MDoGci3nKJZZ
-9gysSnCL0o55tWyQaKVkbMVzgGzIY/ZsdDmWq25713o++SJerm545htx8EHgwIdRWWXm7qnH8dGd
-LhV3eZ83GeBvRVrCqE3IGFT5iVqby2amlVqOqBcZbnVOEiH6QCXYhqCpdRGKq36OY04AhByaplAr
-VZ0aJLLu6noQV61HfD9p8H9IQPeNvMnQHAbzFdlSV79w9bY2mqlptDHlJX8owrO8hLmST0AwlUj/
-2OTsyMOH5RR93ywA7Qa58JREM9COVKplfQaYtfw9rAw3PdHBS5wYnV97J5qSmZoTKTYCIWoSF/pU
-WIg2oeaAK4ej5gaW5djERf11QOEcYQ9fqWDzaUllkaIR4k4Nsx5jIRA/4AFa0GlXQG4KHFwTL7BI
-P0otKwAKMfZpdgyPzzJd1FiA44qzrGo77VwJMPW4Ntw4am9ZXOl7EpnUcjJJjtKrxquQ+h5ASk7J
-uiBbZrbyjVRKBvAM4SozUu0wDZeNXvczaASF8j7xzQGPlSU+xZNMboCLBEXd3uRCUz+iTyX7DuWM
-wAZUZ3XRh2KAPzHDeqOmuAFdGkmJQIaeB3vZ+oggGJUPkMFZMEtlPODxLUFi0sSLIfuAoml96XmR
-kEk5xf1NL1uqRAUcYuUUC7j4FSm7GoByK5SYkS1JzpVSH7wF21Hc5oYAbATU5c4TKlq4btOAOVY1
-5hCIxbB878VYoU3UMlfuFEB0Av5H3l+wcQGuhNyktDh2udE98w82jR816scAD4EPhaC/k64xk3dS
-Sm0CVaYWH8bK7LtZSeqsRNRmiN+l4EjIojZ2dEn8ZOgnYN+ki6JHbgtVwKZ+30AbhXra5dkAmSLV
-L8mq4ZoUWK0RYn0uq/INpX6kjOpBp5ggFUuszcPcLKgLWTwNqGul+zuKILCF0tyrQP4ascvskdv8
-k59lcCaNXMdDJQYXqDDfwzo4VSQFf3ZfavLf287KsdqEAj3uK0R4QApAUA0KNH4qv5i+T7pOAdyk
-SUJ6DcAYiueSo8utlRjIq8iy0v5GTUsjmSZnQEM84IWOHqcNuH299Mg0xpr8viTHhqq48GSZ0l2d
-vc7iTMPAqFC09MxNvPDGVkwZtju7/3AZlm171+CmguWNflcoqgeSuouhuEnLZVXOsiRpHbhGCjPJ
-ylMIX4XkoQMUocQGl3gwoik8bNJ2gQ8t9Qy5WyyrVK3q2jPUuNTXiDrCMulYCDc+oRD28BzAXsdF
-X8yX5K87XgqpVyIbZUlvqTYxqxJdDc9NfBwCwiDzMuTMekaSPZBemb1o02nRd/Vb1+bFd4HDmv0p
-icDTTkhs+LcBXlOJA/YlQBA8LCOoE0wr79TrchiWeuOC8StwQEdqLGuRggFbRXUBYZ76zYiBC08b
-beS8JCQ8ScEPJnWKLi5REVj2keY6aGphhMIrmroGaG2oO2WDn6FUuyjeuH7JOSxZIr8Q4X5G46Hc
-n3Qi1+FCuvnyPqvQd3RaAbBmMtQ1fBcLkFMI9oW67tQK2TemwGOpQP/zeO/fInzyGKSOgdjJKg67
-qRdF/2ZR1lH1Rf9j/Osqr3mb/tiXNsIiX2/oMQK87TMiwPu0htDPFXh+mjxFn4zYji24yuqKVpe7
-r4FoTnRZP9CypMjH6uoj01RErWHzB1095uzDh3ht9Vl39WRsvnX3+29sPYz7v7N17XMkKhPHL4kP
-twE7AscLzv5/5/532nhy/wBvMPy12JUECJvxsz0MmnrMIdhUCV3Xn3Wo/i8aBhJF9t+cBt8eBsU+
-thUgdvKYvR4/BPBPZwPDYCN3xHfU9d//dcPAbBhz0ofNBlU+Jt1B8p559fT2deWYQxSSyDi6rD7/
-YDH8janyZVOZonXzsNpO/EX5tV3nW1/YrKfnf39cS789/PzTk0Pc6nvj5rLuerHa5saff9maIysF
-qid/XP2MWc3Tf3+8v+c9f/WaNr888xfFvLhf9qu77R+vcn3g/fW+WDzd5XDK2fy43g+3rvHJM9/b
-aDT30nm5aWgcD5KPPOf/3d7PP/1Qw/F8SJOdliG6H97yZL7cVsBaJ+EOveDTxQNjHx19bU+1lfGV
-cmgPJ2X2+a/Cr9Kjt3PQ4psG12OuaS/Qwyz1P/+5/TCFsFj/h1765QjxXH7+z9ZFoyrzEhd9OWdE
-oFRiZXT0wNjU0eZ6x5Eh5Tf6Sx1+A1862TS2bp3X+OYXP76KQMBup6KEroxp0UOvekTWfv7rD9Lt
-65ZWl0z68wXW5/WiSObxH/X99iMFh/sCo/3G51Eujs7nCCYW2x2so5NDB2bsYMaUpBOmzBWZu62t
-cXzrkR5+2V52J+b6zXpoH+NWMD+aEjYXfrL9oKkyvMCe8JZVe3Q9x1lqMyCrWWRbgmDm4KtfFJ6f
-bY090cCY5zy05dv0npEBa7lparxqFUO3F9jNfo3n2fZ6HaPFF1ivlzzC8mjGe8Tfvu51MHromFz7
-8/rzX1sDQsPq5hc/vn+9+bbl35cQ6MfCgDfpXsnKA1vfyzw4sO199YW9TX8t8vtlK0Q8Gf9/O5T9
-7heISMeG7yPKHr/8FwAA//8=</cx:binary>
+                <cx:binary>3HzXctxKtuWvKPQ80AGQBpkdffohgbJkkaKR4wuCEil4k/DA79xPmR+bBerodLFYzRreiHmYS5ky
+MDu337n2Bv/5Y/jHj/Txvno3ZGle/+PH8Of7sGnKf/zxR/0jfMzu6w9Z9KMq6uJn8+FHkf1R/PwZ
+/Xj846G676M8+MM2LfrHj/C+ah6H9//6J+4WPBbnxY/7Jiryq/axGq8f6zZt6leOHT307kfR5s18
+eYA7/fleVfdTlL5/d/+QRbkX1U0V/WisP99f37x/95g3UTPejuXjn++fHX//7o/Dm79YyLsUa23a
+B1xrEPODSSSzpXj/Li3y4Pf3zPpgW1wSHDSffuzfRC/uM1x4HRXvVtV9/vD47qF4d9Ninf95TU8r
+un94qB7rGuw8vR69xTNWfnH6Uij1LJSoLtxf4nKLmRF1/cT5H8/V8a9/HnwBWRx8s6exQ8GdOvR/
+q7Cbj68J540Ks8kHRojkUohfirGeK47yD9wWggtT/vqBYn9p5pfibv73fxXvPt63afH7+2NWdFxj
++9ceqGrm8X+Aqq63r0nlraqyP0hzVpNl/6WLA1WRD5bkDpH2L02a5Dfxf/sY/Gt7nz9G1X9DXbOP
+7l9/oLKZ1/8BKrtxf0vtmCG/VWXOByaloKaFl6efA5WJD4xawjYZ+aWzA5Xd3OfN/Tv3vrmvovz+
+tYX9Bw87uP5AZTOv/wNUtlu9Jpk3qsySH6QlOFRGjwdE8kESxnHOcZXtoKj63eqxuo/q15Z1XGHP
+rz5Q18zn/1/qesqt+4n82fLfWlxY5gfy9GOienhWXZAPv2Kew3/p7KC6QOlzYiXHtfH7umerfqqk
+/h8WDf+5oPi78vIQEBZPJdteTfH60ScGUVkeXPpKlfXXoc3Dn+9txoWzp635Js+qgI+PVX6ffW9/
+/J1W9i57vK8blIa2/EAopZakjiSOaVm4Y//4dIhaUCxcyhGOY0nH5vz9u7yomvDP9+bsjYQiiFrE
+dCTevn9XF+18yJAfqLC5LZ0ntUsHl/1m82ORjkGR/y2Tvz6/y9vsYxHlTf3ne8bevyt/nTYvloGs
+bTqEUWLZJueWg0WUP+6vUaTjbOt/TUE15iy0rs6Wd5fBQm1WarO8XG7UcrlbXuNno1Z4pxaLRaDc
+7Xr7c126vfrprdfrn726ujnbk+CR9VgzvdfWA3ntr4eaXefHWI/31btdrtTCXay910kwpJdXSaC4
+2yeRFMZArAgkduud+rr0lp1SG/VttVTXaqkUaHpr1/POXO9seeWqxZl3YgU21PfqCuTzFWRxVVMz
+tq52y8u7zfJ2Cfm69+56696coGSRE/IU5nNStV06fgdmd9DwGbib9Tr/wevl3XK39i53arO72y3v
+dpdaecvd7u4OK1Lnq4263lyvNqvVarFanauLxdrdumdrWMK383N37Sp1rtyLNVbtrSGwtedenbnK
+VevF9so9O/NcmMv6ddWdsg6Bun1fdU1dpXYD61h6V1+/XwbqUi2+XbimOiU2OWvgFTMUiK37hJLO
+cboCGjrzdp7n7S7hEjt4xZNBqqVWl9DZd3iFgsB28xGcCIdZXit8tcHB2Y5gT3AndaFwCO9mY95s
+Vhd4Xd9Alt7WvdpBbvC33XLWvue5F+5yuVngRHzebl13tsHlDjZyuZwFGqo1NIZroK+lB42c4URI
+/+vuclbCpYdrXhf5SQOavWkvQIjALwwHkgBJ8IjVqdXO2zyJQoEFrAp/3RMKINYpBcwutEd2csZ+
+7GdNf4U4dzdrdxYC3niXnnu22exgdHcw3A3+eXDhzWqx0Apvl2uIdOetl3dq6X1drpbLO29zeQl1
+IKZdXgdKfUGEW0KK0NNiC4f4qq7drXqyps1qc7m5ftwE6vF6vun328u7SN1O6nugNjC3zfX15TU+
+Pj4iUi4VnODiBk6L16v1zeJm/ROKXa9v1O31ZjMoFagVvObL+cXFl4vtevFps10/3Fy5i5V75Xo7
+d7G48dT9+axB2NkNvEUttttzBIHtGuL2EHeeAhE4/4mAtPPgXeu1C/Y2sJgzd724gCU8nfj5Bl/P
+/nnjnV19/ep5N+7DCTuYA8VrHjEnkj2F1LouQ2dWCELIVwgChuCeuzBUd32GtbruqUzA5lD/GsWD
+1JQ1gsTZTPFyA/N3f643kYJCZ0OHx12CSfgVPsJd8J/aQvPzR+9yeevdbq533tcCSl+pr2ffZ//B
+gi9XanX7sZsjPNz0Gkbj3izgZYtSLS7uY7WFnW09z1beFSLhnVSfFhezX3tq7S2QCtR2jgYnPMya
+g9ZrfB6kPN9qdDyBz513d7uZXf/mddVRc3aW1ygcZDzkfcuwQOEMhnOJgDPngbNZduByDkAwLRgS
+7AueA0M7g6hg3ghb+Ah54NgaNrnzFlu8xdnLDcS/xlHkD7yHJ7jwKQ/5GrfE7edTlgWu39xCeQgW
+8L2ngDhT3CzdO5yCJSgXWphPx4eFmt1pDbo4F3f8uLrE7eECuBVcebNZzNF2t/vqIV9tbhUEhWuQ
+jGYLROTE4nA97jffzD3HG4SIHVYEV0RVA71+XmznUxfbDfR/8RS1wPV6VYB5qFYtF2vY8xzn5xiO
+ta1w5bV7j7vC6dztxezas5ggqPlqGEaGiAN1ufj6dZU9N31OgRmaNjexf+Yo/yQ7yNoRtfxJyjFU
+AR+Ci2DqfLfts+7MCFm3MLkRueMwhIvXiT63kr+ISovZhNqU285BpI9F0bC+GEJV+XZylZRTupjE
+KE6w9rzg/E1FAC8lBJzRAypE6sA0U7AWit7qVSYNI1fTyFrXZHlxgtgRlixKmDMLkwBGOqgXGPd9
+Z9JmqKwx6l0/z/xVwVm2fF1wR1h6RuWgWKiKwjagw1B1oQ+O+lJcW0YRL8Kh8YEf/Q02f/zls/v1
++jGGpMMsZlKgK45zQKptrZBXfhopx5Fs1QOEUbqdnFMMmS8NkNjUws7F5oRJix5E+ymVpkWo1Shb
+8yzw7NBJelXak/ElFUH+2YgKpt0woIGxlCbrdo3d2Y2ntW86qm7S8bOwrWRw+8SIw81IWnY/6naw
+Fo0f2UQNfcszFeS8axalE/JABcLQw2qYhj72osZijUpLM86uwoHauevko2+5FABGroRhFtpLJSSs
+zDJpB7cWYpxUa9ltpkSasJ9T0bf5IiurbD1ag9kvKp40WrW+ptZKpnb9uZdMhFvb7misAgrbG9qp
+fyhELiu3D/1wVPmUNUQ1Q9amqjeaylI2p86oGrPOL02jHT6TmmTFLjSmMXWnsGdShbyH9xAWjv2y
+FlFPVUPtpFCCB0GtOGdj6FGZ68ozKmY2qoommroRGbNPvqkdX2U0FLlbcGpXi4n7Ua8co0qrhW1o
++bULU/2tqJym8+JBF5PyI5JEbuQkpVyYoaS7ITF6242bUluqCYlVLpJEhKFH0kQ+TGZrjqooC5a7
+uSWGTI1DW1drbmaZqXx/ypKdDmlTuY4xdmzp6Cq+SrvCMlRVmPwn56X1M4s1sxSK41HuLAEMcDG2
+dmR4hizlRZNYmqzTIpKRKhnhxaKNy+oyLYNeKJpk9D63g/Kmduz0m6N1+r3KmRg9pxJd6+mKxrHq
+uBnvRoumfEHDJqg/dVkRBkue02FwGzEkvRsPTP/Mm67Lwans4do2zaNFWU7TTZV0A3cbY15BnhTh
+edwP1FBhO5HOq2wd3iVCJhdWXmS9NxUJzT0zsCCWCPZrLOpxbKwlkX36rW07e3TjUNa7TphFqwKd
+JakiJZWeb6TC47pug4VMiUzXWdklX+Rgs8jLoK7JrQrRmG6aFXmsIhoxraAqeZPVRVktRzFV+aLS
+URS4PQz+kRIudlkc2L0aczGMKkm0kblp3zTJug6T4ZtuusZSQBmy89EoR8NjTDs/aVIGVMEUmvyC
+skDam6Tu29T1rbS7Gk1L/kitvglVO0V9o0TUZNcGK6vkduhgIwtkEOPTMIpKlUPRaa+ahHGlA5rn
+C4PQdpuwPMuXwhBlryRrmsHV8KJRcVPHn4tIS+GRerThi2acpq7RcX9H7IxlKs2CMXZL304TNRrG
+xFRIaSEWVSUgLauJ6ysuiGgVGdr8yhSR0ylu5V24rmqnrs5b0rBsERtZYXr+YJFwWTVk7FXXlNJU
+RuHUgzvZsrzxRSa/xGZk/7B8S0xebTJ9U+dVm19UfZ+UqtJ9nrqmPdjrxvdzvtCJbKtlRI3046ST
+3FQmyRO9FkNk3+nCF4k36mwIL4Z8ys8rRzrw+641r/PJQKiVdRvXivKMfWr6UEukrLTtVD84+afa
+tALiJZqO0VrHxliqSORV6hVtlFG3R0yZlEGS9KIpiqr3yiFstVcPNGrc3kntTCWDjqSb5lXwLTF7
+/a31rWzyzLzKw0UQjD1TfV4EiWuMIvwudTkMqqRVm3lFGPm3bZFSVWcZNDGVk1Mq3yonfCN6HnoB
+SapETbFjjS48KqiXvMyDbQjF/7RLvznzjZFHiprTcFuWJn8Y6tb/zCxfNptg5NJRREfBrexIdBcW
+pv5cOT0rFAlG40HzoLs3EpqOyOgmuaE6rbTKKxn90CmsVeUkMD6ZcMn7MMnDcMGqxN6lSWV1qrb8
+rFB+V4pSMR4Vn5xBhMzTgtaVW/Mg2jZR3H7zEads1QZ99jmsSH/bZO2YecPUlNehk5OrPo11pjhN
+qb3QsR9edF1rTG6PDMLUkFWiWvI01OtBT2G9DP2qqxYQgCyXJUDx0O209D/Vo+GPCytOxCNNWXZT
+RtxKVVr7LIbJ+0GyinTZrytjDNo1/AdJK2qpfxHJ0n6cyrxuXUH8YV0EVBqqb+HlmyRI2CfDlIIt
+G2byZRyWNN86tkkz1UmLfMkDyAhy1+1FEBdcb3zTH29FnuezNAs6ujTjcaQCWcYcgqLCXNilQdku
+TcuzMSH6ax12doWcMRQM0b2OBpfFSUUUTesudgOh/TNiOUxvjS4rG2Q0c6DKig26YSTQxCO2PQnP
+4syiq0l2Q+JmJi9CzxAscJZ8iPlnx7IdoH5DSvyLpM3ysxIx01SRbivfs9uovW86Rr/WVh93Ki5Z
+XClm8+S+r7IKVhJa4ZfaxNLcyMzC1dQVLFLdpOsHI5pSrXg1+L3XxXmLQJOUTe92ZdZMrqSjnSiz
+bcFfXwfwH90YULw2nOAHAg+zN2ZijousLYtQmXloJsqPpfE96HwYlzmUpuUGXZ1eU2ZNRCUc5uZG
+Y0p9b8wQaVxzcqLBK2jeFl5PUytBqIj9ZOk7UXtthBI5ujeMLFR5NHG5siwdDSjJS5YuwiCpgmWR
+1Gm+DSIDYcHgYMGbaju8deqxyVVZ1PKnIenQnuNW4W0s/MF2ncYo2l0so/CyokaWoQKuWK7y0S6a
+VZCJMPWmjFXDIgtlAZ1PWWBALB1qPqDCpq2cvpqczdhlOYfD19xe18yu6+sgr8Sl1Yy8VnEapOeD
+tIpI2YbV3YxD3PhLuyitTz4MyVr2fVwOavC/yCLuiTJyAiYrO09+OGXmEG8opvDTGETZp6KbksuR
+luQqIlO5gsF2KxmOhvDSIkR+SCbyWNqzyhtT21fCQMWvUosYgxvYfnST113Sup2MuIn6G6ZS+pFI
+vdEK/bu4rLtpySsj3jrj2DVuU+RNusho23OVldySbkx0w1RmEl+7eVw2iZf0pii9PBpRKY1hFjAl
+Eqf6WjkJcuYUE5iZA+ezXMcS7KJlaTQsphqWp1B9kG/+WOoL3jL/chgLWF2dzbo3bbHr6rF/LErR
+344izYVbGl1gqjHJ/doNYPXnsajSO9qayUObmCTwDO4XH01ejVxx7VfwEFPWI3J6G3UnMIIXZT+k
+Jm0OjN4UlmnbBxv4TLd5nYXOVxklo6cJiqGBJ8kJIi+2MTMRil46AylsmA7xFhJRHgtkH6RAuSCa
+sC1prSlwaRUhWT9tZP7q4/y1k/nVifhRlGMVBeFf0zx/f/zX7veI0NM8yb+/n+eB/v3psnusmrZ6
+fLe7L+t3yzZ/eJoSOrxmpvz3RSD810rmrs2zDy9aSL+7JwdNol8DSP/h4LMO0rNG2e/u59xdIdid
+/b25e9E++t1n+9Up/H3+776R+CCow7GlQVvGZJQDH/2rb+SgF4s2rE2x/7MAD8yH/uobsQ82lwyI
+gcBABDZoHNu6330jQj5g32hZpulwaVI0kN7UN3qOKMH1sHkHferYxBJUHmysiRHksY3ekdKsSQn2
+P01Trdo2p8U2mFjcnNqQviBHKUEzDFMD2HUi3eD4HvhYGo7fJg0dlJXUI3sY0sSaUpX7kUFvkG+r
+6ceeJk5usxnYo9hhOwIcMkHZLMd9emaUJ9WY6kFpw8yvG4fwWx3xePUWKpwICA77YLTwbO44pjN7
+/R5X3TTJwIRnK2EbnTc2Zec6hDaL16nMbvtv8O8vKgRdPsxcSPtF7Cj8uvQFyWrl57Fc+K3BVJUP
+6V0wTNqLEmlcvE7vIFaBK2bCykyBYQJBYYnPuUqtyWFywLairSRdRqIflmHaWb/ix6/Rs5Mamrli
+JoAdxxEo0WxmHkREqxVRXJl+pWIa2l/MSGebphwm73VeXsoOVCRjDqwddiDmLsWehiqdmmHjyEoN
+CQ0dN5QDtoJJxVirCjkWtbJ0H96+TvMgDM+cWSZjtjAFHNae2/77NGVOdJl1Y6UKndtb09AMWSqJ
+d2Yr+An2jpBCiIFDAYybO8EHQrTLzCyyNgGptCtRkebTsoza0q3jLD0BXB2RJLA/4EkOxIje9YEk
+WclzYeRZpbqojjdtFPM1R5w4pwWRl31VOOvXpXjECvfpOQcI6tgUU8E70KtyayrXmeWXxiLueHSC
+zjERMtuaYVOwh4nC59ryMzGNMximZKrDzo3jKR69JmqnOxJ0+gSxY0JkDheYiAOaycR8fM8cpa64
+qONRqwCVsdd2lX0Rcu67jAJH4YOgb6sIZlPkTBAHYLCDt/zAlTva+qKJbK2stKWKydheAClxVBBN
+wQl/PiZHblLiwJstjCUcJBTLYCwxBlOrsTJTr7FTflHHk61kFlQnHGwO3s8DIljZI3XgYB12x1Vt
+gSs2FZdh6AQrgZIHuxxCz3uaYHcr2q9vt8Z9ki8EGRlDD3hMWaGZoZ7y2RKzysEJdz5m89yiXHBU
+cmgeHNhiLcuwmowQgE4k249JUcauIXJy+d/gBcYOZ+aUOYcTBT7zqQ6lo1VRZxEgnIIvo67gJ3Lj
+MVMHCERR/WA4RsoD/62kE1WR5loZlSTcBXCUbFOe+T+zsg5vJeJVc8K5jlogZn4Bo+GOlB5QjI0w
+rSJONEBbh6/Srv3GKP1ua9tZvF2AjklNe85cwnbmhex5MUenIOiB4KnQNxy3z2rhYe/ZnHCog7bi
+nCHR1pMUnRbO50RyEHFDQ0RtyvJKaQI4oM5J77IpjIGUlsEq7wuiSs5Wvp8kK8Ka3lC6y1s1mTQ8
+EUVemiWH63BsW5j1VI4851dGGYZ6OmQZC7s7fpXXNKw3IWmz+oQGrdmNnns2KHHUOjYRjFmHpcdQ
+ByK0hqJSYRQmWzO1u6XWJbktumoXcGPYVnVZLKqksBQBfXcYk9CFDhqrkZt2NPSJUuhlpJFIrvBI
+7Mspxl0P3L4fUR8Z3aBVaQpss/tAZlzZTQ+gsDcDGxBh1fHrum2y4YT2X8oclG00RISQ5GV5NNoE
+nQsLmWIghQAeHSfuRNr8hGaP8rdH5cDExq6UU6ARtDGp0XltkNpur31jldFAjfIbsAX95hAHvqBg
+CI47likPYrdw+pygotSKALh2DTlQt6PAWl730JfBB1Q4erCCEwvbr4M8mxe2n9QOWkZJIPl1IUa9
+IEkdr8w2jb83UTUtX6d3TI4w2XmOk8FPDiOCnxR4iIUhI/G4p6XXaWGc2b4ZuEJk9c7uRtl4Q4Aq
+8ASfp+ge8MnbYNC6oBqIfV6dxX1RbEo0S3Zxa1RnrWDUNZPYOhH+jgl3rjbRkEUBj+7s83AwlCID
+RJxDuJHFvjZopbULW3bxqs+lWaowN5ovr4t3vuPzsCDnnS8h2AIhLR7Wgi0J+pzVgVadX+fo3KAB
+RzJAlUY+vL3sRCmNCgZdU9PkjB14REKnKek5LdWITszCTKZ2OTTs7cU0GucWChIUghijpwd6y8e6
+KKiNFoPhlP2KJICTk9i5MnXCVFqZJ6zzSCx5Rm22or181Qc2rweOaGVGKdqwBB1H7vp2NY0nLGOu
+Tw705Dho1s/WQYFfHNQv8OMoDcOpVGln1ttQGNmqyDNzW2RMoE/Mu9sBcGyiMkyG9W93BTykBVgE
+9TU25OSASScZxJQ0yP6T0cibFODyJYC41gW2qTdFxadYlaHPTnB8xDLnB1eQIWyHw24OEgT2JLwh
+Vo9S1PJbVaKZqEorDlVkdsbbYzXGiZ+qa45tytMg8J4WRVmPNQ1KFFRh0Z3xVrebDH22bUTl3Bxz
+0ChM0dM8IdYjKgXEAdwBhYhg9tMk7B7VKtT2hOcGEa9bbgcqjSLh9VFRb1lB2ouBFrHKhaxdHXXR
+CdIvzHZOupwS26I2UsbTeNkeaeb3eak1IkoQo71kmzlZAovpdm+MLaAC9AFDOkBmUakeVI2VP5Cq
+n2CzE8YWCoUG4eRhi5uuSenk56/TOsYRogvKTwHwWloHtBI695LLplSJzIcSgx/GdNcZduqcMJUX
+VjnzRAmByoAM8MMgFk0xUHCzRU/OAtxclyM9M9M222gMDJyILcdIYSyemoTPidY5iJdN7+dFkWUg
+pTEiAdjD8Mpp/IYm43iiODwmPNRCcAEMz8xT98+jmEZnJRrsEj1hakaLykCtG6KHe8Khj1CZ0wxS
+I4RnYrD/OZU6cEKJzj5CGJsGZfI6VLrIxNsVhIJ6xvNAQ9iH6OtoBaUd136hetahuESgWhSDiK98
+HUzfXre5IwrCgwjgBxkHWPTTMP2eFzl2pkMjQCud6tZfNklTuwlBYxGQyImBz2Oi26c0H9+jlBej
+9qcxLpXk3WeBvu4it/3yhL3NmfFZipEoOrCjRPxD3AWW/JyI1Qw6w0hLoSxemOcagzQ3GemLjQwY
+nVTRD8PqdflZ9jGKlm1LPAdigeqBhU86jdNegyINJASordAb8jxxfdnZqQqZH67zoQsWY8TkKkcP
+7acxGtua5eUyJH1y/fpyjgkZiuQMUDoeqSQH/Ad5mrXCh+U4sps8ozTiBSCCx7cTcRi3qQPw6OWI
+H9f9FNUlBgSGqLIxqtjHvMFshiz5CT84pk1HYt6V2BLxQ87Gu2cyPsUEBxlhnHmcD5jWIVyZvbG0
+WLfO0So+Qe2Y7ARmZaVw5i7ZYYnQDjUfsq4oldMw/yzpRr0pEUW9twtPAPDA5B3yFj8Etp3UqcgY
+ICLGdVadF22YLQZGohNw7BFeIDZsohARoahDySV5YSRoQc91qhNepL2krhWx8K1QERpNJhAIhA3s
+bcTTswV7+hFTZzTGbPtJRLJdNg62V/q5OBFzXyIdMxk0opiDXgp2bjOze2QyPhXMzJxCxa0fnWM+
+hiwtnW6LeSaPm92F6Nl1aZj+QoeOfwa8e8tlWZ7IL3OBeBBZ4N8WQZsAaIs4LAQwZdrKJkhRCPDO
+xqDjENb5Rzowsztnbd8Td+hlGm2qTtqnYNojboDdAJp+NgFc+6K0M4qQmW0mCzVmMUnc0OSj15fR
+OaEBddvax/9vtlEkHxsYNJ6ih9APYlprO0M2mYgiNAwj1dekWjrZdMoTXqYeCyoFQgYLenr29Lla
+gTkHQ+VArTzEqFwqnGIz5hh9oL48Nfr8UoIgJQjKROw/MH4zH9+zIMRKblYMEiwShnHGsUi1UCaG
+8j/JmrCHsM96/4SfzzJ6bi+AqmzM9mHIFrO2aMc+Ixkmmg2YvylUmWcGxkI1+6zbfvquWyf1LCu3
+vwMGGc7KkBTrrLLru9dV+NJcLQIABeO96HJaiGrPyWe5NoOubzFDm1aBl3LnIa2cO4z8caVlnqmW
+nqoqX4acmSI2reimAWWdn2ncl3HdR3FkW7pQuWFj06rbdg1XyU8EgxcbDgwrY3weGQ72idxzUObZ
+cUMYLZpCVbGBSUyRR9FXPY0Z9arSpx910k2RwlQsMCMnTTGu8bpYj9gsBrlQzqIGBHp02KiuptJJ
+cjw6pozU10sWJGPjSt8Kb4u6IvEJYkcCH1ol2Co7QP3n6HfALLExd9c3Jhyf1x8RF5NbjOwlXker
+1PJoHbKbBIM9PQZ9+rpZ2j6m4ZVR1/pTWNG8PLHfOiJ59GMxDIDfmoGZ28Ndg53il69Mukew1yHc
+tWub7z1HPZ+bg1Tp6Ce7Wny2dBC+OZVBCGijAznDYADjB3ZlZjJluoQls5GmhdsEPplWsrOi+oS4
+j+kWGy8MOxBsJ1/MxGd5HvsYcShUgOnIT90YE2cxWtI/ayLaOifqxmPEJGArIJDSxL+DEIvBcTs0
+GgyPT0DWt6VVtBd97hhex4v+9nWbPRL8MOwDMmgoOmj2keeOafmUjU4OvpzY8R/ixho/icbpVkme
+pms0NMMvr9M7whoweoy3MCACGGc62Mam1IgwwFkgrheO8IwQDcyqCtBRxzVvV5lAyxkpEawBLT6w
+jYhnZVA3caHkSKtAYRSv9dH2y8nGsnNgga8zdiSmCtRUdI5yeNT7qT2xl0XiIedp0OJxFivLYtcv
+wjpWeKyhR7EvavuhGavOXGnkmhM7p2N0ATeCJCY5MUxyYCtt01upTRzQ7TGGqoY2ohf2iEZjlUfh
+p76gxbnoQuNEcXdEjRhQQAngoPjCm/n4Hred09GsMQKEugYogZ/Dy8tEF67j1PxEaDlioQJxjs2P
+wxOMyx5Y6ET61un6eVS4niY3bSd7NfJOrDF/Gnt9HhgngJZjrGFbPbdP5mewxAFruncCPQiZo8VJ
++cY2JtvDoGFxPYkoPWGhswUelAECVRR6DXhiB7I8yMOUa7sJRj9XZhClF7QCfBRTFi5ft8yjVJB3
+mc3QDZRPiWRPV2ZWJhlniCY6TvUCT+mIs9AI+zdjYRaajkAkBEBcZjvzVniPSh2i9cbHElRSNjgu
+JtvScU1j9NW8kQlTnwiRx6wCCNW8j0FRQQ8f7jLNiVdthLhlNM1N10xXWaF7hcHuTDk61icUdYza
+/JuIMEIFmBj7uufMYcA75qSEc1ejDrZ5VJFlnQTOxhyG8mzC0OcJ7o6oDBEZSLTEb4BA6/QgSiaO
+XfYDps9U35Ul+rKhaXdeUFj+qSriiLGDxAyMAaOlppwXsqe1oaTW/+HsynrjxrnlLyKgXeKrpO72
+Gi9xHDsvhLOJpBZKIilR/PW3enAf4rYRI99DgAFmJmxJ5OE5darqcCNwjt2y5H3dgztQ560qRCkE
+mz//fSO+8xbxEtGaBEmBUrSnXy8GNYcbTFMMZUZ5OtT4OdOPYU5SVjICIBfIf8L/PTrixgZaipwE
+KfcbKZsqIOhw0VDKRbCqJU2dgJgMpDYlu4TNoEG7cK3//pjvvVMk1ekRgj7iTMfX8Mc75UaSsSdQ
+q+W6g8yMtbuuj5uyTaKPAPaPVjreDX+slI2ghYEVBLa5NWI5R6gGg3rY2mWsBIRh9oMHe+eqofmx
+MXrMTXCnnDxYb+ai4zocoCPw5gDZJrmFUI3WU6qnHXF0u8gnwb7+/W2+u2h2DCs4DqiWThade7qG
+ooiHUq94iQJUkC/9ln3h2TDvg2yK96vmyQdrvlOeHT2sEDEDVPXA3F+/V114pWU8DyUqpbBs+HBB
+R9d93RiX8DuM+29pH8x1SoL5PFpd/0GweZtLH7tCCKHIqEHwPT38QaJyF3diKG3uwjsbQQ7S8bl5
+IWyy19BpsZ1mk74mo/7g5juev9fX0XG74qQgjwagcHodDSahwgCfLFkE4hBaGs1OxjK6+/sHfRsF
+UHXmwCFBKwOOdnq/LvlghYg4ABtm+bfG84XXBmaSwz5hTn0zNm1e/r7i2xd6rHOPEs0Md2B6Gne4
+6QkPZmQQvRH9Wk5iSG+p9W1Tzmir7NN4SMt8aIKlZCOTH7EW3lv9vyw+TOEDhDz79WZaiApEmCAN
+DcYR+o6c4GACu1d8rSA2FGEpBuaPmjAIWs8AFoe//v70b4NEjDsEhHC0JWLICE4OUIaOBNJkBInI
+tfE5/ry0Y7IeIl4U+39eCRApkCG0cv4D2F8/KWqHiPoOt+TAaD7Ugy/WDeoV9PT32XLUv/59uben
+NMY+AmH2SHc76iRfL6claaUzGtdJ1E0/cYFAHiLbOmwZEDgzKAhqtul5XPPxILc4efz76m8PC1YH
+lA4qcpCHAMRer25slrVWY3Uwx+RlOGZBmcoh+ucjeVylQKMf3R5QTE8SAZyQAiztFRniSuiF3JJP
+S+HI+f/wKAUsr0DYRgFxyqvR4PoRsNLwIlc/3oKUziCKDYLlIy7YOycf4HYEqBLaSSTXJ1kU+qdp
+vw52KJsgSWs6gVNPw745B9/PXRSFIf+ckoIHFxybHfDYQnV0sp5uok1Nx09EiIx33VJ0n1LgXru+
+ccnt31/he3sRzEtIhY6AJXjpr3dDL0WAemvDnZ+v+jyQUwIJUtLX0bZ256Oeg4sJ/fa7dJbjM5xU
+xg+OwjsxBmkcXilQJxDiT7nBaQeJ2Bwg+WauIVE5AVG8TYouB47p8vkhiki6lGkipodENNv8wcO/
+vaKRYUErcWwbF0l2yphSxI9oKXfoq3kVPONjiAx6KxzGyvKm06A6tu19Q1z6PwQcLAx+AT4yws4p
+9m+E0FOzoAjYwklXBL/wfCk8fwpz236Qu54cd5w8CkZPmKMAQAxHZvf6A7OFDz00iaIOVp3WYdHp
+Q6gW+UEEPQX1/n+ZAvEsiHHoT2s1OOD1gYhjUUv0KAztbL00nuxUIEk1ZTr4hH7icNHG5JY55vYT
+up13zJp/3M5vfsZJcEvGYDVIbkUt5rkvXZrPBySG60HlPWTO1O9UFpsSpxnAG8iMu78fppMb67/V
+QfADYyUEkgoE5/W7npVQQuZW1EXT2It0yrZd0Nhlr8TyUZvhvc/651LHc/1nBu3jfEv7RdSWUrEz
+McT9kdPqg896Evj+eyB6BIaPbi4ofI7//o9VyMLblAvJayYgnr4IwIJlld7Gdj6PN0mDz/lo2D9m
+c8dFwaTHaYSYCVbGRzvDPxeNt2SaU0WbGvLz5joFvak+IlcfJKvvPFoOPC+CDAJ6nPw0VbYQizAC
+gKmmcBPoL23Yxe2Zifs8OoMuTEMDlI+I+H/fICcB579HQ+vyyNTC2ihGXj+aYjnjYkvguOACydAA
+Hq3wVe71Gs6Q0ueOwi+CL+uhsRO67X9f/M2WQT8fex9sBZDtEWtPruR5MXlC2JBU6WSas2BmW5WB
++PrBKicRPYHcEyRxpFFo08KS55TuYzsBAYuKoGEWW7NUW9ypGzk5uiOZO5pV4Lbuh3HYx5FvPgjn
+b44fli7QfAYfLkI7JTkJdVSqgLWyj6swUDy8jdJxmR6FMRGBpUCTa/NBN+q99XAucOcjlwNd/eQM
+cvigRIyMUbW1yVJ2KxTp0Bd2VWr9XP/9272zFLB7CggfBCecw5NHG6HoggEBDSuGqmPHpsHXDvcy
+Qto0f/ABTzKC4wcECwItdvzJYXZ8skdlm02hs7Bk2XSgLjkbxgOBnruKIGC/Nwt6/Gy1spK9i6/W
+OF0/+IhvzuVxebRGkNSBuYOd+vqIwJOIIgfmUYVNWhyINxGsK2YA0wGJkR+o4O7vb/btqYiRYeG1
+YvMgX/zP0u+PEDc2rmWSIazB9yM5a7th2U2Cmw9e6tunerVKdHL2WhpTMrUxgz47yOFvkKmqc2De
+hZzeLUucfhBn3lsO6OyRnA0hBZ7v9UtMB2CnAgY+NYJYMMg9LDc2wSuednFny2KAR8Gw20wnkv2/
+v80YSkDQYEGgBID1emEOqBEc/ohUcaGyZ96ijan0P9KB8JEgqwUpGogOOkA48a8X6dTWcbjgJ9WG
+x3mmgRrgLTSMHyBwbzcGBBBBBgQOlQxy8ZN3KGHp2qySyjqK0PVJC6F2RIjw/F9fGFY5YkRoiQKY
+OoWmtIpXPhZE1mMSITOD5HUvAv3RfngbPjKERJS4kGii45od//0fmxxQPdviqZA1WTZVch7geltD
+eeYYmvV/f6A3V9yR0YScKkbxArHQ6RU3q6PKVoi2niAV++HhvPGQps20n2Tqal0octEARP1gv7/3
+fGBCxOjfghYA6evr54MJUJo1E96iFHxCyxhUdh0NeelIuH5wkt9bCicK9wvqFeAiJ9si7fgiIP1C
+B8fH5mbkqq/UUoTPCQiG/3yYjuo9cJCAqB9hvZN9HvhJbKOFu8+4enWguvs9x9lH1IO33wv74Wig
+DojpuEdO4q2OQ0jUoWzFBsy3L1Z5X8M1iF9B96qvAz5213ARmj/qjb09XK9XPYkTLNsUJFtM1HG4
++LNlFOag9BKd/X0vvs1F0NQEgoZrExJ09Ddfb4vUbQKmVChKSGHFbd9aX265G6o+GaPLkEvWl2Jl
+8Rlcu9jL35d+7wFxiaGyjZADgWj9emnn9UiIc6iHsszVmY3aq9YEHyFJ764CUBvdfaC9kJG9XiWV
+FownBgevPFqWfTyqFhyy8CNc9+2WR02DQBgfLRrQizspqlQe9ENouKwD65k9qHXU0d7Lue3Ppj4y
+5oOQeNzWf6C5eAwsB0EKnBpQRaGafP1QSzMk0+QTWTM/JYemnfzdkIqulvMRq6J2oR9sk3eOAFA/
+UHCOuDnS45NvxU2SkCWHh1+RI9swJkTPKieqOEOhYvYLeOVXS651v/v7FnnntSIeg3SDVWFUdJwB
+8mdQNuSYfE2LrBtcPvt0kP6cCQtIV6GY/0g0/85LRfKfoSWHg4eq6uSl0iHYctpMstbGNAryM6R+
+FdgHRVaJjGp+1iZK9P8clgE0ZoCxcMHBj6I4iS1Jvq5aW5h9DWiGVsCW2EO2mvjMx2r58feX+c5J
+QOMKxxxAMdq5pwwqY3N0AfjS1+DR59USLmnVefrzf1kESDRwDkjBTsvhIBwb8PlMX4MAve74EAT1
+sFL/wQ36Zl8APsE1hr4fMJsj0fX1vnAo3tBclKqGtny66wC714Ge1wPfwuzr3x/oTYDEfodzKlIP
+nO8E9drrpeDSNh/J1VMtVRo/MDCz2LnwG0SutWJzQGvc3GvBq2Qdp/abXC2NP9giaKG++XSon0CV
+RIJ8ZIJATP/6R6CcayH6bKfdlgYtdODEx13U3S6d1zCOy/pE977MRA97zxL6SS27Mihg99VWIVp3
+bNpREYR9+Nn38cZfRAsuRnK+dsVIHmG0BoTiK9taOciznCya/Bx6SVhREREwAqPDdhlauQvWJmBx
+xbdhmYLaLGj3yoOhco4fFjdSoqqM8/X433M/xc9TznvzOzTBuH71kc/iT3Ofz/3PqU2MrSK7iRBO
+gLAblKWEc2B/YUcpLoJcZhLNMblsT44PBg3ywTazzPdRIgZbbWG7rLREh62Yr+E2C7cEGfOueAS8
+EyWXsKzTwU+qoX360qIgjGWpIIsKhwpvps/rpSPSDvjxyrGLcZa9qdC5HdbP4UYyyCWVkYzVPZrk
+bSU3Q+cvLolneTOrlMABk1IGgBDPotJn+LvZ2NfxBJPA9GyefOPjnVmkI6bqgg5zI85mrsl6MD2o
+VqVGzg9jX9jVFhDT9nSi8OncRhbA5Y/F272yPhx+duOQReJgYEnzddIoZ5e6m9VIPoEvq9gnI6gH
+2dmG8MLi6aLxUzMwS55C2wQQtcZ+GPznMRvBaaUNrCN2TgeTqWyedvIO1mUjDj+JiaVfU7bl+tto
+547bCiDTYD9rJQG6lssgu5mjlGU0PONxZNx9JpxpUUU03sImspMBgbtqF83Wf81c3jVfRFosE9nD
+QWBdunM4J1p+l3M7LksJ2UyR3K1rrrq1NF2zwkDy2JVFji02eNt9nXMo9lF3DSM1j36LV+ZKsaSe
+3BU6brofCW7sqKl6QopG136dZVSg4x+k9rPKeJD+irxPmhagtJ54AOvaJZe8EsUyh7ra7ITBHHVD
+1dpgeRxk+iDZ1oOzbses8IetSYfhuUjbQLbw4eR8w93S2Xz9hli5REFpbNL628kWoEEeiKabjstI
+DnPaVG1jYjuXovAR+6XnAWZp6HtmGrIFsm1h8FQkm9fQrCfOz0vVSDJtzyOnPrxYozHxXxIYWjaf
+Y8rM8AB1q+vqlDKyVpBF+LwsAsOGelFiC657uPVD8A8w3j92BOwRA/vJDIvP65RfbZvMkkcjC+v3
+BVOIQBVod5oHNaREYUPOpq1D57UcpmTbngc4D3K+74MNNg1l3gYeFJFBkmEOLuM56kdaHVvgNKi5
+IVzDlpoXgAFLH7XoBVxaAiUnrcKlt/5nygm6WDXjGiygMlRboJI9KEJDAcVcCAfdsJSBH9ZnMCyJ
+bEqoytlwFUUNAUsVPj+gJZebKpr2JZ1mN8LhrQl8cJ/xEeYJUO1sjMrSG1BkbIkAm9ofvdwk5yWJ
+Gjrb6siH0PoiD7spMZ9aBdvO+Xw2HR/tYXaQButqQVGQZ/UYZyy9GmKZ9RbeRYIP/NwgWktwpENq
+xjKGh01aRQkhY1sJuxZjdO7jHuHrC+vSzdr7Aa6MLd3pgeZr+GVmCrUPsrsijeWxJ0nya2e8c5cF
+SEM62o2NT9ZypZsNdxp+qkVQU7LK+RZeu9t0NsHPQ0gwCo1qJXxYo5X+LPoIPY+9kVv224xizS/D
+oNXBt1xEWj30ORT5YP2BrATiIYSk6mcUIyaX0YJsATaOYlkugwxzQR42FMj2MTBq7g5d12TRpS7g
+R1UhfAXfc9PD4EjYbTyfme8Oa8rgBTytUxOWWbM21xmL+A2F8mAfdbS9QV9tRL+nz6lOHwqR9u0O
+cNPsohJNb8VvsnFZId4d4ykhT1EM7PsHnknETyaTGrCAJYQe8LPQcgh5a7cKPIQuPoBuHXSXehtY
+Wmcr0vSqlTSanmIbwQq6hIPiNF6RtKXdfdSKbroKcQOz2ykRbrtCvBuffBJu/LEZ6MR+5F4U/Z1s
+SZHfmSnw9AlcoEnttSIir3k4LtsBuepmysUNII3u4MTLfimqw/kWtFXR710jHP2OLauw51gIusvd
+nEXD8JOyRGYQFs54Dzvllzn+JZIF6DQca+cIuxp7JHB3adyjPUWGzWSfh81P/oITmUDanzjWtY+s
+gXXwcJasOtP5PkjnxoVnDoUCg+ftWsj591Jsa/BraZNpWEtuwsSSShuSRN+j2TkbQ0E/uMzXUGjA
++7KCE1LTuJJSLmC7uSp+ZKXOPJ6crrJtmIZfue3hyF6qYtJQy/ImMvRlSmQwPuYi6QUyBoWNzksw
+w3wWVa3aYhhW2tD2ZkAgLdx8KIqlgwYdfY/pWpB0jUsQZWAZVCiHeA7qgbbPPXihcwkNlbAIjWEb
+Vi14IOBYhoqgkeSUAK0oaEVSPLoGjdNHtpL+ZzOMsgBa2S0t0OAxfAwJELMqxl6Mq3xq5v6Htr64
+B8ELNzbtA+7usmF1Zw3OF7tqecyHCtFneipCNH5xwS7tswap577blPyZidT0Z6Ny8d24rtkdhKeN
++e9aeG6KcHbQOersYlgnbj8jUygASfOU9ofJw9ziAEMTZnZBzhJXxQo+nmdeB6C1gO7bP6owx8fa
+PDmf5y0Ia2CjPCj5CMcDWJknsCNIp66Te5ml7ArVzdaXY9/5F0Fwf5+PJpqS3cj1Cgq2MT0Mo8N2
+nxVbmOyTYGgOKD7gGjJu7RiA1MYmXo/9oIJqAWkcXtfIVw4rrrfnGFzMrpoY7pgqbRd8FDigwhlo
+AavVVNu82vZciwXW5slSgDsGtzjawEHIrUstNqLdRQPbi62UcsjP2n6GDzTUMEVYBwTXUBkel6qs
+ilpwPkLLkmoOVUbq2EUuBMmu4fcId9FXHathKaON6i+JzJsvaePYb47Ozl04w/4Eb4SQYM+FQh8p
+yGdYuUIbTmEIW2gkqzCOGbOrkfWuvVPKD/oQJVqO50ef0nBvYxO5Ly2U5lOdTDkRpUz1ijaQwtbM
+NO2THdvg4l1J/D83x+8AJHxr1VLBFDqKKuQoKq8Tj1wEvMStxyUi8x6e1IONXuia9pdNrLyrwWwW
+eIbAmfggiJ+gKvdCflP4NPC2XTuyj6H8TvFrB1CK0nQcQPvr26hCsdPvZdLhHwHDIgdv2mKAU7wM
+m8e5lZKdJQ1bYe2KTAUUDFlQVdGwG2/aLiv4Po8kPG1gPp2Zfax0gJY+9S0tlddqq/gCZm9J0pAn
+OPp9kO687cf7Ndd9+rlvGxlWa0akKXuXj7ps+eTcdZo3I6TWTUybamjWPKwVvuf4afJBBAtj2afn
+Ku4cLOkdSZBd5jAChQk0xTc0uUEw014k3X7oF3ITgVqlvoeq3UpSIGaWU+ZsU/Nmwl8btzltdwtd
+kPFluUgbMMWH/JJ2Mk8OyHELYsuODu0vGMnCCz2D8cpT3424TyQXIq4HTem8N74J8CyhHipkSwms
+H1fQPS6Ym9PHKN10cTEw6AAqHi/Nvc8bGHuPYN5fuoUhuVzWFUne4kca1ZlKGgen5oTCdpE7cbtN
+UfRNJ5RfiU71sOyHtatBMKRSVANbEBhXHyZf5ijYvhHVMlqSJRHhfWQNLAtSUBz6p3aeYI1dt9rA
+eRzHElbF4MPj5oOHf0BuOfLaB28JrF0CFYlLFaaWVgoWk0j4W9U2ddPwIj7Dp0qXvbd81diqA71f
+IDeRO+aEYWWDHjU/EyuZsn0Lqk5bLpAx5XtmGOBgTxgcfLly4VOykiMhCmpOuQcIqXc0XsAGZY6z
+g4+WAD5EadP0Bxia8/ErlzEGOxQ5JgnoxiJ2obORt325QiLZn83Qu94Ce4u6Gv2jJTyfchNCIUZQ
+s+B8ZYIsBzhpOnk2JMU8XiJXQdXW4rNI2PtR/D2BtKk++pxDDg8BC/+Ktn7/K4Kt7E8+qvUn7F/4
+y9q03dWQgpu3j1Gl33pp24cBPvuuDrChnmw8BPoQtPHwMLckQMzsYei8z13WISkIGIUjPhKK+JCF
+LmzP467XD+izp42vUO+jevNmiO9naOzg8D01Y82ZzHAXENxaFWi88MdiXVIIJIMDCtSli7NbdOVh
+TuEhZqJ7cPSDeU/yOXdf5ECL9twkLdJhswT5zncL7qFSiyHGNAv41cGomRD+LBso50uQ1oL+Qdpt
+1fXSTyw+IBSra5AoGCS+sc8gu7E0KxMv4RUAIgX9HcyR+x0YQn/rJEVlu0g2bZUNbIqmZaFxn4Fg
+BzvoJOyjHUtRnoP3cjSMdGE/vazrCqVLw+O+LTX18Q80S1ADGRrCAd6Q+UvBcvW9HzYSX8RQpx/C
+ICtEBTh7hm17ARR4D+VKO1YyZeCecD6Fj4tiC46L8s23bBjXT5lP2As1G7mzcWTvKKFrexiR8YA+
+aVKoivMeTaedkHLar0mvxY6GrmAYxCC263XqXLDvktV9z2FJ2pYp2cwPGD2rHk4vQ5zB8z/KD10w
+LwGAm8a/6CBZIJUfi8GdLa2Ov69rYnNoejb1MiJ4+B0cn+V1JKPgd2T79dNCgIPv40lnL0vTyQee
+wiUDksZOX9isQYqUopmylBs4PstZBxIuTJVX0f92U0C+D9rJCPFt2z4LZWDLopXv+I0UU4K2ab8M
+v8JOz/B53mjb7jaSdB2Ym529JL0bZxQI2/S7yRL2bYvH5s7iCr+F+7x55iYtYPuOt/Yjn8x86fop
+RK4/4JuX8GBxYdW1BHlg12GuSmUTDdpCkGwdTG85t5/ojDK8lK41qKo2WO3X0K2I2zDq3bAfA5EC
+kQ/haLSHj/ViSzmJND+gcxk+Z6ZNM/iTaHKTzCmOewTZZQ6gCjV87SBrn8skdzmqUjAJCnSbyEZ3
+K0ymc5xkpy48er7Jfo1Q2O+iyaDtaRJjDrnEuy6p6U1WKRvZprQ6xyaDS31yw6aCP4J50T2skQUO
+hMLPaozPoBNmjcCBAf7eWeHu265Jfy2KdterFrq5cByjJ3a0QBKzn11fmKq1x45KwMLmPJzyzuyd
+o/QBd7oS9ZKK4VJC4W3OZ9Vl39QSk2snMXBiH2LuydcGCau9yJuZ3nPKNgftYwuNATCWlME7fJp2
+Rejy9mwKkwFW+cmY/Cxgrg0S0MC6y8TP/jFZ7WiqOdXZAMujjWBEB77MoUcrct0vC/dPrHGbu0K0
+wFghGrUR7MsLWNhPoEwgncWEjhXpYHB8OxvdnlB0xw9pGzef2xlC31KYKY3KhiAHqKN2C353QvaX
+kPsdQzjQq2w/L2LMK6hozG1uMJilxCcM8QL8mlUesqwb+LrFruKjz4ZyKUg27Rqk7WlFuiQ4T5cV
+j0m9KuAF2a95XuI8Jz/Q4WNfgjHRXxPQ6b+hTbBdNp2VGLLCO/q1WBf1E0hgdzvbsf8uUx+fKzzm
+XKFLjvLXoUsEtwxw/sGDWyk7jwfdFVjXbthRhJl1x4J4icowYRPeLGIGcJAo1fcdzD1Q7EdgRSB6
+5tPtgip1LWHkK8NLTDZJvy2bTq/zTM4vnWiTr3GOFlqpk858bzWcp0rXAf+sdK+yHmFPdlE5W128
+oMOMJNly2lz5dHJzueElXsM1OhCQVsGCf7QNkpQgtGG9sbxTkHVNJMMQHCWeCahZz4XIEvzuaIQk
+BMQNdUhGzAIot2V2KIEgK0Xx74WaDqwn6zUrjg7UGVqxppx4lDeV5qqwO2RN21Al2ssn0PTZbWSz
+dSl71Ee+6ptj1jYlizobMngSlsuY5apqYgj2L4p5m1+iZUseMk8TxG7ihzv44Rdf0yYOt3OKYRIP
+o5HqhwHF+hr2EWrbi0xQVyq4YDwFDkBqGeEGhvhfTOF9twy4AhiHdSZCbJbfuSHIv9p4RCkHFnHy
+yJcFV8eqNqh+srl13YUJZHzZaRTJyH1jZet4CMmTKBSs6VAzMBSkRQIzJ42s5ar3mDhbjkk3LSWO
+ePadkLVrdnxaYX4kURFXXdO2N0OMegI4EHrKh25i8mr2MEo4MELD80K3+a+mx0wM8NeRxXQLUowQ
+c34egCznUw0aMlsrhxk0vC7SEQT6DoAY7DKhm78WaDb9WDtDs70xKtqn2YKMfjDSiyqaZ/0cTCu9
+zUDuA9d+gCVJ2aZ9N1cU/o+XaGViXgYab+Jz07dmrEYzRB1MWRfkXgWMozD7KW76z5aSfK0w0iv2
+lUlCd5UUzUZxFRpxX8CJN8ecAiPyfVzYcI9vPHpkbpA695EmzyAXQe4O0Xuk67RL9VUHddx61qJL
+9JCTdeYXcI7E5ciRVvMSsYicUR645RA0Y57Xc1pApZ42CDIJwLILzPXxNxiuNdGdd7y93IZtTlGA
+pVtcUrLpG7FmuNWGvEEbs7PzcCZyNIp2HszDp5SN/mWiLphqfMP2yjoThTVdNTZ317L+qyHt+J32
+XdJUGTKUH2gybNcyxwChGjXz8Mm4jXS3AawYTHOPcSRGYEpEbGABz6yYn0NMsULagZEo9lPCoiar
+i6GYtu+tJ4HGMCaDU0AKg68QIFVHZajjNj4cCQCQOIuZ/shSgbFI06z9+rwyG34u0Dg825aA4+D4
+xT5hZhP9gWkNHd8X4TA8wjw9+WoVkZgOEpP+ORC4dcsAFfcXTySF8VJG1T6cM+xSmtm12xFtabFz
+lo3ibAbWrctoSEJ/1XQUOQvmeI2fs0QDXgxdBGeAGAB2V4uxLVwJu1LldkUhVQuYI+4/tw7GCbBP
+9wMp3czds0kweqSO8nDId32HH1NjqBKWdsWU6zrwm7tG8jyhlt26bap6IHpiB3U+JoBM6Am9YOhW
+VjQ/On+EFLZgmu4KSYpiF8GuB8nGOm1r5UU6AJnKLaZLkc15hUtlxOAJhZ7272jLA1j/4juI6Cyl
+6/htYhZOpyy3U1wBY0ZZs+Ux5pkpkqnxQicR6WDTGcdAh2CuB5R4HnlfDd6nt1au7dUSkHWonVlR
+CjUetL2KuxlG8nw247qPIuQYYMA0oAH3Y48BQxLivns52yjAf76oT2Eskbdt0gf93gP1TapsENld
+34E1ULrNjkDc2j7/BFu6OC8xUsf+hCDe2RJgSDDWGT7ziIlahAOwGmlzu2wwxikBlLTBYQFrd61T
+B4dO4NC0mLF1ouS6Y0zfo6nSo7bf1BAew3f3IlxiEabh4Yb/XSCbLgkmxDxEPqE3Y++MO4CuL2/1
+0IRRncIj4s5QGDjC09vA9X3I1gjtqpBbZAKBjkKytxSQ0WPPZQOOh2yWsFIKM2Ku26RFqZbiGsQo
+OmNTtxs9gXkn6fzaXYq5CM/mcTRLOaL//8CxqwyYNV3BgVUkCvPAlMCBEuDKNKUD3QuFaJY2B9vE
+mG4Fc+IRrUwmTVMWMB5nVWaZe0mGzgQHjir1HJhqfKPyNfvNMenDIm41Zqs0NlBepl3nA4xraVpf
+Y8Dj8rCmpCdlGIpNwxsj6XI0YUTeV2OPwXnlBm8sV4B0EfsVMC/4sO2nFR5qaYU+7Toh21+LazSJ
+5i8MFLkADX9AIfCzXTF0qggNGgFinTypNqbBHw0F7qYOc92+E46ZP9WW0PaBoUM/7vqc0K0iqA9u
+KcbUrBXURTMvg0B74Mxb156zOIKu1zi0ZcoUzgxDnSNznSuLHl+PL+kVCgCXpDMmH43JZzqHqKtD
+iC7v0fIJAWFMoUUiZG1bmrZAT2rLzXhrBVLeGp7c7XnfcuQYS0MwBW1Z+fI9YluAOWrROl7Jtu/C
+88gw8jD7JL4D99f3ZWoYBcKK4Vzzrke379qrFAAYb1Lz5b8mQ0kXOv6K7OxuyMDMI2Fq6nZ0nuSv
+NG5xnY6L89/Xjcw38TbwX5OChQeKg5jdjNv/cXZeu3Ej2xp+IgIssphuSXa3crIsS74hJAfmnIp8
++vNxzo3VFtTwxh4MZrbtKZGsWrXCHyqbEBTVxtNUSDR7J7pPZ45RGz+ikZDHo7LHmIuuYziqqvvu
+VBqN+XWdUNwa8Q+CkoyUC3ptmbXjnpO3TND6B0rVtQnM2FqeAUlr3ysmE1xkXqJ6vxiFll2jWMo8
+KR7a6UuDx9gC3n/F+qAxnO5Xp6PZQrZu/9IQctQDilH3xjDmjE5vp/qvmirJrJNh1K+LbIs0Kkmi
++4rrE3uzQUyXDEdg3wJkdjSMC3thXytrlTajmbK4V2Ih32XJ6tZQmo204cR95zoTwapzbP2hdaus
+vewjx1AMmMrJCmOnoE2JjLZrnI2tRCrLQmHFCgdRLb95Q1uwItXMg4Z26pOYE5ql+Ui15VuStkeM
+NIl1xiUo6GuXEYNwYy3r+3xTGth7lbFcEfbMivKD9N63Xa3+HWmllEGlkpZSeDLrh0x5/RwwL0/7
+vScrRF8MlYr7jhRED2xQPnc96T9eWHwUhk/QR0aY8UrvSLJjhQJ8hHGgnxProCdNqbOcSxiBv1wr
+y6RfilGWAZtkeZ7GTHuMRdaljIK77rXKI7q1E64luT+qqbmzkSf90XHz3NJpFndo9tbGXQsWPqJl
+V+bYb2wTYpVVovsW0fnTD5m5jHelLvryMrKHdXPWUrG9h4zI/C/TNtHjTW94V/Y9ubzpboaKw9Dj
+OwvENnnDWzEjkSWecf66PGdM1OTJnQEbdtx1A/ZqcdQz4ldA+Xi/i0FS0RW6fZ8LvA151TG5Qg0a
+9E3PGUzvqp5QHCyZYse6te78Hkx9eZDLOPWXjWtz5SxwbrB0miz1Sh/ckUEPCPlgI32bnKcSePx2
+zaGJ2TS1SfpXx/TtkKExooC27vqcqUm8LHnhYl5p5NolpPf6l+3MNJ4RekZwNWME/G0snMnxC71k
+ho/5WXte9hr/5bKbWlJa6RQWFoiu9Zu5h8W0AxTBNiwu4VxVsqfMQjhe/0HvhLZ4RVCbgpzxoXG1
+dKX+tdBka+w0zHHSYE4Ld+sjRwzjnYT+b4iWXP2Qz+bypkByvfBAuLRQbBTVzoEdYgeynfrhMKOf
+fkHDR599bDHVF7KlqsDdL9L0oHZXzTwsYjBfMNJNn0CpJt9HerMvyHmK5MCcunxqs9T61a11go0Z
+Fq/0/JnNvTV1i3mo57Zzt7PwpfsBcLxZfSPKEAHAjULmGK0V87dqjTvrwkiqqAsH0CBsZIidvzmP
+qqV72DInTqdiIcUDedPu7FxLml3fpfKyR22CcZOq5K/ILOkEiNqNwqSb7XnvpCtownS0dI2Kodb6
++Dq2spJnZjKgBYr9uuzrcTSLoOTbXVSi1pklQ8j8lTfzcN9UK0mtFuHUFyy0q82dVVkK/0m9MPXL
+NSq6yEeYyHrRDMVEqIpdY9hnFLAPWIaJJvAsTVvO0y4xHoHDogygi4TcwKnRcKkHQXcm3vIAP46i
+5raozKYguM/VF61jPMYtjeOHv4rGudd7e4r3mMWW352G7ChIK5rVfqHFFveZUTSPQ6usn3Au6M9U
++Vg7fjdUkC+eJUqG4tpcFmO9yjuZar6ZR3SbpthybsHqNnnocg+vjNrdlqCkWSP0ugl1iH2MgUtx
+iIrWyS4Nwged56QdxA5TpPQxy/GN9A1r1tJdDS5J0s4zaCs3g70GxjKCHhb5mj/B68KPt0TPIuaP
+d2toV8Y6+FyRzDhGbppfPSK6MmTiIy7suYxyNCw9+8LOXU3R0J/Vl4RX+YQHKyRjhbldHWg5sS+Y
+EiNBcriq22ZPSyi+65NNn6OYbfGk6cn4Db4Hx6/Cm5dhVNmoPkyk28sg1rCN9WXkGud9xvl7BSdA
+gJROxaDLMAm2OWkWh7MyusYXKS0GxE0AR6Kb2FPEpnY74A1UCvNQDOi+cRs40U4qigi8aBdvX02D
+ll1ZyxzZvqt0hcnihDIRBpw0VM/cxbZ+NVabfKsIKXiops54XgtSotAFAyUf1rwYrxap1+kV2Zl9
+NTe6Ux2sqZrSwLJKQDVkDnRrhJhEF5aTodGAWWM2T2JZ9cu0jDxIa6bxfUnR9U1RE0Dx0WoEDla3
+ib7mbtwssClXxwlo/DMGYNTbXTYNacq+pKeeBwW2ayP0WbO7EeNc/9AKzUovlWFbZ7Cvxx/2VFg7
+3UjG9obWPTOvAVLkQlBq7d/eVKY/F2arvwq6r0+ysYFORA2KPoGZx2RvQ0tqHqZTI28H4B4gxJjB
+oqM0LYqRwyTzYDGQIUd0c+5enQxfYX9M6JZzkwxOF2R52vMpZoetP7hNJf0q6eWTB/ToNSmEetJb
+B0+50qjUa4VItAizZNLuySdWECotP7zjll+lHLunXNW65xOrRQYHCtwJyDHZkbQscZMieWRXK7Xb
+2g9+igAMrQYU5GlzNU7n+mJU8tUSg/xq6s54LzUKVL93p/6HoccV+QhFUBNGjDXPSx6QlC4azcuU
+lNQOinTqazAr6FYj9mkiTDs1gCw4+mVz4C5M3hw5WwPy0gvmklrbpnYoNctJw4gXKAJguQ5nNWIf
+BKlhpsCW0Qxjfo4Fr4FNpmDYIvjA0u+wlbqqXNqdTOTy5gmBqeJnrqauBoW/FrdVQea5W6a4YazF
+eLcMvWySaq8yxtqtsss2WJxc8mQRLNHdGnHBMBt31fcm1/NXCgJ43GmprY+GWHRYK1o7P8p4yR6M
+ZRI0jcTMFI7ro24C8BpMpgt3qG+nIWpvSmmYX7uKSv+etpMpgxbk1fcFZt1LXC/ll97OSbFBgGdg
+wtLIfEqspYaBv6TmjcaYOzmr8Yx8TabNutamBsn9GRm34TDqVa750+hxX2jLmDFOYpj4aNuAWrIE
+mUt/bqvh1wTh4rtNCRqTb5icT5MkgWyCGZe3q+0Z+9y2X+OvYhCAiRomOpurRsK4wqpn3nNaIj/t
+4yEq7pU5q/sSc7KG1qXMXkHUUYQsw/RTgSwu/aTfdnHfy7Q+W5u8eq4ZCLOhvUKlgUZjQPeZHSSe
+T9OJVtRq58l1MjSVE3TSwOk3nvlDezy0xwR7j4TmeKFrS3EmywjgUB+r4T7uIyAW2Qa096WcN59x
+Y9Seqc2LW9Oi1c2bz7TbphviO+g0iOdGopLnhhjoAXcbRIkDZ1kIROb16IYOTbUnmorNix7PhrVz
+9IK+7NSl4gbMZGUH8EpoXFGv2UylM+EsAXEW8AapV3W/jFjEhFqLDSyZO6PkkCMAyyMGsfesJWaj
+QjNZ9LNZY/xODI/Vq9tY0aNFFsN7srXxTZgrU34I8Sk2M8JaKNS1OXkSUWpFF0iyzre4nbvFnqNA
+YAOax11ZW5juMYGd2pjM3ezoN+H1yVWx1N2VJoktvjPEOH0OhWzxTLaX6Ba+xfQwGe7wNslBdmcC
+zZDLqmAUT+ZWR4wlpfVKH28m/DldfFabMOzpxab1QZ9bkD3YgDeXPGoPtMExkiRYoFz9Stk/rICG
++77XS/t3IxOcx7Vuql638ECVxswDLW8yiXMnUiWyhsxLX1p3FvAdEjOuuKE0l/YMPYqbooNcADzG
+jm5Wp8DRb6URBxYhWesp9KI6bkiJZHqxWhUd7CYCp04DA/THvtWW/Cb38J+nWC1ng+3TmRhwM3NC
+80avC2ooO3/QB5X9mOvV+Z6ABweQmZj6t35tKYqwOY2+SZWAtokNHY5hPOoRabk9md/YhdkVUPwf
+KuqLNjCrhmzPwbPWd1bXQBGyKvSzzGjAM6mVIScBO2uTXYbdqe5PGpUohrJyBmzkzcY5oJzE3aF0
+hzeTXWnmawUYjmhlcg1n1aSfJX3LkaDx7931RmPeNXSgqzCazfmlNbg12XxyfjMq7Ib8LM/sy6kH
+++VXXp0+zQvjMnpSs3UNB3tmhwOuTHYjwL4ObahGUs07OVMMuxP6BR+uA6uRK+0x91QMkG0DINYW
+jkOHqZ1SAm5UvXSQSJ9ns69vKj1V5llWNPq+0tQgD5v9cB44Qz0kEtQELUHsgOgnFNNFXjH/FNsk
+EUyd6zswSqcz5Vkl84YytXsikEGzF6MUiA5o5TPensyc88RHiDpwTINlM/iY3Ot8TnE0603a49eQ
+yugeVCq3HbxlOvC5tCXoVnBvJMNuapzC3OMUREs7G83uuc6M+ddccQehyMXEOcyGpf3ieEIrrgD6
+ppcZ0aIMnHmrqpgx80MAl0lj3yH3ekaHVLuEtcgY21nn7FUmcv7FjI9Vu7zPvZC+VeHiQlzSEMbh
+cKUeQP+WqWvlWt03eHCNdZlYdfoV0MEwkHBNzQhkJtXAjCioLHnQNSCwzmJaav0VdNoeE90Yu1+X
+dtd6hkNig8sxs1ZlPIKwWN9IvCbw8MqRUf80xDlUkF2HBJdzrjHKf0Xle35WMa7wB2bybh16VMVg
+LEYNdUjqa5rbsbNqLx6SaMh2ubZ3k4y5l4AGS1yS67r+0jPGB1ilp/qbBjwCP+Y0t6Id4BAPaBSl
+aRnKHowQk+7tAMhxQazQqNypDVzuFJsM2wFpxqTPexzq1r1fR3PWGVauPCYM5fYA0na+Xqd+pf22
+EhlCBiPjQwxoGj/7VeQtPU03f0qRRzDDEa93VH9AAZJk5uVCr7i3CDmdyCn6XYAhAsjYMAzgUrQk
+Z8SgsW2Y3yLjmGPjHp219JZTRIpIcINaNxgZMoKr7D2yYw3aTEipuXs69zl3k2kwmpPAyNGM61bK
+5aqbDIZWmLV+IXmcp12CguoFYjKCDoteaRrFcc/2nZWOqkKblUvk5wvhnTkiDZ9zVMEppgGcOGC7
+1ky8WrmRwx+ukNFEbXXKVViak/yZrBUxUEtxo8HivqRH62VggP2RYP3QFW3xFWCi2eyo6tXTFCdl
+cq6ReDPbSBvz3okNFLaUaNiRg10NgqmhENczyc1rm03uF+SCPcBHuBVFu8JboXSupjHcdG5q4EZv
+OFaYZUo/X624bm47r+7u56WydLAbLgj2ekvty8jMu0DqI6gwMnJc6aPK7r9VSUGdmyELSpAHxBnh
+6VzLe8IBMyQ4ZkByzarQNMBv2nhHmFqnwMxyMI5NhqLR3P53D8jBm/xar4drQiNzYnBE0TNMjOJs
+QVlVhQAeGA8C82lfFvhxfdgCeGsv8E3Rf8eqcs2DjtU0YGwaMlwluo2DJMFFc3diNik/UT8ffpax
+0c8k1Hn8hMbudL8k3cQN09jxazssy+/YAWa3zzsvf/O4pDG452AxiWgzt0WCJnPAhS6knAE7nmG3
+TDTODSwGEj9K7/wHPfrqtW6cdPYF0vBPTHHp0cz9sFzX9ey9ov0CmoeJsdUyBVgzIMum5v4ssnJ9
+S6mteCpRgGkbS2eSQZZm1rCN86wp0FOn+J6i7Ypxj1ih20s6dUw9043T0U8eYNGqXkvAJ7rOx48Z
+213082IMvu4Ys8U5kFoCyiiLu53beMCuuVuwVHJjiTc1A9n2BucxfQkd3davrLjCbCAVc1EfyB/z
+b21NVCaJA3o0Gg2hH8Bj+QO4aXYHr3UAZ5gapbYDER7dDcSnJCDNF5RpaT1+McCKf22Y3TxaNnME
+ye14VdaF+ZAVpqzu22wekdrx0mk5M9xJfemTvkcGde1MZICaYogOS21mD2Nj9nSe5gXSyqKvdBvJ
+XRBNXQ03d3dUSZq9S2VNuaj61u5CY+DU7OIhVcRHb+6q80oqY4SOO0vXo7dqER8sc+CXE+g8P5p0
+bbQArbUaRYNMLNmbWwOcOCCRMUXXEzUOgC4nmh4UuLlfktKATy02MZcqptceyQQ42QICBnjDoBdv
+c6eix4hM/yeiUFubdVGzJBCQA+6g4pgv8EFAepTQg17aVHGRd4PwDm0x50xZYQiVZwp85wO1SoOx
+cWb0wOctyEGzWFsR9AVMRD83jKIAYUKTJIwiaDLkkY5zR2+abNOCFXCZdcDvwhSLSZfhwcj1BLjG
+fDKWNn1TLsjeoCgcslzYf10btLob3VWZBGdE5k+Sy9g1yfe1WdpftNIAyDMiGnLXa2JYg9aNxtmH
+/gaaqXH0+jF30uW7O9rii81AS9+JaNW1MPE8hhN4Q8VpkHclqWmhmdW9cAf3AffG+kXXegvAUl3H
+RkA8pH2IO1x1BSVNq+A1d+YrevIAPoHjlucdxKtpJ9B9HwJ+Hv0xgvN8sa5zDUaEBurPPk/jF4Nu
+GojaVpUpk1i2mG+YpbaAFJw23CUAN8ABQOC/RdWSyBBE0soY3nGbAwh7/qQJtq7m3mP6RnIMJN8f
+TXTSdnE3ODdDZmmKUF0Ii95flj13TZ4+elHu3TE2pOMyR9GqbQ0uVfuurUFtUakk3V+IbK8kDZQa
+BihLf6ghO/gQq6I3O6FVse+9NpPhAhbCA+c1LBdytUu0LvTthsn0tkh3ckpoyxYgOsydKF3ndqs7
+LYLKuJ73dR93QTRO9PbQbzKu+mmVX+OcKOYjcJniQERZsne7hnQG8ebu9wzh7ypty8EIp05nXp66
+sAp402zIwBrauPCnddGeISDyjdWCJLqbruLRVA5SLS24S4PWGCmaP+e1AfEmr7z7IY9Wy6dYT0ga
+IiE4ELqhfZ1Tc/0apdMoAIRvfWbE4MZXmfVmG6wzfZhgxYEi2nQFFwZu9IzuyqWJNeCzlNX+Yjri
+GrpYd+N6MYBjR5Rk9rF0BsyivGZWRHrG80a/MOpdVT5He4CiMj4rRO/da1WCiobnMbG/NKeZaQbj
+8D6MCPs9FAvu+nMjk57m9wNeykPVadSiA2P3HcVqlUFDzOr63lgEsAAwYz0kmkhn3gVHbty1Klma
+sNOVkIG7QoEOlD6Or5M5a/NuHjuR7b3EyzlTiWeTaQFAXYHPxXEWClqC6U8V05jZjasmpqCsIcCT
+mC05kAuvNdIL9Me88nqeUvfOSvOiDc1pLaBp1WDsbqH8MNQe4SnwMlqz/CnySvT7JVkjFS6KltU+
+TkiMQ8Fb7MKVIE5ukTGl4sUWjSboChnRQ9o65BIt1hcaQM+JJGThrP4qKoWhegrv46EeFhReNhuA
+awwRhmcws5IhZN3b163F3Dkw16UBWuw2GVqMMhIgb4lcvsYg5UZEAsiLopMKEm8Glh0W8Id+1lGz
+fK0Lkd1KUOn6Bhikd0w31qEQrZvfbjRR/NHXpVdI95CMK7MY2AxOoX8n45uHgBKlIgWdOvdWNGYr
+DpF01++xNuvXUEwn/RIymflztoS5NWcK4Jl4CcXnNIaTlfmoXt1CLjAFGH5zTBizY3AQAALiRDkq
+0+8TTA/yoJY6H2zSdetx7DvGyu1oM97N9d47X7R4mA8z3/vLyg2uziTdjPOM7sn9YE70kNA4G68A
+RHBL1qBPbsgOuC4Kva8nf+1pYhzctO1oYBmwCb7QkyxIQerJAC9V5e69XdaAYblu4tu2AEnsT7zl
+byDUp9ut0AOKoxfwwTSt7u/gSUY/8oYOcjCZigpDKrcAJoKlyouXLBzmuEkWB3xWQbuizBDW3aGG
+J38UNNtQhjWa5DGR1UDlq3vtCzpDdkGTrSp+xKLtQEFEOS0l2NxFAya9ah5FDQKAIAv+QlpoHvtp
+jyl5yClevnuLvU7k8SZYkJlWrQUKh7QRnLQsHmQKlyFgCmW/WW7n3HMH9ea+jmLm3GzdbqcPcUeK
+3zVmE2zRedkbGc2dXaYG2tiWuwKMTNzydsOgLmGiWnVN5lL19lnMRHvZJVK4LdJyrXbdT9yaZ3ld
+m+cuPRHDdxGYp4SvVSNue8iAP7tIX29t2KKDPwOsGM+Glf7bHdyzCG1Tzal5N4m06h0uXoNztQ52
+0TxRF2hPmkdjlDFQo4PPtzOy3GFuxEtRrVInB6Q8+uHF2aT5lF9gFCMBaerQtKDGvzm4hnqMXLzK
+IkiYtMbA2cY04QEApctX0KUTfhse1KW92cDl8etxwYv2c8b1piXwp7gB5gFIfyLXoCNyRhfyiNxd
+iMXyWoA/DISl8V0b68gf83Y8OPms7jStQOxVi2I+3TCGRT6Kw+fLHxO+t+XxaoWO7yJjyxTsPdca
+Dms3AFspfahXlEMFUObxTAclaMLubG6ZUXj+asn4slMFsODPFz92FcNgjtUNXWfqaNqbfsr71fEJ
+sy1Gd5WfR1y5u05EHKQSW8BdTlWRAmuiixbDzGZ+nlJRwRHd5RVoE5IYGt6tPTyf+ImOuefHP9GR
+xAqA56jtSj5HXEviMCPMMIs9IyBVempJhQk8zMI72Gi7Ypgt9L3c5VBVdACMOQYavtByAE/inXhT
+xxIA//1YmBhuqrfC/EtZrFVE6FFSEldlTLsV7lwMsKOgG5n3tV2Hn7+FY22IbbVN4cPZ1E3BxBzJ
+pDSzrLB5BwkCHNh9k6ljAo+DLkVaqCz1htGvcUJE56NtiOSesK1tDwrrSPoCgGRf5z1zeOiAxp0N
+zIQ0V4DFHXR1DnrOOzQV3O3atP/N/mGzOLRBGtvbDmR9cbQD3RoGIvgXxn0I4UG5ov2bNl9LyV1w
+TieI0fbnr/bvB32/3tH+WmwNYkrTQDys9JmKdl6uF9a9BI9hghVvh7B12/bBs4p4//nKf+9sVkZ8
+xkLU2MGPavvJ/pB86herFqlkZ+OQpF/EYFu5eJv6H7Va/nufmASybWBk0MR5vwpLp6bXcqLNWQwX
+1gZ9c0txwVB+/uKAtz6xb/4+F6hvEz6YHjMQ5Gu+X86VXuSVGju1G7jNBlrDAR3Hb5BrxNnnr+/v
+MyHR2XBwI2fcg77v9nr/eH1QubpOpdwNUWu052QwcLGgD6cBAE9YyR3t3BO26x+uaCLEBAMeasKx
+eqGgwm7LkTPfJNr8I1podHlDtnUSuyS/Q63RPaEz8tEOwTrBhQjhIv90rC4+4wghmdwSjbuResVb
+m74JG6efqv9hK2JBhCa8kJKvdvQuU8DkZBS8y7V1WrDOgwfmSLUnVvno/SFXLgBP4YICJv79F5sd
+cLp5wioDCAEbaqG3nmWJ0e0UPVYm+PTCPt8iH21GT/dAD5CWEc2OTphdd1a8uNsWEZN3P1cIgwQq
+jh1tNxYkNSciybFI0XbSPNPReYsS1Yhjm5LaGwtyYJjHnYjL15SBHvjQHOjK2ly5fbVZEmvD9PT5
+I34QvrgYECETxEqM34z373SN3NW0AIn6aArA6BROdOgX+q1mme3bInLpQpjyIE0Ajyce94OviQgs
+02Y0mQgu8ihRmYy0TtyWk95Ho/tiQLzOuIvFdIZZ2biP4UfvPn/UD07DlpBhzWIKrqTj0NLP3gDG
+rmCWBTw0tFC23I+aecqV/IOv6BgoutkClSKkn48eC7maOKu2MxcZuVCg3vM+O5h9L/S9qHTQyGmm
+L7cC/G9yIqB9uDIXARQ2zALRS3//KSNw/2rADczP3JE6GjJMFEY9Z4MmSS/eiO2AXWeonNGJhT84
+Jqynk10gdg2+bfvB/oikHZR3B4YpLzZv1EVf6dMOJVjt3qODciKiffCMyP+ZGJhwVDa78PdLtYVu
+rLNVws6H+xdqHdAyZXUQb1MGSPcNMOXnXHin9Io/eEBv04bHP8iig6IffVMI02gwTxySVCCgo3fA
+kaC2RIdYh6Xwz5vUA/Ph4bKB7Q0imO8fMIN0Tj+JB4wQBAq9ARzT3Fqn9N7+Pgqb44KOyaqF4pt9
+LAmoTy4uHi0+MBoCArf5nIPnS7LpRCr2wSqbNh7/I3oioX8UPkf4KmVleQyjHTCijags0DqJ/c/H
+miyaI2egoWjoqJ+9f2NKTyZF+g7IAtBIedshrlOHdacNp87XB49DYBao2etccuyE9wsxUZJxRf/U
+X2eUSdPS6AIAiycUh/+Oiv9ZiqKXhUU86c/R0xgkLLOqaHLyuPkFwTNddmkP/qNRsP53MKyb5eVf
+txxivJg1AlG3NmuVo7iRAuumf0DGbJoNJVviNvtmUSr8fJUPHsxxiYtS53KzqfPev70Z/da4y1tK
+ca9lZFgkzhVmMv3edcYkaFR8ypzn4/UoATAyJb87VsWfDH10HPo6QBC0nvkfdqJMV6MYpk2mZ/X9
+qDrzx+eP+MEG4RGxMeOWQfP/r9IbfXxYK7zIJalSmLs104V6WP99v6PJQ2PMMreo6x0JDXu9Dccd
+0oE/Fnp05yoIT32WLyfcK//OC2hFWVwlDncllPijsxvZCXJTm3ymibUdSG1UWWDNzF+A7HsHb3bh
+4OaxYoTXD+Xh89f4wZcj3UIv0MKrUNBLeb9TplRP2xbDEr+2ZfwMBch6hpon+31RI9vh2zmQov3n
+S/59rWBMwavcJjncnseXdjIblTfjou1HZrUeLFBZ3wuNieSVZlCe30UweIVftwn93M8X/mDLuMh6
+uhxAl/N3rDWL7yUJLHqD/oRa1U1mydLvm2b+5zyWx/PQvTQgXCH5fXR/1Y2Cy+8C/PIKtzrAa4wQ
+edMqh6NQFKV1YoN+tHW4mukGbm8U0Nz77zeaWGKBU6UudVV6QNsLbF2RaqjSR052jR7hcm3RtDuY
+JNeP//46HV4jbiMu28fattYfmYiT0ruObQv0P2CmO4Hm065GU/FEjfrRBnUMamJySItS9ShnRvOp
+MVGcB5ls547fA1j4bipUPcHftmfwRPqz/+GpKKURuqXsIVS/f6oVOZUaiiC7U9ZNGsJyb2xgXohk
+ndiNHz4YVf6WfPB396jWR5kKWCgKDSi4RHAIcAZmYNLXnirO8tLS+4cV5s+pTtgHi24mKdQ9vEyu
+8KOLYTWAKTcrPJsFxzZmVFC4FnDwNbo2cVmGn7/KvzM5NgcVqkWdyq1gHsWWcs5h2SKrAyVqgFwU
+pKtqi2e4X06rYIgvs3GqqvvPF+V9P3izTKGycnmvZA9HX0+VXhLbjCZ8j2NX7tJp0K9nhYKYlw7V
+WeQyOhJp2x8SkJF4AGqMp/x4cRgIlmjkndi6H8QbD+ETQrppE9uP08tkBpmJO1QNtqaLdxjpAuGL
+UYr//C1//Mx/LLN9hj/OYWYPxaRHuN9E66psvxs3cS2sIqUVlKY33Fplop3rM/M1t0CxtikYRSNc
+7uLKk+knfKo+2l988f83ViAyHJ3WGjG5yJE8cgx2PJCgVX+ZXZsDCdPji6mnRvv84T96xTS/uUu4
+OTdTt/fPLu0VbwpkGX3HMlt012AQOUs5n3iqjzayg5G4QBzf5FtuT/3HGwYZLAs1Uicgode+RFnM
+HLE14leMt0+lAh8+EDXXplAOtlc/eoGoIwMQECQcHSbiYdSBCGRQk5xIOD5cBVIJgYfeB/H7/QPB
+a4oaA9tUbILj1N0jUyTHkEoLBvTn3+ejN4d9D1crjXeaD0dpfEdy70JqZSFt0PcayPTQqSfnvoEx
+/OV/WQrhZ29LrPEAf/9MZa/6wdP4SI0amls3GhImnC4wXtBEc/b1f1gMtytacKTY4rgKR84mQR2a
+hHdiALMfxwHjSxDi4TQU5f7zpT76VqRoXIDIMXPDHz0XGCZp9yWtG9O0ynukLNwb253cE7Fq+68c
+B05Ekp2tPcQNcazFXBWTvaQr+67qwU36I1jRc4Lj/JTQodo3I2yfzx/ro51Bsw+IImglZlhH1585
+QBovbUZn6GlVQbZCj+syTMLI65MTH+vvZ6NbItkUXHx0Mo6fbZbCK3ow1RubujskUXtfu90FUDn7
+TO/S6cSDfbCai+4y9gl4vmxws/f7cB5NDbdxxuvWrNkXcelpj1g7Qd0R43qHRF90It/8e3/QWRcY
+55BHGDBdj85yqtsA9rUaUjsz9pdGrAs9N2N++PxzfbgKLoccY1oZzDzfP5WmTbZaUWcC0YYCq5zi
+7gYI5ylPpQ/e3ZYLMWihOKDpvP36H4GWdj3sKBdcfTUt050Q0QaZgPV7IcvZ/ma0UfH7nx+LLUiT
+yUCtngnP0WOZdtGlcUJJgMIYyXpp/Ewr5x89qmksUA9IwhIBncvjOKU0NMQmqnWivKtNVHR7tGPo
+LssqAIoBQU3nm504zX9/LeK6hf0mNSUp5vFAsJ0aGDiTB56vaMcrZ82ia32czfmfozuUCt3Budwh
+uhvuUXR3S/A+AEBylDGGelfm5a91g5p1dnbKBuuvB7JNQQXu6JTIBu7lR4cKpd9OG3WIiKJd0pey
+1ppdPiT/3J9nFUpT0onNLIEHer/9AIKC9naQG+6g4bZ+XrlI4czLnJvX09gA28t6DxAdPHkOP0qX
+7ck52UfPuYUNKnIiCBPH9z9BQaWzEX5BL3UFWJm0M5MrmVrlv97/XCebxxYXMzczofH9Mjry8KPc
+2njQwtzQM+dfFSDjs8/P1pZrv7tS6HhudiHbLNzb/nq/SJdWfTf09vcRjnBTa/d2elbqzr4Who/j
+DQkOpC/8Gk7syb+6C9uqkI1o68pNMOjoG4IlRK1X2d/VeOEl7lU57Yw6Cgo7C9f1+fMHPF6K3rHO
+9AGTHDquMKCPgkeKrsQKNBRWsK3iG9ROomCcy+lSQ299p9vw1OjsJbvPFz3eIf8tyoyfmaZBinHc
+2stQHbLmWiU++h35PfyAYre6ixt+vsrx7fz/q7jkvKa5GesdnTeG0DFywDxaAs1pBlSiba1YVJQC
+eOWnABMfLLaZhcBDY+KNRcZR1O/qGpsya0MjJhFrzY37wIXGjamG6B83Ps/1bqmjjW/ZUeSsLUvB
+TZwhMZTRAXGVf03ZtlXo/OCNQV+NSHIUF8dRJCDvUWckyFiHmakxw7bV2X/+jf7eCUxnYUEQp+g2
+0R95f75gHKyZZUNOjNKmoYrtExQWi3+NvEx+3q1ydIopSNAEUBSPCIJGPrpZL3ouXj5/kr83AO0I
+pFkx59imTc7RV1GFNhjxipQapkX2T6HQcygg6G66Es4pq6T/tu6fYYkEg8VoETAtYb507FA3o5Eg
+l4kpFlN0VGTIGTXI2k5/1WllewP4tt4P9jieIf5qBCrNjHNUcosTsfGvb0eNjOeJAL3lbhzOoycu
+WxTWy8R59lIYAC0yi4Gy81PZ1IeLgPDgnTKxsfXjRZB9QUY4fsmXtvR2ZmtaFxVedd7hn77ehoiR
+FEKMUFgI/5OjWDEWhfISW80+ZngJyOXG/YpuChRSmSUnaryjJ/r/pchysWplho2d4fstb0ZOmlck
+t75dQv7uecBwLDRxKkjo79dhoMtwi9cmTT4Qt+TxcIH/S2giEfeX57f727Nwv/f9/eX1fh+G++uA
+f78O+XsYBv4Z/xReX+7P/XN+z/U1/3oRhvzaWXjBr+0u+Ed+9/78/DY841ev+cPn/NYg+D/2zis5
+jmRL01spu+9RHVqM9b0PoVIAiYQkQbyEgSQYWuvYzixlNjZf4FZ3Awkacup9qqysKJDpES6Oux/x
+fzu+zd/YfCVfv/6IX/L53b1/3O34Npuvs731r/2d7zzxIzyC7ax/wq/5jWfbztbZ0i4/yzdeb458
+/YXr8lVP/MnOsz2Pb3x0D/Zud2/vPIfPeJ7neI7jrD/m8Xm+b/0y55JfHHgTnuh2bX6zdfZfvP36
+o95+Z3vOlePya956uyl5eYen873tpeP4u4O/PijPtuGTt84z37rlR/dXd9vt3dpNdNT6afdwyO21
+2TuHP/58Dr46Lv9nVX8YsdNATZ40rUra0s3BPz7t/HteynOene3euTvT0quz57OWTox71zaZ3DE3
+fPfm8fsxtI+29+3KEe0z7SjrsvmsnZPTRVu3FfXLtMMQPe5ubxlnh/5mSLYXB/fCcc5E+0/8iB+7
+8ORGHkhdnaCkfnNwn+6ZLYzT52NEhsuZV1qX3ZvrHfnZ1B+hjnS4ufAv1gntH17/5f/HJ5+1cWSu
+Hp4O/tPhWNssnMPTE2NpX26YWLvbzW6z2XibzaV9xQzbOxdbpvO3y8vX6XhpO1dbxpuVx7JwnZsL
+x2Z9evsb5+KC2bffnjHhZyfCuqu9eRtVBGmZ0F/uo3vPuqHHzs3q1+P+Z3PgxN4htUMRI01c+E/H
+0GNZstyP64Kn2275Z2dv+NW6qkObN9z/2qLlaf9yt9vtr9G+uTs3RV4j4p890OmW0plKkq+T8ri7
+P/rOr+0utv2Nv3b6wcfGuXeH1UwyMAyEZ2MDnfW37tG/d+93twf3scS2bezHi+8+X8CrHDf25v56
+oPtcrMjtbsO88/bM88r2rp4Te3/HULuubLs3TIgny37wrrAkvmtvXe8GO7Q/rAbm86n6ekH+7D1P
+zlZpKUyKxEzFYB/sR2zuYPPc3za+fftvy8zrYUQvHPfC5yE87O7nT6C8nkM+e4STg9eCtOE8rl39
+iHk/0AuH1a4d7tyj61zsdljr7ROrBWONxWeX2HhejXn1ffqcrWe77gLuI4PjP7m74xGDzbw53oa2
+/ZVZ5DMm7BLenlX4iNXe26+2bLfZHXe3L7vQfrldv/T7/fEptu8X+3to7zB22KHjLb99eWE2YvO3
+ztUdNpb/32zvvLvtLweTv72z79lFJtsO7Q1L9evl1dXXq/3We9jttz/vbtgpnBu2A8fz7lz7+ZKN
+aHtz4d6xRG1vv7/EZu+3dL1Lr752M2/+i+5mc6VF9pbtgX35cOFsvSuW+usPfrnjj1ejcOde3Dw+
+MhGdn2dG5HPrxcnt/XoHq1QKBlsMu+QF/zF3NweXLY+lbzvu/t+bnHNmHoCq+9RoArN732w6GMZQ
+0ixt0h2HI+ufpba2uu7etc0qsr+vez3mknWxs/lBrIN/u+7KDDQDz69u+cDOvuJA4POr9bO73eaK
+/2/v6DR379y8HmzoVn/dNVlRV6zc3etxYbvfsyDXqe6vc/Dor+Y0srdMIbofa+272OOLdRjd7eOB
+k467Pbp85vMBWHeH/1kQ+uvhj4yc1zMmZPLTBNGlLFH3LCIKoCMZYVyEai4VcTmXR3VaVfHvZkj6
+WJnIRBG0k2FGznAgrUmgunHQmm0y1fMl4r79ldaH2iYijkHB/aShj0FZ/ZjCtkO/pg93GnJ6Dift
+c/evk7vR6+PoZGisNyP8lB/CxGYho2yMglc5T5ndqml2MaEy5cdIDhw+7+DXdP3THqZ6QeY8T04l
+Lsv3U01Vc4gcM8frKGnue2quUTRVNkuQbiFJbLWyeerj8amXoBqqwV2h9Y8TiYEzzri6S3fggs6F
+j1Yze/JA+FdM/CyWTHXDaRI3la+IpZiQi0SpsZSXHFn+dF+0JJ9dI2lepH4aL7l8i1Rv/GOJgYSc
+SSL/Tefruq6IZJCTx4om8vsOCZpF7lFlH2wy9kEr6GXpUtZVuXWUZGcW+m9m97umTk4TtTTL0bxO
+u6jThV3KhLjER9ifOYP9vhWLqxMFBquL4v0LNaiNBEXGGuqXMPJlaxL8SkYC9POJ9NtW8HZLZGaR
+G6KfzCML+FWGIi7zqEySJ8Rq2ithEPTbz1v53eQgA5clQdiKlLqTwxF5sGE15IjdpLGUbIac4zKF
+ulLohWrYXYoVYltyX1V7ZUiGh7/ftCkzIcjjlj8uFBRvCmnMUXxQiJkeJkkbn8FVCTsUeLTrHLFf
+FG11/Zor+bmSjY9dSz0jbnCyyPFxYhLeD6AwknEjNAmyaqZaH5K0KLeR1Z5LgvnYtSaJWQydaIr4
+3U/TKCKxHnSxymcbtYRbUdeeB9W8DxZ9PyCsh5R+tzXU5szhcj06vl/rBIplRJyIfstUTp0cLSkL
+H4mGFDOCIGhIPVoVvJZtJSmx7qD8X0VIabchuTEopydfPh/O9zv7urOYEu4E0kzJiiHT+aRpcpqp
+8U9p2tSpk1OmIPHKKqo9EJTUoHbNuYDQ715VJU+FgimSaXFnvB/EWVoCNZSRKWxHVKjkKU++ZmEY
++JS/JWhOGNUWRMQ5LPNHW7ZmaZE5TrUPM+c0iSECAY1eDbLX6EwKTiqWgpuqreVXyJ66n/fnb5si
+lII2BxLT7Njv3w/93AWMNtp/CDqPMhuImIpeYMVF7kvJIunbz5v7sCZAIZPjqqtM2TWF8mTHFiYk
+bUyNwlhtQlJNaJAdrVJ4tp+38mGSrAWENLFmZmiQ6tc18+a6ZwXcoBekQdEvzs3W42yeFG6mR9pP
+SvZNJGqrRPU/b/JDP540edqPGboMJqApBwWOypXU9CUxpM7N62w483IfuvC1OpLMU05XpBPqJ/tC
+tMyRiFJl7IRz3e+QkMsdSraLM/PiYyuEm0iOJP+MLRWkzvsuROx9SIwa8RgrbTWvjoYFIU192Xze
+a6eri7MLq4p1xSyXTQTi37dCwbwEipME5D4IxNvJGmBZhv1uVozBhgs53Q7lfMZj+KFJegx/8lpN
+txbTnbriM8lQJqWlvjVuG8mdwMpojlV2wrWE4OXRMrtVRnjuvM9fdB3+txaTWCXuSYpsXtc0Psn3
+L5pNYz+IKXzOzo/t3hm9cqMcZPdcxOnEMaRjNN63c7LncFrs9Tqjncp9+lK4INHsn/vr589f5tVN
+/NnbKO/fZtLbCEEGWpE35HnaINY86Qr1PRcsnaN5ZETZF429h2pkz18/b/s0JvDhDdeJ+3ZtN2mm
+NivpVNiqzuhQm2j/MA7G/u/uq6c9uS74N+1MWYFMV0E76k2wqVE7+kKd2T44My9Od+/TVk62F1SS
+kkxY32bxQbY56Dk7hVOdWcsf7kmnraxr4s27KHEjqck6Xofa+5469y/a5vnL3TmgubQO+2fT4sTs
+Ul+WzVJMM7VHNZCDLJT9BQ304+IYD8iq787MhHUuf9bcicm1AIljPmhudL6jxW//KOz9L+fuy5lm
+fmMw3i7d05hJ3hatgUL7+lYIkzrE8BxQjo7p6u7z5lvrPiDheG7AzpiL07p0XHeVFa1tDi4XOxZY
+7H1d7B8PV5F93brP3AnsyE7ObCznxu+05lFBO03O1vGbne+LL24AlXqtH13Fu8DONr19pmPfe80/
+2Cr5xIqkKtIWqD6sLxk5Of+qNkLsuOfPzf/Tvflk+p9mUqsChMiIhDJ7LTS0h4AK1bLp90NqnHun
+c3PlxGiYRtKaxbrQTO2xD7YxCItKhkFbpCjEncsDPHE7fuzAE+ORmIKsoQP77w7MjuCzXMMHzes8
+xG7s4lWeMcSi/evcW5640z82fGJPxjAH8VTTsHIn79sv5VW9V74H10SBoaFUz/N9sY+PyrV2f2bG
+nOveEwMTdlOsl+uMUZgzCGIxP4ctpzwnsA2n8govdE3HdPQzRvqDs+V0Ap1Ymlku0qxdFwZ5YX68
+ldz73MGxGtgV3Vv6sn12H/+dASBPi9rKVcSA8rr3FrtNzbwQ1ylbeyAwWR+Ka3FyUB3rIncgK9+0
+14BGNs1GvbR2Z3r5d3b1bdsnvYzM35yRt8JZxR09/UvmR/7oz27qtzt5e85n9rshJc2DXBJqHchV
+PLkQJPBDkrmpWrsByiNKiKKgGqrOL33RuMly8/mrnRqCNXBGHZNMYiS1l+SSvu9VvYvlIMrUxRGU
+TvGRrQR2ITUx6Nt5OWPC1ZPNiaYouCH/ktJw00Cu9H1TmSnrkzwANA0QD7ooraKgTEvJztjQ095b
+W1FJLOI2sIqYnPpVVGmGx9SiQtkhlnJEC9zYN0PWOuIs58ekyvMHKsyl67/di3hwuFZxaCc3TV/n
+z5vTRIl+VdNWILThgFcecvnYVLXLb6AIZefm4mrC3u7xvCB3OBw31EdqVMWfrAMgic1iGcLsGMVQ
+WA6SZO0DmrxIWzZaqaT3mTR06PDnRjXaJBy0go1kdX6dJXPwReuKrkTXaRiGXZ3r8g1JvjXoxyau
+TLsSwVl+3i8fDt+kwpGyRA4CWeaWQkrR+45RYZsVnWHAFpeGARSckIUz1hCUQOROrR5QwKJrw5T4
+gOeH54aEsB9ha4WmK5G0tfhJpejnhIdOz5frIynMD7KOUOAHL/n+kQS0M2NRqiYH8lUK/0GRbRhh
++TfyMTSEZKvB3M+VzLYbD9MZq/lxsSkMGlUD+IPx0L9GmN9MEwT2hXGmaNdpOvOpJqf2oUMT8ogQ
++rnind+0tBY462RH4lUgxfr9S4btSiK25AWV40Qnw5USdLecE0TcSR96+XyQP65rXJj4vFBzooRW
+PM2UDA1xyksURh0DhUKvaya4m3V45o764ZLDsCF2oVApQ14fW8D6xm/6LiQ4oSRLPziBEAX2BOjd
+TvJQsZlQ+T7ul9IzsiDzZDFRDyRZZi9aPktnLNjHpcczkA69FpGT/X/qaZuXYQzLmtVlgtjQvbAM
+hDs1FSnVsDokCndQJVDY+9u9u9ox6q7JwJbw1L9/71yLcqXMAvSP2hJhwllN/Tw3lO3fb4WaszVY
+QCooAibvWwnHgdjUnAyo74FZR6AS+EM5i3+7/1RR4UUkPGtretLJ0ktnJTU68nWdeKyKQ6a2khsL
+iAKOiLq7eT8F/t99qzWVlkIXIiDMHPVkzsiz2GaL3IHtWeJwn5TCsgtA5Z25JHw0KKasIaXBSxFy
++1ALghgLIb3ZbB1DiAtXFJElzGDnbEVTEzwz10YE+6d22AVC+1em/H/8mP5X+FJe/9vst//6T37/
+o0SDc83mP/ntvw7xj4ax/9X95/qx//6x9x/613F4abq+efnj8Fy1f/h98fO5i8vi9DPvvoKW/noS
+97l7fvcbr+jibr7pX5r59qXts+61OZ55/cn/17/84+X1W+7n6uWf/3j+mdM7cds18Y/uH3/91e7n
+P/9BiGS97P3H2xb++uur55xP3v2f/13+cf3cZ+VvPvby3Hb//Iegqn++iqeRna5g//ES/uOP8eX1
+rzTlT8obWcxrDjT71BouKMqmi/iYZP1JNjbp8GvRCMU3q8Vmmb3+naz9uYbVqA3F70htGH7w/3rE
+dwP3PwP5R9Hn12UMU/af/1gX2JtdnS2SOgQylfH1UgRDXdb7BRhVQqFMuSw4ilnq36I0fuQykZ7Z
+jj82oq5xYdKUCZBSjXVydMjKOYt0IjTOnCloUopl4aK1UJ0JhUDNPH2ZtYqN0gpiW6TFWsbJSW9Q
+lVTvYytyC44eptPo6It6I1ifl3TuzYduVNInxPZAz2lJSfF1C4oI8XepnVCATsYfZjL16oU1hCnO
+TyhMh8Joo6e0QqzWHmQrOJgh0iubNIhUVJPVUJiejMRIe3dse/2LGi3jcJMoUmbteyLx2XWIQLZ4
+WYOH6N00TwNkNakieyJ8nh6JNaqVL1UD1JpazqLUcJCzlfrvY5aJF+LYrVT0vkpsDQyRYvNewCRk
+iENUqfaQSiEvlf1T3MiR6HSyNXwTEzEGHIz8tWmHYz1dD/Ko6zbaxclPHUHs8HKoLKQkRRnaqjeC
+QwBSIkrjU1LUiAakc9iol7lVU8S9hNMAw8o05kd9mEb4k1YUGDZI94FrFuo2NQIjaPU5YcQlG7RC
+rryEVTNfmiXoS0cykkCzCQOjl4zXWOy8YilXREYLlhXVrWilzZX49BwB2N1CVFXuL+M0pOgYySpE
+wOsJKmOgyxZF0OIqCywifv2jSK3+rmuT+FfX9+O+i/UEBpYiAhKsdHBnYSqqV1SdNgdOQO1Nq4Xk
++/cE7i+6vo5bdwliiEGB2aWWg0zuuEo/S9K3QE70q7BQmsxeq2heCJh0iT3GsW7apkFVjjvDb86d
+ycqt+1GZQ2tDma51PbdZFUL+WhGksWwhjB9DtVwVsRah8qkukH6IVWLcBvNY9ugJG+EVzDm6sUrn
+pUGOGdV9G51dKTtwuGFzylMEl9BZNRG4DUFbVp4ZV/lTir5jYHeIi/oN8ccaNopV/JD6pgw2VhqV
+PzAR+fcBmjz2XpAhpNbqnH2Ja4hGtlXKSLFLEqrxQ4fWaNot2QFEJTM+1+PgCxzFBG34YgoZHqHJ
+rxfkrnSQy0bLFlJHmU8sqoU4WJqAyeo44QXFfCI1nwpF65dhjtNzTCU3PuBEFB+bJR5AYiJi6MRq
+p+V+giSf3Ss1ow8uYjE58kpVvtWEBTKwgqZsgHxxCgoqCdA9ZEmJzX0r9wj41gBInNCIC672xiSi
+otppCoUUSZWp6KqaELXCRSUWUuohRWHQ1MybGYnoDP5ZIFxCSYtQcY3S9D7uhaTHzSQIuReGWguS
+hCOd6KbhMt2iyWzeC0rU/6Kat+KA16faZSorY+wWTTyh3tuNBkj0utR/DNKUwkYOR+PJbIoWnzq2
+E8060aruQqNMvkhCkZIBM4mdRM4/uFw36ZfiK/CUNvJzCfaRi2LwGKEimhgqxkBoLS+Y5vky7Fa+
+plou48MgqCBw4ymLyZgQF2nYxOiJAOoiQpQ6Afq9YPXEpGOFmOoy4c0SM8up0N3d07WiW6pjeBBh
+gBx7Yl+3gbQxtSu17LXJLdtAue10I8rcRZeZilKkodvDWT7xi5Gy1SHtqYI3OYzBMBQCVfU6SWuf
+DLT2jb2Bmu8NGrrxT33MkKWPkngWKSFHKNsvwhDJYRkK8K8K3avOpVBK8FC3BPeiUgHTQOfp6ush
+1iGtAtQBGssRqtoJTTlqIF+mtPXDIZvu2zFMcuSkA+NRjEfRuGgxWqPTKKH1rVhATCCfjoa014pj
+Sq1ZOw73IeYQTXwLLgOkwRkVQTVCMs4WE8Ty7TCts9sxbaleYSJrgy+YSnQDcHHejyTKoHZADXTh
+AUcHHpTlen4J3HVpd0FGBMceky4jj6YKLbBQRT1zv5Wk+whF48ZusyKNvFLqlDsoMmHFkM8GRA8r
+S2y5TObb0NLzl0mvMGNS1AibrgsWz6Q+Z5+OK6ykBMEB/qI1M8ubtBxF8hg2sl2EgGPsURj60QNo
+q36HqyuAspOFtEFqb4KjzWakGSC1RCRh1bQFAi8YMargcca8RrQ0bi7gKFAWpDRNCUxnyEPDNaYF
+mhA5QzwfB1O1dKSlC3d6uV7CwTCFL4rRh/pF2AIDdIOshVPQtWEkc+GAw3XJPQG93JTC7m8QCZbJ
+G6bZqJyoamQFYAR0ZMyEKjwtUwyhZRStcSEcqoFsCCFw38W5PkSbYizE+xr9HABFkEqtbYaqd+mA
+WQs7z4gr4A2jFGWwr5c+gcieRAV8GU2NL1otAdJTChYkhbBNe8tRlUD+JpqlUG81tUG1SylqNdyJ
+Rj4rzqgH470ZrjLpagg1A22LSVftQRlkBGxNGLAOEEqAPmGfT9+XdEErK3xVpRPzXn1AhLfPN2HZ
+T9/DttDzbRtr07IV+w5jpZoJs6wMh6C6V4MZtQEFywjEZkBs21TCXnf1qbaeRgMCn99DbB5dUzYC
+cQNSAQIx+SDWpYLMDIIzbIapV4hB1foTiWwTW9OSiKuwNhpU7AtzvIXJEGGuxDmeIJZKVeWYLY9o
+akX4M+ytsfRHdWY+lMLMLDeXdI43qTyzZ7V9O0uMSsNySMeGRy9BLylYDmvRUZtXNMp3rWgA/Zdp
+03yZGinYiKEX2jtSj/CsoplXOwnXSziiMnhDB5QCijkgwcaXVDOKK4BR9eIpbTHdylhKIHddEsgb
+K1LMdrskhVo7YVko9Xasx8Q8hksx6N44m+tXdaC8/XSO6PmozkxhO4xDQ9RBwhWzjxOONjtpFEpi
+HmMg6ohHmGwgVK4gfQpvVdQcSIxFu+sbgY5ELa509DEccy/oJelXABugXvloJGsly1CE2ySOJc3V
+QnDxXjuHYunVhV5+baNJQmxEKIRLsQVc77TKwgHAGMO5xI0RA2VKwQZ8LZsmCHbQ1ZhLM85G9OAH
+nC1UZnZci1VgHt9NNNnrTZgg27EbEbkPOdAUanQlKmMzXYRQA9Q9RDGmMTkl5nLTWm2cwcYEP/So
+lSvIDVzU/RjpIurz7dgHm5Rr8U5JXx+iZCntykyMWSiUOurMjriC4NBOhuLOoLytbVWLsnqhxIL0
+UFiTnO6ZgTrJapCykDutQIJ6CHbqT+SLJj/TvitydxzztN4kvYHWfYEQn+KHQqZ8Mycgiq4CpOaK
+pO5i3b3EfFN0Aq9QgD27xVMYWCCoOt6GSw14+KDvqq8BaKHOXgzmImcvwFBeSQuqo4oykEcYfjVQ
+IkH+Fi7j9D1BtoAprc7Y7wZ/UeguOGB0cCkqk7QpalZcAmioYfJLTORiEpngIWRntFgmjZlklBRc
+uks/1nfpYuaNUyS6wOm0kNQH+hUEWJopiwelpdiXY250ti5NyWPWLpwfYq0WSQBA5bpD49pUviax
+mOg2Ou+YsqCNTYgGcRlqQBZHdWfiZpKcMF8WcKDkYkFzGgwOlAP1urcGtz+MaB9YnFCV8qdVm+Hs
+CV2n3poQVkCWFT0nRDmcp1+lkc6GGyCkVTuBVQstCMowe0GvCYkZLhyN6Cf1GP2omqHLEfvu6tgD
+Mz64WQbCwoPOkRNzXNr2F7XfAgRlIcu+WvqUIKRhmc2hVlcYdL/oy3WYjPqXZYHhYNe4oCE7GqP0
+UEeiXG8ZcVW250Lt/BmgfeMJQtPHbpMq2rfAnIF0GbWUO2LXs0np9G3vxRJ4J6qfheYCa1/lThC1
+4b0QG3p3M9W4HDzg2AWayOR9KH7XNZpuD0NSfFfMFbsWDu0T8xmscjsImgMsWwyd0BpjhGGQh+vp
+SkE1bKOIo8mFpwD+th57E0EeqeJJFomTQR2sbAMkbbqFyJ6pPkOQQF+BpRn8BHtipc6IcP/NbJbK
+ZVhrEbDezMyGDWenWuEMFaaJ30WlqG5HWIyHZoj6wh9SsftpKFlpeWOYqiqKcrIocIDAY+8MCYKk
+WOWwfxJiWb3lljbLbm7UC8l1KoikTVqucwIdNq3wILDBn556ZYLr0iAy4fWJmlwYtQlSXNWH8Ucy
+gehqMyES/M4AC8pFaWwABVXsl3Yjjo3upabYPiE3jzFUR7W/bcaoNDdvfBV/OQLeXvxPvEdc/HFR
+kTeIkAhl7R8EQ3swv0Ne8n4hZHn89rz9MaknyxMQRsU+ciXMi6rwFZDj1583fRotfW2bBFeuuChI
+kNJ3Em62klIM0iRXSAqbise8DhQgZZzCbHqpIU4bxgBmFC5YpgNMY5idqgoLyRsBZ0buGMCS2hQg
+fMO7alyky1qblx9Vl+o/BQUlfRhXGudNaVyCr63eJ/IZZ+KJi/v14amrRggKhyI+iLVj3ziEyQjM
+ZHB2soOWGpedcTFZo2tkuV+av98UKmC4f3AFESI7LfGuMjFqUvTWWGcDeKoaAtikgGNJrbo540xc
+XSPv/UB47WVcTfyH8sVpmUaS6rU09SNv1YrlRRQU1QacIxAiwQhvYf+BfRv7xEnySbkcFe2c/N+J
+h3vtVLweuGhRGmRKntZ+U8ludR3Ed44PobkRFtISVb3BxIqCwn22FM+EHz96pIg74jgl+Eg+uH7q
+karCCRm5QA2wDqm6TbNi8OoYVNDnE/3jW71v5WSqpKSjCnWqBE4liAanS710svWwIUXWzTAo2hmX
+/WtWyPtBxJm3utJRBODSfQoW0Aoxr2JTD91uVuIrLZu0m2ouOYAYhSDjzkgrSZ6+S3qQBtsolaRN
+n4DQdtMaDw7esqX9ivni3MYZMUN2YirizO3bXi7B8ZUG8KiukjuHGQsirIZbdj9NS3svxnrwFJNw
+fk6UQvowSrg/Cb6ssQGN3G3rxI8uDFGqRTEhuwX1AY4ZRTnr9jiY6UHJ0uQp6pf6K6mC2U9FC0BG
+oiug5k4k9krhgGQUuCt2uQF1NOAY48ZNo37/fHx/83zogxOZQbKA+JO5jv8bU6DMak3s0wqxSVF4
+0DqldvHzSmdm0WnOmIr7B+Xb1dkvEVhGmvZ9MwxSBp11iFxrms38oonTxHAVkKIklddpKjoU+cCf
+wy04fF+6SXsoJzmi6iWri/tS68ZncqPRbP/83T/M7fWhEARF8xHxAfM0sRdIDAlDQRi7evMD9Hey
+uBXaJNtOjeETLPnf7enXRFGq182ViIBEz/su4CRkqAK0DEfDQKA/BewLPf+/MiD+f1jjTVgDQIYl
+vxnqNXDyLqxxiKHR/bF5aZ7j9m1g468P/hXYUKw/MdbMRpT5JQRV1ujFfwU2pD/XFbuq3q4x+FfU
+wn8HNtQ/wQ1x7kA1DWVSvBRvAhvynxbTCQFmphaLCjLP3whsSP/es96YQ0yGyi2EmCkBAXSjT3P3
+h6nAI1Oo7GmEpK9NDTkO0hUGW2vn8krO5Cc0PI6zFUee1HH1yE3RUUDuOTL80cLoped6Ga1dYsah
+XxkNdWvhENmA1HGH5j1OKiQaPWVMAjSc1HuSoQAm5WVxxQYXX4ZgLm2ly9JtUye186rMIoZQxNVJ
+hkGOAGvSh9d1G8zIvybHIekrP+rmWzwlm9YMcfFEpuBWU/M1bYRpJdhzIioaNsgG4G5ca+1DNVvN
+JdjXwOM2Hu/UhJBHMTUPtRm1F4LYqD80LWj9vIEpbdLsJgUWb88w8Z57o1DvzNRavIQzuh9X2k8t
+Kq6AdIUbUet06gH0qadbgO5IBAi3hG9SB57KN0Q9qt0kmM11EoeGg3QoyUGTbG7KeZ6vUDo/hoKR
+r+L60iaTuGSpyMU8DeQoA17n3qIMFpBcRSDoUY13LWdfv5ut5NiqrYwrBnEluUT0tDWE3kuXuCTw
+od5MQqG5HEkmu14dunAYwYi2peS1euHPlCPaityOHj5YtJGaQnFx1XmJmhv7yGyuBnNJvK41Zxed
+6AcYAQKa8tybkNduyDpvix0b2GCLTQWcOUm023LsMn+uzR5nPB5ELHruLel4u3QSOEo1SnHiZcVe
+C8rdoE4quhrVws0BrU5SgOqv0kIek1CT80Dyeb16PqMFPryg7kBet67cB9+bpBe9irDErSkIX9hd
+PEI1k0+e2W1ezdf4oUieiwUIqyZkvD6Sv8pdTzZmRszEnHtu58VXIdM3+J+/qkHCvMa5b1shsaBl
+aPZ4Psiz0RLYUC3VmJOVwXmHK4f870iVXBKgi9hVTXMfGipgSABfptV9hQzc30cCjHg9B3W4tM11
+L0yW3bTaeG/g5ruUxu4pT+eHZNK+VFb7K12WxBGaYVOV1pW+HqputEnof4FnbJsdSE8gK1zdusJp
+S62adu08TLnXEx82LkAmT0+z2pi4LSG8X6lIKCLxn7C7HYclyI+9mcEbd0Q1Nb90QqVLiaPPuLkJ
+OjVq5U6ZJRwrjUC7jfQniuYURFqLE2YwUuyiDubKiwJikTiDcWo+FKmCvio+pdpgLKSIZMEZ++Uv
+2phWLvIK6WTPwNrUQwrd51iUVVhdKQ0+I80Ta7kyZVdjDdS+EsdR7uVjQVYE+R5S/LMp1QAUOofW
+EFBYXn0BXabfTD365G60INToiIYASEfPYcHbsh6O38BaDSEYYzO+CjvVMDbA+pZ9gFyUABfaWF3O
+S5z34E3KmuUGHYzlTvyw3vXD2KGQpMyyuUtHVSOwKEOchflqBa4+12ntqVYm3ur4JhKnU6oidIyq
+xk8USWOh+Cn+SmvL/crQiOeMcpVx6ZqW1T/axiC+x7oXLXSXgl6HUx3hCAHXaXVbAYyu5ho5eVG+
+TMlB7S8BZx3yeNUOFKaWWuRS4eCNfBMPFwrQOLEspzM607A1GElfxWFuBXcKqnJxlqrQHnB0ZBE4
+1rlMHBTc5tkNs66uuSoHOCokY5nwP1VNtCujCJfnrMftV7JdiTAk0gLsqW/M6GZAUlK2LSknDhMC
+peh2mZFaa+lKZXZXeWuQFteG3dIduNDGwlVjFTGaj0IfzteW2JrdvQCEq3WFXJO3oBIY4FLWhnSX
+BgVYUKOKwYBljdBMtqxOI5zRYHkpWzW4Jd5Ah5RWPFseIByyFvW5mQcychpF+4EnU70maEqFoyrM
+z+o4glLXYwVYOKRHXC4Fe6vllBXuss2iId5+MRp5LfuxpVbaNjTZNG4CuTdSrxqtfnaUSQNeayp9
+PNko6U53vT51x4a93odIOGwzbbkQhSi5SLsGXHjRFTdaWF9Bcpk2dWqObjQak9+3YXkMISbalSWO
+RwNlERu3Gbluc0UfD9H4LIXJsgGNfDU1urCZrai027gVL5ErJ603n3aizmIrgqzDgQu4ZZpCV6y1
+wkV5pT1wbZ7tReo1Wzf62Ld6CWllQya0bQWbqqEqUUml2EvBhntQ6e+ycLgJFe5hFfunsxSxDmpK
+t5pDMqdh+tCIWSpcBq26hUIMbbbqqMRTSTx7IiCVTRtcxddFqVd7wgK1HVuLtitD4Uqr9eUiFbJN
+004UpEdeGBQHHO3ioc9wfA3Bs7LkCjHV8ldTAbKI+qnwI0G6ji1inWJiVHbbmkRMMh0QfRdgE8rr
+YJ2huYygG65tOxYmYQWHxvaAWvdVWZejM0eBT9Fexj1L+VmN2iOhQnGPIzdid9QPQWFM27Ko9AM5
+ZYNLDiJ09FLeynPpCVK+1Rfp/7J3JtuRIlu6fpV6AXLRN8MLeC93uXopJiwppKAHAwMMePr7edY5
+q7IGNah5TXKQoVBI7o7Z3n9r7Xs1yB93dSKT0tdYlJXaU6c9tIDwWhu7I1dzIbw3cPnn3tCHw8IH
+IrY1egFMmQfhYPVfEnZkiJ15elTImhnQmZCWzcA6b3JTNdCsQvRJbE8jJ4YXWKeC0vfdOGr5k0Mz
+fFbSWK9535o0+vSYFTbmPfi/ynnraK3Ooqy2zXVH78HiXqbUGE6mxmy29YJVz8nPV1O66evSdNg/
+xK1NeSFU/CGoFpekuqSXepg6DdWX+qTv8qBdNy0V6NPJXnVRhrT6Fg8FffBPhZcQfTzlEiV7bRvt
+j2L6Els6QBznOmTkWcZjvtB7T0StaE41sR/7dl5dsnBLz2+sfZ6thnGkDwWmRpVmRR1KHnTflJZm
+Cn4RoH2vBn3gNZ1MZziMssuWnRj5Rgc0hVbVw+4C8Hw0WlY78BnUYPbbouhtTmizq5NDlmmOR1l0
+YhfHpRQLkDtAY39szCbP4QNujKPf0Dh7Iue4TMPCrYyUEYQ+ibfVo08eG7Sd5jIyU+nKMxUgdR92
+Vt5UV3fR1XjV5TjTRSk1bU02vlLj40gZlRZizG0eAr1f141CytY9LMw8H4OdTfZ963rLGuFynihK
+R3OLVRBS1nuih9QZdqtp5D4oH3xu1GejCOLEnVumQyYqseenkLBamfKzg6vnThkqRgNy3TyVp/qm
+lEZ9LOCHmBoG+HwtDYbspa6XktUPRqcC7nYa7dFc+w+nLr29r/v7HH0fKF/QbY1q3a3G0u+18TbT
+Si4hL6DznEMXxU0+Puc2cHRnGr8hcr/KnAK1sLYo1mZ91/yoBN9+Gu2EHxNyeFP47Ysa3CPw/4a5
+LQ60gYxMywYe1Fexq6XYGx7Bp84QpC8FdeC+0Z0NF3lhW6MocGSNYh+TVOgS/efynGxdzQ4O9o1K
+Jw37OHbtM9Y6Si8Un58GamVMtNhox3vZO+qBF/gtK4pbg1V1r/vlcaB7PvKgmbnyuiOoZrFPRufA
+SHR/Y+w+OMbmizNgB8+zp1FrtqNlb5yqIqdcNu9GYYycOG2ybd0gopDxterEVQbjPjObr8pv69hp
+8ifawx8yqcGqJt38i3rmD58nlCzt/IjIpttDSh+dMoutWSCpLwRpl01KCV25fhkqOVed8zTQ0Bxi
+6TwTBKGiwgu6O7q/Vdhat4nIDd7sTsfb0LZ/1ikdICkMdpWB39NTF+qXThNd9aCBZ1dqD1VdvK6e
+vFhLS0O1lR/dpPotxqHY1jLVwjyxsp2VQXeqrn2/1RdEqDb0MFkqeN1KiK9p7J9G3Xs08NFGaTqd
+MzvYs0ttZTqexlkSvU/vQpT1lO82kmF0TENvGQC2jAdPWKwRSlyLwHmAB9jiI3idaNpG3yQDHtG1
+jyycs+HiD+9c1TfFUnE3agYuOBBGRt33Nh223dJxidNdEd0MtotSG2sSR7Oh3LnQZLUrAvGdmE6/
+S5X/2aNqsjIHxj44runy6rMabYRFH4NIne85YCi/katWryKrXr+mKqCtHmPczs6r94JliLtFTP7J
+Htw3fe3WH9JOp7vEzl/IpByegLejSbdpQp8PHAOsrfO8Sbvk2NfLS1nrp2YlpRoJ0VW53s5p3DvJ
+7sZ8uSk8fXpdxvFuFfO1ZLG6dJ73ZN/0Jqy/Oke9ifSsn/1DPhboRZEj/lKVHy9OIR5pP7U+HFu9
+5jSIx3IyYSfpKt9SH91HTp1cs64VkRusWhzI0jwlJqKJRRq8PQtVztvcNpcrLrlrmfgiShFmnFAU
+/EYElYa31sU7LhsR3sizzQpe+NSjRjzwPcw0CuAXwwXl+qbOix+oMB9GZWoJGU86qlmCcbuOTj/s
+7NES5k5NyC5CbtuxfiuTGXpalhIO0lZTcm9ThYOoRB+You7Z4uDdpWnm44EYaf6WnWT6njG9EPHQ
+G1m3K/NJFhvWHptq3dYsYGxhP2EUkc5VdFL7khxojU68kl+pd71wDRboc6t0+FPfH28sZa2hMBgL
+iEkVSA2lysT/NdFpFHewYaj4Kc6dn6cZlcK6eErdTTWm+xiJZH4qdMWPjtomb8qIy8JfoxGxGQNb
+vwTHkkhvhPrE/UNPBobgTFiKzTw5K9Ns3/JbacpFeKcptdWdDL2Q1Yipv3NyKbO9yR5zpv2dhSdQ
+NSO5lteMtJAZ7XeSiOk4slilqHXc8iDEkD6UBvKykyak9cdKre4Z+ST9Bpqbjgy1M7JiKVg8xax/
+OtX6ntpWcZXd4PPCtUF2bE3lT9t5Nd0inDp5HPzkSlzF65DPJxwaF6ktoo77wdTPtTcHp6aGUNt2
+4Hn1znTSfuuOzaW3tNPsBSw+aDDDdJpIXECouSnAY9o+NyNw+m01jWG39iNEq3Fs5vVqq4oXoVsj
+K3PvTNnGY8eNWVvjjpj5V4st8JR56wUNQTT3qo36SickWqs/YRmWvSxRCIw++TudrC9tq5gtnU6F
+s2G+DpVcNvXqfnMPXWZ7hky0nmbfzZIDieBAnI6VaJ960ARPyaKbyWaV+ZBuKzk+gmwld4TyG5wW
+Wqme01ZJa4Oep3pER1MaYVGgut0YrHNLDCfgDncesTO71UY3GbWFjW7GalVfniy3PesZ0osiy9g/
+JpPo6a4tzW+pDxcTMCgx23jQZMfIptrzEEzbXBdfhUktlGqh5JW5fkBqp7teM424UV7GyWhuuYx+
+18ADjB5Bh2BuLTixfPOR9ZHFn1wIqqiDwDq3zfIOmPQDU4pCNij1T+rQj7k+tQ/zTBx7z4G543pe
+m6ei7Bj5fNVZ7rW1ESeGaX0bvSa5aCdW8qCn4VXwJXrrtfD5rio+2X54dUadM9POXUaxVEfYutER
+fnBSmn5CUlFV3UQ/dT1SmKe1/oY5lMffTj0GuoKqvgfu7hRjC9GwW7Xa7nbN0QnFCYt7FQEALG9N
+bU2Exg+y/4bPcLnTlfQRWJS14oFOkQb0576ravnYj+hcQ6/XcokvqJ36TYCICLGUJGXqd9cE3vuC
+VgaPoT1pGyJqFfzsUjO3Yi66jZkW1lYEk2Wvb5yp4KaQlqa+BCyGdmyGhagU+I48JLmEbVXv0tCg
+CPAJld5wMpRbXm1peX/yTu/o/mm9fQ2kyKw+AOsJof9uLfA4aFHY7LoaxYvnZ4pOxOUqFjmFdarL
+gzeOP3ULbaf4AG2TcfaMo2jMLjKV2PStOQTHbPande+aaW89FAuFYjz9PpcC4GA5RCynQXFUAYqH
+2KBRLT1J1xdiNzCwfne1n5M0rfvLn85Ni2ADu0z70lCWKtih7R2Ti3Lb5lhAronD0NhTjoAL08ih
+JHIMWfGI0vpEGBcrS9mBIMM1c2lQMKHnBUiMAGzLa8tPj6KCvNzAnXHwpnJI7m+ZY0vU6q1NlLY/
+v3dQay/Z0ukR1axVNBS1EaHznC+Vpc+vJDt/tavVH/S8BlkC4/mxk1ulkp46xafy3GqH67hCgqRc
++2UqK8MMpe5oYeewM6xUuT1ZZbbueRKCADSKfzuGHZ1UpDeZN98NrZbBVhdWktZnrxSz8STRgcst
+Z0zTUVaJvm1v/a3gmmaWl0NpJrL4XHvUL6yDKAFYXLv1WqF2nD/noqXFnVaDxXl2Jh1xY9/rKKP6
+vxVnJB+gnegbsrNA7jz7BeVT0zwyBIvmwfKXvH8pFnrKDkOCxYtwhL8FcrAwxRoNnRe0m2FtpyY2
+/SZwECYWbb3e+W7Ca6CakXkhQceY7Zu2HajA6LWyeOZXMVGiBGzvW0MveaPHwE6zh0q2vc2lO5cf
+CW1i2ibtdc344xhd/ZXz3vxh3Tbqd5QmyHpl1sbSqpAj1xkl8l9jWqCN0lwahGMa1hHxqb9FjE5G
+PdB9UjXDl41eRm00PjGAkZT2nXLUp/6263JX8dYp7rMhbYNuM5elYInDXEbnxU1/mXADGVdGvd6K
+xsnq71ItmLwtj0mnxSNqVaQqqHLBFx074L92s0bGrK/uJrmpQdl+ECcpdDFIRHqDj6e2uOaKzKpL
+v9HMJkHoabRCHTnYtDICmls5IYaEQ00GTX/7mStUWQSPcZSJxJXzJbCr7DDCPhMOUHm3/X3M+TAP
+flG4G6LN9SkGKhT8AISglDuPJ+syu1WV3s/YYHmGUGTREwsHoKX15L6bY+Z9oMW3HzkjmAI9oXHW
+dx7j/5DF3cAgFSjGTbiN/Gvq02zjDf14WdtuPafTYj1WTk4jDRz0VqH8vviTdeiGwXxd3ISCAVPu
+yaieNwm450vAj7pn4mBMWnORXAqrQ5Yo/RE4E6lotXbNuTWmcu+L/jMzqELWdXpiWsdPooUj99JX
+7hwmbUdggpm4nIKpfemT3D76tmZEwrEOmr/+1K7CDLqYocc2vc61Hi1mIOIFXtnvZRKpUVYfrtE0
+T+jUrP2MRDFcxfAo/X7fdP6jDcT3G176OfCqI4INEVbMJPFIYP5TM/h3aSDQ92hphP9k5wUFbXG5
+t0mRfW8J+0hfB9//npokQKQ+GUdEo1oXFwUhYSrntUBg5joVBXNDBbDjuP9ZjvV/VOM/qMa/O1v+
+Z//U//vd//yTYPz7y/9FL7ruXy5n69+V3zZ87y2O6F/0omf9hZYAHSMdATRxcGP+l2/K+4uG8Fu1
+BBoW5Dng7/9FLxrGX4ZNbwf/E7vo/5Ze/M86gn+wixalQdw65AIYNrw0nd3/nZJOZ4pPeOR0qk2n
+rvrUF6OKVd/BVAnTooWkdEbg4HL0KI8TtohuI8k5kFl5bDFrXEuopfekq717cfNCCBq/n0DuYXva
+SlXhHKSg6Os8SiidUs3bVFTJvuvZaBtLGx6cYHYRrQelvTM8wMR8OshsAJltNa1jDV3Ee9B6KVlb
+Vqe7yHtrbA8VUglqL52fObOHy4ACjqFlNrKjRxIl82eSXCvwoyJSQrpn26A6UmS3NL7WWWG5XDyg
+N71ThBG82JjVCGA2rBTX0qR5ZOibyA8sJ/NOFWP/oHKW+qYqwEaIvP7jTM2UR52dBPdF6ZQ7WRmY
+XUycT3fFAjVWaR1poIZ6wUenk/Rj1ckbrEty149uesRlFdxRzvucD0W+0afOOpbI4JF7wEysa35d
+6YU8gsFlj12J7yqT4OZWn17ElJtnm13vLenWZj/7uXdYtBbsYNat9FU6Dejmgs8uRsOIQn8u9Wek
+ZBhuysB/JdRUxKuCSrIR+u1NE3X63Gq4f+UIno8RPvWJTyPxrxnbFA/MzLaSj9lyFm7D9YEdKuqW
+aT2MTRpsaqekHSwzHqeF86po3obAAOEorpSh06foKebxUoxQKoMRMcoOcb44fkToQLG7NQRGeVrR
+CZfOYt7yVprhqlvVMUU2daIHDJU890YYmHm3NbuVpR9JV7x0rkSIeSuT98lZgJZlVvZa84DTr/la
+4XY2K7gQxPfN8sGy17ArA2pFbmcl942wH40mt0LfbplanahPpR1RNtU9Lr2ebtcSwhJ00tsrb7hx
+FPy+pVsVF48ANoYGy33gX2gftdFk4pNGurUQm2/qAQtQMZVAHf7Uxmy1anioZ0f5W/rNO6IMZemG
+BTaVyQHXgXE8Iukeil81cJ60N5NSQe5cUsnlsmJwa5x6X3cenWsRkYSlZW/LjoI+Im9NA+tEbK9d
+1hpnYWi0zYWzidfLHUIii0o1PC7oC9f85JbjXBrXws2bg3K7NLZk2SJp6ai1Jjj1BzyAb4Q4dAsX
+l5/SZWq/3WztXpLanWO9XJZDHyz5e13gXwkV2oTr5NwU+D0vVkblaw13ncnN6PvtYyULsZ3t0sKf
+xoW5N3rl3tEIURahBVH8sfpiPKUE5kfubBGhgGTgQjZh+VElXrBr2OG/GlMEu14k3nnt5KpHjpmU
+uwwY73Gd0w6NgygzyPAOfe6k7Prkrv2NKsp8Dil1Kybxh9EFYkqsFkvH6F58kWRPZKN14MB9wK8v
+6FTG1AMJEsBKVo3fbNbCdo7FtLh7zEHDVTG73DbFZwspxJ2ZESFEyjANIEhax+7Dgbx59ANjQEgM
+mDz7g/ntePnyupQVvKyWye4Os/bD2ljZph55YFyvMJ8WFrxHT67enYe/ZZPnhXXVrdF689qVBltk
+6NaeMmRHHY25BxEsLcHr2FAt+CczDfO5F156r8xqtSJZNPnbrGnymkGizaE9GN6TbudZjHMAQYeW
+Cue1yVq2gU5Q5mpmIBLFXMSGZqF/zbQi2AnPXzGjYIYHHHAAIFL8gqjadU1eaBrIODGr8mEe0JXo
+6w1/bNNFTwEZKDJKEf9TR1km6303IaOL7S5Yotxk+g8zUPVfKXpV0C6cKWHa5vo+Q9tOv2x1820W
+g/3M2hB81iRCJFvTsYaznizOU7HMBN+sun4Nqq56WrPAOuZTbn+qPjAeakSW51lWCDeyxVsxXQ5W
+PHuN96fT+XEoDhTTFSeXuXGLvDyXhtTec9KLul0+a94Fbeeyta15OnAWgY/LcRm3HpXaD7PRgc74
+s3PK+az8bkG8d/MS6F3Mj+qGN9dRXcS2FNZBn8QYAz+igLCsKZSm96W7g7+jHmmW4YzQki8B849H
+rspYMwTmBLfNYtuzxb7QHAUM6Q6/XTWmdwa3ZTh3ln9pkoYZzsBCezFqfz1OROM8gEoQIDhrCF2y
+pBiiNqEGmyTb+lELDLnBipSOzH0AgYNZateBXXeKMCyJHx0f8n6W2fKR6H197ixu6Uio1D+XjdOc
+WdfBQEuRF1FQ+8yzVTIML1O15hlSA9s/qExWbwkN7pEzGKXAk+g5u8Vv8ke8GPp1cj2xo9IIsYjm
+9heOHnHSRcVqUcoqBDgqoMNxl67e74CR1z1gYPI/M2/kgs8SnU3a41Wty0pfYpKJmxvOY3+OLdgW
+edMiDhIMpXORaWcHHVCkgxOwBxBu812P1fxq81DvsoxLjbwRL/mAmkho6lvPo8DMNNdNZCkjqpMO
+Bsas2Y9IzDziHrkPSieAz5k/CBaUx9KwrVcvgOMMR+kbb2hhskhxC7/r0KlfzWybm9UoxxdOve5S
+5ol/EH66XpFZiDDLFoEZuH6BeLl0BjSNnAPnJBy9PNe9GLYyt/aE+z3luDfjwaWBd1tlzfGWTpzk
+rnEeF3OIZ3MctjY4DT8Cr2dcuIk86ZmLO8tjo/ScporrctbPUjl5KLu6jTtEsAeeYcgGy8z2hd67
+R+ilCiNP3r0h6zYi7EP2pnGN5a4vVXucdHIUwFeS3Sy1Yp/rGlQuNexPeeEGG66pAAGCtV5VaSz3
+ogiyNwq3xCWYVPNEOGuzcyjL3BnYdbZ1Yywx7rNyOxaJe1wAku7RXKPH9UnSNNxxy3PWj1GRFWFh
+WM+5ZeDpCDZ4om6ETXZuh+bo19kmL9etk3TxpPx9g5Im06dw6n8J68coB/ceJiHAO2024KXUnard
+6rnjzYRsJQ9s7embbPTd4i0yVob5g43C/GjtRl2g/Bh3cDRlKFjw6ehKu7NJtzXONR+8Oe4pMF2j
+uvoJvC74sQhNQvE7dGvcYAUJPXb+yxAAqGpwvBlk63BnCslzOXb9M0CxHSs/hUNu18yFsU+S7HOa
+xHqoHfRxaceTGI/gwaGR6G8Y0+Ch23yF9xvVFlcr5vZizhBeVJBSAq50Y5az9qW3MGsUPnUb0Aq1
+MUjS2XIEVMCLs3nFJYxqA6FUMnP3EmJVvku9HjZaCr8o4K+PDKjqlxr1aQt4bkaO7jqbNCesYtA9
+suHqYb006eRGIlnSm07N3WhgtnFGWDtQAP5vrM8yOPflmm4HvW4f4DaZXqei3FUk9B5tLZX7LDOD
+x2Ball3Px/VA8ydjIQ3BeerOR7evrAj3iYuCf3R37mJpR92GZW5G/CwToG8M22vGeY280GmxY3dT
+YJy61ninRPS58tI37RaNJYLbnClKVIqJdrJG5YaGuzwkluqijlMlnHuQtiTr17jTjOVRdmmKJgUN
+dZ6D2KipJccF9d2qmiSuUt7RpvF4z4qeSJt8+rGsPttIIJc4t9VZS72TuBElyJMVThEfzqaW97ec
+BTKeEsIJVvfCs3LRPQlnhZUXuDiNBmdFYGbfarWd/KsARwptJU1ilfhqLJ6h4Qv9Y6D5UuT1iyuC
++8Xo2j3OpiUy6rpDFuHNsdCRSyUN/jujJmOuQlZMatIxSRd2laIdP3SZtD+jMc5gH1Iz9riH3Kiq
+yODyCqpj0R3c1I/2rwEH7klWab21tMbbWphxdsVQVI+4lueb4aHfOMXwPMLGX6x67rZda+88zW/D
+eqlH/kyNkbS9u3yFAJwG4920SGlHvVVwKDcvaz8depzmMPwmsf6LDKuK4l/8zhnoJPbNYMS3TZtu
+5OPGC/HNnYbK8R8rMafbzgGV0rQCuVzpNMdlyIIDOhY+/Nwqu8Eyl3AgJ+24ZhW2sAGfgmrmm5lf
+M/i4ExZteuXwBLPTH7QKd2RWKHQ2PnN4Nl792nslUoeQunEtN6mbhL6sYhRUizxQlM296VXT87ju
+fL0xYpFW00l4BW5WS4PTdK8FlNbGXvt5j4QqGsb84Np3iqptvpcP81T/0XyQ+vGCG5i22XSY9k0/
+V0/QmdkB24V+UMGaggDOMIuawWAHde2bh7/lyf8HpfwDSkHCbOJ++J/BlMe8/Y9d/9l8//zHd/sf
+T2P1T2TlX3/735k0wV9EBRD975P4bFH3yTf+t3Tb+wu9dnALmSLS2jNvjqN/S7dN7y9aJvl7ZL8R
+dm3aqMj/nUljWX953JrEyKAu17F1ef8b6Tb/FNjJP7AVRON8E5oWyN0iIhCQ979jK/whcpsFLeMA
+ncQ2Ju456ZiuQ221CEa9MobJtERRaUs8ky54bBXA9PeyYLTya50Y88HIl/7JDBq/Dt3J4ixaW8jG
+z1Gi5ruuidRLSfYTCd/Zhul+yT5zWIrAPkCMC+3Vh8fGHO5MjsrPOk5xp2Lm7iplh0bVT4UDIoxd
+8bupCy3xWb+6jMltYhpJfqmmWW/u/HnoCXJJDAzjwpJ+3DX67Qno05L/Npy7Z4fwzotN1UMfe00K
+A5pw723nokumWPYB3zFHT3jnAx4PkW7B9VS1pf6sNdtoZA1+/la2LXrXlfZnNiqSC/wIo4p+7HVr
+SFi5WYUY0f0iBMV3f+uEvnfbuoCQouM4D55yxHOvCc7m1zwZ2qelTtuFX6LSDwyS/C00XsVT4Rrd
+vccOd+ZVB9kv9MkA2u7LZIs+s/lV4Ih+SYj30KLayfsvC5mRFbZNn/0ZhqFHGrvSk0459S3qO8uJ
+pmD3TgZkcvM8n1YaPz9zC0ot1Dw9+e5QuT+AbACNV/6CCnyYU9xn3ZyLq5/2JjL0WeFIrXBv3SFs
+DEzurXZ5LZxbOEcVcKhGmgt6TrO3WWYnLRewiWVhWhfAp+m1nzzgNqQOpglL6BpPxdAO/taZdfNN
+GGWAeabNYIsrF1MkV+8dtntnCbN5Hk+Luwx2vKSY8yOvH/ond67wGhF6UNzng51iIO9V2NjJuBn1
+rn9bQNLvkhK0Kc3c6s1p7eGcF3QxwOJNcBdZ5dhDqA0jsQGCK6GOjKKq7qhRZjSrzZtXYXDrtIry
+zNJ+p33tP7ZtwhzVj5l+bfJlfWgCOIpNp2bOXqx6+nfp98ZLrY8ESRRcWAqqgM9ehBKwv9FOtXNe
+0so9OsjsQeunTr1WVSY/4NocA2zJMd6pbqkZP/gOKqxARTwSThyB8tjC0tC3i/3kKm+59+x6uZPU
+ffahxsj0lA8BYi0W4dxDQOQhStdrAzSnJq0VXs8tEc5mM7XX5PRov0ZvmN7SchrpRpdj+Xyznj+1
+9jy2VKa6ydkWZeuGzKbox/SsqW30IGCGDMi13Bq9h64+RToBWtbXFWrnZvoy2XSXuJCGd78a6cpa
+lyIwntB2Ple6az2ofoIEL1VlXhwUM0QSJg0BL7h50a3kppl+YRSQv+mYsMGB9Hm5YamZHQ+d3rII
+dwqliCmgS/CvLy81S/CzNKaaIWceYb0KDT2n1vflG8bCuYoagl0+JcEZ3UZZuv178keBcBblCo0Z
+SeccydNQ7DSGxesc8A9+oP9N3wM/UesGZ7BxGREGI7TA3RXlOC4QeeAGIFjJ75hSU36bo2bPPZ8R
+mgeIr5QmIrJs9LOon92cSgxE4YqhMFdfrspY9BLZzaRE2PiKY7gnQUSKp8Qdr6P/S0vz4L02rIGD
+SyuHeTOkYn5Fq24+AzwlXN9zIS511TQ19vwm52M7Yhfe9FRiVFE1BDy/gi95tFy9ZnarZXaF5obs
+CyqExHFf97ciXHspSn4OzfszV3077yAAgjyuDKGmCEw6R41eT+stmckXO1dMnclWtt5kpLmBv7BY
+bk3po1XQJ06wlXcZCqSLkZZXiC1sURTvPeUPz0FSBtca7aC6LSCrFrKnIfP1XbJygB/slQSHzMUG
+VQbiQ0dWx2vYOjdzjFkmX26WCszbQVfwrHcM9eiDh+Vor26NH1bHIcQR2FX5xp4yvQorfPQWK4nv
+3ZNWgfJZQAMeZItQh8RZFsvYXzPzTuJOf0nLHp2A37v5Sa96OF6/J/OQkbDp/yhsnXd5Vw9EOvSA
+7jHCPHKVbDOfJyAGhuNwWhftnXYbdRFEXhqxn6/GszWjmI868HATX3wKgAtRak7EYTXBwwD2hAwl
+L7NkkyQGpdSIVbQXlVvrC5zBaEQm8zMF8eC0n1SdWF20KrH00erovF9dfkvfksgPrlaDTqYQAwB1
+Pa+4ci0W7H2jy+e6bHueKKsLp0YD5PdYz8jdsRHzEkgAlLAxlFg/uwI4LGomZtqt3pp2uq8MGTxg
+R8J3GwRA5yeLfINXNtNRxsmwLATiuKpfD2Zho8Xn6Q7uh6bXmGAHTZdEagGiHMi/bNsHMk8c9OtL
+5TKXo2FxugT57UTixrgRDS7NiOvcbXkrDEjKWR/Hz8lSGjrksTeKLZc9MQ/OzHUWscYQheGUaQpx
+g6YAFFX4xa9VEk52z11kFGQraMYU1e1gk4zpL5xCKmBrPlboXOqzmnIfQWRJtqQ1ragM6nYucLms
+tyyacYW9YA+26m8C1Ay5XTKyyOIFFsbcpoi2BpQGK3g9gjbUrN4obfVcVCumpboSDP2eMpPHvPPA
+J7vCopNmHSawlqXs65+qmcUETdAEjy2ZD8QqrEt9Ros1vCcDFqxoaeF1WDkEOnwoImKz6F8h5QJV
+6OM0ggyyPaNmNxJDoOxPF1JFDUU9dlwhS/huiTR56R0uO+H4ZNTIdWHpxgvnffIZEH98akoRj4IZ
+Pa4jnlN+QMcjQ4h54hdeAWLNpm5qipADyL83hNUZu8T211+ppvQzk+ekn3yzsr6VY1gAAVpFRGdX
+FekhQUW9hvgGm/uFj54RkXuMPBj5veDNzGoeOm8u9IdsqW2SU2ydN3DSdeeZYe+W0zK6HJ6lTkCm
+ZujypTPLIUcoPI5PZmrNNHNYi7oY49+i7z6bHgZSB6rI8KvxTop8AMxIjApSQ0FZVbpsUZV21B2h
+YtKyNz/vepgMOXrpg5qG7puBWj2ZjZxEVLYTSgqcV/6DW7cpL47XpfeIjeAHJ17/t1p3pnsIpqyP
+Ap30mFDTWnntqiX5XQqxrhGTKwy2Pd9SLzAJkZ6YcX+HqQDc3SRmlXLBFp6sIJu4Y6pU8xvwVpE9
+Z3aDqTvVA4B4nJzoP0XDLYEhjcUxKX1kN67ibCgc2+Fdhs9/7mbU8aDceQDKPVv9GGPLkX8CosXo
+BQBnzyM1AR2HTnpTYuIWrB7tnLiTCB2o+0Xai/cgGtlc86Xxr4kuMaBhETauJh/yfqMPtMARAi0s
+Ed1O+WX7/9k7s+ZIkbRL/yLSAAccLic2hXalpNR2g0m5OPvubL9+HiKrupVR1ZlT3VOf2Yx1X7VV
+lYQCAnA/7znPsRPh6m0ydtmrzGCdbQkG5cbOoE082MAM9M/z3OmqeDdManwMBLGw3WgLNteRY/n1
+iVXWxiUeN6eFCGWCV/Q7xdPZzxSilSjHyrpumSJ/SeHR4LJsLf5rYst639hei4BrQXkjuCGe5jRl
+dBUwgsNubgAQYdWUOCfT7IIkyAkdtTuXm7jBqZkON9PkOMMu6TEKrXkLGw9G4LLIV1llQsH3EsNY
+dUMFJauYAeVZrAuSz4xzewONGGvmKrRSwz+paseMHpEw+awe9MPB5yp0RXI3CET0114pi3kekof6
+pCVH3DQY3SyW3AqLYwyVI2G16/7XlvBHsCtuAjaUP99Ls48+ey2+xs2PcNfvP/r7Rtr8AJ6VgDFk
+Dqj5h23sbxtpuK++D0zDFFL8Bmn950ba/LD4ObEOEGZ3SCaz//59I22LDwJvgvAJ/AeI6e5/Andl
+yCglq4bg9+aoo230v9kcxZ/7frPuuugERP3Y1H1H+R8d5e9E+R+DZP8elP/RUf5nUP7iR8njP0H5
+Hzpr3skryxX7AeV/dMV+gvJnEez7F6Hs5TdmWu0T6gnDVVZUw+XPyP5lADkO65xftpsD339qI6vY
+amxqrD6b/1PK/xGDgs8hzHeU/z80r/6D8j/wMgerR5DEe4pEKbpPiCzq1vIpP1wy0PUtHtXSubBy
+kcQnf07+r6ciu5y7cIw3yf8F/P/R9f2fxP8j3L3HlBj134b/P/qQqv3b8P9Ijz9+qr8H/+8tSuU7
+xMvfgv8/0Ih+vF9/5P8f3a//5P93SJM4sGczPHeNmnjMLBnnhDCK81B5W20NgqWBUZw5h3aAASvP
+i4h8UIFNy3zFL/LziIBsverCxr3orML/VffwkXK73JI/1Abg23t/vv6m2oDllfT+qgx/S23A0Wf5
+j2sDhFjuxB8v9DIVWeyJDIJZWRzdP+YYyBRJh7avulI5ol2KJd7x6vYBHnQZbxNkSw9CRtZI3FZd
+fR8RaMax5Qoef6kO/EcRRYA7EuADb16bRMEGR4/5PBsQRnGxjOPADDzRDxSBGLfdGDSPtq4SfoD9
+yx6+tvN10j2b6BzxIN+F6Op0Ck4WBgOwRGibHmSHchOyV7nBMIUYVdMr/WyUE6rT1PftfVKRccKN
+UJqPdZ8NKbJdH98ZZubfojX79VpGnT7NwwErii7D6RZ7kV8xdNbe/diadbeOswglJsoSw17lunNO
+8pnE0art+66ir3gY4Cn4IVuU1ir6Z7swAZZTk1Scg4bmbROn0p02dY2oh2jr2sEaJ2f11HRt+0D2
+H03fSXQBC8TrnORkGIr5kt1fC3VO8J/VpPCR54wcnd8OR3WugW4S0wa3qB+DaTJrTEpG8uwVJSVJ
+Ve2OD0HGmn5TxL5zm03S+obWHxJIzbXZEnoK5gdydEO+Rglw1Wbyiqk5Qwgx79gXWNV2NiLUmwrQ
+IOqNJuJGkge32Irkgv8xBSMwcwaV/gKWce5xheaW3Oi5t64IBEANDKKqe8ZrUXUwbUnWnjdeb5BD
+YHtcXig14dcvxs5MgIxWXqnXS1l5/KkMa/CGEeacZA0ElErFFHgG2DWsS9hL3RmlLbTY15misM66
+YjaxQFVyJNORMXA2rWa6DJzBdHZhJ0O1jmt3IvIC1g9zXiOmz5GUk7nG8oLikZA9SzZtOkzseUfQ
+yeuhjIqPtILI5spCImdmj44xik3vTVP36qCPFzd0JPqgBGIc9+7azZx6YCRRjx58gzq0L7yG+iDU
+NWPAskOhDiMeGGGrMMeyto1do+03U4was5Yec4x1OMdFswa6mnxyzbmNVpBlZLCJdUe3FobXxT2f
+uNEbry8Lt5TZ465sAZBXOwxYld4O4DDIHHrca32N6b0hyf6GTZTEWINCCJQMvMKDbgNwhLqZord2
+dKGKMI66A7Zg3ZVzXdFtZfrOF4a5UGrCBoz1Fnuif+UPc8A5zfq5RMtQM8K25aPTilmbF3ikbf5x
+oMwrEyImOcpWmUTzTCS5lQwbvpvIRV4ARJUbA9NqDQ+lmNzgpioS0W3nORJgYlTrb+euoQJrQY60
+hJue/Lmavth5kvPNaabpNa8dlCA/TSGV9EUTZAyV/JLhQGw91jYB9o3wZJxv+xiu3FrZOWavcXSb
+s9Ek7nJVTK3A2AzlY+mKqTHPMb5LNhoryEcnCaZ0x7Is+diWNqyINXnc+mK5YuVuIltuXE1ulsZn
+vhyIahuBYCauhmnKV65IOzSKBclSlfDjid1pootFAVKFZ4Q5kqt3zfDVmIRg6gHHfZGOvW5tHxgv
+9Bs7wRpKcHk9ck8A2xbQSsoKmv2VYr2XrQN0KiQjz4Ha2QK/P3EoHfmMr4ocYIBFc2knaPUNYwe0
+eonp6rpOF3+MymRu7sn3SzQ9FQbjTR038YOX+FG3G6U7R2d5r6o91RzkJPNxsPQmiZrxOiGzo1de
+14l5N06qHEECjvLOb5KkPkchYTjU2QReD6yacMNVQt0IZu2dO7Wm6YvixP4eyQ2z63BA8xN4BdPv
+LMR+8nvA+wcDjj/JIgSC4ID3z+MhfOARDfS/HavsUnfoC7agr3Dtk6a9m5ypAi60tAbg4uEsAXyh
+TICK6vwt4nN/Ng9lAyJqy8+1v1QQVNSp7ZJDMQEz4+zFmcYc3k6EoZag5lJjMAHcGdaBFnN2GTRL
+1YFFsUuzaw8VCIkc1JWWuoAxVSXy1hCJ9Tm2dFjtSFhSATE1DbhcHZgS4H5tkZxWaCY3yi5RToal
+iaHumwA67dy7mA5ZeGLEdpbiBkiTwVfCOtQ58Ou9q1Ja1vN0qHugUZjqh3fKwM33d/N7jOof1ztM
+ws1/Vv0crQ/t6W+p+jlawf+36udf9QD9ZqH4RdUPmweW1P9aEPpf2asqX9v3lorvP/I7DM/9sHTS
+82CxXefQo/MPR4XwAd6ByeMIpktCwnznqPA/wKST3tKJY0kLoeYdDM8yPzgBDE+UQ2wVvH39v+Ko
+sJa8zPuVJRBZSJr4NhCqiMYw+v5xxdwoQ6ShUiCwrME5CUtDDncdPAvoWZ1vP42EJOlQ6/3RvkKS
+J6TcgLmtmFNrOzyZecUAupkKBsmz0xBaB9K8TAB4fHRfJwytd94SULyLej9+iarCRMQl+383Qo26
+VRhCMwZsGCFXjB3TcyOIHN75Gf0HjAhiR27ZnWTJiVmT94h6T5X3YPKdW6zHMllIMSOlVnXfxo8s
+fyq5KyLTHHaWAbthbTuGKTZORWJ969Eiu6ZXj4OlMniY+gT6k/KqJr0PYhzBxKuhiA5Gos67PiDc
+ZVhZ/5FyASJe5TRK+zRLdVNcuWmlsHk4Hp7pqB6NjWsF+YUnvNZapZENBA/VO92b1YLYj9OSga7d
+tMzWCsvyL/t5HL4apFsU/oGpLrZ2k5SgY0Qa3EUOzPFV1AkG7KKMO3MdEhma15X2HApHKAN6HCv6
+IPazdgZ7N4QDbbUVJuCVNBe7ZhoF7WWve5ukQzBkzwzJOmsX25Om9ltZ5rQSuhDFJqpwqmwSP0iv
++tFXL/TUiZ7RNzCqVZmWESCMmCDyAvP31jVzhjtelHm8LdyOzpyy60lM93ZVf9P+mA40PjrjuB7y
+MlI7JlSq/TRbDkV0g2cml2BVE4L/Zqj1pmBvSKa9rrM3vHnZc2krqlHg273m1SJw90nVXNcuufZt
+Xi5/QQRCQ+xD8FBX9WRHAML4Dc5WwsAILhnNOdZqClzzm6hS71sUjCxb/bpJPmIm0TAEWOs2a7tg
+1XI5MNlxd27W8Ft1Rj8EA56IMcvUVxMzKDOWZ7lMQLeVhSuTdVX4xl0Be5w8jDsMTz707ekUYA5G
+V/R+Bl9s/W2IWz0MB7pyjK5fycgv5rNxmPt6n2GPntejcozHTFqaxaVZV4AZzZkMVj008cdZEgxF
+pceeUwBX/iKTHgMeIfLSPrcb0qergHV7tOKZ4t53siBGXsa801aSZMxnIeqSKSSJCL01uRtAA0Wu
+yPZ01HbjKgiNjB2LUdZ6nWkjZU3dLkPX0WUNuo/xRLgn2KZw8BRELx47L7aKdYhvX6wihAPr5N3T
+8E9egkcKMA8XnilL5ZZnk4THA/bjw2XMjM5WMzd5iW//izU6EcgIzhx2COmtfn4sa9F13u2RfzuY
+Z/M/bid7kfLf7/2H0p+dqXcysDJ5sZE8Wo01skR70RhY0CdmR7vO03pPDsVej3Fin6rKyPaHv+Iv
+eQ6vq69ET5uvXzu67Y4L7X6oxPt/uQSP9dK7C/QHWuzdawE/dg1ElnTZ6/s3pB0cfvT3WYn/QfD6
+ASfGxo633RKX/N10KD7A8ZG8ID0mImgf716RlN0FXDwPlL9rm7y3+LF/zEqCDwJMocdr0nJBSLj2
+X3lFHn+HYYBzZAvjNg981/OPRX85DG2rNYULjmOtE5KK997Qif0syv7zuzP0J7fL0ZpxwY17uDQY
+8XA833OPlMtOy2KhdeUbiw+87q3eXYNd+PLvHMSzOHWBDWvxSCIziVv4suzyTQSTbRsVJsVAuHF/
+0bnnHlj9729Hjy2o6bG2cT22r9Rz/Hg7GlBBWCgQUvEXA+Mkp7HdjEY2XZXkBOWlEzm4HVkR4Hwk
+qIULcj44Io3u4I7sGBys2gbL0xcsGGZIZstoCA6CLiCOtLIXGCZI7zDJoxsb8Ap0LLLbJ1I5fryL
+WdYDwWmWCb1hGu64dxyyFWSQwjpbCa9X06YCFvXVVko8F/HQf8mUUPMmgFBgrmsvTMQaIukckATL
+QQDb41yllJMtFno2Yca3xivLyxKIYbMCRB5LkkOJ/up4bozLpmR/v9aEkO5GsjqgqQbXhgFXhlgJ
+UhSFPMTUux7nsMG5LnNrWJeFTgYILBrFhaoR9ehoe9BQkgYwfXbKG2wFC8eON6B6vGwNNIheAct0
+um91CmaT3XtOV9KMieLBtRN3oEvPsz93puOcQdRNyUn1dvLK72cJ1FuakXaMI3F5UciYBChNgvY5
+rUUFdv0EWI+spPtK4wlb6cS2CjQePGr9Gu8e1rsmbfslQYk+RjTCl2vPS4sLzC4jFF5mfg5ehhkG
+U+w3Gs4bvOD0YmprAIGebFp8UYDqg49WbdLxHRWe+xLlo9HyF4/Nx6KzCbuxDuA8m7zDBT7beboE
+ItA8AL2kcBA8T3I/svd8I56nfL4I0Bq2SQsiYZWmWWWtdeuOzbnlFQleX0zBznnKi4dTIJ3ka2ip
+8FOYlsM9OBAslmPexxSG8L6dAFjgLWPFplVzO9Zl+WKbSXLjgnSAFRl72UOU+vWL7ROfWdv4QK+p
+JZjCjaos7yE18+JyTmQHxIh6GOzJhZ62oZL6OiSGNe2rqPOfRBx4b02Dz2xVl50RbzB+lhdu4liX
+VulxJXSVtveBKtK7vg3kaVnk3bCKKrd5ChSa6SaSRCRxAxjT3qCXEdfZGDUvLkhKyvQKttYkOgTA
+X8pogtd+SCB3dDaoVMIoIQyISTpYTunYi19LJRr6ZZreZYWSZ6VF8xe4g41pYgVauw32EwSUWUG5
+NjTmMJp8iOa4Dfh4f9TjR3phqd+w7KzEzTPboKdnVoo4bLMhf23tsfrYl9L7klZduMeKiPkM46zx
+NEbxS4l/hpusMZ3HUGoKt3XqgREKWQxRhIPfEuioHtqPGfnVjJI4B9XRD6nN3U5YeynsS6wOi7eh
+rHNvHM1r1jYIgok9A7DE6lhaxEKy5rn1DVgRbB+mz54xEk9GG6qwNBk+q+syNRS5+Doct9oxmQUa
+iVGF2wHbI3p5vVRqNrmB0rCY6Ow1GcX0dejwvC5oM+DVAzCVceX2k3E6Wy7NDalV5B+7qlyueilt
+6GUddc9rZOQsPrOJ37HA0mb2KTLI2e9yeKvWyrQTgLbsYuYZn5guoOyYSFLsiEQ9bGqdYZORbdLp
+E6hI6R3Fh2KT8Qjy1yoEr4udpy7BmvgThcKjjBSSZ1zB+68MKn5wNkNKJew9Ro9sIq1x46ew+E6U
+j/sF+c/y7JMyKfC1SAczI4+xqXw2o+X2T3vaFjfciv4nlenO3MYYWYGaTpTlbsv0YGOxAUet2Drq
+FF/MKL/AvI7yC7fQ6i6Pwv6p0qW8lnkrvG0zh2W3zYMiwjdjE6etU1yhENWzBE64GghSUrpkP4nc
+R96zwtk0NhEkh2mdskWJ1xjYely+hig+Wn7n30ahwV9qtK63CctS2bi6dQTNUNsPmGjlieW4RrEZ
+5ka8uvFSneTYOj8lnJL1W8sduQ/sUJv3FnvUM9/o034Vkon+0qaxerb7kcutMTzFa48yRp6kIqex
+ig1RolZQbGDttklgP2aZHV0DlCIcT3LfhpC+uDFZc+JaDWKzGk9IHslvSNX4WosBXztG7kaSlz54
+X7tMRDdMfHDEWlVf3S5npMeH6oYXEjPyE3OLBujKwU+bHby1RNiqK/5v0NJUhvl2BO/8MMSFHrfZ
+wZ07yz54gn/mv8yLeReOIov6Ze1SbACBoRvHyYTXN4YV89bB+sEBfHADpwq4FbDuxSUcySz7jEkZ
+77ACJHCmbWYsEIIWd7GH+5JyWWxa9DgtBmS3rawrcEO4krPFoOwfrMot7K8VJN5FFV3MzBKj6LTS
+B49zv9id297Q9TZfTNAgUvFDSzhXj/VkJcaqD1T+1By804QtwntxMFRXsbFv6sVlHc0ZXOri4L5O
+D05si7vqI82fxVsRVNnbUIY0D04H/7Zz8HKnRm9fDZEWOLzRWz6SlyruGTPhAJ8WM3jR1/hzDw7x
+2NYOEec5PiUHmN4a0WIjNw+W8t4yGoKFi9EcxDSm8/lgQFfsqr2Vt/jSlZOwqcwXtzqW6fTeSBYL
+e7+42YcxVq+Ob7Br9ICafSWWgPGdYAZb/tLsmOQNB3M8IQIezyT+8rvmYJ+npni6mOqclPjirudd
+hdEeOak6rfIik4SozWHgui62fArM7ScZu5j108W3T5R/eHAOZv44890zWO3uJV1wMKaag/G/l2AK
+cS3qJRDgkw0gN2xCJ14CA/khPJAfcgRmS6LgEC4w4HzdeqBcP7eH8EF2CCL4osb6S6dmdlEeogrh
+IbagDhEG+xBniEdNfZqzpBwMRd4BFAOBgCUDoZXTPM4i7cHkMUWMlqzEALbu2j0EKASvpzv20sQq
+xkPEQi1pi/kQvBiXDMZwiGMQfIvW5ZLRyKJYPMaH4Aa+cvsuZy5qb+pDtGOIm+EhWfIeDSMdRRfd
+EgORpkskBL838RD4vHwt0kNq5BAgqWjMu2gOsZK0j0XKKFPgvD8ET0bbVP2WZGENb2XJpoRLSmUq
+sauupiW7kgoPgu3Q62wVxCHly3NvEHTxDqEX103blFcSWRh7XmIxwPLqt+AQlomX3Ayv7eJFWzD5
+d+mSq6GL20IlcJR72SdNfQ2FKLlzK1tie19yOfMhogPsorwLltxOraT7wFLEv0PyJpVE5zIRnzTo
+vM/jIfiTLBkgQUMvs4QlGcQL1vepZY4IDKX5RCsQ/yB+LIbBN6hhLIZv5mSPN1RWEzmKDukj2mNY
+7h5CScMhoPTzncofdl7wDpY+ENey8cvRRvbjDmL0QBSjIZUbNzXqj5kBlphV63ASTZb3+PNDLb3p
+P4gHS7mUiyCLsIqhGJ/dj8cqGko3iywH9FS64h67fGmsKgKsL7VPnhnXJ2WeK2+Y0DIyx6khmFfu
+9C2f4M1tU9euHizZmR0EQaqUzgHMJHAOAW0YK6cwrXPG6+V9ZWvf3HBdCV03/exBYK6g4cWWvBrb
+PvmGWa/9GDjO9OIyP0zw9rplAf88DV5HLcYXKx48ErAVfcZdbkf3XuPMb8WQ5RhDbdqySaMG4ruo
+8pfkjMv4c1O25bfu/1MpA60QUtRPRP78dS7JfLzXML7/zG8Shut9wFBpmubyPZUmZsd/SBgwqSTV
+RJZn8dUK3MO/+i03aX+wiUPagc/dRt8Yhs9/Khh06CA4LAV4bJ2BWf0ljd+1j77cwscXj9/Tx4OD
+fuGLYwljAHAOy6gGpZD3D5FuU2PeFtXs2M+UOtr5Xo9mHFibMW6aESBVnVRomJpuivLFLFLgxx5W
+MUAPjdHtQBmoepM2vKa+AXjq4lerVu5ZHVS9uIyKBb1n0tdQXXvR0Frn6D5Uzhssx9Tp2FhuvKlo
+IuEdNVYGrhETNbrvvdvOXh7hTjWkJ2XbdqxzCeaEK+36k6Rppm6il4ICCePWj9wAEpEylvZhMCG7
+tC2lPNfBZL4YpS75JVFE5NGCAKXwEGxS0hTVF2nCvUwntj73MbGxASivHcf3bjKZNBEkmpIBbn/b
+di4MZ2Hz0nmGEaVPGeifkHwf72eAfmzGUm7a6cSoOsu5KvCLnCXT1ERvPZOcnsBz3Z32jdvlC8+Q
+LtIybEibJCGfmPdNMDdPahasx9sBiDAZkOiR3TS436ioDXFWsEqiok0l014U7P0TChMcd45XaRgm
+XApJI3SU3wMm1Z2+7YSZX7UDYDCnHZ8KppnwYzu2lmjMau3GHXF3S4zJc1zjzFeptN/EODpf+yHz
+bg23o7nCA9p1xpcW3zuLuWRV9rWFGAO/QtVFcuHSWH0d9VZzYedFcwLcttomtnRA0qhmE3sCOHfS
++4/dkJCwNCdRrCyEgk95KUjoSiKsGwH4dSdEHq1CZjD7kGbnjQ0R966xdQw+QqSQ+Cq1J33j7mY/
+yTeanS6D/cpqz6TsvukSWwXp9KbedfzRuwjU6aeUreTKlaO+jZQTnzcsKZ+nttIGeTM/Wb4CxEhX
+4KsiEpKS00EWS/YXtSI967RJc9MwWNhITHBnqUe3hjajGqhWK4pbK5fFF6MshrcIruEdZ81+NGK2
+sRsrdLuzAerELYmz9q3nbf48uIoUMQtjOp4X4uae7Q1bXdMhBVSFrW5XZWUVT9omIvnAZoas/z7z
+Ypmftjk5/jdroNmI7GTW09CXrm3hgW8GIO0iEXy2PaNK5i9EMXvyH0xFnH4HqFcDEYpT9J0HWlWY
+gjuFkQMsTXQbvTl2428trer14LA9DisDKiPUim+11UVwKKA2SEXZROJV+R2uBns1Djlgfe56zbct
+c0V/Cz5DdBc4ZZz8ZBpRFk4pFg/ry6UAKNwH7aRhpgdpn7ag3JB3PjZdG9J/5drgbSzwHXImZ9hO
+yXmJeSwCyqYLoiWMPsbHdjRqqgIS03iuW3wR1wEJEvcZVRiIa5NEyr6g7liMG50aKC6rph3s9lQT
+/Iw+y6ixbb0GaG8PMSpNkgFdTT1x3ZWTkP3a5EXdA/aPe7eonsthnMJTsq1RcTlEYeesbW3k45pd
+1BhhACPCs3UkcRijMljysfKLiKnZZtbeJbWLkjjLWdePkliXuZswK6yahfmz8XKLOQL9yggaRZkw
+N1V2xEbSLDK+bMhcCJFxwZ1Kh/pSgKxiuDhd2k9OsmZI5FLdQSq4vrG7NrlOqFjPIcEPMhSvPYMn
+wpng56LhSgRjGKPaCEmCDxvJmoQMQo1VjpvE8agQYaLSuOMFyw1KkMED0gk+2N5o3gyiAiddBvQp
+hf7SXdT4BTVLqm1P/DZNnCtXMllGDRu7q2QwW2741HczY21pA+z7ZuoN8wLUBnHPNjJ3AjTTaq6d
+FJRONVaXbWC+9J33Gij8INd245kxEenA7zcDu8RdoapOww4cmL0O2ZgL/CcZnIlB+0VzAa06JuZo
+ibobb1Q7Alg2izKgZUDbVvAA2pHEH4QWko8DaXvrQjGo6/et1UvxUHrw2FalXxKcU3SDqIvSCuCy
+m1ySjNGimiweqYYxvgQIO2CKLGZ1cQbqhSrbIUz611YDWN41nekXN5OIq+RGuY1DcdPYims2VIXa
+MbecEmg8/NE8uOm/na481TbPM89XdVZn6BmPyneq+tzs5ST2sHYokfFyKAECTam5nHpNyZs5B8Ui
+SBLjYHDQMqEYNrAHDf8egALfPRg53sxM2hjspD/PHcOTIyFJUrFnTlaJ4SaxpNCnEUj34lbQzJZf
+DRMS2ItFYgrIRzzEFt48nffTaQLD3b1GCgr5dvZWjnTq8B5at3CfsIgG/tdp6LPnuc/kJpuN1zQE
+IB6oud1LWMWbqC3kjUeQMP6cSqWjxwhPTndKeTxGsoywq5OuzChWnaLgOCEeN2KVajDgxXF9ZwBP
+jJ7aAVn7pOvBhoGZQZdBCPaBzKzpHsrU2czw8nMqEMXYaFKISQg4QBPdDuhb5TroJlpRMA5GlMia
+lERvyPzPbzlwHYhgWVB+GlxeCZdtOk84NxOGrMOpjR2hfsZlxv4SKA7+t4/mNE6XIbG054bRMW0P
+kQ6aryx77nx8eN7Gq2V5K0uPaLHNOMJS9xQRNsOpnnjNNV/dPhI2XkyuukGz+IoVEaSY0JrwpHI3
+8X0EIWOmA/zd+g05E43KS6d4vvNigtRsACdixXsvZ73yqTQYfZDJzgXp1M5Bz9jUKMsDVTwQBrdO
+obtZrbocS+wqqasSmh/vI3nHQ70NnxpatwhgN5WWu8gxBHCLuWSITasCU+5uG1B+0jyAvy94/fqz
+u/xaT80WgDnTFUx2dVCVIxyfRLbttoQ+xjeisMykPW0pzA3WjmTYcJWipQL0mnNsaRUWQUq869Fv
+TjSIhCdgfUTfCRHl+En9Qtz6IKQSgNk6lI3cNaZdXVeFY+jPQgUpWCzgwuk6cKCmnWfSm9R5MzUy
+v0Nb6aYNoqDqPhkOtegPkeJBuwdM3uq1H3b+OROiWJ2qqTPdU9qSy33KFLc8lU4PpIchT9fYRE2T
+uNy5OXL1LmJO7m1s5KGrIM27L8lYmFvHrovHATX4HinBuUxqUexdbSRngSAOyKSkeIsDem5GPLhi
+P1aJ13+ppy4t1kZnevqyr4XFSrHw+WrgZZjg/gR5PXzrJNN2XC6KlpUT1TfUc8UDPgiXajAf9bFu
+vJOqNfW0iw1CiNXKCWoLNmpt9VRpZXXoAZpSc724koNMM/UCr27U28l1m/EMsGMv7NUgep9vmDH0
+vbsJ5Nye87qNb0EaCQOeYKR6vL4D01B1Lb0ltsiMwhk8G2GW159QsUFlFMMk+Zx9x2CCVYKJaZOA
+T/PvY73/7gffI3XcgK3Yv94Prl6j+MeB9uEHftsMCsk8GxMYviqCfkBzGPL+nv3zPjCxdiiplez7
+4OWwT/wdouN/cNkhuuZi6RKSAvZ3u0GLETlcY98U+AkXj9Zf2w7+qHS4piuX/Sj7TSwZaB5H4QW+
+dGMQeaAlRKaj9TxW/qexG4B4OUl09+68/Hqe/f1QgY0ZBZ45+J+jEbAIJW8EAbDNy5sW2nfsbHRm
+WGd//Si2tA4fxnb84wpgKBh1w8OQmWRky00jyuqCVoH++udHWTbx7xWiw4eBMiugRFuYC9yj82YP
+Sd8Q1YUIgSi5T8CgX3Sx1FeuVu5JNPJkTqCkrDDNUQibdn3BvkCrU/gHDDKm3yuJsYeor+WfnNsj
+cezw5zBadxZjjW2CXfpRsIr9wu5Y+bJ2mkYgJE6anY+mLHZxViWXv/jof3Ys1ihs7fhi8wU+8iUs
+2YBETlxHogX3OgWHWZbiZA7TvRe7e7dsXnQ8IFaGpwAD7mDjPbF3h3hWbcFHn+If/1WY6Njrs3x6
+rAU+1b5Qp7zv5oN3OR9GM17q+AruqNUE4mtetGN6hjdbt1s/iVrQhnVd0BISz7l9a402EpfSRrkt
+eseytz8/PUeujcPfsuR8hS0swf17dCVqC38aq+Ye9dqjRJVLduE4jv7FvfQn14DZ/j+PwvPhvbsp
+bGa2PAldh47PgHTEfwDpZa42NfbKzb/zgdB8HQgQANOPLnfTtHHIdmbA4a6inR2Mxq6yeUP9G0eB
+NIZohjS1aFw/fKBA9VU2J5BYojJJXkBdtVdGb3i3Pz/K8lveuVAOF2d52vrCkS5osyPpyxBSVf3C
+DWUbkJASqiIJ6cRSWwWV7sKs4vSCoFN1Jvqk//TXD40NzWSLbNme4xx9wIKBpTXkQU+dn4ouR8ul
+81NZxinAQvcmNwJmotLzbjyQLuufH/mP30jEQwTJwBJ40N3g6FFlDMrDq0JhAXV09WWSFuUef2i7
+//lR/nhqGTUtlw6DFvqieXRqI7PuPbPKGe7Z1S3gzNfeocZu9s76pGWsrbq9dJpf2IoQZo8up8/J
+tDEuoUsCqjs6p3B1BlV3S18OcVxSKRaRhcugmrtiX1mCFtGW/VO0sfyYoU7PflfgCvGC5OHnH/1I
+UOVb5cO74yFERh/p9rjjnl0jA+qUP8PHQIlHIEzIjkT1NlMDTI6uqU9+frzlVP74LV6O52CQw01u
+4/v88V6ZrDmEPpUxhx6iCNNHnjxmSoW7yW3AOZFU2SP9B7+4vn984vhYFzDfCeHwLbKODhrNYH/m
+kF5VGLAG1oTS2KROG+yqZNK/eOL82flEZ/Sxnwu6HbyjJ44Y9OyHNJSs2Ppg0PVhlNzOoZmaWyCq
+RU5nIX6FX3y8P9wki6mQUQ8ZSI773Rj/7hXCOMxEdIQKgnxBrXnj11u8xOkvbsXjK8cLkyvGNeMM
+2r7nHz22wdZYuVkpudJhaN6OQb9UEOvTRbGCWF2Ot305/WI9FIjjK7cclG8LmQMWizz4jk6n1U/5
+5AjIh/YAN+4M5n5jtRBJeGB8zcGND1ddF+MWLslCjvDnO3Yqpx3zr+A+Cac8v2yTNrFug4m08Eb5
+fVDuE3+Iurss6thMjlMOPJ9S7IKiSTc1cTjQh5Ub+1HJmpI/eqcbjDdaDi/4GRHVVp0mMHWDB9Bb
+SNxNPNdfjZZhp4Dv21bBZVB2xJuaRkTWWao6gYTk9aYQ144y22LXNoVNRREWiNo+7ynqqS9tCeH2
+MipL4kU6d/B6IZTzIeFXpdW+1EuzROZHxbqzOjdY2uIMbDyq5qQUCenJFfvKobtRlMRNz1VEPu8s
+DWKH7bWbhdOFU0CQvxNQAmI2bjTVIjgi0aMbRvG0dZURVfQdqeHVxXFN+xOuAYbIgla1PB5H2LlD
+5ExbX2ps/iTvRkrdOTne4iAPC7h4czU/aJuH2UrqHkIsaTNj6VqOa4ylaTM/uE02Dyf20M7OSjtB
+/BYY9KjjKprq61J7nKBmqOVFN8djtWqSNlDr2TD+N3nnlRy3lnXpqfQEUAFvIjr6ASaTmUlvRb4g
+KJKCdwfmAJhND6BH8U+sP+iW0eWtFqNe/36piFuSCAI4OGbvtb41uicPZ98LWWeOGrlEHZgBwhur
+uNVlUgzf2QRR1AvzcU7lrdYU2AKjbilHXFh1Zy7Lc21WNrmAXkZQF1z4MT0YszGPl1JOFhS0eume
+J9GqGgF/bvUiEcO+Yz1oTD8FEaRhLJCEC5BaML7JlVI8RLgVUVoCqc080W9PCc8tTetyttyeOAcc
+6DeK2oBwapLWbC/SOK543t6i7DApou4zXVnTh2016q8UJxyQWbVi/2j72sRIOGpEhw6VMr6qs/Du
+wHNoJfxuuM5oWzGck+JlMj82HHnIx5PlSuiEWiESrVOFQIw4j98o/ZFgoXcI0SDfifgl7/DfHcs+
+Hh42iyTwZXLntTCeQH9KjjN35WBmvK/KNJ5ovhMzMC4Z1P6McIHHLgaWGQARKx4TeNYpNvy6tgI0
+8Jk8JwlCXqoVUzYs5ImczmWQZB5TvHywU2siq8xR0svYEp7pO7pFnjSpXrzFvt781dgvUxK7CHkt
+98QMLneQm7Qk0NtkuHcdBd1i5jZzDOVbrE9d5jQfqFBRErOS4amYKXXhsaFB+SjbYlBJhVSrA2gx
+VH4NLY8uyL3Vu2g7YVSB3TKo/VKba2atzR6x/nRKmBTyMer+dFBonMIyX7HUROw9AtCEvwXSiDOk
+fcwnbdtg5TTMTFt8syy8d1cxiFYYUwNfMw5nVHiaXUg9KOKFYg05aQS+oa5A6oXuEr1WZY1T6OCR
+eTaUzvvmKqIUkVKJDGxfb2giis3WqYOxVjFOcL6qHvpshWKG248evMX8ADbVJqU+9Owk6fmA9C0i
+jCgtk/BmEpN3BIfhZ1FTaosoAtcFnWFvVM2FpozzY4ry56oi5Ib1SBnoXbQUY/EwrNVg+HMapwuI
+qxrr+zKu8j3ptDEg9QUKoeTXSo9t3vaPFYNH2ys9ylc/06ZVRiNqv7OlkSMxY2Vh/cC8g0AIzQVV
+bbZpA2YST1M2GKFRE52QtQxxTOExcsYlAXbJHJVWN0uTWYOvURLPQxnTbtoj+bATwKn2hEBSjjb0
+UAezsm8TN6tFszFar41FtMJBxZk1B5ze5sdualRerj6B0U+1abooPQnYHtUCYbctBcNHGNzKkz7Q
+/CWXNy6TcIbcNjG2aQAFSw6lP+indIX2TQrgNRnsZhJao1oQpYjtUxmq+nyJCV8IOgU1oc+k0rik
+BTXzvewX+SGn3r3AmkJ648IzCavK4t3gCjKAd2cEVE7skrec1JoAkhE4X6DmBhb93im2eNdpEN94
+Ggl4t8xmJJRShRXQQCEswlo1YhKFi4SuZ+XFqhfUJmsF2rEKGpq7LBMdF71WkHIuObHDihJbyZkX
+u7C8+QL7fW31SXLp5UN1aXZUQ9EtezTpWkVYt6kNG8M3rZr+bTwmrdh3q7KkZ2qMC/u80+nw2lZn
+lLsR8VQcNmVFuGA/kxY3erPe+11S6zSC+pzeUD+4c0ZIk6AdU7szC1yvqXQoE2bRe22LVNxZ3kLA
+Z1ZO1DkhomEEmqn1F4qGfAmVqVWGaErREVNz4BH1QAFY1NUhfZI4+DxSPEcHyZ5hIdCyJYeUoBiM
+/E7T8+JDm3NE6M24VYfHQQotVEW2gG1rKzOQBmCxkDrsWJ4JewXc1gzWA0OemEVTEcSKkuU3xBGf
+nXhCBZaRxkCRF30UAHcqmrbLHyaqTF/SfCFVytEUXO/DgFpyNEWqhdVaWMtpavrCigYUMZTDY90s
+j7TxDdIG3aT+Rm8J7WZeJrp7hhFekNBd98N6v/SKd89cVBlowrIW8buCRyIZVOONkgFKcpf9eAHx
+0lVzX5D6dcne4adCv1e/z7pb3DDsHSuKLYRmZxTCmIUVQjibM0ILe+q0ExBRdOVjeovWFqs5lCBB
+w5Fawr3A4/RBGWj9kZnbF7TSI9P2QkfsyzY8t5OQX6i/MVn6lMCGtrTQqrJt/Wwobf2DEAHP3OnQ
+QjXAA0lFg8hMk3dUn8QDo7SNrxCqxuVuMmqMaD20N813tNl+GKq2AQjbGXReSRXCz6+qvfmQCLbI
+JOkN6tk0t7BQWfrcS/K1Eu2Q8E7yndXr6t6Ox3qPrWRQdhwt5jcj69BBFgbCPdRFLrn1RjI48Oct
+k+ncVFICcCZa0YiaTWdmPaBlw2JUQqTuTQe1AkTU+khoQElUcCelCFwI+R1BGpUxs2KwWfMXRzqm
+D2oAAgMMTf3BFobRwq7Xqu861Mw+qLuExwXNt3pc66av/XaqM4DFKqIrpoOOHMi0iKv2CoG/AwET
+SKAMDbUvuld+VjVHnjBtFPTqTJioqSZatRNC8/iRNPK+z4gtybPuDQJW1WaUGh+KAvrDr6ZeG55W
+sfCI4rru99JOx1foHss9VDSQVkISvhCw/fOSC5pbtdzTu3eSE0SP2KRwT3D6UaWg9D60tCsDNFgq
+6EVH+qsBIzuYlNhUg9xCd+ivvGpybYmDjfq5StxAFE57Gpva/uE1HKrOtF7WW0s5J3WFyGoOdESB
+rd9wPhrns221100LFpL1dBa4SnOrtEJiq7wmpF/TRmpF6k9YI65oI2Rx5kva9J5+GtIhOxVqIU7Z
+XDF9O6VL4AxrssaekY7LFYd2Geher5/JmlSscDZq/SETCVE1uXCybzkqnJvGZgKjUjKpb2vfb7m/
+yuS+rtqSsqfoC+PRhTsjwn6YJxlCrIEzoqWpfgNvpt7Q0tI5YbNJ7/uaHTOi+VWcOjVNcyIq1j6i
+h1e4tBCtiuylWtkCi1nFDsRmJHcZATkf8aAMtykty5t1jbU7gWcwoEgNxNNGZ837qQfnW1wliGYm
+bfgAClLpsBVzk42LpxDsPKIJ9nVhpQTfmXV636Ueyqc4r18gJGrDLrZTzBH0VmKbaSSxL7iH7GVc
+ZvPJQVkKv0aVq763dUKq94vnwkDvZOZCAGu7a2TnfIM2I5KxX3h12K+tS+opH/8JRKP1IovM+6Dq
+1LzqdudaV/DGKmZLhOtlKFIQk1nX0kucq3m4mZjo8GCmbfpiEdzQIr7Us9uVDQawlypjybeU5R5F
+dcIf5Ys+sNdsUPkPciBHKWPLkVxKXZ1I/wC8QDmgUy0yGaaWP6WggF9EBZ5BvBBy33vPFDOtZHyg
+fmXqHGXMmpxSFMzSuekz0O9k7sYqae3FiJaChHTDJb2CJl6ES5yY0jjedPANknwmPA/gCn9f6b5n
+pexpdfI3X/NlNU69J7IPdF2LBx46zTvqFqunhlad4hfqJB4C3/Z0cdewBOJnsYz+vWqW8mlUes4W
+tuU6/IihM/ccfxTa5BS7bwfLxSpWjUhwgrpAMxGQwoUrdkxU9TbLJuxEhpO3V0k/qWboIhEoI8rw
+eRMlFf4euo0NO6es700SWYiuuHMyrbgFIDt/dL3uXhiAS5zIGbrpsQLvG/+ki9+OheBZkf+MbQCQ
+spNuxG2X3EGPkaUqFH18DpxLygaMWVbBiVIRNJux2dHYab4pip5255XqlE9DVzk6K2tffddKsrn8
+SgjnlXwBNd1jy+GNNqIxnldV6/N9yjbHCSUBxGwOR6tyIkW1kOuQRmb14dB2BmU9K3/sE4NJMIuB
+8JwpaSaHHaO7viScYOwONDNIcKkyb9nPbgwFtc0VcUf+eHVkp4ZwVdFtfl3BHiAJpbWUdwuKMCdo
++3HCnO8O2Y5A3Z6o6SyzLzi3pm/CFv3TBEeWBQEMjhpWJu5mAgb0iWVWKRnkWjaJ0EuU8mXxipXd
+S+bkaJ/JAHtH5mQjxrCcMmevLgjATEXpZVFllsl8FLmRF1GWNMBEhGUidS01JzmrbIPb37RbNwUo
+vjwqtG0nqtKMeSn4HLMoq+3lOz95fTVybN7YsVdcRRKQNpChVunLvdPkxSY1UNzkKlM0jqSsmt3g
+T9UocD2Qe3vfupxBQ5Td4o182owzOlQSqAgWB2D2ClVm7KzJHdKdLJLJCVZ1cI5Ae+V0bs9dzGm0
+AgXDLI7Jk6QyZ0Pxml7+ip3ReacPO4hgKtXixu7wTALRrY1nt9cV96wzO8RL/ZpOhW+RDnVE7297
+gI8qdC6YBvnfzVNVHJNUsZywbUfXjkhrTB6Svp1PaDuQ/rgpsRhiN3RjjlOjWZeNWDxnC5/9kPfT
+TMEhR2U397n7TDyP+0SIpfhmiKa8BeyyFgGFcc5JBdLuLCirKpVBimb0XeqS3WAmSkAI6VrbBI4v
+bP19A0Mm++e8No4CNATFF6SdYPExhLINn8VyonIh+6hYvel2yXXl1sMYiByq7zl2paCTvtnAZT5A
+RrtMIYrU4ZMh98bE6ZTX45hZIkogByUBornJikqysj/qNTN/kItHpWiYVg/isr1MV4WmScxvnMrW
+0FpX5XJoTQoqlWGOe50zFi4tvcNBllDSqXd8PjmrVtfjEAIwUeVBMyP43NveqhLLRyoPFF6pIwAh
++g4bpgNgKVxpwSH+oHa17ESl4pbB/5BrAQfJbQdpxooVJMpctjvWOcQvkxR6tdfs3nsHX9RxLhwc
+/XkRvZ5HbTbl363WQu1SM/c0uIrTrPdTG1SRURQPEjrCLY4DrDYLdBstmAgXRwS6SzqEm2EcS0nJ
+Rk08cbATASECOV46UvBKp5NWN2hGOUiJN6dR4lcDf9INHzSmTw6D9suquIQ5OfBxng2SRRZqT3oP
+xVxZ4h8q3bsnI9l2ukNmxMTSNTjRyioFc75UrhZ6lLXY/A+S1S2m6h0iLULuJPjMtvoOx37XUuvH
+yivl80yWoPDNfkCqGMsa+UJaD+uhTZvqtWR/cg3LjipHatEnI69DNy7RjmGDmbTZiHdTWw8tVv18
+JNi9yJMyXFiLz81hGpM6wKqqG/mWVW19/Cyy/0fahv8frPtbV+iX9sNfnPsIXUEjD83/2H28f4jX
+PwUG/fFv/y51MJE6IFdwHdrhVJl/+vP/IXWAbuP+xMnQ4EMDsfkp/iF10Ky/WRSoNc+gPI3b3aEm
+/g/rvoaUnu6K9c+gZvM/se6bm6Li18aJqaK+Rz9v0sGgfY0a48+NE3MRq9tXFDWYn5BgF5ot9bfN
+DJ2ekNvI7h2uuOcQG+nsu7w7j11rvzb6DoHvqUowxJF5iB16acOyfBYOyVamelAT8OPdvKub5nbN
+h3NRZ5HMOFQU3ZuYG2yRGGbKov3o3fxYxWSKKtWNbL2O+nMdWJoIWXd3gyFEGPdy1xrWTvXkMyK1
+/RKnjxTH93Jyr4tyPR+SqQhAZYWc5q/H1rqhzBqJ1NtNsiLulRxDTygsQGKf6Bmp9pg37Uz9sIr4
+Dq7PWe0Sol6P6n7QvWcJ3WPJtaO+tB/GaN4hVLocrDzqUrZZTnZmFsuZHgMBK+eDpvc7vKFHZ6uX
+97azr432maZM5WdWfOTJHCnl7JYP2V4M9r1eOJGmsG8YH8vBwTdADc9Yxb5m6hsw5RZI+Mk/OCP2
+Y197JL4nm/bcKHbWMj7UanqKhWzCEYyNyVYaU1qO2dxMXwwO8LZ5ZO0OTXcj4Pc09NWoUwA9kghZ
+K9jB5Y9leVhz0kQItMQTekg6gOgcvhpvOTom2q+BxDGXChSLZ7O+kp8IZt3wx6k5mJ11k+TfeqCP
+BkGEHG4Qn5JCoB3rEkdbctuqMhDyKcnmXWY1e8HrdC5Zl/w+cRArUshdiBmYLhwi3Gx8QIL9EPc6
+OkmUk5anTsa+1cUZqlSOu89CHpnYI2LyxuUdNGSgytsxfaStshQ/lH7YNY7YOcZLit+8yI9Keaun
+QTd4Z6vS4wCOjzZxRLOSRyRtOcg+PFxZ853uVBGVjmec7fu4KNkuOeczcu0poYCTx3PgWOmuj90r
+NjlneBMOjmM/FWl7nawWGcfyLEP7o2V5mHm8wSF+jBMrLIf6so/TC0zje82w9rMKvGFqrZ3Wuwe+
+qAOJgLuME5tbin2/iEvbnPajV+7aIt5DHUIal1M4qQZenEpVI73I5pS7KhikqnuSHqJZmAitPhDX
+jTx4tbdMKYPMPdlRnCujZTHeMzffpVaik24iIs2bzytzPes8dY/uj/yHGJQDXc99OcdXpWEcicTd
+m3YcQNdLWJrTbx0J3+zBzmIN2ys+9bOU5WxPw57cojIN1cSA+zl+S+T4ZKDaCYeS6iszwK1IyURP
+KEonbnda1HZv5TFfX/a0dLpzwLd40EbrrUt7hndvR2RIvlIHySMirZog71UCE13kGRzX79xheWss
+JXDL7I5JxwlURT6uVVciFYSmgDXYHEcr6BIzdp7wCnZrJK3C1djSdfrwomSmO8E5lWcuuvs9atw3
+bxr6SClkS0SMVx7qlkSXKrPf2hiHDsfA/LLq3Pd6Le6xLZZB1W0JtL1Khu4I7FPBuVbglvV1JacS
+I6ZsF8thus3b9b5quKGx6E4zWxXOzjibZfrIzLMTiU66oHGW2EVoed8M66Z5LAThH4VDAZudlL0G
+jp7R0Vw2NhGq72ZodqQFMYn2Uc8NAg271uW06yt7Agal/SimIYeqZRymbI1ahxwhPCNo0OKzhIjh
+WG7xDVaUKUntG5tfn4hKc/XuhKKdFKis/pibJ0sagdBkSSbsrIcapldHby7wyl9kg3VGjO5+QS/f
+1OsPD1MLx8VJh8pph4bl7GCXvtc9Gd6Wd/A8ixCr+tomkJNia30n1ezMlsbBrcS94sZ7u46fSDLa
+yYR6RaJxelDPNM4wg11c9s54kUxCBJUykzBBGTEdzf1ES35dVtf3NPctX4ZzLalOFB+/Q828wR58
+QaTizZx7B7OpGr9en8mJKCOvxC5vJ+kVQfT0G1rDi6qCPq0FOFGLAKp4F7WwViMUpXLnONWFtRKr
++p/vgv7bO/4An/x2CxT17X/9n597oA1j9KekB6gq27/9+xZIB9XHzsd0bZ1zm8We919qT+1vqKLh
+Hm9KTxpiNOn/uQNy/ka8uce/Yp9jaZrDD/zHDkjX/oZLkN0R/BykV5ti6X/9zz+pAvtP//0rhVL/
+vAOywBbhnrFdkz0QioANM/irbqykVjrFHpxh0pDcrYCz2K+Zgmxmr665FLsMFCgIj8wkORY51npe
+YM+wfLkWVRukebPF8tjJmO+XwTMSsm/shGMAifb3yBLTq2bARoX3azKvzFQDCm2pfFJR2xXVpn1M
+h9OwesBY+Q2WASNJqUN4M5t62ZslOFKgAXX7OoDQyX3dMwwZZeQ5H5ZYzdJoIUDrpsdPnUBS7ZPv
+lDrJea/bHn+bISYFgh7M3idihNz55KydfOjVBLMXudocZuPZMZbdSFXrVXFSTk2W5YKvqUqP6FSw
+GAqYvwaTzhnz9JRfcRVO7vDyKrJVpMipFc8VJ8kLfHgi2QN3VfU7fV3NpPApqmn5PQ1WjDnpIJzL
+2lsLb+9YsTe8zNvJhK86r3aK2Sgr8DsKqBqsFmxlIpTKTD0mV9VFhK4s0mdM6OZdJfmJfrbAOw0k
+p/cqGjQoNmtVWHdr7dFJ17QGUveYIyqjFWUlbMUGgxpoqeSDH2Nt3hdm19yphB9/wximrvyc0nu2
+9az8Di+oXgiwUaHcWYtYALnWPFR4jkwf2xvMNooRRoIqpx5KX3c0r82+j2+HIV4/lqnA72MX+qtI
+YyjCyClTzmdNDxM6nScsZkPn0X1NbWd6QVOTGMTWmH0auGrvDvdZayUHNp9NfpWQ3vxe6kpMactE
+5BFlg46puxtsaQUeNssyVJLWHS7LydKHQIP5wI4n7afnVG8pOEAAgr9R6XV2k2nU5v1+UUCXLMqg
+PA5QAQTlnomStySs/dIRKGP9jgUCE1Tt1Ce9BHkQ2F0MdKXuBnmbczYGIFkZ2kucb7p+sx14CAnd
+ZurUDYODlLi2gcI46JRB0jgDatHibLsx8nxrC7uNy/YYShAdOM5UwvcIFKbMZhUe0WF1pqrElg8A
++Tz4Hjleqpo9mjnSO02SmjZH4mh5B5WHYhmiia071tmIO/y5G1XPL9dNSpzMEJ5CqjtuEypuZj3b
+Zq3m+1yXHJjZu5czOZNT2iYHDFIAq/BWjfAHVymziM7q9EOOI172ahXaE+mG/BSOdBYSCsJhopyM
+dOoxkN1fW+RLJGW0NeMLRetw3TiU4/x2TPULRd240/Ingxp6ATxqh3quDVW7dy9jj/jSCFwI9GoQ
+1OZ7sozN1pgBb+10RnFHYmobDhv8evjJwcaD4jx2P+nYtP/kwqMe+u8jPs9XctEhaUOVsp+8n3xt
+7LewtocFiz2yANraoWXX2fcOjlQOQynBI7T8JHZ7fAY0bzaQt9a1w3F1G2axX47B13/o7X6dTP+i
+5WKWx5LKmRePN/0AZu1fp9JcZ/O9CC4pJvrRGLCqCjnu8oG/MaTS8vuLfdZwAWazdbRpLBFw50gS
++vPFjJK8QncyoV6TOhiCSPnIHW0I2TpOX0jU/qps/3Sp7b5/UcJ5MY3K1YqzIKPSA1PawZyVlkYV
+dbFCobdEnvK++cB2g1PUBzGmxH0lDqCkFGLWY462N/r9vf9Fmrf9QjY5SGj6EVfanx50ulIUx9RG
+QW7pxgMhlsTiOl39hejw37xOFlodWivyLOMnBODX26a4TGm3h8iR9XS/5yWFGosQTblmJ2lewYTu
+DlW/DF/c28YW+LUkgaJy2yuY2Dk2YSXi/T8/7cE1Wo91tffxIgeNj/4kelr9t4fL1L/uw1fpU5D2
+8y/e8b+51z9d9LMM0cl7ty65qGt9Gwm2R0rQcjqwajCyuvvFxT4P3c93uL3eX8YTnrVkSGcuBpJc
++FNcVrQ2xuOEA/yLL/IvASifL7X9Kr9cquprFCHbw+wiisABoP8AH1zghnb4un/uwwfpJ18Mm794
+Dz5f89OXSYUfCBGHJV5gGtCRCgij9wmj9duvrrS9lV9lv5+v9OnDdDWjXDRgQdydFaqBPPb+I+XY
+K05bD4AHD7//6rSvLvepWGYYNRHa2+WW4Pu6U/ekjUT9Lr3MDnRV91++u22g/+7utg/ll3fnzWmN
+OJbLyeA7D9N/q/3jj+Du8fd3tf3S/++rwNT+81VMKyenY7vKumN3EeDsC4CqfPWmfn8vtvpJcY8j
+UzNpQvf+RRd9L4L7D2v/+nj3dxrLn3b3vy5AX93Lp6ljLlEttYglfPMm3nedXz/C8T3GX81Q2yP5
+3SP7NFl4ggqB2B6ZcoYUKOiDxH9zLpzjVwYC/asLfZoosLumhI9yIX0P7JOpEFj1Zcd3pIVNYEW1
+L/yT8I+jD07v6ffD4qd6/Xc3+WnmWPS6KPttsAMc32FADu+rYPU/wLT5qt/sdD/96rH+fg62P5/E
+kmHObM4FvW8wc5BKzNc1nbHoBlD+AoSRURK6gRt8tZhq29j73Z1+mkUwdY12tz3lNnx5rENSTf33
+4/XrF89zm/V+d5VPkwelEXgf3XZ3d/qxf2wuu6PxPb6G9UyjqX1d7pEMXRnX1v0X1/39cmqrn2YR
+8JS6RWDFH7NxedVcxCHVHd8KHuiLhz9AVzKKVP/HV9PXF9f9uUr8MnuVsxwnteC6ww6CZSCjZm9c
+6OGXo+bfXUcD0Ojo2E2oNHy6v75wq1rdFlNcw5HGimOEHlc0A+9UBTReb/prkOx7hFvn3uGLZ/vv
+ZrVfrm19mjuzDgyhJbd7DEEAPZY7ut+7JSx2/UE/i//YNfxH7bf/9oUnna7YLy/hL723fZP91//u
+/0Sa+uOf/KPlBvZaxetKQtEfdSWGw79o2TqlKNpxqm5gut2I2P8sOOl/M6Bh6yo4ZixEdMP+VXDS
+PAIlXIyLKjUpjd7gf+Qu1jig/HkmMDFoqUC7N2+Nhn/Q/TRiNTN1F7dI7CB1GkgtxYyX4CCHuSbG
+x5bx5Qyz0tuj0qbJYm8ehCjG5vAjs6d8U45p6bsaF4Kqu5WPyWn2qPeG1LVx8xc2SgQq4xraPnwA
+a3WTlVRBbpLZndYznASTd4xntoKz3UFAUuM9GWYdyB1laSN9RNuulqQvuDECMMtroaaq83s+tmTT
+lGP7sPTuluae9x/rYKpv5IxlGF2rOnJng+5Bp6L10Sz6GNCVh73lDgMUEBXenmlO4WwRq0O4Nt0h
+D+GfchwMBdCmY6YU01xaQ9GE1Iiq+NyCQEGzDta/sHkqQUkwX2TbuJcRTHrON3scXO8ttmOa+aZs
+pYhsoWT9bqKkCJ0CfUxPLk4qxUVeSSRN0l5poTgoudLNy9OL9zWfZA0k1li2HGkSqwEm5tCtu9w+
+dcQkER5NZDCBb116Yy4atQ2ntMbqqVYaF831pspWMwst8UpNABctEQIQcld+6chUIOyGUBNgVPyU
+c+e2zF+LxQRDk4tWZ11bycBCp78opwTpuNhaHJsIuuos+5rYOv6KgpKqvpssQ+6hf5DXpE7NDZLB
+nVZaB7vN7KeFlDTEyrRzJmAaF6mFArWbdacnLX54ED1Qh3FRBQggA7Ai4g8laGAjhXU5axQn0MIq
+sxj9QWnfgLMwCPWlP8/K/Ee6pgeio2/wIrmEOBB7AQTEB9132Xb8Vu/YXwzwvnP74OXi3anyoTjJ
+eJ4Rl1VI4ALU+d7esxt7OKdZ2tE5zJu4jtoqJhoFYVt5mzZ4FHhOhbyf1JS7bfukP3aF96bwZJMd
+oDI9pp9Ve3fAdZPvM3aOLBiMLo8PEqJGUxiEjtQ70Mxn9Wq/pwBUI7fO6dbggknsFdli1u1GKz2J
+wTkHCUt7CbPAoRrL+75UWwQcqRm09g/R57dQE/OT1NwfuK5CMK4Ekusle8dh13dLEsSLShCgeg+5
+6URQ9uvsulGpWHvIFPRbuyaEGVVGakz7dcy8zbnSMXr69NwFuaKQyLYjQCKp96uBtHhXO7N36gZd
+vXChVlWho7mX8zidDNt4xAF2VSryghHv5Bw+pTvtTBM4MjosgrCU2suv7XL95uXGa9W3BRi6qshv
+4YU+zfZck7+VGN29U7vGj5JeSX0qKYwwaAx7py/Gc0VgCGM0bqcjjfTmPclJlzuQhJilO5ju6Iu3
+0K5LapeAsGifSHEO6HW8XtxqDduqUw5JMtu0nyVieWCbWhah1588WrQDYI/TSL3xOyUxS91hxzAt
+cEhsWZNib3SkWB2SxlnQA+ak0ASVi+TOB0WspkdJS3odzhVg99i0JuDll4spC3OPwsn0TnEnqKhU
+aALQF7V0DalaVzpBMKtsB1JeNL0N2jVNjMATVYFAPWGvCqzfOw6OsC+Nrnfh9KHJqgsMmnLTZtf1
+fE8Zrmhf5Rzrzw0pJfdL506ArgHVFby4DsKYbCGd9CUfv08lUt73Tsv/axZWaexUb2FWSSSrkJ8M
+PXNLk8X4HRJLbp091wW61JA4nhwcbzCh8uYZwPsoXbys21sxmrzQNFv1DG0tTDy3JDvngMWbua+A
+ZtNdGePSw9Yz5BRf/YG/AzVPYE7eIH9/kkmrY5kejVbfG0o6DPteeNB/SOxr3WqnKkmyVSkviBBU
+g0Gp7T3QwiSyu3F8ntLySlOrpzgtr1vZnJeJsODVy6tUH0C3rNamCsw4tNvzm41T+aYbVwWui9mF
+wu5wKKjaB8Tmab8qDZExTUwSm13kL2pn2FudMdlVdTz7pdCv21jezylazKykEOrhpzwUhMRcN1S1
+9kq2wcpV2wX2NV9mqRj3oO3gSjcKHUvTaUPWAOsK/h9VZTGAQYstF2AcShSrAO8NMra+YOjG+zJL
+oRAVZo64Y53PtcyqQ0LlbrQUWexsYpPK+CUOfVx9q9vciHrbyI5Z5cpIh8q7RyUnz1e5zHvXqPT9
+aC2vueweuxrrGCquy55ACr8jvPIoE6neFRRqEf6nIcEND3VTqkcvbdYzSCfGyeIfBmOcZDvbmmEe
+q0SqNQ6rSMoQ33QBPzTch6qB67zjV0H+ahgvawLQkEmOk92qaKHdptWDh2PPn2NuPbYF/VZd1Pvy
+J8W5VfKdu65LtCJHWFPlLWFNoLtrg9TDiHSZmvpLPxJHYKFnOAlQlzQgDOsSgaM8ZZU6+mUbK77M
+7DxwbNxWlP1yUJNZ1t+VGP+ux8nU38aszh8TZ2oAkUGaFBFcKfOW5dM6Syt9Rt/B90BIhi0jckvz
+Z8zP0A0dTRU7rRrpdK/uZJwJ+jvf3Awgj6/OGGH5lNdhN/7UZMe2rj8DoxhOwOfRa8ukBjnnduVy
+pyEBejTmAsr1JAh5akX1DGqf7pc7zy7QOcW4YeXoZj9Nh+6DMVTKIzDI4TA26vho1Ll8n4ZucVAO
+bPJyDBoeQ1ZLblJt1a4p49YjhoImpluMLh0inwrlf10/cA2o1+5ql0fkkMpezItyYbPjcvHxtu1d
+Qa2yiOjgIaSoEw2+nErbIUIrahB/yGRVcYjS49a+LHpbeTTE/G6TgnSd2nM8PiidaHSCCdMyUaIp
+zewQX5B0omXQNycOlDx9A4Btsuw8ze4I3WTwkrEZqKzrh86AExhYcaXeYp3Uvi/WWO5Y7PRwRLsk
+ArTM1cNQQ2UJe2MZ4Mt71esw2a0BSlQk3RmkfITwoljGwOlc7RkoHuGVCUmMhwWQdeTElbgcGnD7
+2BTb4mY2RPddZa6jX9QsQ87vOS3DbjJz9WYituvEbkitwsWZrauhyaROt2rVBSkRvfq9cKBwHwCY
+xUQRTHoq2HkoHm6VZmJPDigeSWVA8zN5l67KhgmH4YBho2ygN5ag945CwbEVJBPTMv7cjKYfwEQQ
+Iv+XvfNKklvJtuyI8AzCoX4DCJVaMpn8gVFCC4dyANN5Q+mJ9QKv9etkMDrTbn23lVVZWd0iPaBc
+nLP32iaOx8Ja3Y9umd4X5vLd7pLPC4fCYBTDRTEWBzSu3LMl1qejlfcy1HWWbEHiZ6jZ/qWjL3fW
+ihzWPcmPV986vXL6jWQjzHc1ZyEbnC0L2M1gowTdCAuLI7YjNm175CRqp43Zyuvj6ME3g98039W6
+tZoTtV7tvLpjK1O364aOvDoSrISy6uKCgoaH8AmRgmCVhzNY3XVymBBCoPFSHeGtNdYLhF0IOZBP
+W5uebT2MSmlLPu2m6TWnotlMai4Ig2FcAh984hRopqgVxeoSt19uNP5Vgjwv+9TmOMzvqwVvwGPm
+Zem8c2q/xcGCzmZjcVTluI9mec1YGYjkrPZRVcOv68X8nNs0bhDdlfUPADFNIL1sW0nc1SUeuJcB
+jwCZc67s+zvNs9ZDAn6l/EDIKjhsThryBbng0Oxk2Wk/8mjiZsxVuSBsixK93skEuGQoyQ37QU7y
+JxsnxJG5V9xKf3HuClSH3ncB0Su5BEE2vAhsdvturPuvni0dsNyMFuFicqPbhLXm1ewi+wbC25rm
+TGzMEAEX42Nuau2iEUOebIVHaF+w0KqKVlu8N1ynBvZGPBlzWdzGTRr7YU2CxVWUx8YPEuXqoE21
+nyrz7M3QgNbHa4goCGBiW31TXOWPxirEl9wvowdf+l4Yz5Nz3cz0oKsqGpZQ+uN6C+X3VPPVDXlr
+Yzh2ZX1MDU4mpT25O1xd2GNK/9sgpmEPUNS+QAvF10kvLbSmpqn5dTRPN00/Y8oCW3brt4U4sJir
+C/z33o6gmyuJdR/VL7cHpB4h0UYqttqU4itrfCgKKLnHp0rY3vdSlf0DR107nBvQfBaE7Q1Ll3Np
+ozE4wBkFo1r6LEF4MS6zrCyvLDuOsUMJ0T96AiyjJpvKCITF19gxcT8hjmzCXCoPKh8kRmIVOoPY
+6KZDysxZBYWhFV0vPqpDEJlYefNav4TzyKZ0druDT0rqBovHAsh01BauGNsLi0J5S4pFGfjM/Hhv
+e0AFfObqQuBm3c6+kYQRLccA0xrUzqacHi0u54kOJJbIoaTzN2rCvZrzsgujKpsA5cryacn0hlMP
+crEDz1I/2J33CVUthObJrMMuQV9keqtoNYJKYBYwOzpjORr8QpQKmrtn1bGo6jpGfq+lZXOU8WiE
+FdsPDMSo292s167cqnYPGbGRh4bEpS0+dn0v62K1TpS8lqVhlk/QGetPfiyKoz76NHfspq2/DVm+
+PFh2mu/TymY3yaYjBJFn3WpDPEAbtrUbb9R6tIVVsW2jhrff7ipsO43/PXVNL3SzxTrm9ihfh25m
+exJX+OdWqfygXFzsIsmYmXqa+Ilr1Hu3IfBBmaz7ZVoTimLDWgW4P+Y/OUx73aboh25vC5KgeuVY
++5obdihluuzH1Fd7ztgZMr9e28RJcZHRdL4sBtiladTJixbOwzE3YnkJhBriuxsB7lRFhRVdwt00
+FQbtRG+fkTP3W70uvrRuHm3LCv2hVtOjj9mwbPt0trdTGUkrXIAnH1DND98oesyBR54LmdLZNGHf
+E13gLJETVnbDoadP6iT0jKQ8kG/xkADQup2LaNpFOql9uML8+puHvGArumXaa3NGw9BZ2gNdYufQ
++1X5iHnH+kR7yTtCMh2/G4NZ7YHTxtvU1wlMUXhBMerqT5kd4y4V6ZWi7nKtG3Z2MOEak0iUPHe9
+0x04Cmg89+ypNZ1QU8nCo+jc7WB6fUDeY0MEJNMOq+xjM0RmspHCqcjk1bv4TqnIPnSWro58U3GA
+wYSo0EY5qw7uBb80UmsfbnLSJwXCzSo6GilJVcJohh2smx1pEdahH5Lipc4H/mZhUzXSJWdSW/kN
+mlspj6peLbflcMMfx91nVUFp1/5zbaT7stWsvTHZn6fSqrcFdsUHgQDnodOXT5qPHJAfFh2cHHin
+QSwxrXbgQfH0dcmSFzLD3OOKGw2EOTbHQiafbWOsLjp/6o/gQr+rdrgsYmTEHQkMW3uYSP5QREIv
+A8DxuHO/sVH+abeYk6cZv7FoEnziYl9luryXJbZtPRNz2MYNBufE0245fFh33Wyru8asiutJR+Ld
+glPa6i6lLiLAnzlPP/ClYXxwIgoJ87dc79u9Q+pPWChWY0gIQ5CN2ZWH+ylcFMpmXf00p8a5mj1l
+HaRevHazv1uSDqXOqOJ90XbToRY2YYwyTkD7tHeOmc2Ba0Q7O5Pc18STtw6Vq8AvKeYo3buqm0mF
+vWUg6vQc7WokwXSb+4it9KQpbskhRxtVDff1VM+3nUUQaON2yDf86gClYwk1Y3r1ZPUlJ4EzBOmX
+vSBftbYsaO4zDOTigNnyM1IWBWLGSYIZ3dllOXjXo17uHG80+cgU/3ct0fZNj7XMX6rH2mytHSE0
+nMSU69x1xRAmq2t7yaa7pTF2K3YUHyQs+Vjkl2lu9Zs+Lr80cJ8/FfF8m0IIg+3coOQy5+9GN5Fo
+kWPb1WIyrThZU+quvc+ZPVPOSEcY6wjjUM+61zruyO1ggI4AL6TfGFBW8EjFl51CJNrWSHhlFt8t
+sn4l2vWpIId8XzXuhafDonazDBEykgbOSv5N7uONsa1jnWhZmJncb/xj2GkntUPds3PZ6m0w9MO0
+1dMXR+AwMNPuoRrBXUXoYIKYKYbMos7ZNDU4ZlXG9zn0T866hEyRlImAdBj2zbyufmnzqaymeNtX
+0dVozztc4ASlNnIPBePWrwkwd6fuFdk02JVZfk7hXDGxdvfOJIygMaLp00SU/CHGv8pyPopdNKv8
+lUS3H7HZ3OQIwQ42HIvQydyLtkwfhqb6mi488lm/FC35wDmppEFcZUiynSzDfDgVr5i38SbL+g6L
+8M5xG0lmIHayLu131IXqoMgU3RW/fqIqfssWbkZUAKkpR5G0g+5zBAbyU8MWgIccLvcwi3bXdgBp
+G2xygVUk19IA+DKmyUXVehd6qYkjaiuAjfgONgoF9jaCGr4b0oxcFZttkYuBm8Uc02KAWbgPbDPy
+dxBw+f/E7XMUC9Yx/2qq2247JNMQRvH8IHtObXKJnnS9wvZR3OjsGo6aprUckZeFG2x+Zpb+UsB/
+AunRP8mIeYcUcmIGYm5HpCXQbKqpDXqkU6GM66PUu3BW0Uvi1c9ZN4EzSOtp66jkWaSVRTAWe2zd
+mO+hjltoJusLZ6jNPbvd7LbPxq2ZL0cKdpezWVzFU/2Y1NYuTqzLkQJzgBj0kEEGL4pla5UDOW/1
+0Zf5Dp7vVeGynQN6iw0BdgdolQ7f7Uh0FWV7Xcu3sJBT4qxcoumW7wZoy67tj2LGNUe+8lZQxK1q
++w53OpHspKCExALdKgERIcIWV3FuM1dD2+i1QdRGvyKmuyAqvGOUSjhjDXQEyQkFJxsSf16gGS9E
+nF4utftLccAPliQrjwX6QFm1oKpWnDAMA7NHkAc42NTjC5taTtJkYZW3x2a0LzEv4XE2y19L3V70
+k34HMP0GD/SXHEDAdexHyY6KK9NERzXLYFcFT4nKVeyi47ZuqF11W+LdvsCdOwzlz5kEZa+cDnJc
+XomP+FL2NmeP6XKZrB1/zju2zfhokbEc1l3xXLn+lT4MgT8v1yoaXpMKfjfc+VY0B1zhkkRDjQ80
+Q/YXeyk5Ys41sKrkJi4SJN4jargouxqy/tGwamq7SWxUT7Hbmoeqw1JOPtanRKbfHOk7YWImRC9j
+e30clOVT6JVdfcx+n+RmJK5mKFon83YcayvvkFtL/GN2bVKIUhwX9xlWKmenGQKLa1a5OEfBqlL1
+U7pjvnp+sjYa5ngiYYvD/gbZrhU/kM6dWGEXVd7enSL+uHQ63JmjZ4AN8UeqXp5XGoAKACDeARkD
+gVCxWieXgqk6eUn7FZykpQcfTsuGDIn8E1OmZz6NrpuWoTMh0dqkSZk8Ghik8rDrSuNFJhwkvJqN
+OZrZfZqJJewTgfgnBb9cREb2XPaEpoYAzDnQMRfz4XeeuJCohCrAAYBD6pA0Mkd8hYiFljldvOSR
+YDcsKRSSp6Apx77g0VXiO5pgDSCIw1f5iO2zn641eghHpZz2mGdputeW3nOPZVa61j+91//fDX0L
+WgboT8v5/01avv7afq2S//XffwjwzX/+1P9piBoE7ADw0y1b8B8YjP+nISq8/3LRdAvdYt9Kn3JV
+2f9PQxSbIYZAH20+SbsmmMw3DVH9v4DDAAvFR4U60AboeqK4f0+Bf6LZsWiqCqKpnfXvgd582r83
+s55fjh0GSBvxsWRApOlnucwlLrUmEncyH9eAFy/pK0gdBXClNzfs7h8BxlvJ0Kn6Yx3fXmUDLrFW
+GFt+K+je6BQsU8uF6nXyzp3ujp5t/mRQzA9H0RZ4eLvEfswhiLDjYgsFPSCKInejdZ18TloqS5v3
+f82Zm0G9yvBwffkG9/ZEUMBRtG/R6UOWkZRYChaib8qZNZhNE3rnOcqvOckSJ5R8gERchURvxCn/
+3ARYrEQRG+bqVuWfv7kJHJgK1gTwZfaM3oiDCwWVvT9Su/jgdq+qodOBMJzyVlmWadMB/3Ogsqoy
+4u4rUkG6IXoe58ziTG340SX298Hdv383zw22+kfWniNi0lMKaY/lNdF6yGYLd/qiAfl0oyoiJkeH
+fNv3hzpR96w3EMESw4CLcwGVrzf4zQ00ImHjIeC63MyNfmRkCz17vTvuc+oWhywjyOj98c5cmoMS
+AWYv3GkIs6sy5c14haAuMczM4E7teqGGPT6gy0P2K3/m3z8yT5ikhK+Xhh/55N1InRV90JPXBu4S
+izDFqyHa2Etl4YKtCM98/8JORGDrjcSKw4UZdAyQW5xcGGkFTgGJmqQkcCMBoal47jQJ0okM5878
+AXNipM6CdvgDcO65cXFdMyQZpCtH+s8bCuHLKEzLZVxVAbmahlTcmLMO/aNKk2e15hB7Y6J9AE0/
+8xgxPmEogGjv8l9OPofRHRHto1gAppFjCq34yptcYh9wOay8f2PPvKHIR6j8GTCy4aGfvKGLpQYX
+VzQd1G5ZgmIA3jM7o3cY2ghSHhHkV++Pd+7SPLjSeL907Oqn40nlxnLyAIPWnXCOpka7Ah4djnAP
+vcX7Q60//WRS8SgAWzr3EKXOuo69/RiEgxU0JtMUS3Ja3IC0XMJM4Or9D0YhIc42oVk4/qmgTUeQ
+gnOJ2URmBYiJCJ8uIET1AUv+7G0Dab2G0bEEr97/t9fSIYFpnZktnCwoGgeI1ov5IDJ8POEMse0j
+cPK5twIDnMC0h09ZnLLZdX1xOHQyb2l9/zj2y31ZS+IIcP1vXDoKHzyoc6OR5ueR7AA7XayYhbcX
+11Rd5lgNH3c7y/iiSqlMAIl1j/o0NZeLWoYPFoAzLwYzMl8zmjDGPI0kIJyMuFaNpBE1woUhmVY3
+wQfWRvSRfeDMU2MICychpkWBNeXPC5sa6oE9ZB5y5PFQrUihIXTz2qN7RaDT4/sv4pm7yE0U4AhX
+fySYiD8HiybIo33sUVzl1FGF/Bz5nRxQm06Hhj9nU4wi+fezIys27zyOG3aKYp093yw3CzBb/Okg
+V7MxjQKywUNhRukG5zK244hT9jQZ6oOV4Nw9NdgWrptMhHmniaNJT+I4lQi2fV1xYdIo3RYlsbi5
+MD+Sqp7ZdbF8/9+RTgR5TqMPHt1yJDDoWVAS0Jn/xHyN4RgpDlS4vnfKB7XMlbHN4Px+9PKcWXp8
+l8nLW/cqrDEnNxf0kUcgMdjMflr6/QLO7G4h8CiUdifp7aycBqQOL++/RGcHddZphs8D7+vJoG3p
+KyP1LCyCipua+kX+TKbtc+JU7U53pLVTXSI+GPNE+Liu7etCwAy6Hjj+lup6Cw56q602ZSXR1STV
+BanCxQtQj+x7XVrlF7skV93W9PZoKsCK71/x30+Zt2jlw7PD5uhyOhnoonYnqwDaM7iTcU/Bf94U
+SRt/JaNruF48beXPye5aa7oPVsK/Z6H19eXLsVkLgcGcbC1AfPvAxKtqExFvdbse6reQvMwP/HB/
+zwqWy14CtxYBpvzX9Ve8+URHtxrSlKg90jSH5EsMLysJ8aDW1U5EU/2lH+z4A0n73zeUYXySGyDb
+mPRwTia9BJ0K3R12FGVPrQGLdGXf+cOSUy7OBal3FmZkt4r1NT8+yuQH08O50X/v6sFuumvUwMn1
+0kFK8ZTUG71p8MWCeCZDStk1aC6f0E9jk1bRosJm0mlTK6kZP99/nf6enizWFH1dNVnIODz+Ob4j
+05RtM5OGOUFp4N9f80ZAJCcZbPevR8KgblpcIwNykP9zJM4Spr8UrJprB7IKq8XDE0q6AlmzDiXq
+5IMb+/dXikSaYwX7ROyF/8iX37xIHXTXbOoRBDpmIX+woIQ5+aWhkVPO7/uq3sekOr82CmhmNlvi
+0/sXu962P/dyjO7YRPKymzOM0zyAfnCcfOgYPcFkfGk0wODsrDL/9Se5jkJhg42wTsjTyYzPF+LR
+S6M/qSvNJ6JW3EBp047/waV4pDuRueSYlJj/fG6dEA4SzLUJqpbmjui+aN5geR6TDya2M18+OHET
+BwTBWWy2T3ZVJC/bpYKuSFcR3aUPkhnmOHSB1nenCxqd2r/eolre6vClbcPmw3BP3vyOMmAt10ek
+aSjqitErbux4BNwTT+Lu/Vt47l30HJtsL4KrmG1OLq3MUmi5KcpR11XdUc8krSFDlKE5q+KI8EC/
+kFZv35PyAX7JTT6yrZ2ZY9jWcUuxpDrUvE7mGLvIx6LV2YxHE3nK9G59eSe8wvXQtLntk2lqNvGK
+IpVPIiUU74OLX//2k08Bw8FaaVszteAv/fn+gEZALk45ZmOgUnvlYaTOpjL5GIMB0THt/SjPH+Dq
+2f/BhMPAvunzkJl2fvsg38wAPXpAFA8cCmYD4ZnGLzyOHjmWhjvkj+8/YFhjJ1dJcZJAE3JN3LUG
+R1voz6ukx0OesxhsMowXSBkSYRtRw4CKB5RfpjT3iWtVGBBMQDa71OvjfuflRbugdfMxJthzbry6
+vUcSPDLIetmlpvR+VnMzV1CG1YR8Ee35sYjX08xYJu0xHnUCuhyj69md2zadj3lIiyhwdYXseJnG
+OTCjYcR239KP3JZsaSCPj4n9q1uyjEK60ZQuvKFBXiNbcklUGw0b9Cxy7B+IqmmkotqavG0G+1IL
+kJTz19I8mL5KJy2+61YFwhahj55S0Z9AS5ZdB4PWGEiBwtkvNPxDsaeuknJK3Usy72O5aU2RG6sa
+fNm3zljYQaEJ8L05+/V4iz62eTCyGdTrOLfx44wWDyMHl/mt7wV9DkcVpEYsg2sm4ew78kKjHzqA
+kTKKLyLOIJjlbCvKjZHSSdILhE0b4ffV1eIAl4dx0E5b8pAxf2ssAYB/ncW8TkgjgEPe0l2kWtgb
+u2RArhxOUiPrALasLMJODP2F3tsyDV2OCNDHaLDe05bWe5hgUDU3k1eAwvaHiTaGSwLBN91roK3r
+BjzvHQts1NNzbsjAhO0h9A0h29N94Y6wya3Bz7FPI9psQpXWTR0otFQPw+y7HPD8ob9PikjTAxN5
+6WXasPVnb28xj8jSGG5kYZlN2OHmnQJlo+6Hok/ODZMI1C/kup/b2u1fBLJ7bBk0PafQI3cj3lhJ
+ZHzPRkIRwnFER7f17AnIBKLTnviCSbbTjsRiRObQpfO70TFQM6dtgpcc6DFJDPSA2BzBLMm7MHFh
+YYSTUU0zybczOMvFXiWLFeUn2FcSbU2QmYv2mtQ5PBJ4GDCmCQtZNJrxsWNtqhKPRSDTZhm27Fmh
+wtXpmL54ES9pOMalr4WeWwwDtpAGy48opHdfSpF0QT9o8kvUUHSnW9YtN1DMdW4VcTUDgTiuTQqt
+H/lPpd8BDLFGqOe7cpE5SVGoxpD64HMJk8VXOrYZJSXS+xTwcNfO3RMZ8CMMHWcaviPLl+SbV+w9
+l9JNnngbuA0IJlF5Zvr0GXAgsufYA8kd+HIS5jEvrQjhZjKaRojcuu2+Kgh+6he0A6sJbMdWGtLy
+Wie42bVUE0ZF3xT7seoM/XMpovlr17Roa4BeJM0NLEwtf2gIws0JLFi6NfGb/HK2FfTRgsKIagLb
+XYwfnwyMOxpJBE5UXMhymqfDaDcpXWAzjROkl3MrAuwG3fwZxUh6l9CwTIglQUm7GY0yHzZDq3sv
+ClKRsRVjSV92cfQCuxXVNn2jLy0teXe2HVrOlfEkmwQVLMHrdXKAsG+2IR1+s732EHYXn2MgO/nW
+zOqkvusrHST0oCL5o5/60kITsxScXjRvsH6im8uh8RV2NH/pkTdGVCyTucI1ht+InHvN9C9TYXRf
+Z/53dQv/uCpvo6bwh+vKqqwe2pcdAeXeVDao1sfBwZCGDhq2+zFjBnQ3BfMUzMeqSK+nfpngB5Xs
+OK8VsSr9Pp2EAB08SP1Fm8cx2vjUjQug9oD1LmK0mP2+iRehNkXVI3DXcqnd9nY/+lvIJ2MaQE6e
+sM2rFMPOQMJQDy7YQanTLjOAPeAwLvpLpzbu5EoTT5xuVPsMHFUPwVpLrsaytpKdha9DuywSxGqv
+wO6y5MZXjglOnx5ug2ZJudaBJZLOqep9Q90OEWnJX+VgWxZAwNQB0lEKms3oBgbtqs9mB3gum0/s
+QR0SKz0fKgJ2fapw9xWRwt2l0+cFpj2HZ78bfFP9Epia2kNVjqCo8znqOx5I5GbHWDey7zqpMCkO
+Kh1ZOglxjRcUCM8wX7mG0pHfao2LGyCyJbTqZtYOaTn5D6YVAzEyx8WqA9nSq4Hkq09JaDcj+F0R
+9VLHMGKOxSUt4RKxDL0PH8VVUb66sJ+YGzI5sDvp67bYT7M59mGPWAbjGlW+sPO4pCDqbP2b269G
+63SYm2MbEZmj7MjQ8Nv52c+5c+cXJ1bxtYNg7dbXh3JnFn5+axRenh+dcpAqqDqS12nIzeay6+oU
+sUE5ZGN/45aqa48VCgtyw7pqsilgzLO+m0zVjIEzlIOxme0KVkljEtSwM3Ry6sNlZnZGFpoJNB2o
+MmZwpHCvA5OUonlbWNChbkp9LJH7IT6kZpGknrt1RL9cqG7M84M79UpDVA+iYQNFPi7oWpP3s+lh
+NbNAa7kVbeuSyL9NW0xp8VK4teXtB89pyKSfvIQfQmgI2xxZgMurUA/HCECaRQV8r7gGafo38MJB
+iD0S4NSj4SAgh7dRQN9nttSlidKNwYLehxWDGSLFyQ0Qrbjs5iqyQzyAKxzYRoS8aeke3qDcZ5/R
+6BJ1fe5IDgkIeZefUaYZ1wh8kI6UPb9uawL4uzP4Ltor2uvFbUf0CjqFOm3ysIkly9g46UWzZR0m
+F2SeI5PokWFpXupMN+9Lb2abAaK4e1DEDTWbhZBnRM2kDVHziWOLYB4xWL/ofbgY07E0pZCUGmJD
+Iw9Z0COptNU+652JxAYIVjriQzndi7Er8t2oNXq+GRMzBTQ/cuznYx+nK9yNEOr7ScW/EuEmXzPE
+Kx1vroNHhJhU2hpF7LXVlqnLznZoYgD5JbQ3hz1rcHa/QPSHxtw7zq1rN04WNuOKayrtxv+S83nS
+JMFG9clLuhaTaDx2dej0EllgRlGS9LF+uop5r0AGNimS95LUvDuF6+Mqbcz8s0Ih+603ETqHFvFT
+r7y9GH1S26suJpTwrJX2IPOAXUmxvkEa8HcPN5u11xxZ3yiiVG+cKUZlwjEdNWtTKu5X33bfcVTo
+cjt4prtdzJG4gsldCA8udH7MZsqL8Rei2/a5aoYKd14rLlLTijowiUVfrsSzUQRxo8XfEyD/pOOi
+y5pxeESdEWRSH8EYogaBbk6Jl+hRstHbGLFuWLKJmK8sch2PxOl0YwhnX6kN+C/gov5Y8W41hSOf
+usWzRvIfVz+ov6K5N0PDIftmWtyEnRdmjC5QAzVKfBl5Ox7tMq4k27BEshmrGtwC4NHBXZqJMEkT
+h+KVVSvLaozyoOu46Zt0JEeJvcJY7k3C5QHCN8nApowWfhPQ2eW0oiFEyrb4Ctl6LmJBrkxtt3hY
+2gVvnKaP5rJFI82cTbuo/dzhq/WRXCN0CckIwHXnYZiCYK63uh8WIxsG1owRfnybjNEeMnjabxev
+RYUTJwN/be2j4QFrrxHyR0DdEghjEb9ihW9kq8rIMW5MC6sue/BUB7mPNgsOnSHQ98Vjgu9Dm8k/
+DLWl4m8fKwuhDxMEcUQuS98zpj9/2cqWTQcuYmRjB2NuM4HXs2eXU8sUI4QTjZMPO09CtvfrFvmt
+8DQJb1SUz/U8Fmw9XWvRLssqcYgt8Wb5EHVoU/HkwstC8I7vhIlExcuu78wK9D4Qw6tZVqIBb5o0
+Kmic1tUDT0yFtpHG0q9gNU96F56fej/Z3/HFjZHJfrzX/eZJo4jTb1rornfKQo26ARGcPuLxdORq
+WOl+5eUIc1xLXRRBWd/B1W+72UswOiXLr2zO/Itqgvu8JUbNesi7cblehkJ9mhu7mZm9tPLgLWWM
+gqjHfx44pZ+hAYpMbwdf0TGPoxH7l1Od8CMcNEy/gN81xGtXeTIFtpQaftZWo+XLqskBAV1RnASa
+T+2RfT9RcGtKfP7DLs0RY8WE/yGQbjQnQS+mrA1YzhBaVW6BTUbDfo/e2+v4X2rwDE/k3a1Wv1Fh
+2M4rif2IMiqvWMQv38b5nDhh3U/YPRt7Tg/14iB+RoE7q0ApjQAhXn7CCNqmxm7OpMffrWGE25iE
+9q2OnwFvUzsN/pVSZHts3NjmhVYohcttpq36r2oYpm96h+IyiH24Ybs2wyTC+8SKw0ZSqCe1lHV9
+Z3mxXR5qP9GxipFj+Jg5AzaaqgIEELrTxLttxYnjcjro1M/WxZyuCp8fSCWQk8pIlRUzufnbVFV2
+0W2GoexZn0gNAobMJnfDzpW0LuyxxsjSPXE9VjzzxlcSHWGsSfUz09f7SBxa0m+7WEexphKnEEEm
+Wg467KuSezxQa5RW2/BzqnRUP/VY8DdpXmHMR3JX9PhYZT4jWEuPE57Vzr9qMaO4VziAuRz2uf4V
+YE3+eBcpXPFpYTvulq31+h2Czx93Vrl4O+SaTUL2lWH8ctqy+/Z+3eGksiNQTbgOZSVanhTMETL9
+WXWwI4Wk2XLJl9OQt6KLq7LhoMdRw62PmltU1z4HMhFftsQWtJv3B/9dG35T2fln9LWUK1zqq455
+UtkhESGSmI9AKdaoPhcxxyGHIZN9sfdJNhDXJClgnPPqeFtwR8Iq8+Y9YUzdlphKsHKz3b5oFu/Q
+B79rLae997vWu/am8FPp0rGpppNdEs0y2bYGfopN6VfTFrrnrxSLIdGLsZbqG3KQkE73OPvziimv
+LUfOY9LpP7//i06K7P/cqN+wO8NZFWonP0iicGTjlFH6LjkkY5ojPjhiNaAN2NVO/UHl+6QU9Xs0
+Spq8ENRRId+tt+fN5TdKVCo38orgDtv7JlL4qMQzlAqR5WRP36K8Nj8o3Z57DV20LhT3nFWIdlJK
+raKoq/MOQ5WQlXnnRDUYgcjwtqS1Tcd51P19UyVDUFvOB8KTvwemoIixbH0DGf9U9TY7ml24DfBC
+MiLVWk6dr2c0RZcT9rpdO8k+lJ7EUWEX8e79R3pS0uUm/znyySP16jEXOlEjuP1nTDy1mY3+DRPB
+dOvLMsVcEC0sttKw0+a5FK05HsekQ+D//q84aTP88ytQOOL6cl1MUydVR6wkeGAEX2DBGsqRNTNv
+V/vg8f1R/n6huFZiHHiZHERh+snjZejU8iXfk6WM/sJG2o0w2rjwpFKPrmV+FGv+962luclrhNrX
+pWdunTQcmIBtX1pc1MI//aINlCLBlQ97N1fTnabB5AMAwZpl9wNo8sHYv3+1f3+sNB+Z06A2AqdE
+B/Hn5+MJqkalxufT9hxf+4lwy8FiooL6cHh/pHP3lb20gZgNpRgKjz9HavxV2Z/Syo3QcB+LLCbY
+mAMrhQVX4/xMjJx78x+MCCBaB4Vprv3yP0c0YEFLTrik8CWa+h7NmkZaUubCBYYZcdei5P9AcXHu
+BUVJQlNnFe+SwvjngAqBjKitmKm4HVjW/aXpoCK43Vh98D2eHQi1HTxtIXhqJ93FdHCULEfu5YK7
+l81bz4Z5muQHo5x7YnRrDUSEiMKMU8qgcr1+yRNGwbBmrwRlfzkA9Gm3EEjquw5awwfNk3MvI1Un
+Gzkh2wc6xH/eP6emgDp76ytijP69qhZJHGYcu9p2KEqAm++/Hietmt/TiY9Bn7soMMieqrZqfygG
+hFS8+nDsv2IKYsXAV52OS3PldRX7I/Zo46f3Bz0zh7NaGZBZmcAtGsR/XuISeQQv1XW18VIiqXnE
+EVETc7SxymwnC5IuieUVRKfNAJbfH/nM03QRC1s+Ug7mttPUGCqjNd43vvQuGrxX08hhc8vBGA/t
+spoTraTavj/gmZd0ndFQqtF25JGuP+jNytwpv7dFQvWztDQUIopImEGz9N37o5x5iq7p8LXRd/aQ
+X59sCv05ilfbxirUyI2J7XJO0pwFnBymDaRWnmemz7fGTNrABxPa2ZFZh4TBekQnd/3nb64v8rKZ
+Ei8SEUq5HDAmy4zIvuHb2Mwog76xtABsADgzRh8MfOYzYTydLQ+9Pi55fcfeDNzSonD7gYHLvJku
+ukoft86kafc+NvoPZrQz14jKykLPxWwGtfhkeZCFbmK7LBGE0iMLtdV+OtnkXnBXLfO+qdP2c274
+H4lvzlzg79Y4ckqE4KZ+coF2Uw2+P/KRpEYHI7aFjrMGIO9jfVo++CrOvKS+xRSAyAgVIMbAP+9l
+1vZlOyxcYFSYAje8NoVK2h/JmP4eZRWc6LRNIeWgCzl5VfSRylwqkcVBdh9uc5UTl51k4wf7wzOj
+sDsy+BezJwqCk+lz8KqGerJPlLNL4lmDeRPaPO6p9z+4M6Nw+KG1zhKObcU+eTiUBseJUw7Q+JlW
+ym2bQYsDy4C9+4PX/NxAbHNp5iN05U04+bKtUYiY8viaXKDjaCrNNqiT6cv7V/P3rGgjC/ZsD4Ek
+e77Tq8FOY6iJfhfVQTu/YPIkPpRWAlcH0c/c5nDK59f3hzxzXSi9qMyhv2LW+A1xffP5EuyICKlg
+M21ZHJbbxGt2MCmm8P1RzlyY6zEvohJ2hSNOR1GI8mPO/whMfLIU6yJxr9DSdTvPpcaJD/IjbeL5
+8TiXOL+dAKcL22jqg0umWLWxC41mqFa0kC2qKPZpqutZfT/8b+rOpDluJMvWf6Ws90jDPJi93gRi
+JIPzzA1MHATAMThmOPDr3wdWdbXE5JNavXubtMpUUcHA4O733nO+oxrr9ddf8csLuai62WWQPPyt
+H1DoKekaXMgpIXEYBw62cdnNf/68kykKZJJgUVbdz1UHvVf61ooNps/16NJXHTMZkU2/MfMsb83P
+VTyKDIetBCNRQP3xaYVYknvxD0dwe1H6b5NctaElhvEGgxNovpGE2SyLVb02267Y/foyfnHnOG6h
+JSe0haLys65qSPW0rtFrraRrx4+L3uNx7gO73eaSft4SowsF79cf+fdtBXUON4x6AMcIJrefV91k
+NIHKuKpYQTeYd05vGs+5BkHtqJn0DIgiHiyDlmzCiOXXH/zFI4O5AYgWRQjv32d3ETYgDrBwNpiB
+dNq5cGwCvapq/ONzLF8PFx7mLMPlgn36egAFvD4g2JdILr/cMbBEFIEW0ONVyPPC+c0D+tWjs2zN
+aLu4oijMf76YPZsamXhoQUiMSXfCtZexTqrZ0Kc8QbZSPJ05TMp2TFCm2z+/nB6XEbGVz+PjLBv5
+D0sZ7ICa4fdCW4DRdUngIKy+yXDDX3/KVw+oR1AO35CXkH30509hGlfh+ONWFe7CJyw17dlS6FSn
+zK6B4gD0+PXnffWQLJW8R0NpcTYtF/yHbzXPLTTSHmlOZMsqXXd2V4F0S1K9/c3T+GE/+fzWe3QZ
+ltMH//wslUsBaUQisYgSmKNhXDUId/pVKwOV7x0gDCUUCQ83/GA1Pk0fWRHFiFiX7FJEbr/5Xb64
+yIt0jHKIa8zO/ulWziahy6SYs5iiYw8ZIVbDtBUmWWNeXBTrX1/hzwIyNloeGipX3IRLN+CzgAyu
+CLFyJg1wYUQx8NmiiARTJIiB5DPhDYKuDQAKQn/lNOWpTl/rwcANjnxqMOHV0S1wylejmg21z5Xm
+JAhFWKxOPXNA4BJRWv3mHfvsOP34hW1c4ZzzdWR2n41EqgiS2NXJVgt4mYtNOnT62ahya4dMvNxH
+frxIsep2l4BjwWih1YQ1x5Nn3Fr8uv1vXoivfxssaJCKXLaMz8+NcLt80Bl+rqJ5RvmFGiX9cMrY
+TlhYQXfhFIl20MeBKRFRvWuSHeaVNkw+IkSh/5ks959X5off5dMJOkGmLdD/LnxZkJVYJ3OCVMzf
+FZNfPZ48LxhQ6VSx3iw8+B/eSTkBPvZsPiXu6iS0m6B9t5o6Oxta0AhDS+X36yf0izWAE5rLK8l+
+jFJ++fMfPs92Z11i1EHE6lj1ptFmRKxTMf7m2i0v1af3n09Z3K4UWdzKTy+dQl+Zq57qAwlJ/RQJ
+Uirr2oy/4W7+3QHjyy9EJbdE75Dyo3+6TYOAj8XgnG5H5WVrFJzdpoH095tjzJefAhqa1YyOyt/F
+t7EXVSbeNJRNcepvS6XsHiRQDCry1/fnqyvns7tyj/A40dL4+f40lAw+/k4+CGzzdiFTrT05eFcV
+XNmb/81HOTRol+M6TpSfP6poVYseh5tUqa668KMObUnmN8Oi3R7F3f/iwzBt0djj4E7K8M8fZhc4
+eNwliR7zW7Lt+w43EeqXNfiGYvvrj/rqXnHwY1vFsci54dPDt9Ab3RaBGHWIU1zBjPLP4RH9Ljfn
+qxcXWoC3NJ3YYD4fbMt8cBlX8tyVqGf1VT+PArlQOt4n9L228LWy9a+/1ldPBi1E7Ge2Hywenp+v
+oNVBdyYvljOJzJATz4V+1wi0DFQLyW9u1t+/Gz0YjALeYj8OeI9//qjRNoIcBHixIsqg2SVRfSX9
+5gTpnbvXm3T4zRf74tN8hPsYhQIOJ/g8Pn1ab2lYuptihabSPVnEoreomGAUG/18GdVJ9JtT7N+f
+D8LpjcBZDieU+eanz0txlNmGJpGTeHX8VBkz0hzLHK9/fbu+/BSsI7zGlHDu53VJ0wZXwZPCulrF
+2TfgJM05cJTsNzvmF9duOWA5y1PosXt/ulMMAea48hFylcM0XBpG5BEPWYr6xC5G98Gso/z7H38t
+HkGsKjhmP4ZnP98sy80blKgUGhjwKQEK8y0tvT80ArP1UmXYLEss6MQSfO6QmFofVeU8UDRKy8Jy
+GQEhLlHohA0+7m6lc89+cx3/frdY19HXB1SqnFs/b4s1kB9nGpj1TXndH71ZRCDDRmv849XdI0bd
+wx7usbpTdf989fxCMwY/IBwxsTqiNbPifa4IDoD086+Ajv9n+tDfvpCL1MrjdaLwNpfC++dPipH6
+ar1eVyujntKnQmrVJuuS33X9/37Q52OoeDlPBOihcGn8/DEeQIva90CPAO62ahQtvrBORyhj1tnQ
+V/mwAc4EgwoSYqV22IKC4YppKgfj0qh/O4n76jsvSwg1P6sJU7+ffxmyKu0U6GW1mpp8kECGreRo
+p07xp2cBthYcozyYLJAuLsqfP0afGGPaS6NQeqO/DqzxvbT0+J+12h8hhS6q9/Kma97fu7Nv1f9Z
+fvRVVtPH+/XBuPnvf7sY3puub97/wf+x/ce2L9++dQA0P//MT38FXJx//TZLsMlP/7IpOwSJV/17
+M12/t33e/RdSZ/l//k//8F/soFsS6v/zP769FSlpRRBj0tfux8QU2o/L1vkrrFAn/7FrZNvKf7zJ
+f9z0+Rc//i++kKP/BRKEuSg7O/sW7f1/84Uc/y9aFouugRYJjerlQ//NF/L4M24qLz+YD91bOEf/
+Tvi1/9Jd+vXMPnUWPe74n/CFOIF8bhHp2Lc+HFycV1kDvGVF/+EAHlko+SPLGIiFxhK0Appt3bWA
+WvqtgTyVoLi86d+HsZ4eRY8TQvdLoORBXxuHyhxVKD2SOhmjqbUZN9O+HAUR23b1YGCveI0bP7vM
+CKo473oTCIuKhwOKYsJSa5kMV4lt5SYMS07/c5DivyGsEcVpNBjPk+0O10FFY06JonxQQZls4d9i
+2csytkcK2FWZsMNg/rb1ncVrdmebWTuu8Pq027FvG3ere3FmhEHfeg9m2TUiLD3SFPo+zZ6YGAbG
+aijEvE+TWr75ls7vXVfeU6p13prN7VoGAcMmeyYRYTkt3LUgX8/tmSAa6WJdoZWJSGscDe3Urj0W
+6hTdtWQuRXTNiE/iJYt7f0eFpZ26BJxc1ORRnElM+k+6aYn+EM8GVbnd1Zr7+MG8Jn7GCnX0VeFY
+Kj9dI3qxnmwm9oQLZ+q2aAfzrtdcpHGkTGJhihRitFGMXDF/hMaGjDS2Vqmt5BFBtjVv9LxHAycQ
+xK+ywFrkffSLN7Es1K2ujfGbzJYvSBXVF6DWzPpm7Hy07rYC05ZOPSC3Jq0RSAf2fDqOPjK7uHPI
+beDbMXOnfEevllFTrSFPwu7W+V+pYWY3hUVc7cZPjfgtsrBihRMko2nTVnEH23yK8KXpmj2ejBWB
+rITPWk8gKKMLf4wnGS4txUv2V9YxuIZI9r28BeLQY9jgRsZMD3IyDGlUPUwOBgCBOAfhNvipyy5A
+c7vJYTCcTLZDTA0it3adlYa8ivrYfR0xbqDHssmJ14h56doCGnV+QTN7mta+L409Fa8gMtfWi4Nh
+2MGFn1vJfW963U4qP76D4gv5qoszgOtzY3ihQ2BIT53cRwfUhdZ5Yzjy6KaVd5WIJjmUpnqHHyqY
+eI3iQfm92DCQqELdKoKnCtTtXTQa2EBIvK/vWnSkS2Jq/pASbpwcfGviDkX16G6UbZRHF+7+c6Cm
+QNvrucuEpu3Kcj3q5VwQp2H7Zx/RHWDpJwMDgC2+jQh9/QvpjNzNYR7yNZHJ/aOFsv4iSXN4YYCX
+BfEfHEOSTWYgdEQ+46LYre3ogoEGSsocrWe+QdLoxye6A3pn1bW2ECBFfficrT34O99dDGB6D/n0
+VK8KHdGevkDtRteZNxyZmq3ra4QqqEDtyB+CgRd98PBG0QHA55FIwJUm4yUiC7B5tnAwnami7E8A
+b5sbUZK/uIKsH2/m3BS8yhXgvWZWOdJJ8UHkqw1bXVWFRXCwRBVYftD7KDGNO6pvf0fGUb6bZwc3
+XOaHmtsR3tw5qbMRCxjQ+2AEjh+8wOaDHahjPLiiQ15tHDf67nyABuUHdLBKBs0DpptG8SWjR8CE
+9WBbzxIUKi/DB7+QUtXfsW3wXiJ5d+LrsVxMcr6XtiOaV2k9ydFnpcg+AImxyWu6RQpL4EGkfBx7
+mH/gKepDFr/5H5RF54O4OH/QF//J1E/5IXlYXAM5iVWNeyh8vTh2UPRpPz2RYQUWfGqj18GLW8JT
+9fbgpvJK72afcIPkMc0TEkBUshGGQ6alsF9lxxIfgcJ9S1AnrXorSs+cRIrzcSj2rlbnm6Gb7rvE
+v5s0mKy9dz6l7UlfGHiy8mOR+G9+XN9ohjhKq7kKoKSuvESqlaUozZQmr3IIdiv4D1e1Etummh+i
+2HrNesBV6JQ2KlZXXGlva8aTCFPDLW7bwXYeao1sEO7TgKy+kqg752mN767HMdTfkEYCyDhwwqbK
+Xj1Cg3ylu8TpFBvNs5/cKbjuADuztVy7rXHnNUTi6Ga7l7p+gYj5NDJ0soTyXVOVj9iiz9JkOINs
+8hLr5tEN+q3y+Y2p8oyNp/RtF03XOtBJz+kFf9RdMEdfD3V3zKVKLhsz2Eaz/6002ZBqlOwrM7Ne
+BqyoFdjtkxT8KJsJ/ewZ+BRvwNCsqzI/amS1TJr9mjnisaxhU8b+jdHRlw7M2xHfQ8gRIFu1VgqJ
+tO0OkTk++RLnCGbVRRuIyBxzLtH0aQFZnH0HiXUXQOxITRhr0mhevdYzDrrmVmFLeM/KN/30tA0C
+pNtZ8CZxTO9lrd0zY2NDIERohZSQHC8pWv9D2XxMgvm+c/L5OrOHcRvry4Zns3vQC+IpLtkEfWyz
+SKfrxsfXR2KREDWeIXv2riPiFB6sUeh7fe78XdG1WURacZnKfatsMPN+cpnwDm8h6gePSWk3pEJD
+jCYK+juJL9WaemV+iDs/3g5e+ubOdgWQtzD3VecvUfYIuQGbI+WpnD56xzFAKz31BugBg3eeV4O2
+0Vnvy/WQIM1NLU4rqKiGLdi+Y+47pAllcbVSevai4N5qvrrX0ibdekGcUBWnzRXuqquS9Xhv1+K7
+1mvDmt/AQmvavvgyLUMchfm2yFpnM8SZotIgR30lRpO42yl4VrLH7lwNCuWyLA/jZPRAQTvjJRa9
+F+azfbSG4lRrDHNdGc5NhMjjUOjdM3r/HF8DChu289y47JTb0f12AA1213FSb02SOMIhsdvzLiIV
+LkfHt5ZTc0grmFSiMa9zJ9sLkyU8A9QDoCrV17kdZ3vJKQ7dgNpXViS2vOGkrCG6PWnd6kgWwbmW
+dvdZnr7pFqarGEcfsQDxjZ5Vt2YybYoBLL5ZA7cP3QV6j32uvdey1jxh6XB3JqG/K7IWSNuxX6qh
+wbEdVI9er+18vh4pA9igOCuy7NvqGhB4dKmMsdstcW4rS0QydDvolu1YvhXCPODf4Yd6w+6PcpyH
+jcy777GR74o+6290PBL4bhAc23P/7LqxfXBzOb9PheGsG79PNkWLDKl3HOLHkrkvw3QsD2xTL4MS
+LxyJ8mmTzd2Z5WfFxvDTYI+FsL6Ik8Q4b/1E7UmdIIKzLxRLNGPLcOYe7GC43asajxc6mf4ZhYR3
+o+lvXeAVG0vzpwMWoCNxRM9Qp0hmbecgFKNWnA2clcJSpkQK+D0S6ZHVRA/iFaKVJ0vL4LDF81Um
+iZprg/SkHlMCVtVkb2rHwdbqODht8vacuKw9SwzBU4F9Y0bqAjdiRae8vpZdbB1szZMbKCWb2E1E
+OBGrB4izvZFRcqBycO7g2G11q98nA0klnKlCjmz454uTcnK+DaPx7kIcZ4EmihpCDL1xVkqxkIJX
+MNaSLeE2oUZYGn1LQCMkcRCs60FX8SP1qKmW4dWAAt4SRJ6R8RStZNCdFtNsrLw58g6Zai+sVssR
+gdrr2FrK/WE3+XKnGfNT67XWKsDu8t7VjrFxF/PVnHdPPvErV14n3rlW5wEPqDDtY5VClgYYWS+Y
+UWBaDsfywAL/ncvqPTC7c0IRtkU6neLqu69KAvtgxA2AuErSoXFh6X7ySNTOW2GO2TZQZhy2WJNU
+a/H7WE60LXMvPanM4DluHLXrsug4afDSG2N498F+rskxJBGvsE04cLR/Cie7TfMWm6qFX9OZOeEZ
+IkLJO9fs++J7pNlvUTE/0m3b4Lac70w33yRevUkajzFH4ZnbuVD5TsszHn8DpnLs9DtRJgdrxgiN
+IT06VbOF0y2LIfzruLaHenG9VJazqc3+jENQfOrGyMFlr7DMa9FM4mK7z9yJFBMnvgcliI5HQvzo
+CdFYubb2kMvaIVIj0VegOrOQS2/unFoPwnzkDGvqc3COqbShRFtWdRigG7v0unVE4zpspr7ZpMpz
+jwXl0L7XNHmc2hlUc11hy8ActjcrLQqNzoGASRjUbsZGys/WxomesL0pipdDYToDI8PxYHitcSry
+5XHMpvhx6ka5TXNY1U5mb+weStBE1mY8mmZogLTFuR+dF6mH60t5+IR96a1n1+yvMGHwr0uKjh3L
+xbZkZVuN89Dem+U9z26xnWYNRkPZst8MhjhlwYP5bIvHOUeu04+Q2YqOAxweQ489Hvcvh2oV6vok
+N4NIqss0bdx1raVrPbf1bypFZghEMVrXRr+LTVZq6tt+N3UTiR3E2lV19l7m87kdtM0WyMYDS7Cx
+9Uxb2wqncrYoyaKTIpP5dm64n35nVBuZJc2qNTCsou/n7BSpK4KQj7O0gO62M/a4CoQLayqA79Jt
+6KVGHfP4NLnKhy47guwLONlrUKRiQvqcOTuJF9QTsBlWYuQRrz3dsNWEQZMMCjy1yi5Cj5x2UPTz
+XUwCHoPLgUPxQC5ADalqb5vVxaBNDeLKUvfWruLFbjA3rycd875osFFz8ojO54qv4Bb6Rjf19k5v
+ErD+Ph866NqrxeZz0teY9RW5mmGgl+amyqZqJSNN7EaMK6eqR/0CX+UasybH9CgytoOdG+eDM5wi
+dEjhizTPVsqJhRxYVCRR9VhJKXb9EJt3iZea6B+KBP53rGNei8dTK5ieiNna2kzRwyZJpmtOOPO7
+YAIfGumQbxUmzDNepHMrbjO4GLq3TcWsmN4qgN1TS+Zqgv7RaNvXURn5CcOF+3KyiYYWkApGCBH3
+TircMK9TSWqgs4Zpljx1WUzRmWF1nTtc/zivvwGdeq7KRoZJHYTkZ4W0Ucb3pAKM4IoGG5dlPs3G
+VLHxzv5q9CZ7bZo9xmpz6i87Z252cz5Xew+30cYu/IGDMso1Gbj4EkSLMcxbXH7B8o6U85WTq2cS
+ToDnq7pfQwzuV17Dfg9PaQPrM9qXym4uvAYrvWZItn7dwHGmmxvldcT7gH/Z9LyKqfAs2O6lt+kS
+LF9RnRZXg3DqncxI9BMkNnzHm2KETTQEW0I6idfK4zfIlAk9AOcpGk37GeXwS+16b01julurTOxX
+0x60h6xo8pEYO1K+AnqfY5oRtQC7YFVHcEvSzjXIxkirDXfbxFEb8d8MCkmpk/lZJjVN9qjVOMJn
+BWl+QXD07Kn/RsWKr9JfwirqMdl15D5isdYUhyfZrqum5lRF941mUpAcvbg3rjxd+5YGHglPmXPt
++e1B8XW3g+UXOzcXTyDuFk99NBHIy67tNmSCoIRkkxMEkjnKfok68pBSfNybQIDVqbURg3imMOkm
+e0mZRVeqNcEsdJzTJVT/ySMNZCrlUfMEhzrWEyPOyZgJ9Fs6e8eyaoLHIq4vyBTFlpFRMZKeWxm3
+UV3Nm8KGxIE5etY51hN2QFcoT/TtnFXxdUsG2nw1QobogNMM5MSQ0xDt40IEL02pImrOpmqEvm6q
+Om72rFh1e6zwc64sTZs2th5ZoRdwO+axpofj58BF91lZua22YdpltXB4wAWd+qKj5q9KL7ahI2gD
+SeWVHnJR4pZlfhratVSeHbX39EQ87HfSNdS5QaYXAFgmQ9U61go6itXoKRNUCDQWXsw26u56K2hN
+Qj6GHWwXkl6txiHHDclEl6xHq0nHy7hoUjKX2MdPh6YbCrpBE1ADBCtLhAM5AwMw0SLYSgmccj3F
+PdAYzuIuK23aNcGxmkvQbz1hf80av7oijhPnfA88g6S3Tmb0UyKHCMps6KqjFG5K6coX26jWSWc6
+bBZwIr3O4qd6EDW42cEic0bxtzZgkoIJ4Fsd51hdu7o+j3oz63bB1OryqLD8izsrqrX6JOjGdA8/
+3T/D7m6QIIPBPV937JfiEOQR3T5O5uJWdwfnte4M1YeZTSdsUwJiAnZUp4G9YYWsNm5pGEBhBxJ+
+jZhQZoNpABv1RDsNZ9UA2A9PgbcbrcLHdkgPYMlKEyztXt/ZHq9UWV3o5ZTfDq4Zi53DuFbu0WIg
+fYx90C4HGmLpWohxDdrB2GF/jtyTbEB5w6jLydzNQG5pQ0wJKA2erLzSNxbxMiku+mkj6wE8DwaW
+U9KeQxeNmN77J57s9X2jBrRDrpzio1FV07OIaePumkSfTtoURsSaJ7rf4cp+9R1xqKA9KUEvRLoT
+D76zjSx3p3fFjamVJ9rAjF4QS9SZ90mSvjVjsm90bc1h6qhP/olIq3TVtGx1RpnvPDE8E719qItx
+TULMN1e2D37pPrCa31gOG5o2SyO0HDKFcj1ftaKYQnTloRYhTx6wAg/ymXbhNdGaR0wAW79/ZY7w
+nEzea2tMJw0ci4PT+IO+15Qlj3llNPVhklW9Ggboyn5VE1gxNoF+OtYt7nIH6YxEbB/qsr1Gssgp
+vBvyx6xIeSrgeePZ4OnMcMavZi8Y3DXbQ+qAHegSx71KZnRW4dwTAYdTDst4JeGj3BLd4l7WGg/Y
+uuQaJwfYYPxMMXajFWoc1MQdRqKXQsTTjfCS7vvQQ0g8ISGMA/DYamjvm6R+oF0yvlZ269RhomZB
+fVfx7q1GvneyH4csh/JjyUzfBwZ8pXCcG+YqXWepBzuYyWtJBjIS17mh5mPHd05JI8yUeTIFkyb2
+NU6JEY4TIhi8olA3d55WbjjznrQz6/CK8yQjMcaOfQe2gNbvdqIf3hF4mcbfTJlEPnfJYjxQ13ER
+n2mJoWNtdyfq0mYIeg96p66/icxCxdpEBrFjncizQ8/aqh0NUuZSAE84VXYfA58/moWdpa/MgOT3
+7vNM66ep2P/PczA07f/DOdjPA7CPn/vvAZiJ0HGRjpvWYqFDDTW+t91//ofmGn9hb2DohKZIZwbt
+ozT7rwGY99diC2WEuwRfIB/+Yf5l+H/pKKgDCliSg+HkGn8y/0I9wnjrR2UYUkODT2B0iiIb18gy
+Hvth/GWpmNdZSJ9gXoYvOwLj6Y9IUsmuMNc77t4kvtxeTWqOn3qGO/qKZnM5Lnng+rSe4Yow151K
+UtP8Umr+emj05FhiySW11Rtw0USRlX4bK7Nw1/im52xHDGdO5p1pK+dkMOs8Qdk4dwf6aVaxAevc
+vtYWgEFSI+kGHlyW9lvWdYJRqew2bQuccxXIInqh7ZfsgbEYzwTRBHfI3thjfKB7NfyBHOyIQ6V8
+AAXpkfs+TNZWkYRHfQ940wyrkpy+Nh+CfcDGFYT2uEjAkbQ1T5FRkQE+9vK76Wvt5VRlI5qeagJw
+04ESvyomFmCqyCA7q+YYDkTgMgleN1FTUx8YAUHqwCg0j5OtVR3w4evfo1Qxfhotvbz2ogAe3VRP
+ZJVkkc2aqGIOCZAUTPcKiGFHhhm5W2rtiCmn5WQNIl4nqUggw7jlBN2iIrA2w2B/K8wmKXYdEvaB
+zE+W+Tjt7YdgRK65UQ3RZicOeWxEby8ZiemoTeRp1d50MSLoabZeNUz3zRRkj9DrBoY0Uxzf1J6h
+HkTXI5hn7R9egoAKe9ViuLhwggImciwdKFdEragGcJbLH1IVNcQzR50LDHLW4/vcHupk3daZTZCA
+2QY3zKI8nYOalXtbNg2T6OrCnevQaunThUnWkgnqeCq5rSBVfa/JbFShYMo0rHIiz/lbtaD9nqQF
+nb3WqobzGtpcDfogZZ8MPBG9kDEJnE5YRlVsu7rqLngIgnqb9jFSDrAb/bzx4QJBpFA1CJXKXyTe
+QyeFwRSROGSaoZz0Vnkv5mqr9DS+CBxZ2dsmFXgzGzeZIAqUZsEUNiq8kGFxNW0mAMA3pZGYDwGC
+iuc8MEnI9eBuAZPhHhGW0qTW8hL0MWg7YvQeIr+GZjJwWgrO2lHIOZScd98GVfTOOuoaQ2wcp25c
+ivKxhu3AuWrvFqpTp+IjnTY2k4FY+8prmJMWJUCMllQ3ZpBF6ia7SCrz3S1q4W46U9qvYGL8mwzZ
+9y1IoOHJUJn0wiZujDN0u7T27OTdNio2Yru/EH5KhnbiU1DmlVybTeUnm9HO6oe2KGh4KU+zfTDg
+6UR+6TQ1t/aUJhm24yJPwzqS0RNMuvShbtvxqGLjTnC6PPEmv3yEyxlcJamqmXy203jN4an5FgNl
+YWGALMRLYujiSrMaOUJ76Xsfbp8tc86sE1IZ7n/MIZUl8qXNSt46CzUL7Obez8YQzeaY0zlLqrdc
+F4FYxZpB0rGIoEZWzahzeOPIkO9yL4r8VSQc7wKoT8qMjGhTEeppFImd8hKGpracScUDXASjX499
+/i5S0tCWtpDX+XtpeMFh+gBT5ZmjH2QTTPfSGyKx183G3yUMWa/t3q9xXWD0XdWT3tD69Q0C8KYJ
+D3rDfzFI963qdDvUWnCrJwwK1lSa1fusExaBjkoaQehF5FaTIKlOg3QcSUV1VfkAxj+P1hL1aX6p
+jbPHs2InzgvWXiPZ+TVzD5pi0La2bZzoNqBtv9P3uJhFeUj9mdTdlUnHPvpuW+lIrJ2ke9bBQ9U7
+jyPxeTYzYO5PIXPGTrFOylzQHFlVOmpnYozrHNYYSoyIL4Lv7pGqOp/CKImieG2OFK0UpI5oTnWi
+zqfVrEfBAWKNR+d3WclCl0DkN3OkzAobf8rNbQYnDLfD3BPdaeaJsk9dEEh9OOmsduuhKn3gXbbu
+hHhcaaXbkbbwId0M7z5zPhBe9ayPO7QRKl9RXXpU5nZS3s8Bmj5Wdr/PNziNl0ZlnmW3FBPtk0+z
+xlsNNPk9aoO2eTC0diZ1ktbHe4+tJgutyivMcCSYtT+Wvi2XOZDKMjyaLmIE8KGyBkWWOfGRNNhY
+rHUZwzPB1uwuqbm0F9BEWp5YFxEaWBrGwqJolqOZbhwIwLdKo6BYm52hD4eptToeKKMsH2cL+sMJ
+ziM4qAnkJDQHXtOtPEJYurUNprXdeUW9ZAWnWdWtCypKA6qQJPVQp/uah5J5Huw002X+Krg8dah5
+uQVrkMqP+tRT/XWRd8u3hmcKiks1tbv1PL4CudAlUoJ4ssCOAvWpGyRGRWGsMVJInSuhrEc0hC24
+kTqazsemiIw1EAAtWc0tsueVRZTESEB0N6O0wj9y6Cu/s8F1coE2JM1GBu6SGP4L4cJSpVPRE5Aa
++FpC4jNR3/Qoyu4gZAajppldmvRRZi6qloC+0yYeAHJBMvNks/bcPn4T2pC1VLoWtK+271mSsUfw
+T+a4+TXPiXppTIOBv2yTB3g4xU0xxo4k7VePr50poB1iEODwTlPF81eNGTGrsAz2bbiotNQ1llhE
+D30bJaCw7IyuUh2Jh0hTxB8vCwgLkK1MWpwl7ms6591wM9rmHOx45s0rfxj6gNhFkZfbUY7Enaez
+6ZwYiRjbnRhRdIe50xhXwoE7ZkrQnStngvC09quy2oBAhPikCQNiU+VBTuI3Ry8PA5BppD44gPia
+XtCRbt2heWSn5V7b7IfNao4i/hASrX8mGh+mVDYr8U0XVl3vhKIRCDKugGaGMss/r5WgkwcEoDgr
+JPLoftsxQ8Peow/tXaKZ2b072dapV49zuu9JA/5WwkEoaQcb5rmcbPNCV7rT7PwGd3E4lVN3Po+d
+nMJOOjpUZsKuKYyjKjZXFsxabo0sisfSN+p3KG7Wu83HBatI+qikomjsL8jCzB6tcQgeZtVONuOd
+uHuAOeJ/r/2g+u5pqXFUpuNr23xm2sjKEOvnadn7p8RsVLe1loBfI5Eib3HSCkadc0zp33LMpVuW
+WfLdr2XzfaBOQtClWgN0c5LnL6nMeB/0OQW6a5Q8Ffh8IwBfTeFyBTu91uS30e28k8KAPrXpNGSS
+vJGl9xi3NZnmWde0L+4ItngfE2T75DNcPh9lI5li2TZdycJo7Fcj0BgZtnlAm4kGPBG9/mBZtxA8
+GVs6FQMztm/Du1MJqPSV43YOqbKKYjlG2+6tFFOoc7vyhip0zYVnS8Rb+T1mZWKM1FUqONd6YSTf
+KP2nkxrv9bz25kkAcsPIrK1byUFrPY7LLL4yWpPM3WEEJlPShn/LlMVhLWHCflI5uQF0MqqDy9as
+rMsqIY5pjdHIfp9t2g4ryA7ji1nW2A9EJtzToXV6VL+k3N6PU8USQ+HsnOGeGudQYQjceFhzk02v
+L1C5fKhswK9ZSYVP5HN0qtFB6emaKe3Wbpv6xkYOJkL05UW1w9uXHrMhKp8ap58fWYnleamnytoL
+ei1buprdwt7OgS+mAqKswBVhx8wH5t7JBSC4aJb5cEK3D1vVWkb0m7P1kklBDjWE+KDyHxhD+WWI
+8VN9Z+qTPSk6sTCdOTm1YaOZFUIgrelov7IzqdVgZYsATSW8bnrW/V/2ziQ7bmTLtnP5fcQCYCgb
+v+PwgnRSFCux6mCpoGCoYaiB2eQAchRvYn/DFfFTdDLJVLZf5xUrlgJyFGbX7j1nH9uh09x7n+hy
+65CraSIOn1CAA6MuxkUnlEYLva3vOtYt4ZYQCFlYJS8t6/HWI0zU2SadqB9KQs+fh2J549zUSpn4
+Lxw3VORadu6WYXyWeAmrozuktB0T/m0IFxo6AVC1INIVbq+duZXOyufibfhqSQskmzC5dJ028BCJ
+oUfxVNMyBy6SS8h8/M3SCIWBFBAknckYTupaMLJEVTXeU5nlX3O8VNW2EZ52reVVSJushlJpEe59
+L3OLrcLsIjKMAaISCItcrIGFijBTownBuCYw+jJzA+DW+Y2C2mgFfpybnKMi0TYbWGXicYTujEBN
+zVBXPa9ppp2gJfJpwJ7BmLJhCIX5satJuQ1V+jhVOoHZFThrsuKjZfQi5z59bFCLgpFUAy5hYaf8
+MDqb9B+HioZeMNimcRn6g+Vt2zn0vbWS0n6C/VIPO8EQJv1Ux41zJUKfYjJJELYVdu5csM/qnydm
+hrezR+S0ogxfMcVBnRf6CSAdvey49XkachhiXAuNatk7f+QOmcRsdXp967eRfCb4SL8trAxaZBED
+JGPZtvofbM0efTQ1u1dNRVM7GGVnfc9AcMqg5Av5PlTU8chIY6ta9S5BuJ8id4ivgdR2VMJdTPcu
+52S40wAmS3IvYQSf0p8i+Ldy6RjHsDaNTVHpAxG4jt0xlonm2TsbJ4yXW49pm2TN1lxommWsfwY3
+idGyWCQFTu/P1tqO4pFiwxr4plQNRHAVo6q8b1uO0isDKK9YK3C8DMgN8dR0VqECq9Q1bDV9Hz3G
++G9cnp6uGmDiaqz3TMk7FDyly2IEUfHJt0Jbg0GJB3RlTR5+8gZqSX02xgnnaOjSvqSkUcxLSfiC
+6DiMYqJI8Px54JbD5ewJJMcGGVg602NOoM2CFaQNR/i7mstpB8cB8mAjLDaWWfJx0Z0txNlI91/b
++zNbOGnKM93f2BkB3htuz+PFzJicWUUuO5b/2TyHJhsau8y0xZnWufAsSpHoXzMPuQpD76ZHIxUT
+v32actP+Noj/u4f2t8z89Mf//T+mDVTjvR7a5df6X//xonv260/83T2zHLTeAtSObhsmgjZBi+zv
+7hny8cUuScSQ0B1nMcz+/+6Z+RcHQppwOPMguFneglr5Rz3u/+XRozGwRtj892I+/kdJf/mrKfZe
+OO2RvYGcE4pWcwmENB0QOe6R16eHVRktY3PkZYikphbNBUyldvPbHfn7qr9n0B45in5dRdBFtDCI
+gh08atCVYVPBW86bFRRKfxN2mr2qizF7itBXrMmp0T6Amb3+VRixuHuejikQzxk39veGYGZwxPRH
+r151tQ+01htGKBG9sXr/V711FQJ1cb5jV+ExHf0qo/PipNbZXznAmfeAIfJTapt5/f5VXt87W8ct
+Ry6jB7cAdsDL31KDFZKtS7k8ppZ0A+mjToOZZttkofoTjHOD4ent+9dcnvpvDVWeF/Laxf+lE5QE
+TZa37/f75xdCEYI91WgDC3Ova4o8CGQx2Jc854Of98alsLtgkuDTWEA5R2Yfhtd6iTSMS1FvrVij
+5m0FXZiRbZ594LF54046+DGIeuU28tiO3gq7cgpPK3I0tXGTnBJ74Zw4dtKeg6HzPw916f6y2/xP
+7VLLXXxxvaO7OLWINJ2e69WFgRggN8JK2yS9E39wnbduIfUBdE2TnwdD4+XTQhQ2T3FpKwgaSvYB
+YbzJtG7jbn6CH64+uNhbN/HA8tTxU4AAOrqYT3OPo9rElj2Z6brra/NCOkAQbMubUJr8eTgvN5G1
+kHwpvjOi/JaP8Lfefm91aFFjRG1G1iHE8xNzE7ccMSJ8sn/+PTsgLElhYp4ApezVpWKNGF6DS0li
+ca06tLeYj6IPXvjlBh19Wy+usjzN33/Q7FZ1g2iRM0X5WUo32nnppO7w9lnnS7/yDj3Swx9/zi8u
+uTzT3y5paLadaiNF80RLfd2amXPRJDPBNNCsb9+/1HKPXv06Uq89nHJLvNrR58ykVNazhh6qwutx
+mZYV8kOPUMD/xVV42fmY0VzjEXz5g0I7tJT06XyUDcE/YiydbdyXzu79q7z1qiN6ZGNedluCSF9e
+hXQxRMXKob9Sw3sLPCIk95mThz/zqpG3PutV+8HH9daXzK1jOSRMzXmVWZloZMLFDp5HZv7OjnT0
+R0ba38iIcjfv/7S3HhOkMB1gg4MR6tgwhjuW3DY69URs4YgY8sZbo9xqP/igjtEbrIDohRZUHENA
+NpJjGI3UvLjL7IJ2sqgFMBoxBDZt6Q3zn4hSvhQrkot2ITFfAHda0m84qTM/162PEuRe/14s02Sg
+m5RzzrIwv3yUHOn0vu/ZZQzcJQ7ScGKCTqXo8o9wOMayqL/8ABaOM7UOWFPbxlT28kpjE3nSIOJ4
+xWgv3es4t7ZKVeK27OtPkaON+xpg2gagi4Ekl1QhqDac/t2gNVr/tCMF+YNS6PVyszgQ+SKXlFkd
+ItDLv88wUR9p/YgGSOcYj4TLzwHOt0OE8UyPzApHa+9cN12bf0QFefPK2BKpXjHQUlC8vPLUV/4c
+KVadQeJM7KKMBjXuKBBPEX2XxzIZPkrMfP2U+a2/XfHog51MwQHYYG9C0eEFdZmkAWfRIvjTb4er
+8IC5cY4L6OLoKh7NNEFFiWp6ovumMUUOegsz1vtXeb34cBUH36mHG9oBmvny7hUlecCNCx8zjXzn
+mraj2oiF1ql3GUL4uJ6371/vrafFK7ucOWy+k1eAzrSc4dSzLTnJYBG6ojztzAx1RG9e3nwy+8lv
+11g/m49Iqx9d13v5O2mOj0qVllrRrK3PkqEsT0nWmD8RWVSfdbC2URgnxgfL31s3d6k2yYmngCcC
+9OVFx8rLFS4cbm5s2A/kUYzdxvR7dK2FT/iJhGV7//7tfb2y+wsxDo8+MADi1Y92rI7omcJuItRF
+YVOsHaXqNRTbfqUVeDXev9QbX4ENLJeXx4b0Cjbx5Y9jZj2ng0NPZhqYJenpjB0KH9AHxfRbV1m4
+vBxBPbQf1vG6EplOMzqsH0xyQoRYsZs6kOvrefrzZ2X/fqGjpbuYGJRYJsJjza1ohqXMvdPEvULZ
+txhoPiLkLjfn5fK9nKthxfJ2YOw1jp4T3zH+Ojkzt8V4t5eelu+YcOv7Mre9TeU6zMIG9FqrfEJt
+8cEn/8anAIPFMklQcjiQH+eBu+mItqRl95+11r/JlG1+Jv8Q65FpKwa2zpwA5w4/IuK98WYuobvs
+EJQBvDfmy9eFM4nTCoMenG3gzauET8qKkSDL1tFPvv9mvvUDD2dlRDdA+I5ZCl7VTI0VVRRUsuzP
+nE51pxiN7X1s+eZJG7okN2Wq+ePwczRIixDJpBAhFeMY3YNAzpzblquKjlYrBrvYWyIVm71diu5i
+XLI9Cg9rlMK7+cETffWRLJsudRwZwgeF0tGnSAhHUSnFihIhKFyZeiG29GL6P46rxfMDLAOCD5Sn
+V2tLHTIRGWbe2TluDRwHaEAYdeIuZSpcfADheusXsbpQfnoLfPMYm0vsNfCLqsUeR2gG8u9Om596
+4os+Iv2/eiu5cwvBjEdGZ4AT4Mu3Mp6TyhuYZPBWptO6qSbrDC88ctCxaz7Y+d66lMv7jyD6sNEe
+XapdxEbM+riUQhRN20NbV/NELKU+nbz//r9186iF+AQMm7rheI9VuYeMxEQ1X1s6fk+NWlcOUm3+
++CrLNsPnxc3TF7jEi9NeE7nSJ7ubJcxm+qI7zUJqwB7w/lXeuGsU1Es/j2vAOzpaNiYDtX7SILYl
+z4bikoVqg8M+uQpVND/+Ly61LBe+zSJFX+rlD3LNXEktSpfQ0C7ctikxhCmasoCWyAcE7zceEMSO
+/7rSUV1QlJMKmUNWK9/p7zDdiA2m4OqD9235l7zYYpgs0J7kMogmSZM4unMGJo+8hBWF/q7Uz1Uy
+KnALQ3nq4/iaV+Uwjrv375+x/BtfXRH1JlRQZJfweV/ewFllSQZ5EFRF5HMDkaetx6JIGRL1mE6k
+HUocJn20QbDs78jIMX9qk7Zv7KLaSjGk1+//dd66yTzIJZ2F/ixolZd/m6jI8s4LeXOQSaPerjTS
+0bzi+c8vgmbVXLh6dE+PbzKBg+g6K7tcjXFtMu8fEiTJDTFhf8hbpSlLreBbtI0gIi00mJe/JrRS
+aOsTL2eR4DuDT+qsiFzfQrI/KVpt+uCre+vegUTn5YFTDfLpaK3qxgYQcF/iH23t8CztJ3VasYqu
+//zmeTQ8EN6wbznHjW03Q543RayISZPX52Un881oi/hPK0igpsw3gP9y7KCZc3TnMDBoKcSYpU51
+5UWGPRaTFzO/P/4tXIVeJbsWhymx1CS/9b68uddabXn301ggHZlGPNth4X2w5r7udCw/higTGwky
+nLFDW+C3yyAGRUaSuzBauzA+1yZPbA2V7cvBJp5a7y+8wb6uAMFslHTDM/rde8evqg/2l1f1FX8J
+yMKCMcGSBXB8yJgVjJU2wl08O71pbNpRNsUlGmW9P7e7AUvBOPhZfIrsHgHr+7f5jUWNIt1j1AIj
+izLraNMhBs4mRtUnUT1PRBpInSDLoYrPhRVZAcIk/vP9C77xJbD5sHosiD9u+vGXYLpjjliPNW2R
+Mg+NQA6czx99Ca93OYNHSoeMN2hRwB8dB+g5R2Pt8lgdGUf4Vt3ydCpm95SR7UfU3Nd3kEt5ANZw
+dSM/sI52OdZKHNQ2d7BMbbRVU4lbEZ2PNL74yMZ/SGK6wg++8+Vv/3JfWFJVOP7CNmNEeQz4lqmy
+x0gJ+P1Frq0tX9l3qhvmb6pzs7VhFOY32iDjWSVFeZLXZvP0/iN8/bpCk6MwgI0HQosJ5MtPMy8U
+Ge6I1Fc6/Pt1huuQrKonu6BBpUgSXnXWR1Xl65dmuSKHVqZpdFmPz/3NECexaWAGKxD/IazouhM+
+lY/wu2+8NETfUk9ShB3IXC9/FxExLngYTAUaghAIGenUBn5oyFvAlyL54DvwDueX358izTWP0TJj
+YgoeSIBHt9HoyRRpBEmRVm5l2knHcv2My0ZbtEJJczOiaDVWo29O/mYavak6JzMeFgblPWQoJmWl
+Ws/I8dB88/3khOkm5jmzP61HceCibiCWr+xPoU9l6W4ImXfuBw+L3dYTzVSeLGnuZEomaSj2vNRT
+tA+HoclOCUMyyrXbGpE8wdon7ZNlmNTtGuV3xaW0sgZjQRqmLsHEgHyIoZW1tx5VaDxWbD5pUGfE
+IQTNUHoxGsElPTV1yPW+xvqGFdX1GuwdDSK0bO2VUWTgtgNjFJ55Q0haqZen47S44BLSB/GD/MiL
+kGQ9c3CpdXT8jfPeQvu/JE32yGcVTxPjG0tbv3abtIWP1SzqqcQkdDXyRpSMThORYQv7kuPBRF87
+Bj9R1jXGvj6pT7LGSMcdKusogk6IVDGoTfSVq6HrqAHgKer43xzIIfwVYCXtiFgenbU/iCQPShLR
+nwm1R2g05yQsdRWV3NqSuaGvSM5r8d2G85DvGI+ZPEKUI6BPhjJ20Pz7Vh9okkbGtqcxCBCq9+No
+37mja1PDDkTW6sMcQn/pCD+F6zRrJSqbOvK2xH2S1Z0Os+NsFgFzjspEgDk0+fbLTdeXsbcy87zG
+Qb4iXRex+3wIyp0PobnWIUAXUhVQgEgDqr+krROym8EecFfhotWBTFoXCYbeBqGvh6SvP1FLVi/+
+QSha4hDha5TGQJyvjNp+zQE6Pu2GUZvOiTDl7jRg7NCOFhMKX98r4vtYkRScD1aL/zrJ5mkbH8KE
+sfOGX1s/dxE9l3GXr5ND9LAkCGWfIKX/6aqp/jItGcVyRo6OqXeJLkbl6eLkTX2IYtBN1KZFGfkd
+5yo+Stqy2ZNjT5zcy8L0L+bUKC/SzJNiN9VizsGut3kWIPVDe5Sx7XOQs71iPx/iliFnyMfuEMLc
+d+QxT16SPQwYDpFmk9acH4Kb5SHEGaH7yBFgiXZWaNsuLTqs5dozQsKfsQ8kd2npu9M6s0mHBnjQ
+E2UKLwh885IfLVyB5bBcUqWJe5ywYR7CpttD8HTlE8u1KeceM4Z9CKfuc3LfySoms3oE2vXTnnsd
+9gVQl/PwEG9dyzHBX5G48F4GMeTp1jZIw8ajjHk+bZeQbOTSxQ4rTSFvemOJ0XaTxoxxBy7x2sxq
+xc/Yz2lZIdRH2quVqoPz4S5INjwazXV2iOvm8GNeOXak7mOBTHHVwftHeW8YebVREUaANU5faAp6
+ohEFzpeSAdRAVXculqzwovWIDY91DVm/lmjGp1EU+nM6I8heqbmu6wcHYuP4lUrczs9kmLTRdszN
+eNhrea6qc81OfWTMaZypcyMp7fBSWWQLnEd6Wz3MljHJu6jwFfytFmzyjamKvN/yhDz3SiFXNU+s
+sEqhdevF4OzbWKuJmuU7sdeZ7oTzWdGb5rhWONC6fV369rAmy5B0Xywd/D7sIE5knLLpjPWu1ufI
+2abKleFOaXmIEjIc9HWKZTRc6wJe0tbNIOYFDQJJJkXo3fxvHaJfnPTsj1p0EhpQGq7IDDCtvZZQ
+rW/90MI9M45dMZ/6MKeqSyK0c+dheRHEc2z1+IR4LrWZRCu9GvTxKqVALO7xWqTJTTGhctyzA1j0
++a0xzNK7MMKLATDEx0HVr1TC5gZBw66j0TgZy6EKgSQNXlL/DDsvIpbatjJxFo8QCTGd6jErp7LT
+JL2cPA+kfun16fAZUaYIt4OpEUKvwymp0X0KflRpWhmkFCuqR/NTE9ZVgfk2R5sOY6dyrn4l9fJr
+WYgpVkx/pUyyuFGtyoLaNmnLeyuFDbOdRDrNd2kXRQqUxkFCTm+PZqOM0u6TY+DevRk5fZjo/evU
+9M7rVO/FllArbwhqy8/rz7PXMPjt01wbN5UXh06AfDxRQceR6TYS7vhZd4fqRoTgzmiagqBflXnj
+fHeMhsplCG3aqORRZvjkEBI8zmKGaxkBKbjyW7eeVhTy2D34As3iHL5yb6w16Xg5OfCGdpnQ2tdQ
+EnYgA6bYxFu2xLvcS40Z4aZdjn6bNMyii0xTyYWkxahDKyiTh9zNQlDeGNueR/70HBgIROnQO77k
+/lhhlHIWUYivrEV8S6Mlqz/NjYsjvJ84LwfCrZgBs1d3dtBro/95SjADnhaa4V2XmRnpewh63bTq
+dH/6bPfw+ElSlCzSbpX23h5zGCzAqUmKH1aRhiADi0L9SKbI+hyR9I7OEj8YUdT9bJsreyjzO1mY
+TrVuQlU+ZHXSqS380vKm1OxYrCANExab+VF2abjTCOeiA72JDmluSLaIjXAO3MTMy8Btu/QZ4Ymc
+giTz+oGSrmydIG6gxz3ZWdUgiZ4ideGHBc4FU4u7EcuN6yJzpSD8wmEXdSwkEvMGmAR0oVQeKC5+
+lGYbqzMhhokU/FPvovMHHq2iJ7TZxLiwqMxnzjxVjxYHH3Is8ynyA8II68fZM7Q73P3EZzqzALQR
+2nP7ozdagdlDjT+GKpXfaYFgLBQQQvGKxlYwyEj7Kdqhu6SpkX1rexu6AZJQqBjVTCbnJHr/u68h
+pt7xyOJHWG7zt3oo0z0USAPtlOU1P/x5LL8z/JFDYE0muS+UPQKyux3DEgR2pbD4j/6w0yfbvYtJ
+hTc2WWfgFxqbUtM2aVx60BrFkPGStOhLN9LzkMyboXC1HRHSyW08lLaFwr+0vzWt3UXbIhGEoped
+X+C+FwNVi9cpLE4mla+7Zr4VX9hh6Awnlh+bMpAA/uDi6VEKi2ieGM/SgYdJxn6V+SssXMSKMxDM
++qdBnzIcQfFkh6BZJ2cwLiVDDB4iaaR6GSRNUn0Ok1Ca6HPTsg/aMAQ4lBGV4q4xpyGRdXyMOysr
+cal+nKIzv6L3z88iUc5EtbgN+KXZxEW3wxMn5Mqc4+RJ4eMc1oL+OXhaxkFb28b2v8nyPMVzG3n5
+NrEy/qdQMfaTInb6J5EY0V2NGSA8sSIwKnwg4XCWdeNw7ySeXwa+kVWf08zxSLE0E8QBrKZOuxVl
+o3PGw4PvE2rTYEaRvWOnaIsNcHSSuZO9mbu8urbB9q6S2ZHeVZ5GeD4HR0vaVT66GDZJj3cuO40b
+c2q7UUX3OhJ+FFhG4j6OES49MCyaXV3gOzNPyijJ7dNSZGPIH9esfp25nYHmnxNXv2JtYV9o5tjK
+tmx72mecWSHR7HJo9gbUTAs7kLPQjQC1r4RJ2D3WEiN6lJFyjbVIYejCe8sRunc+++7acWM7WodF
+4Z75WeLigKCxCDNUl2MWJIgav7ZWnwzb3q/NeSUbOTMB8ov0ebIVMCkKxehKjLr71dKMTG0QmIbD
+2mEw/jC3kYUHpbD1dpvIOBacAtL2Ajpe9DCY0qfgmCP9Jk9Zj8EeTixVetv1dqDmouRls2sVrvBz
+2HdylC5RYSKxz2uvSK+KEAFhIEUfXc9uRPVbaWo8G/uQv1CfRUmKeqKV9/1c+fBPSgvIJRoiHwWt
+HOPLSZnm0xiTLwvkDJtVq4uI5Rs/ZhwUYQ+pYpgN60tt6tMTmQsov1O3F9hkfA3fD6C6zFiF3bKm
+jmKgkWL2vn4+eo6S8XewbhVaA4pTuSqIfuXEZjXsjnMXghnCOBj9KDA34teQngltiAfkby2nAKiX
+9tmQrbmT+TWHY/U9xR1B656IaLWdKqdpTnw3A4zieEUCrqpLBBVLXWfTFk4vYwqnmczrWe8jjg/T
+2HlbF3TrKT+r/ZmZQt0bM+mGU5lgTZpbt3zWC33+5jUuHmJke9a4FtJ1YPokVbQpaUDzNZqoG9jG
+RyvaNHHtXxnYt27NdmZxoNKIrTXSSfu2njxqkDYx6jV03fBKnxoweyIs8xO/rfPsE1DYsA66qtcu
+qpRTLGQrIz6dMt+LTtLJ4dyZTBXFJEYY3QngBhr7UKBYXOWztbwaXutcDnJ0v0D8EG5gtlXx3OvJ
+cNOVrX9fdYWUjGua/izBV5HBArLcGzOuxp9OmnRslm3oXPXU7p+mYVwgfyafa2dqowx0zkJfcFOg
+UEsZBlyNQLJVEANUfZ5lM1/3IEoaEL7hdI/ethWBb6b9DRE3w5OZ+8O49vS4P/XmsPb27ICTt2Ij
+MiGKcGgsd41Wsm3NVcJSNLcpjDWvCDHkm7ibbpM5TdQJ7GX60m2FDBWnqp/goo3j3oNZ2YUP4TSq
+68iKZgs9do8rf0KcS5LUbIZh4Dl1MUMvMMGYCnr5deDxqUS8n8m4zWrpP5l+EWMdlZNoT0YZ++dI
+wSr5LcMb7WxhbS5NAi8rrhEqozRKmxg7EN26AhYitNph4yn6zxskNr7dMdBn8uFPgcekv5+7AKhB
+oeeId1LK8VMVuuEPyuFk+KTNXVefjPis6p3QHFvdUE/7OoPONnG2KEUtE8+5jpwdEKE8wX2iTffd
+0KV0B3x0NJh0Ja1PsIFYWI2DnZXjONZWa3G5YuDG8MrLhvk1OxhhCRvnsJUdDLJ6uphl54NxNj2Y
+aGn7Y6gtDubaxikL5wzbElspyli7OzcPllwiykH1uYtTVz+Ydu1SU/fdwcqb5p7PGQZ+0iOVdno7
+DRG23/hgAS7cmvqQDID8zjmYhFXSTEAgDuZhPUwpk6eDqdhC/fg0HKzG7sF23C0OZAfsYLa2D8Zk
+42BS9g+G5eRgXlYHI3OXuL0KYCKEPyAsY3XOftmekyI8nQ9maP9gjDZ+maQNUGIBR3CBs3nxUTdm
+h9GrjJkWsMGwn+O1/tt6LRtjFh5Z25Vz8Glr5TykzRfgXxi6Dz3Ef1tQXlhQEJv91lpdAhP+/scX
+X3OCELCgfP3Xf377+tKFcvhDf7tQhPUXQyqmIAL3hcNcjJ7l3y4U4f1FuAUcNXr39KHEMj38h+GC
+dwUupsuUEjkqopRlDN+UXSthv3h/CR2pyqKnZ+KAEs7/Ex8Kme8vm9FIPCwCFIDUIw7xUegvvdvf
+JihpyDtXZCpDAiLru8rIkqfa6KJbqxswv/tpq7Wn2J/Du7LSnR9RRj5jbiZU2KIK27OoGsufblVE
++7lqZbPVE9eY2B8NNj8dkrLEtBtCUJ0q9NerFJVLFvSj6eGn6tJLTxs7ay3JEqSjUdXxt7EoaUEO
+HeZmnNp1KTdtaOQgOqdQPSJUix4bznIcPd3MZPmi44dHWoQdHrGyrId1KNIMV62Jm7LoDodg/I0Z
++59G884rmwX+n0i6kP3oFl/AxnWgMx0P2OAAQPSLh4YDEkeq2/pK9J1+LeYJc3AGa+U85tOWF9MC
+b1m7Y2w+6Xzq6oTRL7WKtLTscsriod42YVg4m9kczROlhgIzIkotpAcFKe6Mo1p1o4eGxwAWZ/h3
+38v9e4pEdQMPX+Bwzmfs71NrQCq2vNq6YQ5jzTuV6ylNyQF67CrXmHFFWpo6p84SqmTq5fCYm6rC
+2F0o5xOItvgrp3SURUIPJ+jR6KXlvmpK60s5pBMhtC7YDyh9bTPAhku7cCfcPNUYF3lQ9zi20DxI
+/Cq/0NvCpVsahZQwxaxv8BNNWKUzx3qM7U5q3G4/p9lKY2cOkDZrcu0YeIuCcFYjx9Ao5nhE1I9x
+W1ooS1YuBxaIoS208w7gmr7K5hHkTjREnXdX0U2GVReZ5U8IkEqeJLVmgLgvdOeB6VvbnZrRkD+m
+WdsJBGixf4phcYyCfp7Ce0erMFH2mpG2G8IMcSDBV5PuztU4Fq+9yEx47bIQ9EdY2NT4JTWgwVF1
+DO9h19gkmSUkQAScWrUvbtvEVzRBLNgSdax5n6NmBMxTNzZH9abNG1D27VIWT6lm7To/rM6KaYy1
+Ta2nMTdpbkaNIttNr9EAK5oB0eRoZ1Pp0WyswGnaq1YkcX2qDFEyl6yhF4HzsIYz1ypkSBt6dL9h
+Y5zlzhKzK9ZO1VfgraNMwVfNFpIojIn83sjK4X6MbHGJel3mK7zgWDH7pmk/ceoMH1yvmH5WUoP1
+Th5X7m58cEp2gMaMeiwxCRthD2qbLzwk4JBjNQC5mdUEi5UBRVZtSZyInrQMazPAgCH9ks1YoFaz
+m2Y3FEK9Wttm6D/TgzbNbV83/WXYhi3/PwJf68ddY28dSgKAC5phXsK3k+22Qu5/KfJ4fMDoD+Wx
+83WmUD4adXFKCTK0qDSRnm6IGZ66lU26KWHkQEnbtcrIGtSalIJigPdRrogk6UxmJgWwJi92jcsB
+yO73ppDjd5HXYbuOnFb7rkiqu89xnesj3S4kvTEIDI0C9Nps6uHKoBOIUsGE6L9LM5qUAV0gkO+6
+788iqH1O++u5Nu1yY2aDxEVc+FO7rsU4XY1+7/5sSD4BLCIL91vRp6rEMJuSxdpxGI1XmcjB7GBW
+84Al2G0U84PyXKzaXm/PpiGvFe9iKMjhGOy62pgORbVPZa3WBc/iCdd5OgV5UpR7lXAyWsf0261g
+SggUXBs9Ux86RXRURlo+lzVeVnsjgHd/iazRZ3VlFsTpg2gFGtz0ZdMTegCf9DDOHrPZNy6AG+CB
+Z8nhOJ+VPELg9sgCV3AT6ssi1cDa+hzWIdqVfBHFMNEQzkaVQLeWKsnOGiLerxzNEj8tOB90CbR5
+ighhyJ0rkJmgGkt9bAeU7iJ9NmkS/NCciHFxmYmWF9owgXvYAAvv3CmK3S1H94oEG78fmWD3ibB2
+7KYz1gjBlHQNz8Ui+UYf4XD3edWCcwS+sddcFZ6JrEGQBO8TmwO9i4RMHYiNuBxlD8ZiBPb0MFrq
+LBwtx/7URa6vwwghCpQ+u0oJP/VKCzIUcr1phUhgugU25qpTKzK6i1oyc+IVNcR9r3L6TgKJT7GX
+uoslnzabvc2i1P5SCmXUp5He0XfzRTieaCqCSsNJ2HxWnAQuFjA1D0EDtHkiVTWc2DoNwV1KDA9f
+cuwYMOAzyCN2o7vPNZT3iUnWEH7xsQvJIO6IPdly68FIt0UXNVs7k+qE18ert32lJ/YKAzg9uZp+
+zMUkMfVv+iwh7s/nsV4Nc0sXYxzHnH6DGm5bltA7cxaKbycx2scaFPZedSOsZGf0JM30qS+/+H2F
+bLI2whz5RgrLm8OMY3yK4CjJTaN38VfXmsMvFTM5NA91F38XyLppjifSuglTi/sWN33/lWAK7Ydy
+B+RA/64+X4Vpoe6jFvvvw7Su4yVL62vx43nJ0roo6/b5RSH668//U4iKv0iocoi+sgyy8ZAO/l6I
+EpzImkYC5uGfYKz4pxDlT6FbQ2uIIhQ77MFW808h6vxFuchIhzzEpYLEfPMnheiRJoIDp8AbysFr
+EdJC8z5Sp0HGbChInKduwXaX2hVuzRzMdGnQsnbFqq5A0wOU/fUi/bdW0SMpxK+rcp91qnTkZMfJ
+elpnMwAanaex2/vSO8/7jVlyCHWS9Tw//PZwLn8JA373YpuHRPXfBANU2jp2IBtQIglI5EAfSaLM
+XrdTxAQsO2U5gcE4lAtEgCXapl+qCDXk9k43kF1uSE1p3aA5lBzyUH4A1JX+Z/9QlhDFE1+1qal9
+GQ5ly3woYZh/h/fVobDRDkUODa5sCJqxTbPAORRCY81euSOcmgLJnUTWbuxD4dQtNVRLky8K0qWy
+Sg5FlrHUW2Ve9t0pEAnnQZQmfeTyUJxRUpU/y0PJNtT14N2NUgkVcPimrLNI7blyDsVecSj8wqUG
+BAJBOQhfgdKQLCzKROtQMvaH8hEzbcFgyejQ4NRLhbl0VUDyKlvfQH7I1x5wEmeBzuYXmrmUqKZH
+TCYHlEhggAWTyKqfgwbfWIwMISdHcE/PIL64xkoXiZVAabEmez+kwj7Tk9ElTwLORkU2RWRexJCo
+2J4ScYH2mSqHM8e1VUUPTaRJBck3IWMhBxLRrIVD+4DepAZBcCIo0Vs1dR3SNQ5bzgEagijo/eM8
+OQQeGPa4IcYzqte5Ny1BsvpYNzvDokykMOipxkrD6NrrmSzJHbL/Uvtsycz9McbEFyAIndqOeEDE
+Z9saklF0JpYz2alQLhk21uyVD2XnJc8KbeLIpCOpnI2JMRhbW8FgBMpr4cpFyUBEj89Zap11mo9T
+3o7rtT/Gctiaoi7Sz63HySbAJaPTAQoL+vZUNOz0hpqTcsewpVJrV9lFstfoJRMnNVsxib8j7afi
+SvVD0sHT6+V3PDz4kZNWr8KtqTuUatLJE24hoMiTkpga2r+8YmChLf6NZuyQfEs9lX9tI1g2q7FN
+3AsCxZLbIqsGfxeLwdzD35m5572nQ3s04uQnsx7EAZ45FYSwdFEyc26McBF1bihOLeUlxgojUCN3
+MJbaWwlf1966qu/OqCVbf7lrjLxpFGnnrWNqyboHuJiBQJ9bwnUgE10qY6i+UjCTNsQGjNd5Jt/j
+a///2DuP5biZLVs/EU7AIzGtKpR39CInCIqUEt4DCeDp+wP/PtEmogd3fmeiJJYBEpl7r72MNXWP
+xEXL13Kcoi8cgPpz91PmaSy0xcAedeFaLpVg7yzBEqZL5ACjhKVgNH6Kx+mnkASLzvnvPwWmMc1q
+XJHmQOHpd53p7MYWVf7KWGpTsMXuMfspWGl5aO7MMX2tsfWiXaSyhRundRtRq/Fr+Kl8Gbfes9Sj
+HK4KpmcrsFTKZA8PG4zLluo5qbEH47MMdAnyp8Buosl3yDAiAGnlRMi1sH2H5Io1t01xDkt4/IWz
+oHfvGVF323mp49FqGAkF91Lehz+lvun23Z9+qf9nZRrmFlGX/8fD+xPPfMdOnxjAYZEzlGn6QitO
+M6GYirwTTJhWWwulrRv4uPt3yDaXNiTDNfEl/mlOyp9GZcx4Xhnu4aQekJVHMzM41vSXBKeQWUTc
+XZyftsebZ8n4d+mG9KUvKpYOaf5pluQY0jjVGOLRRJkQRDcQJrE/xDLC++3+tFzt0n3hqJ9jjlN6
+VRi0Pw0aKD3N2qQwR6TTELZ2YtpJQxcvvd3/L2j+d0FjYTcN/PV/FzTP5dcnYaVF+9/LmP/8rX+7
+ujj/ojrgaPUMiIv8CdDs364u+r+obUx8jUn+dShZKJ7+XcY4S14oIcRwOQHNFtrjf+FphvUvKN3I
+L3Uqd6j6BGT/P/i6mEiN/yeghjBPNxbuO77IvJzzvwmlcrTgA5ATvS6dicBLS+A3l45KbZkFd1tT
+yvkw2rjsIXkRqYYVoSZfEKU5NzVwFoRtYweeo9W7Kk2Y3BSygLUW/REyn+E+mOKYex1dHflyLrGB
+zqJU1bohyKH3bfVYDb90hAW3ssnrjZFYJWDAoH3FvqE+oYhsy8q5T96gH9APl6daGv7LmMtfZE2P
+H2TIQBPzivDRxo7piuW+8W5Ls38nfqS5ZwLLeBl+91jUnc06b/ALj8QWi6vyewjNARNceAHbURb1
+zcf0asNJY50SmBZAAHjpqQGYpcFKc7MEpMqV4/fGLYMks1e9m96tMX2iBzaadWfPODD2fUuLErpX
+4iHnlawm6FlZ1zxExYdn0FriWMfI2BT1CmdEb1OlEBWhXpDdk4xgB3r81ugkYWSWki+TIAwvcnUm
+wlCGjuwFpF9NtzKG/kqY2rRTukMKQTSlJJ3gUig8CH4b5SWMh0fC2Uma8SxeeBgOSdiXQTYOw9rG
+r9XDpirEWbI0agbxoRd4YYzrnmVh/xl4DL6zr7QWCN0kg7k99UPjH7RxSm4zs/1pGX2HGgb8rau9
+dqlSpzZK8xvesNgNW6m/lwbFkFNzeTbTMBXbSohiWxZ2utWNtPJ2c5/WDX+b95+Ax9kjiDIm24Xt
+BmjTkr3wRKClI7iU6s9p8mU0vyF+rExBshUZFHtIk++2at9mbHtWefhqz/EuDYtdHbrwwf6UdvTX
+j9PjgNualxp/dJm/9Am0GwlhMHOtQ+wXBwno6lraJU/1LQqb61TKxy7NTwhNTnUe7TGia68GO8PG
+LFsmViBj9TEWWb2tMSbeODa10fTUx7GJ8eukPfQgiQvOVGH1xcixeE6iTgD3GTaxQuJial4RtAb7
+uSj2XpgGcUJJ0+iB0CFwmtZuNId36Hk7VYutOfzuQ/tBczBfdB/t6C2cPowlBkuEQwiO1K2tsbO2
+btzJ62x4AetwpxfpZs7LrcqYtMdWwwBzeGhdl8mvTxJG7+xw49vIHhfcKX6DarB30iroRH11XeCM
+xiWLbHkNB5+BrINmZUL8+DvDsIg8Agm9ibjTYVf3pbHTLX3Y1H7ygk1BsrVC+Qxv49xnU7PWbTJj
+stRe6UK72xAzMsd/6WLxEukghIyQ9SDWqr3R6Re7+hPjDTnMeAXlLuS/GjYAltPAm0rpepCC3K48
+zjEYvTtlZYCruv5RlH52cROc/2wgGArcN8OPA0sVsCq1PRDzevB9WHA4Epez+Xfy+mgX4Q5hOw+d
+Lr95at+Y8CJZWtfSv+X2ZU6x6nTaR6nLl3HxI/aLFipMod3aFHJB3BefRqal614WzL/H5DGCp0yk
+VXYLdfMSClhaOlSIlSbFPTTirzEpY5xL1d0q+ofRcd4xCnxzcCnEbEc7z0n2hO3TSVRdFphF+6B3
+2TvcDdZneiGP6D00iwNEpqCXZrGWJcklwxIjqMgnarrXHtYvSC7C6TzTfnOefDI3Phl4ZkNUfq2j
++kXE5bwiRPcjLIyCz2tuOodyamrFQy/GHbaLWxX3N8qXNWBlfS9HKyP3MtkqOGZt+SVKlmfK8z23
++snt7mQKb4qSoLth6zUxyWwFEWu/rFGs+2a2wKHmzzBky3GTnY8xuoVNBgu0h6Nl4JJdXSPf2M+M
+Slq3/xhUPn12EIDMHA5v+lKFJ51tUNf7v5Pb/QU6XuWQZ6HbLk744fR3rJuHKstpqVkGc9Odwuy7
+ZV+grvkgrOj3aPm0DNqd84g1G500JGpOCMHFdtaMRpjHaFJbG12dr53KeqhDbPZjvd36bvE25eqO
+InULtedFuOMaAvJvHDWD0jdSyDw1U2Qth2OrtlarhnXWDWsyWf/2prgls/6KnPFa69Ed5u5hnMMC
+niZM8CqxVv0A3VdXUXpI2tqFa4HrLmT6jdIK2G9gEus5IXcD1TidwZC8SCiqzJ33eY6tI5Yq31jR
+Po96++1BFTnlSQoDxCd1Z6hJS2LS2rk7jflVDOjcOGjUjDSHwBi7ahsu3kPxfHAK7HGZCaj+IpPq
+G9mW4q+T81jbXOQcUi5MlJUfY2eA0gk1hequ8VS+xnl16OwwwJ1cWwSaGmsvFjczZyXoJZYfhFmh
+9Xsb87Z7090u/jtWEzxcxhuQcNq90kHzp7LRd3oFsa1mq1/X6Xhlk/ky4uyWhob2QBketBGeSV5r
+nwgl89cujidW69w4yoFLeFYrEsUYfr3X87fT5AHW86uhf6LnPpUEhxA58CRi4g8H4yuJ9GJb9Ea/
+h1vJvOIrqeqGhUhKDWGKtmaRUIBLl1U3xzof7ZuCSLpX7QfzwnpykDMaizB/WDUdfH2lmJWMJNAq
+0ES/vqM8PxCCtjdnuY2icJ2675FXHHQ32jrWjD2li+b/PmQCILM4KhMHfQJmBky0E9Zvpv1q4VhE
+0c1xDpkY1y3xcy5ZR5BnjmYoIeQSKJRx/3yTykHfQLAW+j0m4Llzs13kh2triK568UV69TsGACvo
+JlhGynPvYnUb2W+lX7MVk8SNL3ibqg8Xh++RymJlyAG+e3kNJ+SYrbc3zG6V+EQvDsDRXoSLv3UC
+NkDTIjc2uoyumpFt9hQC+a80sw59O5E8ZV2qZeQnho828U+G0sh7IRUutRh7mtvCCOFsy7Pj/E5K
+667TH9VqIfh6u7I0HiKWimX9ZcbExiKPlVWuAVIGYH8xyyD35EeOnXiiv7Uzj07LMLDLbk3ObyWZ
+FhRtDZQGnYvA8NbK+fQFszADymQjoGK2MQyztH3W8b9NhXkYh5h4b65oVJZbrV/Ca+Zp3wob4MDu
+A1h35YXaEiwpkqR3Vbj459MzJ9JmMfeNMt84+YUX7saKjKG8nW4YEW/d0N9Odesc4USJ7Wh5X26c
+XQqGqTCRYtzMevcQEegweOktm6JtrpuvxKwFUPYuuBeyI4pV7bXVhdTVLfTmVW84YjWg8L8Ksvps
+bMGL5m+jUeyssTJl3Dzl9bXGZ2jtzbB7myZ+rg1CJBWppYx+Wn8zIFJZpxOD5LVd25vB7NbY3K7B
+EaCP12RTeNbeiHcgSrvCMX7jHBoMZnxQnhckJGgRD31zY/LQ4jAoeo54wk1POI+swZiuUT3kO73x
+thkWxqiOnrEfGhcZfVBP1qUs1dEY9aDFRYbR6YHSLgAP3PhuE3jiEmcaCggG2oRMk/KOGADCNckk
+7wzQ10ZZPbXQmo0C7lqUTrvO/hMav0yLKmnVx+NG03pYVCgNUi+Cao7DqXAJt5V2ENuPVX+lmqV3
+zrB/sImc2hvusF8C75IJb3yrb7apQypvNqJGXvyxXXOvoQvK09du0fo15dmahRmIbNpYpG7GXJB0
+EsPG4KDcu+o5735V067SH8T0OkzhHr0dqoB6O0TZq0YyctdPa0sDWhuYpyAUIT/tbvSo7nL9D2yk
+PWYfy/APbXm6i1z6IfUekSA7++KV+OKtFH9No8Jiuj4YORxtKTySTcxVx1/GlPS2Ys4+DM814RMO
+C8TvIWLO+D9k47ElZV2m8daYXTbhmkyRpAsohJFYabFDaX4xsufc/5XUB1VoV0JKjgJwT5N+4INO
+sBNkEbw5Rnoxhr6rIgU0NC1SC0vFizZaEMIZMG1jK4rKPuCJUS83dOf6Zrzr+UED3Sjm05A5G5LY
+8yMqhnbTZp/IVt8XQMRLw5wc6OapYN9XOF3j64AqJ7rnPfUvqrnpKSrDlbvkqESX1kBUZhZbt5t2
+PAWHqMr3rdOogwuDl9suiz9NVXt7iZoIH54VqR6HqQrZRkj7mMLHtnvNc5Lhfeu1i5GXGCSwGzhD
+wcx6Jm4n0FFC5CazQ6idiMK0XWMoFmGvCCIx23OKpg3u2Y54i5rlLzhWO/nCxvJQ6/rOZ2IFygg4
+aDOsC02Yo+wnIwy21qhahksmttTkEAahQ35nPE3PAkiYCL0TiR67AWnQui9t5FFSRkdjcekmsyq1
+8nGnw0VxACe3c4eDj/Sx+C1gYGI8vu+aNxyYgxbHzGQgcz2CKdGCU0dX4M0KtEZRTMjHJfD36kCI
+X7kItpqRbct8m2P8oG3tWrYTz7C/IVwAjxJQahyDotQBHmfAC6N1NURqXJuAQ4TriLWfJuuO/aRP
+Tkv82qQHyaw2WQ2onPvXWqZnL/qD4eTKsX/32rsi0nWnJ8V2jFCHVM4jDIiT7tcrhHxB4k9PxGIi
+OX2EyUq0yWetP0OA3YfcrZh+eK6Lq2Ik+1T6uBH3DkT7ydmS30NbyQ5HgEXQlOPBwEx9Vci5/6ON
+HdtL2QcEk57UxKy01IxV7g7pLRTx2pnCd4DCQ0f1r48UnDH8AwNT5lqrspM3YuaPFTP0Oi2ICPM9
+iqjBjaonPTNjo56cFoEaTSxhET1ETvDFhHB6ghvsgPbCW9J1E+J2SmOsf2dzubYHuyEuzYkLd6OG
+JCQrjVTQ1ynEcKabIabJuPsTKnGWKQnDMk73eS2yfRLarMBI07szjEnv0EWxlgb5qGvFPjL6Xt7w
+HKvaBxxkRhImtMrTjuhqjqQwbCxv3IZxx1riZlNEU4nfGZ7S1IoADh7FZKp9uUDZY9Twtbts7Tgh
+T9V0mQ0Bwp9tM47ucNpbLKSgapjIWrq/y7NFGBeFNAJJQhz9irGaIAQWCfwxbHL++6DcN9RezW8X
+mGBjwsbfWGGX/ZrnIb80VpjXn3JqIoXGDmnY1h3JukM1Ud3Q5JYyqHGG0zZ48cUy0Iuy5Uz3zVcA
+kOEIPXi6pZ3PDjlW5XPO5njoRFPeUJ0CbpRUf9YqVdrfEYD80hfM5EPgmT9zjsvZaoKJsXYddiA9
+I70BIo77CN4u38CxqyAk8o3lOHCXZxeSVstBMEkkL6ifiAjUyt+pplxiIL3HqiqivQsEe3S6wkbc
+J4pgGKI+SEg2CfJ+GQDE1XCcpTeibqWDjaMu+12KQoOnjRiAvr48eWpBlkhz/tCJnKtXVJjqecx9
+7yNGEk7epeRnNKYAJyIe6qelu9pBavbPeq/4EaOHkxhdOgLHHCkiILTHD63W+me0R4A+gki/B8QN
+DK7bsiYfDAHGNeUAvDJ1F9cOX9PznHI8tMKPTyocxcUHmD8W2DqYjfvMqLM8RlXv7lsX0rgwacnS
+1P9Oi4KPxNOs722V6HsRwmOYZ/UF1NU86rJTW1tqy0cvyBSZcTvQywzCU+5nO6Hh169mncFVGi+f
+qWu6Q9u6/Mem5vXAiQJVJIO/bidetfSH8KaU9oqKOXprDQYFSKUo2Ze3bKta7NTQikuUtfHW6+d2
+D5HB2pA4iYZWddTRy3sSpTE+C8StN6Z47SXl7lIdkH8s6iJ6qOyh3dcEeq7HDL5z433rZsXrKh2L
+wtQKbySViAvJmBlhzf7yR1jZx7LibRVq31vrkzAMZVhtS1ezIOOjmgKAJPPLq6MHPRzE7p9vaor4
+BKk9BNawx0WI/N06UQJ1MLLeZRaa7xKbyL2Kel54ubblkHFBmoRHK4cZU0KRCphi8sJNdVcq8oED
+GeTF1PcoCMNbWvOxS7elkYbFZ1GgaAY16/wG4Ubtqkp7IhOFL2axiuopJ4cyi7BE5ALrsfatS8ve
+cFUXK27/W/d5ICSZJLvSRF3booW+dvSW70mhP/4spp8PMOvTpzbLjzKJwQibMXuUMHx30tdeVcgH
+//lwkMxEkOYtX2G5QHbEq9rwwGjc9I3wCdi0PDzuZ8DDVKcthTUZ3sgPjffwypHqjMvRbrkUg97o
+n0mPQWzgcxmyOZZb7odbcbFLnUFqy0R3Zw/cHsiRH1ao18HPxwQl/7YH+VaOWPOX5B6vSZgsNm2i
+/LOqJPHCfLguTAi0gSDzyCNHH2Tz+Vvdan7ZE+FX6cCbeJk4sv8WW1lieiLVcmU6Wqzl+ilhH5mj
+3ou6WOSX3xCJmE4OXBdCK7mFA4QqKUnE0i0+DK6KjN94h7JGqWVEX5qL9hWrTPZE21NBsyx+xlpq
+m/DAs560b8sPX1tUEhsPAvuWEo3+DWRwZZvaK0MivpjgzfTCvou++A6FJD+IGnAThXO2b9q6++ft
+8c86EsJSQWDhW6I/5BUIZ93jP/hpd7yolrCyIDfyiI9DSc7ZUBMugEX8WlSEOel21h0QJolASL46
+rifFJvLnY2ouX/Dn5dhyfj5VM/b+uS+yKxzzeofdggUJc1kobaXvW6Z50PD5hiU+Gjcx8iNxh8UR
+sUP2qGLT2hTdqJ00W4mLcEj41samOKaqZL/AcvzhZ3Wqeh5/Y6jUMKKztBPhiv5ZDry/UqwMhJL/
+eavtCI1T1Xd9wDh50lC9sPf8PFGyYcf5Z0SRT7xC1MbkOkHeofHXnmiZQCLgvs+rxq/FsyHQWqMX
+EezDy5ZWN/yLTPlmYpyaX5mmeQ99/OE2Jmi6U4RLgp713OOttA9TWT13OkFefmwYR6jwGjmFaUVK
+T6//8u2Era3fLzB7V1OIyqaEQRATds4R5D40c66tO1XfhPnoO8PWzsptW8tH+HZ09dqEamekD6Dy
+25JdBUwVOX8Tgq9nq/IO02yRa2edKm98VF37x2fggelRGYjW8zdGZDnbvsrw4YDiEM788qRfGls1
+e5bIqesr7TWafeKSx+nYLcoO1+BEq73mKMssu/d9V90q/uA36o8vhndEK8XOrdvP0tbOPVVvQidk
+99UHbpt3wdpfxXlKD/2dhchRI1w3tW07jG89wTlMGCAotp/sYHeLYOF31ORfcENOqdQOhUXmmalu
+ow3bsRuLAz2ntW/0od8gQ39nhL1Yxjsl23F9q5E3ln7xQHjgQ13FX8zczUCrsBR1iq5ZEtAO0A7X
+3uSAzRpvY18+NXYxBzQvM4YGkSgfCuGtLGW9oNc5OL14s93y3NiW/zAOIFUSfi72ByP4kgwJ7KFZ
++65VtU9huq9yDixQm8qGmUFIZJTwNEp/R4Z6w+U1X3F3Zp7lXCiJPtFvBknUmq8Y3//pY3uv/PA4
+tOZjrOytZmVB6PpE67mkso/XbJFfpQTbrl2jqrdFTTB4kdQvE1lgNCjXCH9jhBebJU0sa+wDxRn0
+VT2IGB2EOPidSsd4dFQHx7gwxiAhHo0QuWnd9NHrUE2/UFbaGyI/SUzpKZCblIQEcDF8WQk4ceJj
+4TLO0FPhrKXOHVFZRaNedIGIa2ODH4G+R4durYeofG3a6peqCWnu5wHTZc3P8MghWVw1jr3q2aVw
+oBC0yGUCXEEiDWy7bt0Nltw42Gc8tf2HEYqNU/FtzDD2Nr22CKk0kR39bEwPBIQZ+4qHaRXq2fiS
+UXB/DH2YHLTZ6jdQvLQDel7yX5aA5lx0JoUlCUbZIIYb8n2S4JthDiaC2Hf5TOcwTkSr+sT0sIlq
+D43W0mfbMXnMLfHVzJUIEKztZ7js30x8sqMRLoSbqIP2y06xtR03PpkzRHqKvPZtMOp+A4rf3JH4
+N5sBMsHyBtZOuW36N1WEGUa+EPRRDR6fRuWkV88a0l9xF3tHWAHcZD/yt65Le9dW0FDKofCPkoWN
+WnpwvUOLSHNLoob1KgXSNtVQt8Yo4ek+Ruwler03g4bYbzgNkwNihTDv2BZauoXNxM1wpPEx2nFJ
+pZbahL1ndY1Gbay/2FaRW6EUPGRtZGGgoSX6B+7+kBndKpcnR1bMvqIuzreycdlEEf+hNc89Aucc
+t7p0fcz4cJq818TXQkJ7hHPM8FnYGBDwoaxUPLsZlhOrqYcCsjKNiVGRpIBbEchN1oxpfLh4q5ML
+NYDQzWMDYBKWt9bprROsA3+VQJeGJ4KNbQ816TwSs0YlX+WfJG6mBn0JMWC6Vhu05eavSiB3JpzG
+OVQlrFrR5ZVYLUPrleOMNtBe77EgiTGFDlFQiepkQcY7srMBG2y0V6ZlDQe0VZEKbLemAsSqUd/H
+nMDnEDO7X8hGkk88+5fjSMuI38lM/2x7FG5qdMXFxlFgp82V/wQqavDbs199C0MVO4lm9P2n5FUK
+4xy0SpgmgjNXRDV1LgVumRDt53gKM4xhiQ7e/FO2kkd9ErMQVzttOSvTFIeYuXPBSnONkNblFqxL
+jSNzydKdSJSjCW6g/GNozNdejUk/fkvDZG9OW/OaSm40cV8euYC2o1DKuR0pQSLuml9qXEpSQcA6
+wN1SaEN73qeo//FfSHusHWVBjY9oIHts6lhe4Xznn9ls4bYyFO4HMs/2BsGoexlMOznHdRheJjdz
+HvU8yvd5r7mbuB6Y75AdNO99Mo+ZLUJB381oTkGr45ixnwmvrImsYpemnJ3obFdzPngvrRZXl94p
+w3szx+M6mgHFZUXo7NR71NgV607P3WarL+R66XuPJtq3C9moLdUX/KdN5C5eM/OU+4BesbNjcI2O
+xutF6yOpjlIAEqf/a1pDvIkIld2H8axOI7U1PXc+b1tHThv8KfJglkmxy0s3vM+zSW9b6O0Z7xE4
+3l4XO8B7Rmt8A2FbZxuroDsD4BZM3/RpLxDrbSBU84hZg65dNcbiN8KQhb4tGfQ9+lz6t+kfn516
+gp6O39E76Vj5n3YJtXLcUisAIMCx0t5W7MYoGR7zzAn3IRruHRZDzpvjaExsyTOJvzMPFQsmAsK4
+2aU2B8Xi+kMD230jHTQPasxRKqFDaD8MryNUdsS05iqa2Dz1uAWQRtcgayWptI+3Reake8eAgtc1
+NhdokCCQmHXIcyRLQQg9ciRU9ZXfnx1v8BB6S1Ntm5SnYjEX835huVid4XLXQ+DHdvK7NUNQhGlI
+6t1UDt41FwNKeWh0xMuZcXr3osjcJImU+GXU1oLo6g3Rbz/xj6pTrF1dW5b9Ut1Xrp6ejFpQDPVN
+h0ikrW0eFqRpnNJGmj0WCCUvGU8wzt5lSfIbaXAQLGHOi2sf9t491SooWXg5vTCqA5mnzL+EmpYQ
+G7bYOYEFvWYuTr6/fTptOqmuN8xzubQq64hzVVxFUvNQkQyrzZyYFiNL+8czqrJGShNbetopG2ML
+aI7yVwuMekqBz4jmRGCr4cznl8p49378qKqhkflacwc7OQG/QUz0xq7dzEaS5uca98JvPFnUJ0Fu
+yfPYGwmprcqTaJUa5UAO4H6yujhMyg2HkPaCNV7O7EYP6bh6iHpAuKM8atoM8w44ham5iEznjHpI
+XI1czfe0XqQaWY97F2Sc2T1yVgMpD6HTvGHowaAzQd3GGMFA/A3R03tHYIbuyYybIMYcplhV5MnR
+ZiyWXKORFge22meYvA9TVdZEMpSo6D1RfTuTOlLdPdm4UjwgagZrt+V+mLAob1GagzQNAOzI991H
+5CTk1hVq+m3X/X3CQOGcSQ20EH+YNpzFsqm7qUsLM6QBC9TexIjpH6Y0d3DEMYedXksvGDrhnGl8
+3AcXYfduikdIRn1UPzRZZJ+G2nM/PFcuiRBsRrW/FJYCg/jZT63fY6x125H64phzoZGQFSHSsEE5
+n/HoDKdc9fYXvIGGCmPqiqdGmGMBIRCEa+/G+Tge/NHqo83curijFFHijztVZcWpogoIN1jUFG9V
+3w9d4C45xuyZchdZ8HmA212hNs5Q6ny92Z5IqpWg+rBF21uNx14Z1LGaZmT0UflkNML7clrwMpSH
+xscA03Y/1ZJ8ZsMwqG9Dz3y1HLyHGeenpYWYz/R/V2WRrhyTiUljpy8hYvcPMlRgrkwQOj3xyCY3
+8FQWXrefBn/6wsNaEAeFgJ5ukXaNlr/QKBUEydIbEuynTTUk2IV6zXDI2CKe55/MaCI461vF2gW/
+dpJdWC3hm/6SLw3AS3swDhVgnuALYikHDo222zpmixOXNfh1kGfGwD6DYO5TiyG5jqpiZJADfNmF
+fVnYEJss07jTOScG1AHaJMcrIbU0BggWQOYmjAuPqs/IP9gW+7u0hvo86e7wq03N75RtbI15EHrn
+JMPfLeXmSkOspS1g4/jYHPWjM22IZomezTlxserqjnFJ8bcKCQnfa5ZFTeOk8X307fDLx2+AYru1
+oBw1zgEsh7pGx2ghFd3NLETx1GIaBE3Z2VkO40lEfxf40JyzWAkygRmbJVbeHd46eTPteQAu0w4Q
+nXKmj4wbHwa9GK5tofJHIFCx99xmOmJWXV7ZQK0gjDGwbso427L/WAclZfpXzePixaPZF0Ivu1Nm
+1qgUaQrv4cQWgmFW+4i9U6ANLj54oIEPhYrpZohu33t1nXG9+/BqwkWD4JsPziau6uw8Okpe4FcE
+TdFyJmtmvsWLWZ4B5aHBGCXEkKxAnYV7zaYvhPXcKSg3uDhb696f3/Hvd9eKW/xrKkp7VwvnhNDt
+nuKrsfYrK8cCKgRajUYNwlo7bWQYgXc3Xbk3QtPdzBN+KWPa/Y3ylP2+kp+QJmOWusbzoTvkjCwm
+L1gYvdeG9mjVRvVA2Fz6KE0Zbu08o6Muw6tUExtXpXWvldFAoa7jBvA7dK5Zl3nvDvLf22ja3l85
+W9M1ytJErYyoo6Mp4dNamb+jdrtSrSUPpjf2+9JI/TvAWvfp9CzzTO/aT0fr62M4FQyIoYLtZC9r
+0GjbuAizlAxrYY03OE1sGzlgPF7Yww4AFrmrwU0Pmw5JRlPNzlnzUoWwNh7x9PKl3OVjlGwsLDIy
+vJh046I1GqGmeZmTiErMJf0TfLxKicBV0wZTkl3aV8+Jne5kKnjilGnH14oJ1DFrrebuj5G1ziO/
+fe7SejpSb7l092BL/yA8M4fViQoLNEgYZLimOqGmxBRTCWK5xbhQysMEKB7Y0BKCdtI43jmK7FuT
+lXEAVllvuwyZXRdpEzm7i/HHQjyvdMe5ufAHzzCo22PVWdGNSXoadGU0XSKiUw8Mwua97ZXrUFiR
+JFHdNl7cxChOcxbKQ4dT4gU4ham3LLv46mVgVWZejBxLTDIKuvO10WjZLWkKZ4uOy782ueufkF7E
+57rSqGD0MT/0WSW2burloCrTJA9RWPHLytz3Rd5daqPtcX8AcNTZ4VSTnVsmHFiCGUOfPzFTqRSj
+QdEh/sIFH2uHjIGk1XQ1R7Ezq+eqK/tzLNyEFeRaG4wJHToS9jdJ0wvXkxHqCi8+nEswi2C2pZnG
+WYEErCKq23uW5QBO4VBlRx1sE8bX7J89J0fRHZo21jIy5rDL+56sUxdXmK7FQUxTDHVRV4e/hRdj
+J5iTc900eXcYLBu0uO6NiiFdLmHt4f0MBBnp2SP+RfLbpu084tLUHdNprIYz4F94s0DQTvZkgOZP
+hfHWi85iNA4+UJCKBW8A6K5NQAMbFHXMOcv7D66YNGC2RQ7uCzOTkYSFCcwfi6bvrbVKscMUrfkl
+xbJoPABaBkuYejh2fPoZeBR1A84HRfHgaYwXSnobELmYvqstl7jhBgHQN3sjaYjoa6I3W8sZ+ipc
+lB51GKXbMoJ4SpRvR73XMwABkaLa+QF1rQXex/ISkNdt9C/TmxE+KYgG3fSJN5LCKpCNB0Y+XbKb
+Mf1W1MtiWmZouEpstNbWnlvaxK2vmlfde4pbWHWOPt9bf1yGeRUGRBMYjV97RBHV5R0VIlaBlnpI
+k7HZNn4Yb10qKkQKXX2E8+XdZKSLjdFTyhhQXxHYtPAsW0/sZs07TgSSrWGKQqqsciqasNzMqTYS
+bskQA/ekVDc3ugUzQ+9Eu00LMV81fcTfqPdrwmNtkxKW71hC2eakmojaUJ5zt/wjAk14RVUePU2O
+GL+kz23tCc0chzza0GkWLFMq7FY3OZrS/2DvzJIjN9ItvZXaAGRwx2zWLx1zcA7OzBcYk2RiBhxw
+zHu6q+iN9YeQVJVSXfVtvddjGpNkMAKA/8M53+HB/Y7JdHzMirl+oIYKrljO5fe2SYN8FgoT3etf
+m20ffQK5o9D2U1k/aIcJbT/ihVkZPleL6TKFZgSbXAK/ow9OOhRWNgdlt0nH2A7f/r7B4FZ9lQ9t
+8/XVXr+r/7WgPj4qhYU9ituz4v1f/7rtv5q2a77+wX/U/8Bj9PneJlX55+/5w48g/fQ3esjCyfjD
+P7ao+tvp1GFfvf/SXf7rr0NBvPzP/98v/uPr/FMeJwV54/2zSMoNevl/MxmYloN/8a9NBg9fTZSo
+PzgloXMs3/O7U9L9xQpIWAgc03GFI5fkrn8hOyQuAgI/LOH7ZHHAkv7dYhD84iyuPlyMOPtAHHtY
+HTTFyILsEOIXIBJSmgA7nMWF8LcsBguQ4w82QouXZQsEbT4/CxYmX/8J2EFZicRk7Fl7ZgWE1iZ7
+A5Hz6+Xyl77I/+l38Pb8/DvsNkBdSVDMKkyYXVFmx1tYauH/wFCGMPLf/C3Q+z3+DI+ZkIOd4+ff
+Q0ZG6BH8gNs8y0uxYQNTcdS6pfFZVn7xrWsUqNSEuETWxYm7EMwG3ezzUbYc5lGMXiSMGakc2r4o
+sDpMMiY/wSUInhtpSldOk2c/AurQiXTstJ62oyvM+6HsLR9nc5177PXYl0THCGDGDHyiruqrARRA
+wWOL1oyKHCeG2BuYsMnM82uzXDNnz148pAQEgosGx+bkdDpgfWniFOS1ILwGe1936zA08myFupjH
+fxM7Vn4QiPAYl7teiu7LqpEYE1Bqfyi6CKjbXqkw0hMZ/8g2UiH8o2hncBB4qDgYJaFQqNxasK9M
+PR+2CjCnZmDvnZpzU65aFoj1uvBE16ynyDZeIB/gCgcv2dcHuGTlzAAbnwjqxQJyGgIyND6dwfZh
+1VXARzdBgNrv2Cfp8FoFwBTWNaGtD2YZpUfpjG2+SoI5uCYy1q3XA0uWfpU2fnHsVdaaq8LS1rNQ
+Cibr7PhutS173Rebif783WWK7FrB9MJiAfgdc+tkWI3VOxzO9lGAV6H4q82RHa0x53uArzHWxdJt
+kOmzqjC3MHWIhaf78m02y0Z84/DL8/VAfPyTPbUD2EOTnmYuJodE4GkabuKujoYry9eFA6Q56eId
+UursOfGLtlrHyoue2ykhn15MDT4Uv7CtlxHgYLYavQQTCrDg59CCwLnhkJDDhnSO6gotOOsZaGHz
+hdWGxotiv871OmpmyOCfgg+r6ZEv66LNUxIW8/lkD3PGyTlQILCPLJx4TbGEWcQSFBAcalbwoBld
+vkcd84K1GIXFrqHr7R+zS8G/rpSAD0rgHcqJFICqD/pRk2+hO4bHbVu08ZVjIkEKzQocomha/zQ4
+voadKhJKcU/GDUiDObIvQ9B7zFLn1k/XY2d0H+QyM6f7z/ny354vpEzwwP3r8+V/M2//Yy45GbrL
+t/zuYCNG3COxBK85igj4TT852Gy+5NJG2SaRGYtP/J/Hi/2LDfHJgdMkXNxq0v/5dPkFpPU5J9V2
+XXK28MT9DQMbHICfThdOvOUEw4UPu5hDDs/6H5/IC+o5lREuhjbqWoDprGszFMQEJLAIaDh1ZFmK
+aTMDKmelbwyy//VK+sujR/Cn/OkVMLHxBb+ds1cIubzCn843ZXhhl7X2SC4UyyNYvfUQHqasMb5Z
+fhG+xo6W8SZhrPzqYBJJaUk03s8MLigdlzUwKpmkY+4bHsXlMU2rXi+zx/D7T5/q3b/b+f94Qi7v
+E0AE+wwscMj9cP/0Ks2kzBowqSOqObO8b1FUPbLxS/f/798C0OsP7wa+P/ISUB7iZKNIwbq4vFs/
+vRtREumsj6hiI92E+co7c44r7bkfKYSolZYjdBH7jEP2Q1892MEw3rYLLdn3dYYt7QxRTpGXTVtD
+G8CVjQYWzq3KpgA4wBnAHI2EoF/B0hnEXRhMsX2d+NEoH+yKfRCDFGPCUTQFaXeMRGXNqJpw+1+4
+ePvmZx5vs9yJzq1ePPjkFqdPBk7LzmKLkrkBRBkR0IiH5Cx9qkzVuCfOD3ROfmrU5eUYtEa/a5Js
+xqyikU3v/JoB684cszzYgIdVDTs+yQbKtkq+yi6iGG6nFCf3msVnnt31Z9q19kuPxK12Hs1YEVqN
+u+xC+4S+PJdlPnq0NmT8rSkQwoNrE8TyEmsbKQSbl3bcuPBcksNC+C9fFdvW+RhleMDZ19nECCRa
+BhzEoPDTtcpVXO0NNArNmslXmBy13WGXGkSbXXPBQmryld9jukMvTr2C7gG3faTla5FGEIUN3PzR
+KsWixvzC54DfOOwuX4O5iNttmgeMwZhkTvI6cirGuFoXs1w33uze1GCKX5IxQwMK7rVFfDJHPvqi
+qdXcmikzRxgAA1busQkwlhVNL/RONoPZPJeUQMGRZljCtciY7axrOzXVc+SyHLnpsDhSy7DTeHTb
+Jre3kDON4IB83nSPzPJ95ziExShWbeeq6Vsxl23xyNWvhk3p+/6TaixZHXXI7nxNAIfVbS1smZ9O
+a6kLOLD0OpxeYNd9v8+5TwMR1NeJwdJtRS+6iNFxXuD+KuHyIEe27eSu8LTb4P4aE4hEqaCiyryS
+hIZKYHpnIs6Qn6snBVtq2w7yqFCYzJIyCI7PYyTs4jkcjOIzKlWKeQCicYYIVdtPLuMzFmyImpm8
+QUKTVywkEbTrbvbvQ1HFr6l03A+zqM3mOMaKstQth/FgWnNs3AxwlDro2HH9Ss3SDyvN2vpNo9y8
+z6cq/XQTpy0OCq3iSQ2DeyLHLmrXid83LBNFwxBbaPfCZCs3PlhCTtwSOgsVALEsMPcDIyuwH15o
+j2urChrnMEPr5SOlikHl5DU/+mlmr99MLNAX9jLMOYXXHumUjVaZ4qmCmIwk6kagKFjKztF5x11l
+cI+nHEjsI2RtbyEcDIc0pX7YNhiLdq4/CXtnU+bt2zYiilgRqWWu1Tihb2cME8zrvs2qTSNt2e0H
+/po3YEVAhOtwmvXayXo+wGTKiRvvjRknxdRA/TwCePYm5FU+9jytQuzKzLyHfpNMhh4vgCUxKU/T
+0jtkBcOR9VAMvmCX5QQhlQy/CuWupO0uAaba60Ygn9tYo+QSBPkQo1yd5TI7AZxMuIp+AjMdPTn4
+/H/ExFFC9SJTeT0niBx2AbypJ69yXnPcJt8zs0ELl+Qu0i8PP98mMhYmdhVpQHNsYGBle2pMbujq
+Um9DBtA87EPrV7K2ZtI1iBpqV9M6mO+GBcSdALO1V8WC50YVAak7b0k9QUu/ELy7M81bRw6dQpvr
+KNplZ+J3HC30bzTc3rM4M8G9pGgukZhACg+QvpbgDiQEcedME3empPpgytN+UiguOL14zC6sBUFu
+9HPy5p+55CPbgY+gH4YPRJGnEPafXulfOeY5Et4mMAqMzh5bo0DVL5Vpkm2+oM8Djpw3mX+oMBru
+KeXjD69Baz0QK7XvBNR0/F/t59Q01rCqz1j10qyMZ7mw1rO+jcGuQxpBHwPn/W1YuOxBNNsFlmxo
+7d0Z3J6FHXBia+G5l1Oc59s4jab3uNBX7pn6jpZCPKCtir+3QcNkCvLCU3KmxPtJh1TZn2X1qhLJ
++gbEWH3TcnMCrzpD5qdfgfNn+PzgLyB6d2HSu6kET+/jgwVVD6UYK4LXIAtXcTB4PICi/G5OEiD3
+5Rl4byVW+ZDBkwODvxDxozMcPx+8/JngD+wf3RmfbwQLSp+/FP9bYKlP64zaHxfqPv04AH73DOMX
+ZzB/7msHZ8TC66/O6P7yjPEvFqL/eIb7d8YY3GYgNJ219Bb8Px7dicA8DWOeJmqJCLCWtACa38jF
+rdFzU9MZMJ5WkdQK6OISNNDMcfPVFSb9o7MkEeCAU5g6lnyCMk3Su87EsbaNzgEGaHj7F9dnh7dK
+/Q6xruFaSPGKNI5O4TkEIfAUhoIJy355xda6pjlqPUrBKh/T03SOUpjgSEHNXQIW/tNA/FUDYf1U
+BC4jsN9GW79BZZP37v/81x8QGDQQfMvvDYT5i+XRIDD+gS1KXDIV42/zKfvMjRVeIEiJNYVYeovf
+51MSOgZTKSZUHrIfItx+Gk+Zv/DDTCdggEqEHujnv9NAEFX4x5LVDgQcCgmiw7OWnGr3T5wrrRoD
+azAPxiiH6nKcbTT3sy7iaqNkax5+rQez0bGfioCCZhXaaiIGOfNYyRpT6D61lq3FKiWxgLBRvzby
+nQGl9NZzHYc8EGOIPsFVQIspwqgU67x1QnuHcFd+GSUChUNCL414in7XWE+Wo0/CD91o05cZyGsL
+BKfYJ3NoMpWmdv1Roun7wvs6Py4aRSBjTBKYxvhOfK+kSeS04cNhAv8JluJARAEDB5n6bX3omBZj
+lJA+7PrJM78LJ028taEq+6aQLZgcakq+3TMdQ68qKtYPBAfBZ+t5qoN/XlErz9oIHlWp2/nRxDNG
+nZNH0j90MzEyhCNH5StjUHtaYbZw84u498hRnpHHO9tC2O50KWXOIzJqFUknZpzNGJF5Rm5aJ3a/
+jHmIv/Wu34bbUfiUngP4omyNzzmBYZnMzcvkqy7cWkZT82iBrGiv46p1niwvLO+sqeryw+C4s42N
+WzGg1oMc79t2aMSm5NFerPAO+XINXiD7SiGaPjgDdJa1b2gWXKFpeAuPJ6POr3CFvTRDz7ZC+ylM
+zNCOo3RTcp3mHPrkaqzU2Du3CKeAiCRD2H7mRYoxCz5GRoQWEsXHOLFNALUioiIk60wKTNsGirai
+dqzb1EXKt05UKLlc3IwddDPW0WeVYVtctUUyhZuk7IGfKDk3r9qqe3XlJtjOD0ipMDrbhs1UHlgQ
+Vv8coss9VRHjPqt2QVs5OGdvGhR70Q2I4VTv6bI6KFeMkQ641PyTtFX+YQaD9QluAYbsKOLwW9Cj
+1twYZdK9p4aPWb3RVd6tDREmDw56HZjrKSIk5pm1PIlKIzTyG/drxJpW7nykNlgvoxpQhOsqFMWC
+mrKfs9va6goEr3P8hCQRNCyZR9nHTKYsYid0yyhW9Os4pNgs2YN5Ykd0hniapiW+N8yS4WFgHY2w
+c1b5FRNUtl5VhhFfD0ww7ylwPHngOsCQ7Q8NYYvgbYC3xJKPaNUlAaKQwiS0YGUWTjNu48KPkdBN
+smr3BdN02A3liIuzJEbpljV33V2XhTNJ5Ek6Rlk5yYFQnhiTK3v3fjz0yVR61z5bkcqxsguaC8E1
+1TN0BDYRE5hVZQvWzIv0u9vH7e0C4+i27MmLUyUWH07km9atbbfjcIiSFjlKlsghO/QWF+rGaObF
+35urZUoRjRgRZr+uhl1ehFi267IcNhHWJL3PRgJGVoY1gqOwW/9tYH27yfUwvKG1auZrop7Mft3N
+TXYaoZBUh5obhedD4SiU1obJLjRNG7TAhW0+A1GL8EeDzOsvm6jpgS9XtvXuGsLGyuQHwzFgChtA
+x6ysR7ptUnEr9nF3ExIhqNJdzkdiioGeE9ElAFQPudSVIzsitsYRFMPKrYP6RRoCXx1NdZfuShAa
+ggGqw348VbRiKwel/Q+MXHBOFCjSbBWPkW1vHU+HL44fs3TFp8hzLgU1ptGKebrbohCfsZXWwjFP
+mT+42VEhw6sONhLaa4RO9Yzgb+K/V67fPRsZZfx2arPo2gZg6myrpiyu7STP021ZzsVTqxKag4bh
+wrh3aTvRKDoMKace5rbBEFrSIebza5r31re8yYtFlhLmHzGo0WHrtT2D9EbF01XMfNba2boWb5Vw
+gR3IINPPtt153Lq9as11LC2w4mk1yrcpj8JLjXzhERNd+pAuefPk9ZH+RWkUdnpdGl1xSV5d3K1n
+0k2BEJbeeIoQbJjrLjW6azBzSr0mRh5fV/4A9Cs1UZnvtZ1SCfU4fb65KQfCdg4aFsxUnR09Tmzp
+QwsvwQP5MowPTs9NA0SRLC2QZh6mB4mp4J6RG4l1RMDo5qEbTHvvSD5m4AUutwYCFFYT5KHXn5XH
+htFhIwi7qYqru8jHB75NwMS3Gwk9Mt8sIy5iFvAGX6NiCKFidzMhHbzy9rXt6SK4Lzz5baKd91YU
+p+LR9MP8znORlG0wZUWADebGuzXFeGGUMyJkEv2gIk9DAQ3J6YulC/cQ5dPfmuK1cwv/ZRAFVHJS
+BkhGRT8EXmAAGn8XITpttqDeu4u+6Jh2VPHy2CZ5trbxWE6wBJCJj/6WsCV0z/1Ml7HqHR4fAEoq
+543rP8gv0iHUJwJnJhM3N57ETZ+EsBhZlSI6ZThTrp1als1e1DqN172tmZPPmj5l3cZiQLhOkNmG
+yMWiAUk4cgMhmXK+gpwx4Va5o52vWQ/gcWe0hGcLedlbhiYpo/+k+l9VNU6OnezyiqV+POCvhu3T
+MTXw7BcLyTOIAdfhk5qmeLF9+2GNEh8WKejGkGworG3QtD24cwKXzeBlkCEH1PlsZ4RAqlMgtG+Y
+N7R4mnqE6cTKzY/VMHFwBgCqfYjbhnrmY3RJs2M08pIaTetDLciwC42Z6X7ZniZxwouxBKfVNx79
+NUeDnXQfTVD2Hg+VXD8iV+2KdS0tVkDRHAwm5g6EOpusk/UlYq8UBVbv2NEOvAjDnyQIg0fB8nuE
+ceGQMkMql2muo0jPN4Gyq5Y226i/cYaTLGk7wj8lkAvqbTYvhVAXFYGxQbeZcIaj9HiZB5tnDaOz
+qdt6Ze+0aLobzrYpHjEcVaR9kHFZZfBBrDE33qqJCdi6WvJL4THAqMBHH2l4xVqh0Aly0rk2vVPA
+PvNHrEMrR8PYYtkUdwAR3GV2A54/vTODqNlFLk/4TT8ikthxv+hhyytP61Xq9DxkegXwhkDPUHzo
+kLBLjtgMUALEauoCy2vblzg29Gsfo9TIS7dFzOt05qMWLN7WLmRmtUjduptR5lPJn5ORKY3np70k
+oZ1plONE5tHwu/ZUCJSqmzHV5n0UDxVLJoPgvE0j6gwVga15RErpDSeFXwquJipe/9JtVNCutV+B
+Wqc8o57yZVZ9d2aPwnQiwgXsQOkq0plkNbfgnUV/QsczGGtFXRttvBBVKmM1QlSm2sCFk5uI0zaY
+fsROhqMdrIUcYoTw7iyxNVcCsU3SK2c9RwluedMt3RtGNTR6Iw98jheVXrCDXfBeAeK4VSFF/m02
+eNhSWU3gtoHrY5kfctZPquCJtAIban6fDE9gSp+a6AE9NG1ojcXuXjOliraZYefEVTHAg+Bo5/NC
+NE3FjrgmJlZB70fepa+n4crMc6Bruq7kHvOGhb0cry5uD+kwJGsrf0b9bi2XS8IM98PikfJe9H1v
+7y1hdgbhOIu8i0lOyWUSFtlnWaTo3rhhXY9U2a6+hhJReIdmpvFeNT0GsTCkEsUGUypvKz2X53g8
+Y21aY9Sw92OXsOmOHcfD4S10CzakMymO09ipj1lUp2SjgSY8Gk0/NNvZHHlExbL2v/qk7cwd0lKn
+WLejNN9ML8PYU2WRT+ij38bfYh/W6c6h3M13wggL5oO4AeUek3NE2FPSQQv1ELjiuISg8j3Wufih
+XUmN7+Kvh9lLhRkCzAQ1QmRAiNPJD8nlZHHZ1xLeV6C+yIpKBghHjGo3GeByCEV+15EFocruu5f5
+NEKdYWYaOqEovjuNtdh+CNx9qso0mvlJg2czuGi4/mK7sHglHQPGC8Gl18BJATBB4GJdXrA2heMA
+Zsa/cXOkbMtDZORKQKrLzWXEDT+WR06zl1Hruauq8hfbH4m1nIhJ7VonNgYTH2bfGjsn7Mq9raWJ
+ZSlp091/Jgt/NVlgS/XXq8n7qmFc9P7n0QLf89towfF/IUKeCYFH/44qI6Bz/2204LKblJ6Ee8jE
+wWHn/s/JgvOLBGrt4dliZY3CZWn3/yl8+YUI2eUnCtpXOyCh/u9MFsSv265/aV8cuJ8sTYW08Yuw
+CvX+bRs2pkq7WOmgSCWQiLJW2k8oNZEGNq7fbJifowvVgZm+p572fiCfpnQb+y+3HnduxZC5rSx6
++S4K104/+6C+65DAhUSGlNy1KS6zhmTATimEARSVzTWNfI4obxSMeWWenDTq/xOhNUx5/TkmyIE4
+3VPHybOj3U62RTbZuEwdOhdOyeQoaJUZWRovgRdDGsCC9mDrAoRLp3X1nkcxJJauwT0WMgJ9C+Mg
+A0XtlA+uYFkfk9MarloVmTzRnRJ7qkQZDlljyAD8KK+/sMx4uhiLsX6zSIi5lvjWbpsIQJFolwgb
+3PFWCzOjiOEm1Tq5LkKZXRa44tNNJ7vgqBgsv3DHuVdGG5KtayC7ZVszhB/RYFWP9ZzTUBBqi/xD
+NiPcO6Rkx6lxUbYHYmZJ1wY/4hSDeFa59jHHpbeSWL192C/JfJtBsdtZGCPQMUzZwkFLnOnZwLXF
+1/tkj1ohoSShjI/Qc28Tx4cFypItpi3NYeeZM6QN3XOURd6SV552+b7ECvkNzmG9tgicOwS18QZB
+XV97RamOhaUAO1gtYj1buRC4wsx4Yxlcb/oKfgdmjn6dZlgyM3+cPgZGPM+uOeTLz3tpK+erSF2m
+TFlskAtoZMaDb5j6g95TLTIoCrQgooEzJPVhyopGrKrOiS5VmQ33MwXkLsTUw4sOd6TO5isnN7o9
+Yd8WpIJEbfHM2lvT12NFhwbqr29K/wVvWrcpKse7oLqLH62kdS9KyrCdNnO8SAHh1m8zKVJgJEPz
+qhGts2/LGDskN+J2nLvgPkxHd82sjceyEUQlZ5U188lneTbsHS9PDiKG6knu9m1lFMnJCdMZa8GU
+PLEta/dYK4vvIo6dHUkh7ik3Ynwn6VgBO2fG+6GVVZ56l91rjqljV1d+dBXVRgwZcYmnpQE7kPj7
+SkxAugbm5A/YIeUA8wyv5pzQI0Eey65rUkXXKlMusvDYeVOy6r8nOYE8YiztW7YeDH2w2mP6y7l5
+sRZnd6x9ynGN1x4bfDU2m3Bu433Rjs2zFSt975gw1zliKTCwSxrT9UCBEzHm1u2P1BhURWaiqy15
+6ol4lureta3+bjAGRLJ+AYaDnSluea3GxyGG1b7KOoubU83xy1D1w5fZtvZT3kzRbZnRW6Cpt95M
+kwWieZZ/o1s6mgZciEg7Fs1FBcEkKk0IP5mkvKxGEBROyPifGrTZms1i9180vpgHYTygMH/R6Dxv
+Bg/fftSgBR6VUZ4o5tX+zDVQwhovTXZ3mzoyQRUZPE/Ae9jjNsgn/73TC9lIDt2uAilyiofBe+xr
+TYyzmYA90ZVSWyY3n6Y9MiQB4jo+auRkJ+KFsYrVsEFwveAi47uHL0S0aIYXcETTQ281xjJ/rwxm
+JgzxGCKNWm86VsjPtmYIN9MuRquwTSaYkxVwjzD9mMA1AYtCFH2yCnCdtbbCazgWPVG19Ij0hBBB
+NwgDc5wcS+5KiF2CamtOqRdtse/xar2VanbvTIxML7kwzXuuK+OJIGtK9Ua23/PGj3Zd1sePMTKJ
+lwah3AlTYOYBuBPlkVYLubqZNwC//HN/Mjo7QrO8K1Uxi1xJBgTMUAlVSV4muCFOpatDie6TNMvA
+PeosJw99nLMt5ral+UTRvEL+1Ry8fqSJRw7ToSgL2tuWFPVvFnXcKgB8CyGD8KcuxRXULsMy+kbW
+tSYjsAZR3HwHGosZtA+uAK1XE2J9Es2TNBqFe9eYLmvc5JA8wrbdGMgFoQqqgt4tLR59OibQXCHK
+iZQcsysiX+ETlbNxrexZULg3WDbijLybMnXWjT1CwembANMK3OOC6f4Ou0t/aSufbaqdDa95DVGw
+cmdzRyT0fJW0QXvTj3wx0UWyq8DKPBZsiNZBrmhlmk7u+fxqIqI8dZNaOfAp5rXMeJLwAlv4fKgS
+stoZ1EcpWCSyX7thrq/ytHng//J4VdWl6+cKLaQCS10vH0nmRebeQuH/aXEiX8xeZ3zDBxz80PWS
+0ilZ0F7O+AXWSdH6V1aMNg9/D7bMKr/tBzf/kXbo1xVt22M1hebLDNmDLKD0dor0kTIWElZB3XKn
+RJW9E0UrNsJFOahF5R3zQXYHcAkBtNyets703csZJBtK8sjGhT1Hn6xVnTu2XepawIzcqlqy/dSW
+sZ89+wqLR0z30i88Tf0eQssFD42uEw5VdZMFMwnMjLQOiWdIwABKXDYgedaenwWYJ5P02Ju93hSg
+XLgqpuh7nmKy9SdGOAWxOMegdZodEZv1jlWh/Zrx/nwqTI/Xfi+iRwUf7IZSIMSvYJ6MegYxy9sS
+Gn23LawUjRO57Uevt9x9gr59Y3kzlGxRNtyLnHJxKSKLOR+hkDsQSZgNC4qm5VSx541V+AbnuVvt
+SENAtBIb1m4SYjZpxHLYsh7IR0+MA7atiumJj3HBB+W0ljVAjF7RKa/nXHkHItySk9X39SVDTnfr
+9IItDpqBS7/U/rc6bdnHSB0+JIkbrFmILuFVEAZCAa5UdphBp5igajkN2WUUq7fcZ5Mcm404aL8b
+tuWgnFOOCgmYVpXeDaqbsKvlxaExRbzl75svAqc21yQYjhcN0UPc62CVTyxQTPKXrWog32DuUSKF
+5fCK1Le8SXie43map4tIONkR1Wb30mvDvBNT5N4CPhq+G3PhbkLbsu+j3u23A1y3de/OmykqC6xq
+XbSnbY+vrWx4VuFElmc22leGzEtGZ4Gtjk2X2zsxFXgIyABBFoPNpX+cRWI9dk09kokWJ+qyim1m
+WG6LDCYxLiZGnesYEtZd7snWvSJG2jq4EvsgItT2cnS/Oee2a2SOUo5mLtcSTyK8CRJUCVQOy0vm
+WymONIk0RJEEuHdJdmB1ZIsC+u/MoWQMLfCHKvSbq1IK49hrDk2DauljHGw8ymTQpFtG6R05bJD2
+j3iBZ1TmeQNYbmrr+EoFjfc+JmNCFlg373xmg98dHdh7EfvfJlr5w9xW82nuQWJTASY3wm2/m25n
+HSxg75wIbvfk1hGc+kaOP8zW4AlgO6qDCgbfoKnn/qKQZQHzyh5fsDbqpzFmDr6udQQsRBQSbmDO
+4hol/viYaEvvRgFSDep7dZmIehm8EGT4xdzMOqF7g35BOnf+kjhNvAkss3xppQi3E2KTBVbfMJxp
+iJzWxI3sIkZG+yIb3Ose/dlS9kOzjHu64AhIw9uclVAlKCGgjA8SKGHqhFAP4rgWz7Yf66OYe2vH
+Nr8EpObnV32ow0uXILcbFmjhe9CCNm9JDvnMDSmPSZcNDHBKY9E4qnCDhF1eBbi/AQDD8aioh1j3
+gUK1LihAUKgIgfHW6cruxp+Z1HWzhGcbQ0L0FKgndMX6rkDnsDOGPEh4I0VwNZIZba5qq5+vMqm6
+zYzq92lckOzzkFgfLnPenWNM7Uffsq3cne2njIjNfSq6ieFCC0iMaRn4Gu4pctCTH1NoyEcLLlQQ
+5peGKq2bYHjsSU1jrYQRHuL8NpDNJVcOMhDZmEeah6RYsYiR28iyEPOZrpUw7RbBR59p6/swMMlH
+1qyqb1PZ8DRrsGyJ0CF7DZ/hXTbn2Q4RnHFw4rB4kKk0f0h6FyDLvntS1N1Ht2ZPHAHE5ySoXurc
+v6bA2aU5nnkanjm47aQMoYXr4mChdthzd5Tb1A+YqjFmvSASvvueK27qsTX1SzgUaHQCcKPJxCmC
+cJFBZ2hMxTH3HG/aLJk5KzFOi3l5dHICFbvphOrE2rc8XRiUZMD4jUge9QxGY/JybG0Wd94dzi39
+o2JedGklXXrodTiAT7e2ZpI+S5YdcZZv3S5noA2/kLMWruHTFIR3oV/eVfSLW3Ll7sOOHFRHFvdT
+CdVzCq7k5D1gK9w4fnifJ8aX6xkPEsxq6oU3eWa466xmbAkoqAFP6i0Av8QyeFLW7BkHZrVmYjm3
+Rd32C8DEUEc15h2g7LLZKOLj10HQITqsmOYIYHCPRiz0JYDD6jbui+xCOUW0hwGs7xLWwPt+CIP7
+Cs/dTmS+tWdyGzxlLql6LcvSehwQfYWmfxMSN3/svOkqLdTIOhTfwI3tNc5FyAL1MnLSLbtJdUwA
+t1AKiugH+HaHO1I6VNRW/BwtRgSyC9YKtajyJ45pDnuX44LlrEpPcYFvKGai2HTOTYuXollRGksT
+yr12MBvEPus6BHvARYILG2bW1iY7677och/lTUd72ISWfek5AVvZwq33sY+edNPrqechNSXmE/4I
+S224A8Znsh5qZtpelr7xFiAscyfzDtzCgnYmJyfe1n2kUR0k896YECE51hw9MCTzUq4+OwVpSokX
+Fpq5njZ7BK9Fccpj+SNNl5wzBBTxKUgc973MG0z4xagvzbkXu4QggdPMsNnb+c5ss5fJcypNZwqe
+5zouNkNQDh1tVFnfMPGEDUfG43OAYWAhFGfGD4bISCckJ+4O3iRcnq7P7xxAX8/FYFFmuU5CYALt
+zmXU18YVThe56fQQHZJALVmvLYQeQrriTay9ae/NSblmyeoTBsBWkU4dzClZiOIqmdIZcn9mXJkZ
+VtaunMSekK2JJC+WDBxi0ZRlTIdHYKnahdHUz8PWbWGCrKF/+RdETnhXaegLWtqmvIoBv09rpJ4R
+DtuBDGKvB+qPkAA2vGu1Jx2Q80mjGEZ7cGkcNso3iHQok+HWtAZ3q5o4OSAXXkAQ2fI7gC1aPFl6
+tYU2EMHLCzW5sEGDDBMEHFRtvYhu4U8zmc/HEeIAcuuiycdDR7IYeKBSNCDwUXiEde+CSERAtpFF
+hJRF9c781Q7c6k0t87sY3gGv3OH0HwEpp5abYhs1jUdZJ+W+/L/snUlu5MqapVfEC2Nr5NTpfaPO
+pVAzIaRQBPvO2BjJdeUOamP1eTzczHoPhQTeMIEE7iAuIlxyuUij2X/O+U6adl9eHNmnogHM04z1
+/IOdlX8ccWecOoiqh3Gqlyt1pNVhHpxulxQtXWfM4C4knZIv3WB5xiJiMes1Ylj5kENlGXoBZ/m+
+BEsjauK0DJpUu6ei1b9GzIJWWAj1NTWLcpcQO70OpRVsSsfvNaygvDxxwq8O7WwEu9oFEEiAE5oF
+01pQr1j5Dpgqfrdiwem5dJysXJq8JgohhsC2nyuJ0mhhxniNMKM9wN0Vv7VU1lFlstx4sW0wn6C0
+a58lyn0ohTtubPBEl4KNzyFIyvI3XbHBYxNpFhzHN9+MKImQPCuXfd4AlHLlGnXwe6ZJqN4MJTH5
+2VgMdM+YCs66tIaHRbriHkYt6hEBB3Veart8qJxuuvfwBrKlNbz+HUK2gOe3cHM1nKkOJcUZTxlG
++qe4naYrLXfD3s1c88INoU7K94pzMGQuPJYWMzjbtTDR5vgaW6TIOZQs5y4p+29Rj8kHqPn5VPvA
+LzLdCE5m9riX9WAehOCQ7RNd+ha0XT2ooSm/mmQojzXcy21eYhg2yjE6yFQzpAIyeSScZB9mLyv3
+BQL302QT04UElcg9LofhUvhsKFeONbe/rEa3206N6IUgd5N9bfdo+mVLXSsoQ3ehIUDWNLNBqT6T
+Tqk+DK8qr6Lo1HNu0dwRFXWwsVIb8bKfs4s7OfZlMuR4daWj32bSr48icZID5vzk0fCVfRqsHLt7
+Wd/6/LQdvNkG8FpT4MIc6OmY/dg/DGVWXHyzHPa2N4pjkeYOn1g9hmxhoydUf47ViAX0FKRop2qS
+KMy97nuOmzkkfdhAK2VYvJGpHncyQgpbjYEwfrqLFRNYWECpyKV6SZO2hZ8EhcOMlPmNS3h8qqih
+2LtpY+7cnMSbF3nZ2eKeblfe3FWoEAbTSUPfMmd27jww65Rrfy5utIxGbYdM7tyW6Uf/kkZGcPWw
+fz+hBEfPHEzFdp7q9B0OCbmCaig3A5LGdYGEtWKnqjcJ0s6WPoXxzouH3xnTpmsrqehdwTJILtDE
+F/Izifmmemnx/COmVlYUV0++8DdUVXtrr48j5tjOklOogSqD0i63mWPE2SqFNHwinSZ2GIGzt+hG
+G7VZ0uFKUxHulRC2g8mXTKj0de5jEfZ2n/BVUKkoQ8IBUXMgfqDpMbkMKQ/A8jYfHGrbuu+82Pzh
+2914nwByfgviiXydX1j7qev9eyaFqb33PW92VxyiqbyNVQq23WXgZ4qcTqIgqhl1sSdifxQ3o12i
+8t+cpGyaacV12J66hqmokSjymaY3zGdvnSPgcfS2BdhRDVOZbRu8Tg8RtdVcRZNrQoDXKbtktAdG
+gaK03qUfkw5RVQ+7qIV0Bpe8VvssYFwluLQ3mpCf9zZQkpHRBA4UBqx85tPRlJC7A9GUMq0DPWO/
+ZyYzOSSQ9MSTFkxu3zEUy+tbz4gSKnmUJkOzysN2z8oCqOQCWBCV1ojHetzTt0B3htIqoRujAala
+z9P0tVgOgwVl2O0dWwZQAQ4+u5BtLdM+lTB9rBBsa5rph+lLFrgiVXSDGP8phbcTjt3MNJPF35PM
+Ih7SKby/6NBDGpo8S9mPQm9CxVymZW9rgDxsUCc8YCmkgj/8AO4p/SsGtL26bS1Y7/H6Ah3FPXQc
+oxt5IDc9VHDtMLY0BpOM+m2UOf7h/cJFZmRrBvsgB4iKRl74G85x1drx2+SVW4kfsW+qY29M00bi
+PnliC8L8xKKKy6Z0nODqEDzE5G2OrLvDU7dwBjRgMc2t39zRVmjCGjWK52qws0s82Pd0eTyiopJ8
+zAX2tYCU4krUrtq3rENHp0ryM67C+IwtrTp5kfEB5YaTomFy/KQzjZUy9lz6szoRfylJFsVsPePR
+7cx+nXrem5+coS28+AExAjbJ1a+0j9KdYZG8HZxA7qFU9YQrRve1I+qE1SeS5ZaKwGgrqVzjRN+Y
+4eRH18HmgB7bPDDdnK5yPqZl76tbYfosy48RZOu5bEe5thRs9EAHMYTFqNvOcZlznqGT3ldg5dM4
+0hAO4GSsUiKZa5dN31EWc/YpFaNoxUbt08RU91aadvpjmSBUVMaYvNITG0WbYb4pswMGhyqcPLoj
+UbQSS7ObYrZGyqa+i7nmLoDt6K33gvLC8pPfBQPPfarb3TTZtjhEr9TETw8q7rpdmSH6MiGho4q7
+hRsHaPi3IoDmhaPdFE8z9BqQEcK7XxobMAXTs5ozT6fc6fzva7OX9Kdi5vq7/1e8wD8BCv7nIgnY
+81jBTan875TZ6vv//EeV/pM2+5+v+1udDf6S0vYkvc6cP/gjwu3f6qz3F/5tPN9/Iwv4q7+N3/Iv
+CpXJveDt9jzG0+4/dx/ydzdXOCMTiRPZ/Lf0WfTgf7Z+o/ViJPc8QosW/9nBv6Qi/R5Za7Gt/AaI
++WYTWx+WuFcbJg7Ep0c5mVg5aLbfe0tzcgooTeVo+jhpqJ6tzMB8z91yPNfjrQS4kBNdUU4yHuIq
+cY9CdcVOTu03jq7Bx2Z1CIqp3OUkLApNexdxrXI3R8Onu8R3MQaTXv5oIOhn5fjged2hLmk6YJc4
+4its9bzpJv27s4NXsZhUAEQEiubs7DbJz0nuB5/qAyYQTt3sh959tIthoxI/pASB0dqdqa231E83
+bpvv2tw/Ln7zs5/pAIiGS9ISzTDmDZj0B2uaKCgaZIYjCprlwtSVinpA2sVaOV9YOZi1mGsXuVTB
+2Vz1TbfLlmrTm1SMZtEhtbCVkuQMPvEqjVir2DejZ+2G9qcVLz+yTtGBklhvhuWah7ZfXklYFttU
+tUyuxt1YE28a4xGsmqMOcq7y3UgEVHTyPCXq6A7JdWrthzKlHaAsrKs0qC/25Iz9KQttNhocSQ6p
+vrApxcU3bgz7znWGLeaWg7LKNRI5FUwvc4k5Z05H44wnct069a6H/iTNsMorpsLRO01doMLTtdeM
+nG2G8aXUsguzCBSZaQMzNmm44iE9Mt1mVH/XACxGym8ZO8KOPlQVl0AOrc19r1IgLe1iPhKmnD4Y
+JVETPsy4nd0zYfeFjb6Z4Z5KiEDBo0vAc63a2P00hcfgxoWKiOru7drJcknPuxQo9YXeYg+onuY6
+ffLiresdskrfzHw1wwqOIasElOYZApd+CkbONW0aWQ+WmubXuLPnfTADHZqNmTNgPG0LyTkYN5xJ
+P90UvTdmdIq8wjmMjLxOLPcvjdBvduvrO+V06YFgan4UVZ9RBNM+Y0aCHcq/Rinu1ig1OaC1nG2k
+fc+Su1dIThzQz5aeGAREHZUqdVTc5T2yvpllhzwdu43TmB9LX/1GS+QpXbEBJ2L4Ar3irob5xhmW
+k8GWg1L9DJUvjMT0Q0tEGgxO5bYO/DHM2UMWuLS2ltE4l3iWqwy4HPSmC00nIZ6hldAuDGfN9HvU
+MmS7At6O/GLv3JA9+06zIU/WpN7YEJZd/+Dl+a9aF6+1j7GUkOzMpKq/mzOUnIZCF1K/0v6JKXLl
+gspMRXchRtrtlI65DrWzx4x2ddE7QSqoJ8DVxBx+LXp8V7BVV3aSHpqu3dHgDfzQJV88CGS0TwgT
+PwR9jt+LF3t3iYPbscZOe4mBI9n8ADb6x1JkAxzWfV0/E5lbWe70TfJqFVm3BoA32EJXIH28KZps
+LJoLg+iVF6zmTFJWtECTNyVkEaxRKszY0+ZcANRRPaMWFswcstXS7KMmuHjYark8hhDq3cYaQWuT
+H+RyWVVooave+Vr8/KrdNMeQR15CBW8ezVG8D+E+tsLXu6W20tASFhvBvp1pNJKX2ZhgihNxC92k
+bLYeY5k9Rgf4d4v3wULKwYtpRPSRx8M2od0wLsxDFP3shxEOHfjM1szwmhYbt2+2zkSHQIcRsF2O
+RAX2NmIFveQ58PmYvO+9qd8yte1HJk6iaM7M2eDYZVQ3zMxE9TEq9LlPmaOQ92B+iaThfpVGdYc7
+bzeoYpcygS27iNabYWskREdbcezMFsz0tIbJtIFZW4zwtov4MaXON8xrfRQcdZmEL9d6bC/V9NnK
+/Eyt3J0Z1G9TYTHdW44yZSuf5acKf0oYZZSVpxOnCemmYWKlTxgfWSWk0e1LD3C2sDkTJbrgaO09
+JzW145WJ3VZCk2+qa5kFRxAa65bBAuoBqlX7QOlKHNrWsMkLuc9kQpR4Zlc0Z2wgMSirxDsgc71Y
+sX+llT7MA6+5BC2FYhXZA1i0tRe6iJWcSrliS6mzPa0Pj33pPahS7Nquf6HhJrsH5nrGs4uA9+ov
+UWga3Wc86V3rLncM95/j2jxGfNIrx52eJSOBlTd2TwK3Hr4bWk07KsTj4PeEyFDmy13hZE84Dloq
+a2gmCHpp7jLjaN7eAZ2bG3wzpACUtcsKoLu8GIdDcqdNAPWW7EQ4AUr0EsiaAioOre5rs2qeR5Cu
+6MlzW0KpHKFf21xw49cyt/2FfewDUaF5LbkhtlblvEJPAX9OBaRpAtd3aIvgtA929tHt0509vKas
+ouGA6/JgK/Uwz8NBMeGIGC6P069AZ0DYaNJhHn7uaepQ+sZDH8QRBeboJdyNWAxPvjDvGb+G2CGz
+MLU1AwjGA8CvH4cOXwJ1X2FqiV9VR8eS27oXrELu3pzd54RAypC794FhDCsJdN30ENxNoY+otsc+
+AHRaJ2XYWM2pb6MfS5Yg3slDjRbcLnIbVS5hC7mfAyfYUB3bnRLgBBuDSPPZN11opb3zZkcIlb7q
+yWRxpnGCkvt02YLa2RRp9Byp5ClbdIvOSRIlthhtgIkRYvqy4u4HLRQPc5R/5FzN9vgrCGC1sWGi
+ZXa+WN3N1Jw2d0LHPTUHERkahQ9+lo655wcrSbrQ3NrREN1Z+r2Qi7qzylbuSAkcfcdc+cSCDoyI
+gx8DHX9YhZ8xJdAZw7j8UlqGDMd6EqxnUtCR16sfDbRIcBAeOqp18XAG6Z4AmjVk9s6pWnkykxik
+OMKiaobXNri1kSU3a2pSyuApq6MLphV32zZ8iFPu+1sud7EBv5yGtfOTu2VZQ6C/A/d5h7pEE4Hk
+11gCG4WV0h0INwSvqZSfHZbXSuPDQsdYicK+lkN+EV5Qf9p55F9cg6MQlKbdZIu1EvYYRkQUWAri
+rUfyZUUNoyDX4JdnLX0j5PT5e+DYVRai2vgKPcSY7ZOx5FdYp6Stowkcafvcl06znwqS66gWo0Wm
+J2AleCaXdFGaCDH1J/043Ik+zk6UEeP9cRDa4px6GvGn58c0bvR6dvChmk37mE4vsZyp8UEBTI0B
+cdaM9Jqqab2lepUCHBcmoOPdGlVSmgNI5evtnxKSP2VAola02vypECcJipgzoVLGvEJktJHkBs0t
+uU0DT37DC+oFJHk+uO1V4Ere5taEEwiE79kfg1uRCy/7849rygeOMclrsIb081ChSGcStgmGC1lj
+v/+jHeZWUPIntHfrPLK9eDNFKZtf8C8hnyI+p5gWlT/flukjXyTiU8izW6+M4uA6d5G9ZtD9S5Pt
+osXm9tVoVZieW3KaA1JmKi9jmlL5OJSPzNJCinyP8ULSLsZwMszBvueYSud3nhBbWmqigkZmn2yb
+8Ag6tXe0LSDkxD1Y3VIUCdNUD8ooXxhj/0DhbrlUMkqlmeFg+IPuECz1h7BqWJBQGGsEjnqOd9qv
+n0RrH/Dti7VQqd76ZkGj66Cuhpff+0ZzJEe7a5zbox7Fck204q4Jsu3iwEl18cstZCmZwbx3unky
+HHckD2LqE0S2dJsv7bwHLALno7aui2M/Flg8NtKYrpnI7mTS3Ptl/Fh0+dljNLmmuT06uVMHNRvu
+4hpu9A1CIYc9Z7YPHK0SiC7doWjS4BMrXEbSi34h59LnmE0XaQbzxo3L4SosPBUFG81dSQvFQZgZ
+8bWlKK+RyL+4khjISVgOWqfuegB2wI4q7i+1ZQ7rxpxJ4jQUnwTulqbrdt2K6LbuxuwMgHqssNRy
+tfiUY49JurNgDy9xdITynK6ZOMsNjan92k1H60xDm7uuBzwlbo8fyP+QmfOVgVMLJxkvYTXU3zhn
+y298qi5U+i66CxDiHsn8LHd+O+iwDCgrgw+/zzHvUhyY0JtdziE3oM1OPkpCoZ3gjnqUiV0DyRpW
+R33feFUGRyJNw4ompnFlWmWwxrgiz7fRXQEVZJ8mc/ZgjqbcGpFZbP9xy7Zz8ZSXPHMISaF49/6t
+NYsq9Ry2zCkWwDPVMHB72M3tfldcy7RyTK+gKth3F5HLvNbrwH4u3LtO5kT3cewyMaSelZcXNCFg
+EoSyueCx2UR0WMzsVrEOOiPEyLrEgfdnhfhTpNC1RnfIF813o12RyVtAX1U8lLT04PeC9EFY+tkh
+7gfOZMK2p+kypyLMtoBAaG7yxVj2neqwN+rZeQHCw7QyrwCJStoYX2RmNceJxNu+Gmlp+OMGHG2+
+oo2v5AhoNnmi85w6n6UBVillBKKSrTauOk1RljNijnQ6fRs6tgwEuU4pShBYiXf/WMpyzWDT6Wjw
+jXN7CEKx3DqSbAaWf5arWA58Kv94i0wyKGGqB/WW13BNM7AP3/CSeU8zcUf8OlxuooBTs+osGy9V
+VwvnZZC90azLdPA/IbHjYUxM50WkrLO0EFlMWXVZFvb2H4th001fmHbssI6DYpdbCRHjP51wQjgN
+OaeYca93+1OUjtHuz8LoqNsMuBj5ermmUYGmmdurRMsKW+MRT2/qNLT4Wo64NsHvHGOII8/URvAK
+nCoJPy5HKcUlz++mulZlWrMdr8X76AcUrzemgTo4IfonfVUKTgRZRNK35N/rtqSOh6eYhWW0gqex
+VQvPCTz6dOp00J9OPKcVPcyDDbEGQOJOUt8OuLpuJGd61i6rCPwHLzF5GCdlYmwm8s9JmPE5nWxK
+r8ngDMZyaaJlubr0rDChIEKyXhhU7pEcE3MlAR+G5ZKLj4UgynEebWNDynM4isWmKseWY7lqolw+
+UmwE42/Mg+LNhcbMMJmTFQFLUes3rNTGD5kQklJzarCu1/p2qF+kPCjbSO8HOgLRYVu7f++Ip9DS
+Q8/V0ZL2Irmls2pPRFwOTwF2w3lXagOglqi7dcw/W5s92cwVPsngl7Rn/WX2c3AcbmVAxFXfGWgs
+D+k4AvDtOBOEgOOnV9xE5HeyTD7pxBJZuCxJslN1Fh+iGJriKkiFfeoxTF6aMpPppsks09349hCt
+pI/ljhBSY+whsmVnREfV8Xuy6P3pHQIEraPcHazh4sc4B2ZouclwMTs02ziJox18sqZfO81QgN8q
+MLt55u35gzMALtXg7gnaTC8mGM+vJYvZf5O8DI6+TMmz90zRAcCPbWJtSSp3R1Mrfc9NP6HaWs2P
+UQygbitrYvw1MVfK4iyu1rhisCcqxrnWXBnHoVM1+Bh2jHeLuyzHmsnTER+D/8A1N1/miVm/yZmf
+HDLJwoWTr6hK9G7B4CNNxY8BxKUGZTlQTUCa3dmMmYoenQGXazyOTK3ogiGXVxYjyK45aL89Z6Kg
+ecx9qgjtpmMnbWYXs8qJVEPRqkj5M/PINvVsGy/8b/wTi5T9RkJJdWuUDPntexQ2Y6Vw/VeoX94z
+l6d3aWVNTDGCH44cJB9LEhJHLcz5OvjBDJVFjM3B1knzGlmV/8MAKfZ9G04yG2xtD4NmYSbYW4mC
+he4SJV9AejlukPGn89lRRfPc4E5SR6gDxmXw09JbpWbXfUVTlZ/nwmRjzEBhY2C3/hptfpMLSKRL
+gXvZ34J3b+2v0Yk4PbCahfairINpO3K7TF6w9WkWuRDTlb+kifV9gpy6CmYInEulRyaSQz6FjvAx
+77uOu6fVJMB2SHZKLE52RPHmCOkLCn9LjW5vNWVJJ7WW4qH14pIAbRWoPUcDZF6ssXeMBVeWx4sp
+jjm7Rfw58rXOXFweUk7UE7bqg53MarwmC2ayM3m1m3SSgclLbTZCs0Re8s30VBuTAt9sGg8RwPtw
+aXx96ky24MLs9aNpWeV+FtpHJ391kdve+OhVWKm6uJSeJEC8xAZ8eyBVm8Ev5DFlBrXHJvllGex1
+YH8DJjPH8gAlCFtCMslHTUVFu8K8RuWubTXnKCEmpzSWzURS+V64Vbd1y2i6LtHM9rW4VUJIv3zp
+TKyuZiuGJzjg7QpHGDPDcibkWgcRE4KYEDs2h/EMHYMe2jr+0jdMnEgtHyWRKpdwpKznLk0cDgKd
+BbwtQjQmLAt+P1QqFuuEBRSSHFOE3pojnlCWQTOXNjC7GtVGiGzat5bu7l1Nde4iq+W7RevZm+RD
+jq7rWDgjB2MNNc64pECDfluxJtQCjr3mBmn0a6uxDd+G0l6DLaO0bkPPxp7jT1hefJwTa5bCEXXv
+4n6xaQQu1aHIzPGEbbTfsyDApy6jwT6NS5A2OwsPCnYDTqcfBeV84OEswtmjrspmhyMr+cryG2Xa
+yjAsVslNz7QbBjyO4VIgQ2h//LX0S3JPYYuswjyiYeV2JTrTkbXE3k/T5DwFOOU+KtOHAyjtJlib
+RRw8G77AYaKCqT5XfumTXOwD/0ApD53QFY0HP7peOr84Jlp0hWNO3zUWRR0T/shjYQFACDGoONNW
+kfdiUmY14tcQJByNWZ3netuz2iLuU2jzgbCdf9ZS3zzYJR+QmnmeUVBCJTJm4+kytq51XNLaeBlr
+JIUBJMKTQ4adqVIJ72idT1l0N/ZRe4eLJd7gqR3JatDBtCH31RUbKGe2E0KZnD7mZNTvcT2XV/IY
+jOq5D68knXj8kUq3fyRAw3K+nnDXs6JPDZNNAIskjiTN9UE7YAJO/c0EZkOFdCEnSOUECh66Yuh9
+Npxz/RHlbk6IXnjxJabD5LH2+gYek+lTXTZjIT5rf/GfaVCPPuivQSbHibW2TNncB9SS7au2uHaF
+a56qBOJUGmiYDq4PMryxW2vbWEV7jsiRY1QKphiMmtu3z5p52zpVydghGDfTNhkMCIkRxs29KgRc
+rZwc7P1k6+kxM8TNb5VP8bVOovyZGpfxe2JdLhkrThnG4pmGZh4eBtO3Bd37jYWEN7LwNMESBc5n
+W8dYdFGa63KE+ZFPX1CUaXOWNF+EE/2CB2/B2jpnTbIxgjrAReNZJHzaoRHfbMTV3mlp92sKYH4b
+1CbE/w7X32PcYSZaaSovfhCnSC7jKI31hHJ7NANKNdNuPIjBJf1fNFO1I6nrbLnIzKOTWwvlawRR
+HybT5USn+vjB5KSUMjKoHO5AdyCNZLkHttw2bUvkfgG3+MxqaFsgNGin6mvAJI2LNPJ/JXWSN+E8
+d+49AxOenaNKzTsOv4qxJv16HOEGDyWgypgSh7lTpacJa8yOyFWxEXSOw9RveGg2wYl8uUVG3emr
+J1JA2FYbx2VOr5QLkivTmzypjafaAfmAaUiECwCXk1sF80qX9rov42fWr8fewABheMzQU3c5erlh
+r+ds9tdW6sXfZVe8zNa8TpDYL4gN7TqXhroMjrLfNWIGhdbYNoY+8lZJ6z7pLjkYTbsJQAYdR1b0
+gAePYSWP+JC2pUElODB2PZmXuE7uGYIw88mjDZreplT5gbqVfB15zmtSY8URxOghct6yx1v6R96b
+SJ5UQy3SzB0LH5kO9SqZb+MtjJHkWg5B1hGHofRFWfmyy12RbrKqnpe1gt6j4sDbGrXs7ty+njc0
+ZBE2dPr0FQJ1+2E2lrXV+DcunRdFJPKJ0ZDgUc5+MTxKInE+iN9k/5o7rlpWKQcmKMbB5cUi4Xkc
+jIoeEzORw6Oyx+rqx725aSuBR21xYQM6yzOuy5NE0QiRoziGEVHaLIV2TvkYvWGrLsHLGhMgmYH6
+92bJLA6CWX7hPM++FTPcIS6BhSqlinVi05AZZ9Ahe0Ft78ge5pjinV0HkHX6XYJp88mozeEb+bdm
+lo5OMiVa7WrH8lEagOlwHLRPeEfmS2PH3R1kGZypjj/Kqxq94ZQncmGnOcmfEpvRtmstbAzsOUOv
+prUJ2EJB/2eTbgNn8b4MExMb1K0CJhIO26AQ2VEl2L2NTgTsf3Pv1XYSazOP43IoqsTbOrMF5BrP
+cPnYuZlJ3YwxbEyLxFmpA38/z17/YkSTvR0M2/9J8LS/lO0c3MNrzxnJ5Mmz5HT3S0w2Y9Au192l
+aEyx6WnTPrp+7Z41LfYYNspy2hU3k44wq3Qz5y7H5nm+NXaCeqEyFMlJZSJ/t1EltlRIxw946RkL
+NkuxofUIJmxNhpXwq/GAXmZv8DwFj/RwYCpHH0U4sZt9ERneZvFuYxGvz49R6rzX9K2SMB3Aa006
++ZXFyqfJz5+fgIhxIRWNYQGyHO3P1ueTm+wmOtQaBYdWenWNZ8/ABZPzhmqc+WY2NzQyQUVJFknm
+nvXsbCR/hlAOBnvI0LRORwh/tQjUfYHodrPKawvRwpmXEGMrWR7YHUQNiMclq4Q0zyER87IFrYBl
+Nm/piGdH9TVE1rimErrZwCtZvjIIGocMKNUlYLa1z6bWOKX2nGwsrxIbWAf6hL1DH5A/u/DP7rW0
+nWVP9eLyMRmIxhMS/tMC4WQ1NPNEuCBTzwEgnC3pzx1H9OxE5NBHjwrsHfLNwLULmJj95wjU0hj4
+RMggyV6GFoHwIyT78pGoVE9p5iRfZrVQmwXOnDI9hw7L0oNoFiQ46kaehAernAJY9rEdv05z5l89
+AxfMyh2o66ylzO6pDE/vssLRRAgDbR2qSNfqf0GE/9+mjMB2hCv/W5b5w6f6rP4ZZv6fr/qbRuj/
+JSzXD4TtEng0/19kgOv85ZkSMjb+E/kHGvBfphTLoi4DLgAtGqh6lrApmPgbGmB5f0naLf6rZkP+
+O6YU1/5XHKEnTA5TAW0dFrj1wP8XHCF8ssREHKaVtpYcqFzdjqRBzYrr0lIWdUOGZxwcb8II1db0
+9KymHvWdHks//3RwpFohdy2GkgIDAH8pdcOEgKK/iIe3QIz3y1vVUJUb8cGLrEEw86xb8+Yy7ak3
+LbL5p69kf2vmhJqqrKE2Q8rbBmoU3AFpZSa6f+8asXmKdYe0C+iDMXknsEdsYt2gzeRtt5CNDGT3
+aKeWpYjgduA1wK2KibWHPSe7BuG8Bl6Zl3Sy37pgS+9tET1Psa42o33mKe+7t6bmUZlR+Tm7PQie
+Gasqb4KqS5KmcUF9YY7Hgt6CfmFQQS4Us5pvDDdkEx50KoIImuVKcb6fdeKMa1xwTBwmNeIKqG8e
+wNAzlvRzThoI13kUYdFLEthvu0FnPYSVcgk+/R7f+coqExoJimJiszkQXmVXjGEOn7ox75mHsu31
+40Lna95r91ZVZa9RLQN5AIiYXyOUrWcmSalaw6KxQJA5NVHf3kDIVakDCSLu5Fed9P4buCY2uQHD
+R45SDb915cFYovlY9icBs+QS61T+WKS5AM4B73DfFTxWwrap9Id0GuDmJRI5k4aB6CHxso8qqNun
+dJzFjFly7JzQxK/eY8h2c5dYMCL2s0EH4Tff0YUNZKfuC6FAnW7HaBn9tR6IMm5bYpQZ66qdfkHI
+bX/VU5sy2QdtSFPzAgJcric7S6IVNgTykRY9dl3I0owSxYRKrmoVuHp9Gw78YMrtdIc0C6ipgpT3
+Lmf6Mttpjj5VlNTYByLYbduilv2TB5ntE3zL9J5gXjduFKLxLm3m8i5zCjzkiY8JCovWEkErprGR
+CqTIxr60VLVm92/68outMQHQGhEyWudzWxhcfL5/FqLMsSWYy3LP6Wa4a00P2rlfex9QQRgRenpQ
+Z1HZREIdpqlzWoCIWjrqc+dG634FUI9pi8XK/2h6sNBWAxQB7ou0d6+e46cpKeZg3KKfEokXTt1t
+Ce0ETzSzKPzI3QTwuQl2nOzKTx6oUBZZraouFGxhaQzRSe3vmCmPT8TaO1RDX3QfHVR2b1MvE+F/
+Axcv31NyBmRcTj8W4VBTXTR600+/9bsI9NuthRRXkrMpTKJT2yVGbacosnCqTVEvC7sCmk793eCW
+IoEDNS4W+nxK5W8UDx+ABy03FI22AfVFjFSIvOXQUX375rjXuei/4ah3FY3U8AYb4lEOWnqck89j
+xMX5f1jycccOPaHPZZ7t8yTr6jHLiQKHXRRF30OycHAIqCn4xCnF5dgCNTMBCTIKxe8An0npgd5y
+1aCorhybpyzFiLdLSWUMeVcwq8g15KDpaeuq2tgLAzz+74Qsug8HwPRZj1n1NfTK9VYDpxaQfDPD
+EpJ8Br2G1NF45MbTTl5LauTZDdukADOzh/jHuEaxQewHZj5+yxuBpYrdoctt9z1La1qGF82v8UZ1
+7Lec6BwqNhNhtXtPapOslYspRSz93FMPp70fpVswBXNE7m6gTagLPaxZiv96KV6Jfxss5YPf/VZx
+gZDOdFIz1CV2sK6znm6IFsJBuR4bI/npA6QUW2DpcGPmdsp/gVgwutCiz70NG5lTv2nHMwnV6WYk
+DARM7BV4F+cpan08dC44tO9piILraBXgqnSn+qeohAXOamYFgFvK2zVBfHMyyfRr58DPGrtsq1MW
+PFrbMsTNVEBDWEhAv06ATRgBuEy06GdJCvQ9c8r+L3lnttw01u3xV6H6XilJW+NFd9Vny3EICQQI
+3YQblSFpzfOstzl1rvspeLHzkxzzxQ6YbsJFVx1fQeJoS1t7Wmv9h/d5lyAGqDXAuciUAZlBDxBt
+CqhN77LQQO4himB64+rWFZhmy8SJ3qC3xsrjKAz1uZepRSOSNhU0/BgTBTgPAMe9cjK+A0cK1rcK
+KT+CMpglMBIZ7QoPJPxHCDqUlIysQKpG+AYu2QrWw61uldJKNlmjF9htKjWqWHX+RwVnMQEWje8C
+B3qwySvsmSltYeqgnYNCk5O1NwjGNob0L+2ew6XjUVW/CQHiidOgMfEK1nKYdGtyJGShweCEt0Fc
+GB84XVs41zdUhEFM2JoETK1Xo/MQItk7W5dk7cU44isO53jATlAhFaZCLUNqggrvgJuC3JdB/Lyy
+SiB/wP7tkZil0d55HGjJeaS4Qz9HSa4bz6JaodoFC6F0SNEZkZPlTO1l1aQVSevanByUkX3Abi7t
+ijMvB4X6XO6igrwYNdxo7Wu4zp1lZA07lCaQLX1LxgJ2C4tTtxCypnevENuJFNjJWfLBbUHzO0Od
+IV4SJ4UXnspBRY0GLoxxphqY2S7lwSYlAu9qBDSrVK6Jgb1C7KGNjVFiFS3CN00uoL62gJPCxSCP
+yKWhMA6OZ0SO2FqFnUlwE2BiiDdoVRilo+LsUKy8OuirVYlhX/o81Xq1OZUNBeq1IkFC4XWFLWz0
+uo8Rl/H1CqldUfN93wgSTKrGHCSFJTJ/JcjeWAxNMbw1wb0153iVNs06kNmjSoBx7lkSpcDhepzT
+r1F5V+40EnkbLI2oTWepR27B1fwuWpBSJ6M91HL8sSt7cDIk4W4l37MpLA0U+yl0dma3xD2qeJEF
+hbjBpBjudoJM1U2BWS7soFqx1wWHBeRfozBNzsgJuW+wLMhbMiFq5TmYdoerThkLBaZ3BMsgIi+M
+dFSf4kOOfzELIMpX5lXVSZBLs1y458i6itSZVEzVRVBQx1gKFO3eyaTMUCORkPSAq5YaS9xLrXLp
+ln12lYaahUFXFwFJUiiPw1xGD+UtOxmHubpSzSvf1XWo7JbLiYroD2p4bsrZdR/GSOpanqFkC7WK
+QxOpnBqsYCDkondUtHDXaeoVoIySShirGK2RV7Hvtu+1tPGwjQa5dFFIvXnrigj0X6WWDJRM0yWJ
+AkIEk8ovMX1i6HSNvPLl1noXtp7McoAtM9gGf8huWgRsgduEKdv9MLJ7U3WWC2VlRoEI1mZgoqcr
+InRrLBdFKoRjRoMFBlFo6OrQEzvCyKFG7xWJBoglNmk1zoljYi3zFihIaHTRW6MCtrimIkbdQYc4
+2TmhjLQ1CUlCQ+hp/QgJuVNZ7uOm8sioslEYcIn95J1S2BCeSWfHwXlfJ4Oyjfe+6Te0bzdkaNjP
+sTUKMbnsTP8EOv/QYIeAVDcQNUI+FxYZQlvkPyo1hZcuKd0PNGUIRSPwVXUNPP5+UzopGU7xduh0
+o6hfYSSTLLPWUm60CBfNB/yB79oTTU+F9LpmyBMjgEhKOwh65LEIhhwNGifvxmxtV/GfpTDS1fFG
+pov8V41t24ihaLJssK2puE/tP08lMEzXGnRAc80c3uEjB3hF0vwLS0qrS2x44ktka0pjcbzV6YUc
+a/Xg0aBMAQjwZye1djxD5LNeZ1Wrnv3DVlCs03VlErK3ZZ0Yd//Z3NanFK8NuKB0le4oyKyulQz6
+6/FWlMlIce9h5mYgZRAHWypB3X4zWF6y8YKTIIOfn9U2JRr4ftIqk0NpWRiV/LLQmuTUL0yYdb3b
+n6JRB1YGzPXV8RuBBHL0Pg5mgQZqCC09lYIQ/rjooJrl2hTTam2SbWbvXGWQrKn5Ys+rd7L3nYH0
+6JXSCwZAJeChpmZRpd3vBWMU5gDzI3AawI+rWsRksPsq+05nP5rpB61M7+KBlRZe4NiFmU3gWB4g
+B70woEN4TXuakdJzjnfnIRGGmWfjmWXAuDEF5Bv94Iky13T9YNACpH8AwKCkxU7ARlpG6nmQieJD
+4+uj8jzLUvkD+bve6WpU8sw4S5R11CnaZR66mrlQEbBDDCSMzhTYrXcN9LAPeRYREkkc0XWH7QLS
+XcMW9Z2V6tELYSVkWlMIEVArMTvd76qwbdFqDlmpVBU5H90KqIQHeDkc76WvtoLipKGb9BO4yP1W
+qAFSvrdYenNNZXpZIjmFB6B/Z7149Np5lmlxUjnU6hjHT3fx4LV71NIGmBfACFv0BH1f1k4D8sxn
+PSSIF8cf6PGCOElhCqaybMoE41Mq6kFTBFUsyEEQOQC9vU9j1CTXqAQXp0UI4wStXwnlPoqCxxud
+3sXeEsJSb2JERx4NThgr1n6jej/AaSXXQNWqCa5Q6iaoMdGkBc2qAtdFEneBqYI4g5vqQkD7wlK7
+2jbyDALzFQzJuvr1l8cvkKYt0Ai6qhLMHw6TfqxyCUIoq5dh4KLWqNFFhD6E8wOtQFGDwjO5HyqH
+Dxg2nLPgMTqm2ran8B2jU2UKJo+38ngpph9thjysNRTSES7d78fMlJOUqDV03IyTrFN0mWdyhkIn
+GgcgVasXIgvEBTLQSFBXpZwyEwFJUswLI4o6CLAX37mjafs8fLE8tiB3yaqINO7+DbUI2xQFmBBU
+LQoNv/pifJ3qkMewGzBQa2pa+zt73uPhC6NPthXkVVUZ+d6DRYuyiia1cBam/D2ydjUaXY4pZRao
+UJP4PMytC8Ce6NEc7/nHE5RmSR+btGroinwwQWtJF7KC5onjkWWCYRaOVBMbHLDI16rGdwbTvKMe
+9KrKcqCq01qAW9HBLmAjQo2QZxE6mTkJ3AQ94mBxJb0tdNl0WmAmsCICBV/cKlP7S0Ue7ZeM/AwH
+MmLYdV3ipUGuyl3PfXDviH0/lbDIfshpPfjvb/8f/LltYUzL1IMB8sgAaXm3KQ+LDvd/dF90EOYJ
+2QHVslR2KQ0KIaeZnQWScqIhXSxvixHYIDHYdkxYLJDYa6gATBPdNmWG/67mYJ5YOjUKigST97fO
+UvpPag4C3uz+1MXE0NJh6TIyTEMWxsFM0vqmrcsAJS+jbiWwnA2R/qIZi+p2aDNsB4h+/DXkR+Do
+XqD2H2f5AA3zmk1LhbRclEoHtkZHXuG9aDCRGcKmcp0xw4kDpqA53Hpy23SO1htt7HDUN4BuTOKc
+nmK60QKehPZnzZL9eiBJGL/oUYlAs6TDOMeJiEDfuSIbO1R2JTAhgsTOFbrgkOv9UQWJ2tRo+C2D
+oZPZLYNMfYlpTXzjkmovDcOC56M1E621w74QQf4UMGE5Du271jAlfaVoQ3Q1hh1HGpno73wMSc8T
+WsUpIe2Av6lDnJmdl0o1YbPyLvjQd2FSOMJI4ktJNmA1YA1CHhDeHRYPTSvXLyjHxAJPtBroCTKH
+SO8bfaWi1dS79RvZN6WNWhQyFh0Uj0tU97sckdSqusr7nMjXbHWq3uTcvMgh0+thq2aJYZFXNpKz
+RtE2LxThxvqpHCX1dedZKM12bhdBjU/Bh8BUQCqrUmRydhVy7sZ5gswTUvRKEP45cp7tlrmug9Ex
+kGs5R7HMstdgVcJrlHbMl36LRCslYyvZAGRDHnNgoSscDofdTecF5IvYXN3oLDCS8L2KgaaFd6BZ
+uKce4SMa9Irrfyrw5WuWiuTDqE3JGNTFSmCA0iKYrhWIepHhFhuSCPF7KsE2BE2tj1FcDQovXmD+
+FkPTVEUtxBKzz+imaUb1ZedxvkdfXwOpwg3Bm4zMcTRfkC119QtX77CjWJpGh41iEuB8c1ZUMFeK
+BQimCukfm5wdeXg05NH3zUPQbpALT0k0A+3I0MrX14BZqz+i2nCzlQ5eYjU5eXorTclNzYkVG4EQ
+kSYlzncWok2oOeRt5IjCSKHcIFczXIUUzhH2CBTMIQttUri3VFW9EVE+pOwSdg4eoAOd9hLITdkt
+JVzKLdKPOIOhPFJgo97aCTw+y3RRYwGOq57ldddr50oY1/EVFkJxd83kyn4nkUktJ5fkOHvZejVS
+3yNIySVZF2TLzE5+PVnmAs9QXWVNqh2mod/qzbCGRlAqv6cBZn2QiCP0UHO5BS4Slk33ulA18QF9
+KjlwKGeENqA6q4/flyP8iXU028YM0KWRlJjtZGAvWx8QBKPyATI4D9cYh2I+408+NGbWpvl7FE2b
+S8+LMaqJtWR4PcgW9jW+DbFyiYU4rjZgPAAod5PZDU4JJOcqaQjfgu0orwtDBWwE1OXGUwVauG7b
+gjkW2mSio0x+Ol6SKfgDVIVyowCiU+F/FMMFCxfgSshNWPLYW3eeySs1mDx7QkkM70uV9lb97OmT
+UZtAlakLn0u1OfTrajYASiYvoAwcCVnU1o4vOT/hhAH2TbooB+S2UAVsm99xnEmhnvZFPkKmyPRL
+smpGdhZakw0R2WUhv6bUj5RRM+oUE6TSx4coKkwsjFBeJMGJtpv7B4ogsIWwncTwSDYSDEk0GR+k
+IJ8skYzZHikBF6gw3ifbJGW2UAqktvijm42VyKGQTWScigsgBSCoRvx5Biq/g46FRz/ZM2mSKr0C
+YAzF0yd0ubZmKycZv6bn1LQweMJ7EWiIB7zQ0WcLKOx+sIOKJmeoajaJAu2AYVTSNfmrPJlspLrZ
+UspNvei1PRtNMdsoAkVV1920kxOV5+o3pSI8kNT9bFTl+3W1zif/KrhGWFkNs60V7tgeOkCz3ZWL
+4mK8hIdN2i6cLbGQu8UeS2g1VlmocYlXiDrCMuknLy28ONBEKQjAXiXlUG782XZL6JiikpfDjYtq
+E6MqnTy6TMy6Qo5B5mVEzHpGkj2UXpizsVc59M1b12bju8iyyv4zjcHTLkhsBNfhUMENA/uCn24a
+VTHUCYaVd+r1BQxLvXXB+JUJebE1+wFSMGCrqC4gzNO8mTBw0SnWbXBeUhKepOBHkzpFn1SoCPgD
+nj4OmlpSgv4dKreUJCqoO1U7UmJvXBRv3KAiDkt95BfiJs+4eCQPq14tdLiQbuF/ymv0HZ1OBViz
+GJsGvosFyCkC+0JdFw9R1o0l8Fgq0P/8vPdvET65P6ROB7EVCad6eN3clcObu6qJ6+0Z1bvLpt/O
+YeB19mNf2nnSf/1C9xaY10N+9+svn7IGQj934AVZumdXQej3JT79cqH5do9dIN7wVM0tV5YU+UTM
+H5lLxdQadr/QxQmxDx/Oa/Nn29SDvvnW0x9/sG03Hv/O3r1vkKj8KmCHDIn9N5//4BoPn98+sRWw
+ZfKUtp0+nFwfdoMmTmx0fviO2P5+e1T/F3WDalsqN/13hsG3u0EVJxzyCRwsa/uYh91gnIAWQsaG
+AHH+kHShxX9TN+B/sr2pbaXjyGw40g3qiS1PXaCo98/5aDSQEjEFgcy/dTRMakhPHQ1CPiHrQw2D
+Dn04GXTlhFgSZWiMbebPv25NIPad0mFPnAwmNj3UiOQJkTd/9rtBs044pVOdIA8zf/7BmvA3ZsyX
+LWaJ8tHtvLkEd9XX9qBvfWG3uj7+/f3K+vz2118ehPTz96atZtv03bzpTf//bW+qzNP9wS930//h
+n98/3+OWv3pPux+eBXflpvzkD/PTDvd3ufV//s+n8u7hnodv0u6/291x7x4fvPujF403Xrapdhea
++oNUNMP9v4/36y8/dOFkM2bpwZWRPXj6lRcbf18PbZuSfeoNn97d0vfxs685aNkKg+TJXbKq8s9/
+lUGdPXu7gTuwu+C2z7XJLfupz7DOgs//s/8yVdViGXzqhS8nwK//+X/3bhqNoZ9x05cbegSCLcZW
+z27pmybe3e/UMywuk9vY0x/gSyO7i22vzqFu94Mfn0XgofcTk6quTEnyp971hLP+/NfHze5K8y2T
+DP8J8/Pqrkw3ycfm0/4rBZX9E3r7TcCrvHt2vkE+s9xvYHs6eWrHTA2sGZI0wpB5mZX13tKosvlT
+LPi5rRwOzO0B46ltTEvB5tmSIKoM0v0Xvd3Cn9wAs/bZ1QafsV2HzKNoe1h+8sXvSi/I9/qeQ9GU
+9X7qla+zT/QMyNvdpaa7Ftj7/YTV7D/JJt+fr1MI9RPm6yWvsHq2Zh8J9u97G6E9tU+ugk3z+a+9
+DuHCYveDH1+/3nzbAPLLEejHjgFvsqMCpk+8+lEeyhOvfazadPTSXzv5fYkQH58Hd3mAr/3Z/ll3
++sanmCLYb/8HAAD//w==</cx:binary>
               </cx:geoCache>
             </cx:geography>
           </cx:layoutPr>
@@ -9096,93 +9103,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Dashboard"/>
-      <sheetName val="Resultados"/>
-      <sheetName val="Queries"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1">
-        <row r="3">
-          <cell r="I3" t="str">
-            <v>país</v>
-          </cell>
-          <cell r="J3" t="str">
-            <v>estado</v>
-          </cell>
-          <cell r="K3" t="str">
-            <v>vendas (#)</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="I4" t="str">
-            <v>Brazil</v>
-          </cell>
-          <cell r="J4" t="str">
-            <v>SP</v>
-          </cell>
-          <cell r="K4">
-            <v>734</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="I5" t="str">
-            <v>Brazil</v>
-          </cell>
-          <cell r="J5" t="str">
-            <v>MG</v>
-          </cell>
-          <cell r="K5">
-            <v>142</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="I6" t="str">
-            <v>Brazil</v>
-          </cell>
-          <cell r="J6" t="str">
-            <v>SC</v>
-          </cell>
-          <cell r="K6">
-            <v>110</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="I7" t="str">
-            <v>Brazil</v>
-          </cell>
-          <cell r="J7" t="str">
-            <v>RS</v>
-          </cell>
-          <cell r="K7">
-            <v>98</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="I8" t="str">
-            <v>Brazil</v>
-          </cell>
-          <cell r="J8" t="str">
-            <v>RJ</v>
-          </cell>
-          <cell r="K8">
-            <v>66</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -9585,22 +9505,22 @@
         <v>518.58000000000004</v>
       </c>
       <c r="I4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="K4" s="1">
-        <v>66</v>
+        <v>734</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N4" s="1">
         <v>108</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q4" s="1">
         <v>10</v>
@@ -9609,7 +9529,7 @@
         <v>0</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="U4" s="1">
         <v>17</v>
@@ -9635,22 +9555,22 @@
         <v>478.99</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K5" s="1">
-        <v>98</v>
+        <v>142</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N5" s="1">
         <v>136</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q5" s="1">
         <v>10</v>
@@ -9659,7 +9579,7 @@
         <v>6</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="U5" s="1">
         <v>185</v>
@@ -9685,22 +9605,22 @@
         <v>517.84</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K6" s="1">
         <v>110</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N6" s="1">
         <v>193</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q6" s="1">
         <v>10</v>
@@ -9709,7 +9629,7 @@
         <v>5</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="U6" s="1">
         <v>188</v>
@@ -9735,22 +9655,22 @@
         <v>788.72</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K7" s="1">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N7" s="1">
         <v>237</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q7" s="1">
         <v>15</v>
@@ -9759,7 +9679,7 @@
         <v>4</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="U7" s="1">
         <v>202</v>
@@ -9785,22 +9705,22 @@
         <v>717.88</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K8" s="1">
-        <v>734</v>
+        <v>66</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N8" s="1">
         <v>248</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q8" s="1">
         <v>18</v>
@@ -9809,7 +9729,7 @@
         <v>2</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U8" s="1">
         <v>205</v>
@@ -9838,7 +9758,7 @@
         <v>3</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U9" s="1">
         <v>223</v>
@@ -9867,7 +9787,7 @@
         <v>1</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="U10" s="1">
         <v>234</v>

</xml_diff>